<commit_message>
chore: update land law Q&A datasets and add supplemental questions file
</commit_message>
<xml_diff>
--- a/emlaw_crawler/answer_dat_dai_evaluated_gpt4o.xlsx
+++ b/emlaw_crawler/answer_dat_dai_evaluated_gpt4o.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H129"/>
+  <dimension ref="A1:J120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -492,6 +492,11 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Ghi chú verify điều luật &amp; căn cứ</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Trích đúng điều luật — TRUE: 55, FALSE: 64, Tổng: 119</t>
         </is>
       </c>
     </row>
@@ -5975,440 +5980,6 @@
         </is>
       </c>
     </row>
-    <row r="121">
-      <c r="A121" s="2" t="n">
-        <v>120</v>
-      </c>
-      <c r="B121" s="2" t="inlineStr">
-        <is>
-          <t>Chào anh chị cô chú ng ạ, cho em hỏi là năm 2022 em mua lô đất có bìa hồng rồi ạ,nay em chuyển nhượng, lấy mốc lại, thiếu diện tích, lí do là lấn làn lề đường, vậy thì phải làm ntn để lấy lại diện tích bị thiếu đó ạ, hay phải làm như thế nào cho hợp lý ạ,em cảm ơn mn nhiều ạ</t>
-        </is>
-      </c>
-      <c r="C121" s="2" t="inlineStr">
-        <is>
-          <t>Kết luận: Bạn chưa thể tự “lấy lại” phần diện tích thiếu nếu phần đó thực tế nằm trong lề đường hoặc hành lang an toàn đường bộ. Trước hết cần xác định chính xác: đất bị thiếu do cơ quan đo sai/ranh đường sai, hay phần đất đó thật sự thuộc phạm vi đường công cộng; chỉ trường hợp thứ nhất mới có cơ sở yêu cầu điều chỉnh lại hồ sơ, diện tích.
-Bạn nên đề nghị đơn vị đo đạc cung cấp bản trích đo địa chính, thể hiện rõ diện tích trên sổ hồng, diện tích thực đo, mốc giới và phần bị cho là “lấn lề đường”. Đồng thời yêu cầu cơ quan quản lý đường bộ hoặc UBND xã xác nhận bằng văn bản về: chỉ giới đường đỏ, hành lang an toàn đường bộ và thời điểm cắm mốc.
-Nếu phần thiếu đúng là đất đường/hành lang đường bộ và gia đình đã lấn sau khi hành lang được công bố, cắm mốc thì không được công nhận quyền sử dụng phần đó; Nhà nước có thể thu hồi để trả lại công trình công cộng. Khoản 1 Điều 139 Luật Đất đai 2024 Các cơ quan, UBND có trách nhiệm xử lý việc lấn, chiếm hành lang an toàn công trình. Khoản 4 Điều 210 Luật Đất đai 2024 Khoản 5 Điều 210 Luật Đất đai 2024
-Nếu ranh giới đường hoặc kết quả đo không đúng, bạn nộp đơn đề nghị kiểm tra, đo đạc lại tại Văn phòng đăng ký đất đai/chi nhánh Văn phòng đăng ký đất đai nơi có đất; kèm sổ hồng, hợp đồng mua bán năm 2022, hồ sơ kỹ thuật thửa đất khi sang tên và bản trích đo mới. Không nên ký hợp đồng chuyển nhượng theo diện tích cũ trước khi làm rõ, vì dễ phát sinh tranh chấp với bên mua.
-Với người bán năm 2022: nếu họ cam kết bán theo đúng diện tích ghi trên sổ, nhưng thực tế thiếu do cung cấp thông tin sai hoặc giao thiếu đất, bạn có thể yêu cầu họ thương lượng giảm giá, hoàn tiền tương ứng hoặc bồi thường theo hợp đồng. Nếu thiếu vì phần đất vốn là hành lang đường và sổ hồng cấp có sai sót, cần ưu tiên xử lý, đính chính hồ sơ địa chính trước; không tự dựng mốc, rào hoặc sử dụng lại phần lề đường.
-[1]. Điều 139, 210, Luật 31/2024/QH15</t>
-        </is>
-      </c>
-      <c r="D121" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="E121" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="F121" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="G121" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="H121" s="2" t="inlineStr">
-        <is>
-          <t>Câu trả lời trích dẫn Điều 139 và Điều 210 của Luật Đất đai 2024 (Luật số 31/2024/QH15), hiện đang có hiệu lực. Điều 139 quy định về trách nhiệm của các cơ quan trong việc xử lý lấn, chiếm hành lang an toàn công trình. Điều 210 quy định về việc xử lý các trường hợp lấn chiếm đất công cộng. Các điều luật này liên quan đến việc xử lý phần đất bị thiếu do lấn vào lề đường hoặc hành lang an toàn đường bộ. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý cần thiết để giải quyết vấn đề của người hỏi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="2" t="n">
-        <v>121</v>
-      </c>
-      <c r="B122" s="2" t="inlineStr">
-        <is>
-          <t>Chào cả nhà,cho Em hỏi tí,em có mua lô đất năm 2022, đã đc cấp bìa hồng dien tích rõ ràng, vậy mà năm 2025 em làm sang tên,đo đạc lấy mốc thiếu diện tích so với trong bìa, lý do là lấn chiếm lề đường gt,em muốn hỏi phải làm ntn cho hợp lý ạ, thực tế thiếu 20 MV,em cảm ơn mn ạ</t>
-        </is>
-      </c>
-      <c r="C122" s="2" t="inlineStr">
-        <is>
-          <t>Kết luận: Phần thiếu 20 m² nếu thực tế thuộc lề đường/hành lang an toàn giao thông thì thường không thể sang tên hoặc công nhận quyền sử dụng cho phần đó, dù “sổ hồng” cũ có ghi diện tích lớn hơn. Bạn cần yêu cầu cơ quan đăng ký đất đai xác định rõ ranh giới pháp lý, lý do chênh lệch và xem lại trách nhiệm của bên bán nếu họ cam kết bán đủ diện tích.
-Trước hết, đề nghị Văn phòng đăng ký đất đai cung cấp hoặc lập văn bản thể hiện: sơ đồ đo đạc, mốc ranh, phần diện tích 20 m² nằm ở đâu, có đúng thuộc đất giao thông/hành lang bảo vệ đường bộ hay chỉ là sai số đo đạc. Không nên chỉ dựa vào trả lời miệng.
-Nếu 20 m² đúng là diện tích lấn, chiếm hành lang bảo vệ công trình công cộng/đường giao thông thì Nhà nước có quyền thu hồi để trả lại công trình và không cấp Giấy chứng nhận cho phần này. Chỉ khi quy hoạch đã được điều chỉnh, phần đất không còn thuộc hành lang hay chỉ giới đường giao thông và không dùng cho công trình công cộng thì mới có thể được xem xét công nhận, kèm nghĩa vụ tài chính nếu có. Điều 139 Luật Đất đai 2024
-Bạn nên kiểm tra hợp đồng mua bán năm 2022 và hợp đồng chuyển nhượng đang làm năm 2025: diện tích được cam kết là “theo Giấy chứng nhận” hay “theo hiện trạng”; có điều khoản xử lý khi thiếu diện tích không. Nếu bên bán bán theo diện tích ghi trên sổ, biết hoặc phải biết có phần đất giao thông nhưng không thông báo, bạn có thể yêu cầu họ giảm giá tương ứng, hoàn trả tiền phần 20 m², bồi thường thiệt hại thực tế; không thỏa thuận được thì khởi kiện tranh chấp hợp đồng tại Tòa án.
-Nếu kết quả cho thấy chỉ sai khác do kỹ thuật đo đạc, ranh giới sử dụng ổn định, không lấn đất công và không tranh chấp, có thể đề nghị cấp đổi/cập nhật Giấy chứng nhận theo số liệu đo đạc thực tế. Việc chênh lệch phải được cơ quan đăng ký đất đai kiểm tra hồ sơ địa chính và xác nhận cụ thể, không tự ý “cắt” diện tích bằng thông báo miệng.
-Hồ sơ bạn nên giữ gồm: sổ hồng cũ, toàn bộ hợp đồng và chứng từ thanh toán, bản vẽ đo đạc năm 2022 và 2025, biên bản cắm mốc, thông báo từ cơ quan đăng ký đất đai, ảnh hiện trạng. Trước khi ký hợp đồng sang tên hoặc nhận sổ mới ghi thiếu diện tích, nên yêu cầu ghi rõ việc thiếu 20 m² và quyền yêu cầu bên bán hoàn tiền/bồi thường để tránh bị hiểu là đã chấp nhận hiện trạng.
-[1]. Điều 139, Luật 31/2024/QH15</t>
-        </is>
-      </c>
-      <c r="D122" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="E122" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="F122" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="G122" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="H122" s="2" t="inlineStr">
-        <is>
-          <t>Câu trả lời đã trích dẫn Điều 139 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là văn bản hiện hành và có hiệu lực từ 01/08/2024. Điều luật này liên quan đến việc xử lý đất lấn chiếm hành lang bảo vệ công trình công cộng, phù hợp với tình huống người hỏi về việc thiếu diện tích do lấn chiếm lề đường giao thông. Tuy nhiên, câu trả lời chưa trích dẫn cụ thể nội dung của Điều 139, nhưng đã bao phủ phần lớn vấn đề pháp lý liên quan đến việc xử lý diện tích đất thiếu do lấn chiếm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="2" t="n">
-        <v>122</v>
-      </c>
-      <c r="B123" s="2" t="inlineStr">
-        <is>
-          <t>Nhà mình đang xảy ra tranh chấp quyền thừa kế với người ko cùng huyết thống,cụ thể chắt của ông dượng,nó bảo nó trông nom bà mình thì nó được quyền thừa kế,ngày xưa bà trông nó lúc bé rồi thì giờ nó phải trả nghĩa ,mọi người cho mình hỏi giờ nhà mình phải làm như nào ạ.</t>
-        </is>
-      </c>
-      <c r="C123" s="2" t="inlineStr">
-        <is>
-          <t>Kết luận: Việc người chắt của ông dượng có chăm nom bà bạn không tự động làm phát sinh quyền thừa kế. Người này chỉ có thể nhận tài sản của bà nếu bà để lại di chúc hợp pháp cho họ, hoặc họ là con nuôi hợp pháp/thuộc hàng thừa kế theo luật của bà.
-Nếu bà mất mà không có di chúc hợp pháp, di sản chia theo hàng thừa kế: trước hết là chồng, cha mẹ, con đẻ/con nuôi của bà; sau đó mới đến các hàng sau. “Chắt của ông dượng” không phải chắt ruột của bà nên thông thường không thuộc hàng thừa kế của bà. Người trông nom, chăm sóc cũng không được pháp luật mặc nhiên cho hưởng thừa kế. Điều 650 Bộ luật Dân sự 2015 Điều 651 Bộ luật Dân sự 2015
-Tuy nhiên, bà có quyền tự định đoạt tài sản riêng của mình bằng di chúc, kể cả cho người không có quan hệ huyết thống. Vì vậy, cần kiểm tra có di chúc hay không, di chúc lập khi bà minh mẫn, tự nguyện và đúng hình thức hay không. Điều 609 Bộ luật Dân sự 2015 Điều 630 Bộ luật Dân sự 2015
-Gia đình nên làm ngay:
-Xác định tài sản tranh chấp là tài sản riêng của bà hay tài sản chung với ông/người khác; chỉ phần thuộc sở hữu của bà mới là di sản.
-Yêu cầu người đó xuất trình di chúc hoặc giấy tờ chứng minh là con nuôi hợp pháp, người được tặng cho tài sản.
-Giữ giấy tờ đất, nhà, sổ tiết kiệm, giấy khai sinh/khai tử, giấy đăng ký kết hôn và các tài liệu thể hiện quan hệ gia đình.
-Nếu họ tự ý chiếm giữ, sang tên hoặc ngăn cản việc quản lý tài sản, các đồng thừa kế có thể yêu cầu hòa giải hoặc khởi kiện tranh chấp thừa kế tại Tòa án.
-Việc bà từng nuôi họ khi nhỏ hoặc họ hiện chăm bà là yếu tố tình cảm, không phải căn cứ tự động để nhận thừa kế. Nếu họ có chi phí chăm sóc, chữa bệnh thực tế cho bà thì có thể yêu cầu xem xét hoàn trả khoản chi hợp lý từ di sản nếu chứng minh được, nhưng điều đó khác với quyền hưởng thừa kế.</t>
-        </is>
-      </c>
-      <c r="D123" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="E123" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="F123" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="G123" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="H123" s="2" t="inlineStr">
-        <is>
-          <t>Câu trả lời đã trích dẫn Điều 650 và 651 Bộ luật Dân sự 2015 về thừa kế theo pháp luật, và Điều 609, 630 Bộ luật Dân sự 2015 về quyền lập di chúc và điều kiện di chúc hợp pháp. Các điều luật này đều còn hiệu lực và phù hợp với vấn đề thừa kế trong câu hỏi. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý liên quan đến thừa kế theo pháp luật và di chúc, cũng như các bước cần thực hiện trong trường hợp tranh chấp.</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="2" t="n">
-        <v>123</v>
-      </c>
-      <c r="B124" s="2" t="inlineStr">
-        <is>
-          <t>Cả nhà cho mình hỏi mình có sổ đỏ năm 2002 nay muốn bán một ích nhưng kiểm tra bị đo đạc ghi lộn thửa trích lục và mình đã lên DK đo đạc lại để làm sổ hồng để bán, nhưng khi bên đo đạc suống đo thì quên đem biên bản ký giáp ranh họ nói để về chỉn sửa rồi đem giấy suống ký, nhưng đến nay đã hơn tháng mà bên đo đạc họ không trả lời gì về giấy tờ đo đạc vậy mình phải làm sao để làm sổ hồng vậy</t>
-        </is>
-      </c>
-      <c r="C124" s="2" t="inlineStr">
-        <is>
-          <t>Kết luận: Bạn nên làm đơn yêu cầu Văn phòng đăng ký đất đai/Chi nhánh Văn phòng đăng ký đất đai nơi có đất trả lời bằng văn bản về tình trạng hồ sơ đo đạc và yêu cầu hoàn tất biên bản xác định ranh giới, mốc giới. Việc cán bộ đo đã hơn một tháng không phản hồi không làm mất quyền bán đất của bạn, nhưng hồ sơ đo đạc phải được hoàn thiện trước khi tách thửa/cấp đổi Giấy chứng nhận.
-Bạn thực hiện như sau:
-Đến bộ phận một cửa nơi đã nộp hồ sơ, yêu cầu cung cấp phiếu tiếp nhận hồ sơ và giấy hẹn; nếu đã có phiếu, yêu cầu tra cứu tình trạng xử lý. Nộp một đơn đề nghị giải quyết hồ sơ quá hạn, ghi rõ ngày đo thực địa, việc chưa được đưa biên bản giáp ranh để ký và yêu cầu trả lời bằng văn bản.
-Đề nghị đơn vị đo đạc lập/đưa bạn ký biên bản xác nhận ranh giới, mốc giới thửa đất. Nếu các hộ liền kề đồng ý ranh giới thì ký xác nhận; nếu có tranh chấp hoặc hộ liền kề không ký, cơ quan xử lý phải xác minh nguyên nhân, không được tự ý bỏ qua phần ranh giới đang có tranh chấp.
-Vì sổ cũ năm 2002 bị ghi sai số thửa hoặc trích lục, bạn đề nghị cơ quan đăng ký kiểm tra để thực hiện một trong hai việc:
-Đính chính nếu đây là lỗi ghi chép, in ấn, nhập dữ liệu; hoặc
-Cấp đổi Giấy chứng nhận nếu cần đo đạc lại/trích đo địa chính để thể hiện đúng thửa, diện tích, ranh giới.
-Bản đồ địa chính được chỉnh lý khi người sử dụng đất phản ánh sai khác thông tin thửa đất; Văn phòng đăng ký đất đai có trách nhiệm kiểm tra, đối chiếu và chỉnh lý hồ sơ địa chính. Điều 6 Nghị định 101/2024/NĐ-CP
-Nếu đơn vị không giải quyết hoặc không trả lời, gửi đơn khiếu nại đến Giám đốc Văn phòng đăng ký đất đai hoặc cơ quan có thẩm quyền quản lý đơn vị đó; giữ bản sao đơn, phiếu nhận và các tin nhắn/cuộc gọi liên quan. Khiếu nại lần đầu phải được giải quyết trong thời hạn luật định; ở địa bàn thông thường là không quá 30 ngày kể từ ngày thụ lý. Điều 28 Luật Khiếu nại 2011
-Bạn chưa nên ký hợp đồng chuyển nhượng “một ít đất” hoặc nhận đủ tiền cọc theo cam kết ngày công chứng khi chưa có kết quả đo, ranh giới và điều kiện tách thửa rõ ràng. Sau khi đính chính/cấp đổi xong, việc bán một phần thửa đất thường phải làm thủ tục tách thửa trước hoặc đồng thời với thủ tục chuyển nhượng; diện tích tối thiểu tách thửa còn phụ thuộc quy định của tỉnh/thành phố nơi có đất.
-[1]. Điều 6, Nghị định 101/2024/NĐ-CP
-[2]. Điều 28, Luật 02/2011/QH13</t>
-        </is>
-      </c>
-      <c r="D124" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="E124" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="F124" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="G124" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="H124" s="2" t="inlineStr">
-        <is>
-          <t>Câu trả lời đã trích dẫn Điều 6 Nghị định 101/2024/NĐ-CP về trách nhiệm của Văn phòng đăng ký đất đai trong việc chỉnh lý bản đồ địa chính khi có sai khác thông tin thửa đất, và Điều 28 Luật Khiếu nại 2011 về thời hạn giải quyết khiếu nại. Cả hai điều luật này đều còn hiệu lực và phù hợp với tình huống người hỏi. Tuy nhiên, câu trả lời chưa đề cập đến quy định cụ thể về diện tích tối thiểu tách thửa, điều này phụ thuộc vào quy định của từng địa phương.</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" s="2" t="n">
-        <v>124</v>
-      </c>
-      <c r="B125" s="2" t="inlineStr">
-        <is>
-          <t>Trước đây Ông em có mua cho Bố em 1 mảnh đất, thời điểm đó chỉ có phiếu thu tiền , chưa có sổ đỏ. Ở quê thì mọi người cũng nhiều người cũng chưa có sổ như thế. Sau này lúc Ông e mất, các cô các Bác đã ký giấy từ chối nhận quyền thừa kế và để mảnh đất đó cho Bố em. Gia đình em đã mang giấy tờ đi nộp để làm Sổ đỏ, tuy nhiên giấy tờ đã bị thất lạc, do có xáo trộn lãnh đạo địa chính lúc ấy. Bây giờ nhà em muốn làm sổ đỏ thì phải làm như thế nào ạ? giấy tờ gốc hiện tại nhà em k còn, chỉ còn bản hình ảnh thôi ạ</t>
-        </is>
-      </c>
-      <c r="C125" s="2" t="inlineStr">
-        <is>
-          <t>Kết luận: Gia đình bạn vẫn có thể xin cấp Sổ đỏ lần đầu, dù thất lạc hồ sơ gốc. Điểm quan trọng là chứng minh được quá trình sử dụng đất ổn định, không tranh chấp và làm rõ nguồn gốc: ông mua đất cho bố, sau đó những người thừa kế của ông đã từ chối nhận di sản.
-Nên làm theo các bước sau:
-Xin xác nhận và trích lục hồ sơ cũ
-Nộp đơn tại UBND xã/phường nơi có đất và cơ quan đăng ký đất đai cấp tỉnh để đề nghị:
-kiểm tra, trích lục hồ sơ địa chính, sổ mục kê, bản đồ, sổ kê khai;
-xác nhận việc gia đình đã từng nộp hồ sơ cấp Sổ đỏ;
-xác nhận thời điểm sử dụng đất, tình trạng không tranh chấp, phù hợp quy hoạch (nếu có).
-Bản ảnh phiếu thu, giấy từ chối nhận thừa kế vẫn nên nộp kèm để làm tài liệu chứng minh; gia đình cần in ra, ghi rõ đang lưu bản chụp vì bản gốc đã thất lạc.
-Làm hồ sơ cấp Sổ đỏ lần đầu cho bố bạn
-Hồ sơ thường gồm: đơn đăng ký, cấp Giấy chứng nhận; căn cước của bố; giấy tờ/bản ảnh còn lại; giấy tờ chứng minh quan hệ với ông; văn bản các cô, bác từ chối nhận thừa kế hoặc xác nhận đồng ý để đất cho bố; giấy xác nhận nguồn gốc và quá trình sử dụng đất của UBND xã/phường; trích đo địa chính nếu thửa đất chưa có bản đồ hoặc ranh giới chưa rõ.
-Đất có giấy tờ về quyền sử dụng đất thì xem xét cấp theo Điều 137 Luật Đất đai 2024. Nếu không còn giấy tờ gốc nhưng gia đình sử dụng đất ổn định, không vi phạm pháp luật đất đai, không tranh chấp, có thể được xem xét cấp theo Điều 138 Luật Đất đai 2024.
-Cẩn trọng với “giấy từ chối nhận thừa kế”
-Nếu giấy này chỉ là giấy viết tay, chưa công chứng/chứng thực hoặc lập sau khi đã hết thời hạn từ chối nhận di sản, cơ quan có thể không chấp nhận là văn bản từ chối thừa kế. Khi đó, cách an toàn là các cô, bác cùng ký văn bản thỏa thuận phân chia di sản, xác định mảnh đất thuộc về bố bạn; văn bản nên được công chứng.
-Việc từ chối nhận di sản phải lập thành văn bản và được thực hiện trước thời điểm phân chia di sản; không được nhằm trốn tránh nghĩa vụ tài sản với người khác Điều 620 Bộ luật Dân sự 2015. Người thừa kế có thể thỏa thuận phân chia di sản Điều 656 Bộ luật Dân sự 2015.
-Nếu có tranh chấp hoặc thiếu người thừa kế
-Nếu có cô/bác không ký, không liên hệ được, hoặc không thống nhất việc để đất cho bố, UBND xã/phường thường chỉ hòa giải. Trường hợp không hòa giải được, bố bạn có thể phải yêu cầu Tòa án xác định di sản và người được hưởng quyền sử dụng đất trước khi làm Sổ đỏ.
-Lưu ý thực tế: Trước khi nộp hồ sơ, nên đưa bản ảnh giấy tờ và thông tin thửa đất đến UBND xã/phường để họ kiểm tra hồ sơ lưu. Nếu gia đình đang quản lý, nộp thuế, xây nhà hoặc canh tác liên tục từ lâu, hãy chuẩn bị thêm biên lai thuế, giấy xác nhận hàng xóm, ảnh nhà/đất qua các thời kỳ để chứng minh quá trình sử dụng ổn định.
-[1]. Điều 137, 138, Luật 31/2024/QH15</t>
-        </is>
-      </c>
-      <c r="D125" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="E125" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="F125" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="G125" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="H125" s="2" t="inlineStr">
-        <is>
-          <t>Câu trả lời đã trích dẫn Điều 137 và 138 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là văn bản hiện hành và có hiệu lực từ 01/08/2024. Điều 137 quy định về cấp Giấy chứng nhận quyền sử dụng đất khi có giấy tờ về quyền sử dụng đất, và Điều 138 quy định về cấp Giấy chứng nhận trong trường hợp không có giấy tờ nhưng sử dụng đất ổn định, không tranh chấp. Các điều luật này bao phủ vấn đề cấp Sổ đỏ lần đầu trong trường hợp có và không có giấy tờ gốc, phù hợp với tình huống của người hỏi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="2" t="n">
-        <v>125</v>
-      </c>
-      <c r="B126" s="2" t="inlineStr">
-        <is>
-          <t>Sổ đỏ đất trồng cây lâu năm nhà e đang lệch diện tích với thực tế hơn 100m2
-Trong sổ hơn 800m2
-Thực tế có gần 700m2
-Thì việc mk xin xác nhận hiện trạng thửa đất có dễ ko ạ
-Và có lâu k ạ
-Đất ko có tranh chấp j cả</t>
-        </is>
-      </c>
-      <c r="C126" s="2" t="inlineStr"/>
-      <c r="D126" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="E126" s="4" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="F126" s="4" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="G126" s="4" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="H126" s="2" t="inlineStr">
-        <is>
-          <t>Câu trả lời không có nội dung, do đó không có điều luật nào được trích dẫn. Để trả lời câu hỏi này, cần trích dẫn các quy định về thủ tục xác nhận hiện trạng thửa đất theo Luật Đất đai 2024 và các nghị định hướng dẫn thi hành. Cần làm rõ quy trình, thời gian và điều kiện để thực hiện việc xác nhận hiện trạng thửa đất.</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="2" t="n">
-        <v>126</v>
-      </c>
-      <c r="B127" s="2" t="inlineStr">
-        <is>
-          <t>Các bác cho em hỏi nhà em đang làm thủ tục tách sổ, đất nhà e thỏa mãn tất cả thủ tục để tách, tuy nhiên cả khu vực chỗ em ở( cả huyện) tọa độ giữa các nhà bị hay lệch khoang 50 cm, vậy việc tách sổ có bị ảnh hưởng gì không ạ? đo thực tế đất đủ diện tích trên sổ không tranh chấp, đất nhà em sử dụng và được cấp sổ lâu năm rồi. Cảm ơn các bác.</t>
-        </is>
-      </c>
-      <c r="C127" s="2" t="inlineStr">
-        <is>
-          <t>Kết luận: Việc lệch tọa độ khoảng 50 cm không đương nhiên làm hồ sơ tách thửa bị từ chối. Tuy nhiên, cơ quan đo đạc/đăng ký đất đai sẽ phải xác định lại ranh giới thực tế; nếu lệch chỉ do bản đồ, hệ tọa độ hoặc kỹ thuật đo cũ và không làm thay đổi ranh, diện tích, không tranh chấp thì vẫn có thể tách thửa và chỉnh lý số liệu.
-Khi tách thửa, Văn phòng đăng ký đất đai thường đo vẽ hiện trạng, lập mảnh trích đo. Nếu số liệu mới thay thế tài liệu đo cũ thì ranh giới, diện tích được xác định theo tài liệu đo đạc mới đã được kiểm tra, nghiệm thu Điều 9 Thông tư 25/2024/TT-BTNMT.
-Trường hợp kích thước/diện tích có sai khác vượt sai số, cơ quan chuyên môn phải đối chiếu giấy tờ pháp lý; nếu chưa đủ dữ liệu thì đo xác định ranh giới tại thực địa. Kết quả đo phải có xác nhận của người sử dụng đất, người quản lý đất liên quan và cơ quan đăng ký đất đai Điều 17 Thông tư 26/2024/TT-BTNMT.
-Bạn nên:
-Đề nghị đơn vị đo đạc lập biên bản xác định ranh giới, mốc giới với các hộ liền kề; bảo đảm các bên ký xác nhận.
-Nộp kèm Giấy chứng nhận cũ, mảnh trích đo mới và biên bản đo đạc khi làm hồ sơ tách.
-Nếu lệch 50 cm làm lấn sang đất hàng xóm, đất công hoặc khiến một thửa sau tách không đạt kích thước/diện tích tối thiểu theo quy định địa phương, hồ sơ có thể phải xử lý xong mới tách được.
-Không tự dịch chuyển mốc ranh hay xây dựng theo tọa độ mới khi chưa có xác nhận, vì có thể phát sinh tranh chấp ranh giới.
-Do bạn chưa nêu tỉnh/thành phố, chưa thể kết luận về diện tích, kích thước tối thiểu được tách thửa tại nơi có đất. Quy định này do UBND cấp tỉnh ban hành và là điều kiện quyết định cuối cùng đối với hồ sơ tách thửa.
-[1]. Điều 9, Thông tư 25/2024/TT-BTNMT
-[2]. Điều 17, Thông tư 26/2024/TT-BTNMT</t>
-        </is>
-      </c>
-      <c r="D127" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="E127" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="F127" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="G127" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="H127" s="2" t="inlineStr">
-        <is>
-          <t>Câu trả lời đã trích dẫn Điều 9 Thông tư 25/2024/TT-BTNMT và Điều 17 Thông tư 26/2024/TT-BTNMT. Cả hai thông tư này đều còn hiệu lực và liên quan đến quy trình đo đạc, xác định ranh giới và diện tích đất khi tách thửa. Điều 9 Thông tư 25/2024/TT-BTNMT quy định về việc đo vẽ hiện trạng và lập mảnh trích đo, trong khi Điều 17 Thông tư 26/2024/TT-BTNMT quy định về việc xử lý sai khác kích thước/diện tích. Các điều luật này đã bao phủ phần lớn vấn đề về quy trình đo đạc và tách thửa, tuy nhiên, chưa đề cập cụ thể đến quy định diện tích tối thiểu tách thửa tại địa phương.</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="2" t="n">
-        <v>127</v>
-      </c>
-      <c r="B128" s="2" t="inlineStr">
-        <is>
-          <t>Mọi người cho em hỏi chút : nhà em 300m2 đất thổ cư khi bị thu hồi sẽ đc cấp tđc ntn ạ . Em cảm ơn</t>
-        </is>
-      </c>
-      <c r="C128" s="2" t="inlineStr">
-        <is>
-          <t>Kết luận: Không phải cứ bị thu hồi 300 m² đất ở là sẽ được cấp tương ứng 300 m² đất tái định cư. Việc được bố trí bao nhiêu suất, diện tích bao nhiêu và có phải nộp thêm tiền hay không phụ thuộc vào diện tích bị thu hồi, số hộ/nhân khẩu đủ điều kiện, chỗ ở khác và chính sách tái định cư của tỉnh nơi có đất.
-Nếu gia đình bị thu hồi đất ở và phải di chuyển chỗ ở, đồng thời đủ điều kiện được bồi thường về đất thì có thể được bồi thường bằng đất ở hoặc nhà ở tái định cư. Điều 111 Luật Đất đai 2024
-Suất tái định cư tối thiểu có thể là nền đất, nhà ở hoặc tiền. Nếu nhận nền đất thì diện tích không được thấp hơn diện tích tối thiểu do UBND tỉnh quy định; vì vậy mỗi tỉnh sẽ có mức khác nhau. Điều 24 Nghị định 88/2024/NĐ-CP
-Thông thường, cơ quan bồi thường sẽ lập phương án ghi rõ: diện tích đất thu hồi, tiền bồi thường đất và tài sản, số suất tái định cư, diện tích từng nền/căn, giá nền tái định cư và khoản gia đình phải nộp thêm hoặc được nhận chênh lệch. Gia đình nên kiểm tra kỹ phương án này trước khi ký.
-Bạn cho biết đất ở tỉnh/thành nào, bị thu hồi hết 300 m² hay một phần, trên đất có mấy hộ đang ở và gia đình còn nhà/đất ở nào khác không; khi đó mới xác định sát hơn khả năng được bao nhiêu suất tái định cư.
-[1]. Điều 111, Luật 31/2024/QH15
-[2]. Điều 24, Nghị định 88/2024/NĐ-CP</t>
-        </is>
-      </c>
-      <c r="D128" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="E128" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="F128" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="G128" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="H128" s="2" t="inlineStr">
-        <is>
-          <t>Câu trả lời đã trích dẫn Điều 111 của Luật Đất đai 2024 và Điều 24 của Nghị định 88/2024/NĐ-CP. Cả hai văn bản này đều còn hiệu lực và liên quan trực tiếp đến vấn đề tái định cư khi thu hồi đất. Điều 111 của Luật Đất đai 2024 quy định về bồi thường bằng đất ở hoặc nhà ở tái định cư khi thu hồi đất. Điều 24 của Nghị định 88/2024/NĐ-CP quy định về suất tái định cư tối thiểu. Câu trả lời đã bao phủ đầy đủ các khía cạnh liên quan đến việc cấp đất tái định cư khi bị thu hồi đất thổ cư.</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="2" t="n">
-        <v>128</v>
-      </c>
-      <c r="B129" s="2" t="inlineStr">
-        <is>
-          <t>mình muốn hỏi, mình mua đất thổ cư ở Thái Nguyên và có sổ đỏ nhưng sổ không có trích lục bản đồ ( hầu như cả khu đó bị như vậy và bị chồng thửa các nhà với nhau, địa chính đã đi đo lại toàn bộ khu và mình cũng đã kí giáp danh xong xuôi rồi, nhưng vẫn ko ra trích lục bản đồ cho mình lí do là ko tìm được hồ sơ cũ của người chủ đất hồi xưa mà bán lại cho người chủ mình mua sau này). Có luật sư nào nhận làm không ạ, và chi phí sang nhượng được sổ là bn ạ ?</t>
-        </is>
-      </c>
-      <c r="C129" s="2" t="inlineStr">
-        <is>
-          <t>Kết luận: Có thể thuê luật sư hoặc đơn vị đo đạc hỗ trợ, nhưng trước hết cần xác định đây không đơn thuần là “xin trích lục bản đồ”. Nếu sổ đỏ đã cấp có dấu hiệu chồng lấn thửa, cơ quan đăng ký đất đai phải kiểm tra hồ sơ, số liệu đo đạc mới và xử lý cấp đổi/chỉnh lý khi đủ căn cứ; việc “không tìm được hồ sơ cũ” không nên là lý do để từ chối bằng miệng vô thời hạn.
-Bạn nên làm đơn đề nghị trả lời bằng văn bản gửi Chi nhánh Văn phòng đăng ký đất đai nơi có đất tại Thái Nguyên, yêu cầu nêu rõ: hồ sơ nào bị thiếu, thửa đất chồng lấn với thửa nào, diện tích/rành giới theo đo đạc mới và thủ tục cụ thể cần thực hiện. Kèm sổ đỏ, hợp đồng mua bán/chuyển nhượng, giấy tờ đo đạc, biên bản ký giáp ranh và các giấy tờ chủ cũ bạn có.
-Việc đo đạc lại và ký giáp ranh là tài liệu quan trọng. Trường hợp cấp đổi do đo đạc lập bản đồ địa chính hoặc trích đo địa chính, cơ quan quản lý phải cập nhật sổ địa chính, bản đồ địa chính và sổ mục kê dựa trên sổ đã cấp cùng hồ sơ cấp đổi Điều 21 Thông tư 10/2024/TT-BTNMT.
-Nếu cơ quan tiếp nhận không giải quyết hoặc chỉ trả lời miệng, bạn yêu cầu cấp phiếu tiếp nhận hồ sơ/phiếu từ chối, trong đó ghi rõ căn cứ pháp lý và hướng xử lý. Sau đó có thể khiếu nại đến người đứng đầu cơ quan đã từ chối; không nên tự giao tiền “làm trích lục” khi chưa có hồ sơ, biên lai và nội dung công việc rõ ràng.
-Về chi phí, cần tách 3 khoản:
-Lệ phí hành chính/cấp đổi/cung cấp trích lục: do HĐND tỉnh Thái Nguyên quy định, thường không lớn.
-Đo đạc, lập trích đo hoặc chỉnh lý bản đồ: tùy diện tích, địa hình, mức độ chồng lấn và đơn vị thực hiện; đây thường là khoản đáng kể hơn.
-Thuế, phí khi sang tên: nếu bạn đã hoàn tất thủ tục chuyển nhượng và đã đứng tên sổ thì không phải “sang nhượng” lần nữa; nếu chưa sang tên thì còn có thuế thu nhập cá nhân, lệ phí trước bạ và chi phí hồ sơ theo từng trường hợp.
-Luật sư có thể nhận hỗ trợ theo hướng: rà hồ sơ, soạn đơn yêu cầu/đơn khiếu nại, làm việc cùng cơ quan đăng ký đất đai, hoặc đại diện theo ủy quyền. Khi hỏi báo giá, bạn nên yêu cầu báo giá tách riêng: phí tư vấn hồ sơ, phí đi làm việc và phí giải quyết tranh chấp (nếu có); không nên nhận cam kết “bao ra sổ”.
-Bạn cần giữ đặc biệt các giấy tờ: sổ đỏ bản gốc; hợp đồng mua bán; giấy xác nhận hoặc biên bản đo đạc; biên bản giáp ranh; thông tin/sổ đỏ của các thửa bị chồng lấn (nếu có); mọi văn bản trả lời của địa chính, UBND xã/phường và Văn phòng đăng ký đất đai.
-[1]. Điều 21, Thông tư 10/2024/TT-BTNMT</t>
-        </is>
-      </c>
-      <c r="D129" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="E129" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="F129" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="G129" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="H129" s="2" t="inlineStr">
-        <is>
-          <t>Câu trả lời trích dẫn Điều 21 của Thông tư 10/2024/TT-BTNMT, quy định về việc cập nhật sổ địa chính, bản đồ địa chính và sổ mục kê khi có sự thay đổi do đo đạc lập bản đồ địa chính hoặc trích đo địa chính. Thông tư này còn hiệu lực và phù hợp với tình huống người dùng hỏi về việc cấp đổi sổ đỏ do chồng lấn thửa đất. Điều luật này đã bao phủ phần yêu cầu về thủ tục cấp đổi sổ đỏ khi có sự chồng lấn thửa đất.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:H129"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: update evaluated dataset for answer_dat_dai with GPT-4o results
</commit_message>
<xml_diff>
--- a/emlaw_crawler/answer_dat_dai_evaluated_gpt4o.xlsx
+++ b/emlaw_crawler/answer_dat_dai_evaluated_gpt4o.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-2320" yWindow="-19320" windowWidth="27040" windowHeight="16960" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="QA_Evaluated_GPT4o" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,14 +11,14 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'QA_Evaluated_GPT4o'!$A$1:$H$129</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,7 +27,24 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Cambria"/>
+      <family val="1"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="14"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -40,12 +56,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -61,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -75,9 +91,11 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -441,19 +459,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J120"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
     <col width="90" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="4" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="48" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>STT</t>
@@ -494,13 +509,18 @@
           <t>Ghi chú verify điều luật &amp; căn cứ</t>
         </is>
       </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Phân loại</t>
+        </is>
+      </c>
       <c r="J1" t="inlineStr">
         <is>
           <t>Trích đúng điều luật — TRUE: 65, FALSE: 54, Tổng: 119</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="409.6" customHeight="1">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
@@ -547,8 +567,18 @@
           <t>Câu trả lời đã trích dẫn Điều 152 của Luật Đất đai 2024 (Luật số 31/2024/QH15), điều này còn hiệu lực và liên quan đến việc đính chính thông tin trên Giấy chứng nhận quyền sử dụng đất khi có sai sót. Ngoài ra, Điều 584 của Bộ luật Dân sự 2015 (Luật số 91/2015/QH13) cũng được trích dẫn, điều này liên quan đến trách nhiệm bồi thường thiệt hại ngoài hợp đồng, áp dụng trong trường hợp môi giới gây thiệt hại. Các điều luật này bao phủ đầy đủ các khía cạnh pháp lý của vấn đề người dùng hỏi.</t>
         </is>
       </c>
-    </row>
-    <row r="3">
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Kind 1 (Loại 1,2) — Đúng: 36/57 (63.2%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="335" customHeight="1">
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
@@ -594,8 +624,18 @@
           <t>Câu trả lời trích dẫn Điều 89 của Luật Nhà ở 2023, tuy nhiên, không có thông tin về nội dung cụ thể của điều luật này trong câu trả lời. Ngoài ra, không có thông tin nào xác nhận rằng Điều 89 của Luật Nhà ở 2023 thực sự tồn tại và có nội dung như đã nêu. Do đó, không thể xác nhận tính hiệu lực và đúng đắn của điều luật được trích dẫn. Câu trả lời đã bao phủ vấn đề về thời hạn 5 năm và các điều kiện chuyển nhượng nhà ở xã hội, nhưng không có căn cứ pháp lý rõ ràng.</t>
         </is>
       </c>
-    </row>
-    <row r="4">
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>Loại 7</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Kind 2 (Loại 3) — Đúng: 13/22 (59.1%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="409.6" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
@@ -642,8 +682,18 @@
           <t>Câu trả lời trích dẫn Điều 143 và Điều 562 Bộ luật Dân sự 2015, đây là các điều luật còn hiệu lực và liên quan đến phạm vi ủy quyền và hợp đồng ủy quyền. Tuy nhiên, câu trả lời cũng trích dẫn Điều 45 Luật Đất đai 2024, nhưng không có điều luật nào như vậy trong Luật Đất đai 2024. Do đó, trích dẫn này là sai và không tồn tại. Vì vậy, tiêu chí trích dẫn điều luật bị đánh giá là false.</t>
         </is>
       </c>
-    </row>
-    <row r="5">
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Kind 3 (Loại 4,5) — Đúng: 11/27 (40.7%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="409.6" customHeight="1">
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
@@ -691,8 +741,18 @@
           <t>Câu trả lời trích dẫn Điều 235 Luật Đất đai 2024 và Điều 28 Luật Khiếu nại 2011. Tuy nhiên, Điều 235 Luật Đất đai 2024 không tồn tại, do đó việc trích dẫn này là sai. Điều 28 Luật Khiếu nại 2011 là đúng và còn hiệu lực, liên quan đến thời hạn giải quyết khiếu nại. Câu trả lời đã bao phủ phần lớn vấn đề về thủ tục hòa giải tranh chấp đất đai và khiếu nại hành chính, nhưng việc trích dẫn sai điều luật làm ảnh hưởng đến tính chính xác của phần trích dẫn pháp lý.</t>
         </is>
       </c>
-    </row>
-    <row r="6">
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>Loại 4</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Kind 4 (Loại 6,7) — Đúng: 5/13 (38.5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="409.6" customHeight="1">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
@@ -746,8 +806,13 @@
           <t>Câu trả lời có trích dẫn Điều 152 của Luật Đất đai 2024 (Luật số 31/2024/QH15), tuy nhiên không có nội dung cụ thể của điều luật này được nêu ra trong câu trả lời. Điều này làm cho việc đánh giá tính đúng đắn và hiệu lực của điều luật trở nên khó khăn. Ngoài ra, câu trả lời không trích dẫn đầy đủ các quy định liên quan đến việc đính chính Giấy chứng nhận quyền sử dụng đất, chẳng hạn như các quy định về thủ tục và điều kiện đính chính. Do đó, tiêu chí trích dẫn điều luật được đánh giá là false.</t>
         </is>
       </c>
-    </row>
-    <row r="7">
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>Loại 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="409.6" customHeight="1">
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
@@ -798,8 +863,13 @@
           <t>Câu trả lời đã trích dẫn Điều 152 và 220 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là văn bản còn hiệu lực, để giải thích về việc thu hồi hoặc đính chính Giấy chứng nhận quyền sử dụng đất và điều kiện tách thửa. Ngoài ra, Điều 7 của Luật Khiếu nại 2011 (Luật số 02/2011/QH13) cũng được trích dẫn để hướng dẫn về quyền khiếu nại của người dân. Các điều luật này đều còn hiệu lực và phù hợp với tình huống người hỏi.</t>
         </is>
       </c>
-    </row>
-    <row r="8">
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="409.6" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
@@ -859,8 +929,13 @@
           <t>Câu trả lời trích dẫn Nghị định 101/2024/NĐ-CP và Điều 116 Luật Tố tụng hành chính 2015, Điều 7 Luật Khiếu nại 2011. Tuy nhiên, không có thông tin cụ thể về nội dung các điều luật này trong câu trả lời. Nghị định 101/2024/NĐ-CP là văn bản mới, nhưng không có thông tin chi tiết về nội dung điều luật liên quan đến thời hạn giải quyết hồ sơ cấp sổ lần đầu. Điều 116 Luật Tố tụng hành chính 2015 và Điều 7 Luật Khiếu nại 2011 là các điều luật còn hiệu lực và liên quan đến quyền khiếu nại và khởi kiện hành chính. Tuy nhiên, câu trả lời thiếu thông tin cụ thể về nội dung của các điều luật này và không trích dẫn điều luật cụ thể về thời hạn giải quyết hồ sơ cấp sổ lần đầu.</t>
         </is>
       </c>
-    </row>
-    <row r="9">
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>Loại 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="409.6" customHeight="1">
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
@@ -910,8 +985,13 @@
           <t>Câu trả lời đã trích dẫn các điều luật từ Luật Đất đai 2024 và các văn bản hướng dẫn thi hành còn hiệu lực, bao gồm: Điều 13 Thông tư 26/2024/TT-BTNMT về việc đo đạc và chỉnh lý giấy chứng nhận, Điều 6 Nghị định 101/2024/NĐ-CP về giải quyết tranh chấp đất đai, và Điều 235, 236 Luật Đất đai 2024 về thủ tục hòa giải và khởi kiện tranh chấp đất đai. Các điều luật này đã bao phủ đầy đủ các bước cần thiết để giải quyết vấn đề tranh chấp đất đai và chỉnh lý giấy chứng nhận quyền sử dụng đất.</t>
         </is>
       </c>
-    </row>
-    <row r="10">
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>Loại 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="380" customHeight="1">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
@@ -960,8 +1040,13 @@
 Các điều luật này đều còn hiệu lực và phù hợp với tình huống người hỏi. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý cần thiết để người hỏi có thể thực hiện việc chuyển nhượng đất mà không cần về Việt Nam, nếu giấy ủy quyền hợp lệ.</t>
         </is>
       </c>
-    </row>
-    <row r="11">
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="409.6" customHeight="1">
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
@@ -1010,8 +1095,13 @@
           <t>Câu trả lời đã trích dẫn Điều 11 của Nghị định 103/2024/NĐ-CP và Điều 8 của Nghị định 10/2022/NĐ-CP. Cả hai điều luật này đều còn hiệu lực và liên quan đến việc xác định nghĩa vụ tài chính khi cấp Sổ đỏ lần đầu. Điều 11 của Nghị định 103/2024/NĐ-CP quy định về tiền sử dụng đất khi cấp Sổ đỏ lần đầu cho đất sử dụng trước 15/10/1993 mà không có giấy tờ. Điều 8 của Nghị định 10/2022/NĐ-CP quy định về lệ phí trước bạ. Câu trả lời đã bao phủ đầy đủ các khoản phí và thuế liên quan đến việc cấp Sổ đỏ lần đầu.</t>
         </is>
       </c>
-    </row>
-    <row r="12">
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="409.6" customHeight="1">
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
@@ -1069,8 +1159,13 @@
 Tuy nhiên, câu trả lời đã sử dụng Luật Đất đai 2013 (Luật số 45/2013/QH13) và các nghị định cũ đã hết hiệu lực, điều này vi phạm tiêu chí về tính hiệu lực của điều luật.</t>
         </is>
       </c>
-    </row>
-    <row r="13">
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="409.6" customHeight="1">
       <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
@@ -1120,8 +1215,13 @@
           <t>Câu trả lời đã trích dẫn Điều 139 và 140 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là văn bản hiện hành và có hiệu lực từ 01/08/2024. Điều 139 quy định về việc cấp Giấy chứng nhận quyền sử dụng đất cho đất lấn, chiếm nhưng đã sử dụng ổn định trước ngày 01/7/2014. Điều 140 quy định về việc cấp Giấy chứng nhận cho đất giao không đúng thẩm quyền nhưng sử dụng ổn định, không tranh chấp và phù hợp quy hoạch. Các điều luật này bao phủ phần lớn nội dung câu hỏi về việc xin cấp sổ cho đất đã sử dụng lâu dài và có nhà ở trên đất nông nghiệp.</t>
         </is>
       </c>
-    </row>
-    <row r="14">
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="409.6" customHeight="1">
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
@@ -1169,8 +1269,13 @@
           <t>Câu trả lời đã trích dẫn Điều 13 và Điều 41 của Thông tư 10/2024/TT-BTNMT, và Điều 45 của Luật Đất đai 2024 (Luật số 31/2024/QH15). Các điều luật này đều còn hiệu lực và phù hợp với tình huống được hỏi. Điều 13 và 41 của Thông tư 10/2024/TT-BTNMT liên quan đến việc ghi nhận biến động trên Giấy chứng nhận quyền sử dụng đất khi có tặng cho, và Điều 45 của Luật Đất đai 2024 quy định về điều kiện chuyển nhượng quyền sử dụng đất. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý cần thiết cho tình huống này.</t>
         </is>
       </c>
-    </row>
-    <row r="15">
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="409.6" customHeight="1">
       <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
@@ -1219,8 +1324,13 @@
           <t>Câu trả lời đã trích dẫn Điều 138 của Luật Đất đai 2024 (Luật số 31/2024/QH15), điều này liên quan đến việc cấp Giấy chứng nhận quyền sử dụng đất trong trường hợp không có giấy tờ đầy đủ. Điều luật này còn hiệu lực và phù hợp với tình huống người dùng hỏi về khả năng tranh chấp đất đai và việc cấp Giấy chứng nhận quyền sử dụng đất. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý liên quan đến tranh chấp đất đai, quyền sử dụng đất và thủ tục cấp Giấy chứng nhận.</t>
         </is>
       </c>
-    </row>
-    <row r="16">
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>Loại 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="409.6" customHeight="1">
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
@@ -1265,8 +1375,13 @@
           <t>Câu trả lời đã trích dẫn Điều 151, 152 và 236 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là các điều luật còn hiệu lực và phù hợp với tình huống. Điều 151 quy định về việc đính chính/cấp đổi giấy chứng nhận khi có sai sót về thông tin kỹ thuật. Điều 152 quy định về thu hồi giấy chứng nhận khi cấp sai. Điều 236 quy định về thẩm quyền giải quyết tranh chấp đất đai của Tòa án. Các điều luật này đã bao phủ đầy đủ các khía cạnh của câu hỏi: từ việc đính chính, thu hồi đến giải quyết tranh chấp.</t>
         </is>
       </c>
-    </row>
-    <row r="17">
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="409.6" customHeight="1">
       <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
@@ -1316,8 +1431,13 @@
           <t>Câu trả lời đã trích dẫn Điều 133 của Luật Đất đai 2024 (Luật số 31/2024/QH15), quy định về việc đăng ký biến động đất đai khi thực hiện tặng cho quyền sử dụng đất. Điều này còn hiệu lực và phù hợp với tình huống. Ngoài ra, câu trả lời cũng trích dẫn Điều 10 của Nghị định 10/2022/NĐ-CP, liên quan đến miễn thuế thu nhập cá nhân và lệ phí trước bạ khi nhận đất tặng cho từ bà nội, điều này cũng đúng và còn hiệu lực. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý cần thiết cho việc tặng cho quyền sử dụng đất từ bà nội cho cháu.</t>
         </is>
       </c>
-    </row>
-    <row r="18">
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="409.6" customHeight="1">
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
@@ -1365,8 +1485,13 @@
           <t>Câu trả lời đã trích dẫn Điều 328 Bộ luật Dân sự 2015 về quy định đặt cọc, và Điều 114, 121 Bộ luật Tố tụng dân sự 2015 về biện pháp ngăn chặn chuyển dịch đất. Các điều luật này đều còn hiệu lực và phù hợp với tình huống người hỏi. Điều 328 đã bao phủ phần quy định về đặt cọc, còn Điều 114 và 121 đã bao phủ phần về ngăn chặn chuyển dịch đất.</t>
         </is>
       </c>
-    </row>
-    <row r="19">
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="409.6" customHeight="1">
       <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
@@ -1422,8 +1547,13 @@
           <t>Câu trả lời trích dẫn Điều 142 và 328 của Bộ luật Dân sự 2015 (Luật 91/2015/QH13). Tuy nhiên, các điều luật này vẫn còn hiệu lực và đúng với vấn đề pháp lý được hỏi. Tuy nhiên, câu trả lời không trích dẫn các điều luật mới nhất liên quan đến Luật Đất đai 2024 và các nghị định mới, do đó không đáp ứng đầy đủ yêu cầu về tính hiệu lực hiện hành của các văn bản pháp luật liên quan đến đất đai.</t>
         </is>
       </c>
-    </row>
-    <row r="20">
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="409.6" customHeight="1">
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
@@ -1493,8 +1623,13 @@
           <t>Câu trả lời trích dẫn Điều 109 Nghị định 102/2024/NĐ-CP về cưỡng chế thu hồi đất, Điều 7 Luật Khiếu nại 2011 và Điều 116 Luật Tố tụng hành chính 2015. Tuy nhiên, Nghị định 102/2024/NĐ-CP là văn bản mới và có thể chưa được phổ biến rộng rãi, cần kiểm tra lại tính chính xác của nội dung trích dẫn. Các điều luật khác được trích dẫn đúng và còn hiệu lực. Câu trả lời đã bao phủ phần lớn các khía cạnh pháp lý liên quan đến cưỡng chế và bồi thường đất, nhưng cần thêm thông tin cụ thể về điều kiện bồi thường theo Luật Đất đai 2024.</t>
         </is>
       </c>
-    </row>
-    <row r="21">
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="409.6" customHeight="1">
       <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
@@ -1554,8 +1689,13 @@
           <t>Câu trả lời đã trích dẫn Điều 138 của Luật Đất đai 2024 (Luật số 31/2024/QH15) và Điều 25 của Nghị định 101/2024/NĐ-CP, cả hai đều còn hiệu lực và phù hợp với tình huống cấp giấy chứng nhận quyền sử dụng đất và nghĩa vụ tài chính liên quan. Ngoài ra, câu trả lời cũng đề cập đến Điều 10 của Nghị định 50/2026/NĐ-CP, mặc dù chưa có hiệu lực nhưng không ảnh hưởng đến tính chính xác của câu trả lời hiện tại. Các điều luật này đã bao phủ đầy đủ các khía cạnh về điều kiện cấp giấy chứng nhận và nghĩa vụ tài chính khi công nhận đất ở.</t>
         </is>
       </c>
-    </row>
-    <row r="22">
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>Loại 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="380" customHeight="1">
       <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
@@ -1599,8 +1739,13 @@
           <t>Câu trả lời trích dẫn các điều 33, 34, 43, 59 của Luật Hôn nhân và gia đình 2014 (Luật số 52/2014/QH13) để giải thích về tài sản chung và riêng trong hôn nhân, cũng như cách thức phân chia tài sản khi ly hôn. Tuy nhiên, các điều luật này đã bị thay thế bởi Luật Hôn nhân và gia đình 2024 (Luật số 31/2024/QH15, hiệu lực từ 01/08/2024). Do đó, việc trích dẫn các điều luật này là không còn hiệu lực.</t>
         </is>
       </c>
-    </row>
-    <row r="23">
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="128" customHeight="1">
       <c r="A23" s="2" t="n">
         <v>22</v>
       </c>
@@ -1641,8 +1786,13 @@
           <t>Câu trả lời không trích dẫn điều luật nào liên quan đến việc chuyển đổi quyền sở hữu tài sản thừa kế và nghĩa vụ thuế liên quan. Điều 4 Luật Thuế thu nhập cá nhân không được trích dẫn đầy đủ và không liên quan đến việc đổi số điện thoại. Câu hỏi của người dùng liên quan đến việc chuyển đổi quyền sở hữu tài sản thừa kế (có thể là bất động sản) và nghĩa vụ thuế, nhưng câu trả lời lại nhầm lẫn với việc đổi số điện thoại, không trả lời đúng trọng tâm câu hỏi.</t>
         </is>
       </c>
-    </row>
-    <row r="24">
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="409.6" customHeight="1">
       <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
@@ -1695,8 +1845,13 @@
           <t>Câu trả lời đã trích dẫn Điều 102 và Điều 111 của Luật Đất đai 2024 (Luật số 31/2024/QH15) và Điều 14 của Nghị định 88/2024/NĐ-CP. Các điều luật này còn hiệu lực và liên quan đến việc bồi thường khi thu hồi đất, bao gồm các quy định về bồi thường nhà ở và công trình trên đất, cũng như hỗ trợ tái định cư. Điều 102 đề cập đến nguyên tắc bồi thường nhà ở khi bị tháo dỡ, và Điều 111 liên quan đến hỗ trợ tái định cư. Điều 14 của Nghị định 88/2024/NĐ-CP hướng dẫn chi tiết về việc bồi thường và hỗ trợ khi thu hồi đất. Các điều luật này đã bao phủ đầy đủ các khía cạnh cần thiết để trả lời câu hỏi của người dùng.</t>
         </is>
       </c>
-    </row>
-    <row r="25">
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="304" customHeight="1">
       <c r="A25" s="2" t="n">
         <v>24</v>
       </c>
@@ -1739,8 +1894,13 @@
           <t>Câu trả lời đã trích dẫn Điều 76 và Điều 220 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là văn bản hiện hành và có hiệu lực từ 01/08/2024. Điều 76 quy định về quyền của người sử dụng đất khi đất nằm trong quy hoạch nhưng chưa có kế hoạch sử dụng đất hàng năm hoặc chưa có thông báo thu hồi đất. Điều 220 quy định về các điều kiện để tách thửa, bao gồm việc đất có Giấy chứng nhận, không tranh chấp, không bị kê biên, còn thời hạn sử dụng, và thửa mới đáp ứng diện tích tối thiểu do UBND tỉnh quy định. Các điều luật này đã bao phủ đầy đủ vấn đề người dùng hỏi về khả năng tách thửa khi đất nằm trong quy hoạch 1/500 nhưng chưa có thông báo thu hồi.</t>
         </is>
       </c>
-    </row>
-    <row r="26">
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="335" customHeight="1">
       <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
@@ -1784,8 +1944,13 @@
           <t>Câu trả lời đã trích dẫn Điều 137 và 138 của Luật Đất đai 2024 (Luật số 31/2024/QH15) và Điều 25 của Nghị định 101/2024/NĐ-CP. Các điều luật này còn hiệu lực và phù hợp với tình huống hỏi về việc cấp sổ đỏ lần đầu và nghĩa vụ tài chính liên quan đến việc sử dụng đất trước và sau mốc 15/10/1993. Điều 137 và 138 quy định về việc cấp sổ đỏ cho đất có giấy tờ và không có giấy tờ trước mốc 1993, trong khi Điều 25 của Nghị định 101/2024/NĐ-CP hướng dẫn chi tiết về nghĩa vụ tài chính trong trường hợp không có giấy tờ. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý cần thiết cho câu hỏi.</t>
         </is>
       </c>
-    </row>
-    <row r="27">
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="409.6" customHeight="1">
       <c r="A27" s="2" t="n">
         <v>26</v>
       </c>
@@ -1839,8 +2004,13 @@
           <t>Câu trả lời trích dẫn Nghị quyết 326/2016/UBTVQH14 về án phí, lệ phí Tòa án, văn bản này vẫn còn hiệu lực và phù hợp với việc tính toán án phí trong tranh chấp dân sự. Tuy nhiên, câu trả lời không trích dẫn các điều luật liên quan đến việc chia tài sản chung, quyền khởi kiện, hoặc các quy định về thừa kế và từ chối di sản theo Bộ luật Dân sự 2015 và Bộ luật Tố tụng Dân sự 2015. Do đó, mức độ bao phủ của điều luật chưa đầy đủ.</t>
         </is>
       </c>
-    </row>
-    <row r="28">
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="409.6" customHeight="1">
       <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
@@ -1896,8 +2066,13 @@
           <t>Câu trả lời có trích dẫn Nghị định 101/2024/NĐ-CP, Điều 7 Luật Khiếu nại 2011 và Điều 116 Luật Tố tụng hành chính 2015. Tuy nhiên, không có thông tin cụ thể về nội dung các điều luật này trong câu trả lời. Ngoài ra, Luật Khiếu nại 2011 và Luật Tố tụng hành chính 2015 vẫn còn hiệu lực, nhưng cần kiểm tra tính chính xác của các điều luật cụ thể được trích dẫn. Câu trả lời chưa trích dẫn điều luật cụ thể nào từ Luật Đất đai 2024 liên quan đến thủ tục cấp đổi Giấy chứng nhận, điều này làm giảm mức độ bao phủ của câu trả lời.</t>
         </is>
       </c>
-    </row>
-    <row r="29">
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>Loại 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="409.6" customHeight="1">
       <c r="A29" s="2" t="n">
         <v>28</v>
       </c>
@@ -1948,8 +2123,13 @@
           <t>Câu trả lời có trích dẫn Điều 212, 122 và 132 của Bộ luật Dân sự 2015. Tuy nhiên, không có điều luật nào từ Luật Đất đai 2024 được trích dẫn, mặc dù tình huống liên quan đến quyền sử dụng đất và cấp Giấy chứng nhận quyền sử dụng đất. Bộ luật Dân sự 2015 vẫn còn hiệu lực, nhưng cần bổ sung các điều luật từ Luật Đất đai 2024 để đảm bảo tính đầy đủ và chính xác.</t>
         </is>
       </c>
-    </row>
-    <row r="30">
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="409.6" customHeight="1">
       <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
@@ -2001,8 +2181,13 @@
           <t>Câu trả lời đã trích dẫn Điều 45 của Luật Đất đai 2024 (Luật số 31/2024/QH15), điều này còn hiệu lực và liên quan đến quyền sử dụng đất và các quyền liên quan. Ngoài ra, câu trả lời cũng đề cập đến Điều 623 và Điều 652 của Bộ luật Dân sự 2015, liên quan đến thời hiệu thừa kế và quyền thừa kế thế vị, đều là các điều luật còn hiệu lực và phù hợp với tình huống thừa kế đất đai trong câu hỏi. Các điều luật này đã bao phủ đầy đủ các khía cạnh pháp lý cần thiết để giải quyết vấn đề tranh chấp đất đai và thừa kế trong tình huống này.</t>
         </is>
       </c>
-    </row>
-    <row r="31">
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="409.6" customHeight="1">
       <c r="A31" s="2" t="n">
         <v>30</v>
       </c>
@@ -2062,8 +2247,13 @@
           <t>Câu trả lời đã trích dẫn Điều 138 và 235 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là các điều luật còn hiệu lực và phù hợp với tình huống tranh chấp đất đai và điều kiện cấp Giấy chứng nhận quyền sử dụng đất. Điều 138 quy định về điều kiện cấp Giấy chứng nhận cho người sử dụng đất không có giấy tờ, và Điều 235 quy định về thủ tục hòa giải tranh chấp đất đai. Các điều luật này đã bao phủ đầy đủ các khía cạnh pháp lý cần thiết để giải quyết vấn đề của người hỏi.</t>
         </is>
       </c>
-    </row>
-    <row r="32">
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="409.6" customHeight="1">
       <c r="A32" s="2" t="n">
         <v>31</v>
       </c>
@@ -2111,8 +2301,13 @@
           <t>Câu trả lời có trích dẫn Điều 27 của Luật Đất đai 2024 (Luật số 31/2024/QH15), tuy nhiên, không có nội dung cụ thể của điều luật này được nêu ra trong câu trả lời. Ngoài ra, các điều luật khác như Điều 117 và Điều 462 của Bộ luật Dân sự 2015 được đề cập nhưng không được trích dẫn cụ thể. Câu trả lời đã bao phủ các khía cạnh pháp lý liên quan đến việc hủy bỏ giao dịch tặng cho đất đai, nhưng không có điều luật cụ thể nào được trích dẫn để hỗ trợ cho các luận điểm này. Do đó, tiêu chí trích dẫn điều luật bị đánh giá là false.</t>
         </is>
       </c>
-    </row>
-    <row r="33">
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="409.6" customHeight="1">
       <c r="A33" s="2" t="n">
         <v>32</v>
       </c>
@@ -2159,8 +2354,13 @@
           <t>Câu trả lời trích dẫn Điều 630, 627, 644 Bộ luật Dân sự 2015, đây là các điều luật còn hiệu lực và phù hợp với việc lập di chúc và thừa kế. Tuy nhiên, câu trả lời cũng trích dẫn Điều 59 Luật Công chứng 2024 và Điều 45 Luật Đất đai 2024, nhưng không có thông tin về nội dung cụ thể của các điều luật này trong câu trả lời, và không có thông tin về tính hiệu lực của các điều luật này. Do đó, không thể xác định tính chính xác và hiệu lực của các điều luật này trong câu trả lời.</t>
         </is>
       </c>
-    </row>
-    <row r="34">
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="409.6" customHeight="1">
       <c r="A34" s="2" t="n">
         <v>33</v>
       </c>
@@ -2209,8 +2409,13 @@
           <t>Câu trả lời đã trích dẫn Điều 116 và Điều 220 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là văn bản hiện hành và có hiệu lực từ 01/08/2024. Điều 116 quy định về việc chuyển mục đích sử dụng đất, yêu cầu phù hợp với quy hoạch và kế hoạch sử dụng đất. Điều 220 liên quan đến việc xác lập lối đi trên đất. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý cần thiết để giải quyết vấn đề của người hỏi, bao gồm cả việc xác lập lối đi và chuyển mục đích sử dụng đất.</t>
         </is>
       </c>
-    </row>
-    <row r="35">
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="380" customHeight="1">
       <c r="A35" s="2" t="n">
         <v>34</v>
       </c>
@@ -2251,8 +2456,13 @@
           <t>Câu trả lời không trích dẫn điều luật nào, do đó không thể đánh giá tính hiệu lực của điều luật. Tuy nhiên, vấn đề pháp lý chính là tranh chấp quyền sử dụng đất và quyền thừa kế, cần tham khảo Luật Đất đai 2024 và Bộ luật Dân sự 2015 để giải quyết. Câu trả lời không cung cấp thông tin pháp lý cụ thể nào để giải quyết vấn đề.</t>
         </is>
       </c>
-    </row>
-    <row r="36">
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="304" customHeight="1">
       <c r="A36" s="2" t="n">
         <v>35</v>
       </c>
@@ -2295,8 +2505,13 @@
           <t>Câu trả lời trích dẫn Điều 254 Bộ luật Dân sự 2015 về quyền yêu cầu mở lối đi qua bất động sản liền kề, điều này còn hiệu lực và phù hợp với tình huống. Tuy nhiên, Luật Thủy lợi 2017 (Luật số 08/2017/QH14) đã bị thay thế bởi Luật Thủy lợi 2024 (Luật số 32/2024/QH15, hiệu lực từ 01/08/2024), do đó trích dẫn Điều 8 Luật Thủy lợi 2017 là không còn hiệu lực. Câu trả lời đã bao phủ phần quyền yêu cầu mở lối đi và điều kiện xây dựng cầu qua kênh công cộng, nhưng cần cập nhật điều luật mới về thủy lợi.</t>
         </is>
       </c>
-    </row>
-    <row r="37">
+      <c r="I36" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="409.6" customHeight="1">
       <c r="A37" s="2" t="n">
         <v>36</v>
       </c>
@@ -2346,8 +2561,13 @@
           <t>Câu trả lời trích dẫn Điều 4 của Luật Thuế sử dụng đất phi nông nghiệp (Luật 48/2010/QH12) và Điều 18 của Thông tư 41/2017/TT-BTC, cả hai đều còn hiệu lực và liên quan đến việc xác định người nộp thuế sử dụng đất phi nông nghiệp. Tuy nhiên, Nghị định 252/2026/NĐ-CP không tồn tại, do đó trích dẫn này là sai. Câu trả lời đã bao phủ phần lớn vấn đề về nghĩa vụ thuế sau khi chuyển nhượng đất, nhưng trích dẫn sai một văn bản pháp luật.</t>
         </is>
       </c>
-    </row>
-    <row r="38">
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="409.6" customHeight="1">
       <c r="A38" s="2" t="n">
         <v>37</v>
       </c>
@@ -2393,8 +2613,13 @@
           <t>Câu trả lời trích dẫn Điều 41 Thông tư 10/2024/TT-BTNMT và Điều 35, 43 Luật Hôn nhân và gia đình 2014. Tuy nhiên, Thông tư 10/2024/TT-BTNMT không tồn tại, do đó việc trích dẫn này là sai. Điều 35 và 43 của Luật Hôn nhân và gia đình 2014 là đúng và còn hiệu lực, nhưng không đủ để bao quát toàn bộ vấn đề pháp lý liên quan đến việc chuyển nhượng quyền sử dụng đất sau khi đã sang tên cho con trai.</t>
         </is>
       </c>
-    </row>
-    <row r="39">
+      <c r="I38" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="409.6" customHeight="1">
       <c r="A39" s="2" t="n">
         <v>38</v>
       </c>
@@ -2446,8 +2671,13 @@
           <t>Câu trả lời trích dẫn Điều 137, 139, 140 của Luật Đất đai 2024 (Luật số 31/2024/QH15) và Luật Khiếu nại 2011. Tuy nhiên, không có nội dung cụ thể của các điều luật này được trích dẫn trong câu trả lời, chỉ có tham chiếu số điều luật. Điều này không đủ để đánh giá tính đúng đắn và hiệu lực của các điều luật được trích dẫn. Ngoài ra, cần lưu ý rằng việc trích dẫn điều luật cần phải cụ thể và rõ ràng hơn để người đọc có thể hiểu rõ căn cứ pháp lý.</t>
         </is>
       </c>
-    </row>
-    <row r="40">
+      <c r="I39" s="6" t="inlineStr">
+        <is>
+          <t>Loại 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="409.6" customHeight="1">
       <c r="A40" s="2" t="n">
         <v>39</v>
       </c>
@@ -2507,8 +2737,13 @@
           <t>Câu trả lời đã trích dẫn Điều 133 của Luật Đất đai 2024 (Luật số 31/2024/QH15) và Điều 19 của Nghị định 101/2024/NĐ-CP, cả hai đều còn hiệu lực. Điều 133 Luật Đất đai 2024 quy định về việc chuyển nhượng quyền sử dụng đất phải đăng ký biến động, và Điều 19 Nghị định 101/2024/NĐ-CP quy định về việc chuyển nhượng đất đang thế chấp. Các điều luật này đã bao phủ phần lớn các vấn đề liên quan đến việc chuyển nhượng quyền sử dụng đất và các rủi ro pháp lý có thể gặp phải trong tình huống này.</t>
         </is>
       </c>
-    </row>
-    <row r="41">
+      <c r="I40" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="409.6" customHeight="1">
       <c r="A41" s="2" t="n">
         <v>40</v>
       </c>
@@ -2557,8 +2792,13 @@
           <t>Câu trả lời trích dẫn Điều 220 và Khoản 3 Điều 146 của Luật Đất đai 2024 (Luật số 31/2024/QH15). Tuy nhiên, không có thông tin chi tiết về nội dung của các điều luật này trong câu trả lời, và không có xác nhận về tính hiệu lực của các điều luật này. Do đó, không thể xác định tính đúng đắn và hiệu lực của các điều luật được trích dẫn.</t>
         </is>
       </c>
-    </row>
-    <row r="42">
+      <c r="I41" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="409.6" customHeight="1">
       <c r="A42" s="2" t="n">
         <v>41</v>
       </c>
@@ -2610,8 +2850,13 @@
           <t>Câu trả lời trích dẫn Điều 45 và 138 của Luật Đất đai 2024 (Luật số 31/2024/QH15) và Điều 651 của Bộ luật Dân sự 2015 (Luật số 91/2015/QH13). Tuy nhiên, không có nội dung cụ thể của các điều luật này được trích dẫn trong câu trả lời. Điều 45 và 138 của Luật Đất đai 2024 có thể liên quan đến việc cấp Giấy chứng nhận quyền sử dụng đất và các điều kiện liên quan, nhưng không được mô tả rõ ràng trong câu trả lời. Điều 651 của Bộ luật Dân sự 2015 liên quan đến thừa kế theo pháp luật, điều này đã được mô tả đúng trong câu trả lời. Tuy nhiên, việc không trích dẫn cụ thể nội dung điều luật và chỉ nêu số điều luật mà không có giải thích chi tiết làm giảm tính chính xác và đầy đủ của phần trích dẫn điều luật.</t>
         </is>
       </c>
-    </row>
-    <row r="43">
+      <c r="I42" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="409.6" customHeight="1">
       <c r="A43" s="2" t="n">
         <v>42</v>
       </c>
@@ -2660,8 +2905,13 @@
 Các điều luật này đều còn hiệu lực và đã bao phủ đầy đủ các khía cạnh của câu hỏi: quyền của người vợ đối với tài sản thừa kế từ ông bà cho chồng và con trai.</t>
         </is>
       </c>
-    </row>
-    <row r="44">
+      <c r="I43" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="409.6" customHeight="1">
       <c r="A44" s="2" t="n">
         <v>43</v>
       </c>
@@ -2723,8 +2973,13 @@
           <t>Câu trả lời trích dẫn Điều 651 và 656 của Bộ luật Dân sự 2015, Điều 57 của Luật Công chứng 2014, và Điều 45 của Luật Đất đai 2024. Tuy nhiên, Luật Đất đai 2024 (Luật số 31/2024/QH15) đã thay thế hoàn toàn Luật Đất đai 2013, do đó việc trích dẫn Điều 45 của Luật Đất đai 2024 là đúng. Câu trả lời cũng trích dẫn Điều 10 của Nghị định 10/2022/NĐ-CP, điều này là đúng và còn hiệu lực. Tuy nhiên, cần lưu ý rằng các điều luật khác không được trích dẫn cụ thể và có thể gây nhầm lẫn về tính hiệu lực của các văn bản pháp luật khác.</t>
         </is>
       </c>
-    </row>
-    <row r="45">
+      <c r="I44" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="409.6" customHeight="1">
       <c r="A45" s="2" t="n">
         <v>44</v>
       </c>
@@ -2774,8 +3029,13 @@
           <t>Câu trả lời đã trích dẫn Điều 133 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là văn bản hiện hành và có hiệu lực từ 01/08/2024. Điều luật này liên quan đến việc đăng ký biến động đất đai khi có chuyển nhượng quyền sử dụng đất. Câu trả lời đã bao phủ đầy đủ các bước cần thiết để thực hiện thủ tục sang tên, bao gồm việc chuẩn bị hồ sơ và khả năng ủy quyền cho người khác thực hiện thủ tục tại Việt Nam. Tuy nhiên, câu trả lời không nêu rõ nội dung cụ thể của Điều 133, nhưng đã giải thích rõ ràng quy trình và các lưu ý cần thiết cho người hỏi.</t>
         </is>
       </c>
-    </row>
-    <row r="46">
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="395" customHeight="1">
       <c r="A46" s="2" t="n">
         <v>45</v>
       </c>
@@ -2823,8 +3083,13 @@
           <t>Câu trả lời trích dẫn Điều 20 của Nghị định 23/2015/NĐ-CP về chứng thực bản sao từ bản chính. Tuy nhiên, Nghị định này đã bị thay thế bởi Nghị định 101/2024/NĐ-CP, do đó, điều luật trích dẫn không còn hiệu lực. Câu trả lời đã bao phủ vấn đề về việc chứng thực bản sao khi không có bản gốc và các giải pháp làm việc với ngân hàng.</t>
         </is>
       </c>
-    </row>
-    <row r="47">
+      <c r="I46" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="409.6" customHeight="1">
       <c r="A47" s="2" t="n">
         <v>46</v>
       </c>
@@ -2888,8 +3153,13 @@
           <t>Câu trả lời đã trích dẫn Điều 45 của Luật Đất đai 2024 (Luật số 31/2024/QH15), điều này còn hiệu lực và phù hợp với vấn đề chuyển nhượng quyền sử dụng đất. Ngoài ra, câu trả lời cũng trích dẫn Điều 131 và 132 của Bộ luật Dân sự 2015 (Luật số 91/2015/QH13), các điều này cũng còn hiệu lực và liên quan đến việc tuyên bố giao dịch dân sự vô hiệu và thời hiệu khởi kiện. Các điều luật này đã bao phủ đầy đủ các khía cạnh pháp lý liên quan đến việc mua bán đất bằng vi bằng, điều kiện chuyển nhượng đất và khả năng khởi kiện để tuyên bố giao dịch vô hiệu.</t>
         </is>
       </c>
-    </row>
-    <row r="48">
+      <c r="I47" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="272" customHeight="1">
       <c r="A48" s="2" t="n">
         <v>47</v>
       </c>
@@ -2932,8 +3202,13 @@
           <t>Câu trả lời đã trích dẫn Điều 171 và Điều 220 của Luật Đất đai 2024 (Luật số 31/2024/QH15), đây là các điều luật còn hiệu lực và liên quan đến vấn đề sử dụng đất ổn định lâu dài và điều kiện tách thửa. Điều 171 quy định về đất ở của hộ gia đình, cá nhân thuộc nhóm đất sử dụng ổn định lâu dài. Điều 220 quy định về điều kiện tách thửa, bao gồm yêu cầu về diện tích tối thiểu và các điều kiện khác như không tranh chấp, có lối đi/kết nối hạ tầng phù hợp. Câu trả lời đã bao phủ đầy đủ các khía cạnh cần thiết để giải quyết vấn đề của người hỏi.</t>
         </is>
       </c>
-    </row>
-    <row r="49">
+      <c r="I48" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="409.6" customHeight="1">
       <c r="A49" s="2" t="n">
         <v>48</v>
       </c>
@@ -2994,8 +3269,13 @@
           <t>Câu trả lời đã trích dẫn các điều luật từ Luật Đất đai 2024 và Nghị định 103/2024/NĐ-CP, là các văn bản còn hiệu lực hiện hành. Điều 13 Nghị định 103/2024/NĐ-CP liên quan đến việc xử lý diện tích đất tăng thêm do sai số đo đạc. Điều 45 và 220 Luật Đất đai 2024 quy định về điều kiện tặng cho và tách thửa đất. Điều 4 Luật Thuế thu nhập cá nhân 2007 quy định về miễn thuế thu nhập cá nhân trong trường hợp tặng cho giữa bố mẹ và con. Các điều luật này đã bao phủ đầy đủ các khía cạnh của câu hỏi, bao gồm xử lý diện tích đất tăng thêm, thủ tục tặng cho và các điều kiện liên quan.</t>
         </is>
       </c>
-    </row>
-    <row r="50">
+      <c r="I49" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="409.6" customHeight="1">
       <c r="A50" s="2" t="n">
         <v>49</v>
       </c>
@@ -3053,8 +3333,13 @@
 Các điều luật này đều còn hiệu lực và phù hợp với vấn đề pháp lý được hỏi, bao gồm quyền thừa kế của con riêng và quyền lập di chúc của bố.</t>
         </is>
       </c>
-    </row>
-    <row r="51">
+      <c r="I50" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="320" customHeight="1">
       <c r="A51" s="2" t="n">
         <v>50</v>
       </c>
@@ -3098,8 +3383,13 @@
           <t>Câu trả lời trích dẫn Điều 4 của Luật Thuế sử dụng đất phi nông nghiệp 2010 và Điều 18 của Thông tư 41/2017/TT-BTC. Tuy nhiên, cả hai văn bản này đều đã hết hiệu lực và bị thay thế bởi các văn bản mới. Luật Thuế sử dụng đất phi nông nghiệp 2010 đã bị thay thế bởi các quy định mới trong Luật Đất đai 2024 và các văn bản hướng dẫn mới. Do đó, việc trích dẫn các điều luật này không còn phù hợp và không còn hiệu lực.</t>
         </is>
       </c>
-    </row>
-    <row r="52">
+      <c r="I51" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="288" customHeight="1">
       <c r="A52" s="2" t="n">
         <v>51</v>
       </c>
@@ -3142,8 +3432,13 @@
           <t>Câu trả lời trích dẫn Điều 140 của Luật Đất đai 2024 (Luật số 31/2024/QH15), điều này còn hiệu lực và phù hợp với tình huống đất giãn dân do xã bán trái thẩm quyền. Điều luật này quy định về việc công nhận đất ở trong trường hợp giao đất trái thẩm quyền, yêu cầu có nhà ở và sử dụng ổn định, không yêu cầu cụ thể về loại nhà (như nhà cấp 4). Câu trả lời đã bao phủ đầy đủ các khía cạnh của câu hỏi, bao gồm điều kiện cấp sổ đỏ và các nghĩa vụ tài chính liên quan.</t>
         </is>
       </c>
-    </row>
-    <row r="53">
+      <c r="I52" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="395" customHeight="1">
       <c r="A53" s="2" t="n">
         <v>52</v>
       </c>
@@ -3188,8 +3483,13 @@
           <t>Câu trả lời đã trích dẫn Điều 139 của Luật Đất đai 2024 và Điều 25 của Nghị định 101/2024/NĐ-CP. Cả hai văn bản này đều còn hiệu lực và liên quan đến việc cấp Giấy chứng nhận quyền sử dụng đất cho đất khai hoang và công trình xây dựng trên đất. Điều 139 Luật Đất đai 2024 quy định về điều kiện cấp Giấy chứng nhận cho đất khai hoang, trong khi Điều 25 Nghị định 101/2024/NĐ-CP hướng dẫn chi tiết về hạn mức đất ở và công nhận công trình phục vụ đời sống. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý cần thiết cho câu hỏi của người dùng.</t>
         </is>
       </c>
-    </row>
-    <row r="54">
+      <c r="I53" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="409.6" customHeight="1">
       <c r="A54" s="2" t="n">
         <v>53</v>
       </c>
@@ -3249,8 +3549,13 @@
           <t>Câu trả lời trích dẫn Điều 45 của Luật Đất đai 2024 và Điều 17 của Nghị định 320/2025/NĐ-CP, tuy nhiên, Nghị định 320/2025/NĐ-CP không tồn tại. Điều 131 của Bộ luật Dân sự 2015 được trích dẫn đúng và còn hiệu lực. Câu trả lời đã bao phủ phần lớn các vấn đề pháp lý liên quan đến tranh chấp đất đai và nghĩa vụ thuế, nhưng việc trích dẫn sai Nghị định làm giảm độ chính xác của phần trích dẫn điều luật.</t>
         </is>
       </c>
-    </row>
-    <row r="55">
+      <c r="I54" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="335" customHeight="1">
       <c r="A55" s="2" t="n">
         <v>54</v>
       </c>
@@ -3293,8 +3598,13 @@
           <t>Câu trả lời trích dẫn Điều 138 và 141 của Luật Đất đai 2024 (Luật số 31/2024/QH15), tuy nhiên không có nội dung cụ thể của các điều luật này trong câu trả lời. Ngoài ra, có đề cập đến Quyết định 17/2026/QĐ-UBND của UBND tỉnh Thanh Hóa, nhưng đây là một văn bản không tồn tại (năm 2026 chưa đến). Do đó, việc trích dẫn điều luật và văn bản không chính xác và không có căn cứ rõ ràng.</t>
         </is>
       </c>
-    </row>
-    <row r="56">
+      <c r="I55" s="6" t="inlineStr">
+        <is>
+          <t>Loại 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="409.6" customHeight="1">
       <c r="A56" s="2" t="n">
         <v>55</v>
       </c>
@@ -3347,8 +3657,13 @@
           <t>Câu trả lời đã trích dẫn Điều 137 và 220 của Luật Đất đai 2024 (Luật số 31/2024/QH15) và Điều 7 của Nghị định 101/2024/NĐ-CP. Các điều luật này đều còn hiệu lực và phù hợp với vấn đề cấp Giấy chứng nhận quyền sử dụng đất lần đầu và điều kiện tách thửa. Điều 137 quy định về giấy tờ quyền sử dụng đất và cấp Giấy chứng nhận, Điều 220 quy định về điều kiện tách thửa, và Điều 7 của Nghị định 101/2024/NĐ-CP hướng dẫn về thủ tục tách thửa. Các điều luật này đã bao phủ đầy đủ các khía cạnh của câu hỏi.</t>
         </is>
       </c>
-    </row>
-    <row r="57">
+      <c r="I56" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="409.6" customHeight="1">
       <c r="A57" s="2" t="n">
         <v>56</v>
       </c>
@@ -3395,8 +3710,13 @@
           <t>Câu trả lời đã trích dẫn Điều 235 của Luật Đất đai 2024 và Điều 105 của Nghị định 102/2024/NĐ-CP. Đây là các văn bản pháp luật hiện hành, có hiệu lực từ 01/08/2024, thay thế cho Luật Đất đai 2013 và các nghị định cũ. Điều 235 Luật Đất đai 2024 quy định về thủ tục hòa giải tranh chấp đất đai tại UBND cấp xã, là bước bắt buộc trước khi khởi kiện ra tòa. Điều 105 Nghị định 102/2024/NĐ-CP hướng dẫn chi tiết về thủ tục này. Các điều luật này đã bao phủ đầy đủ vấn đề pháp lý về tranh chấp quyền sử dụng đất và thủ tục giải quyết tranh chấp.</t>
         </is>
       </c>
-    </row>
-    <row r="58">
+      <c r="I57" s="6" t="inlineStr">
+        <is>
+          <t>Loại 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="380" customHeight="1">
       <c r="A58" s="2" t="n">
         <v>57</v>
       </c>
@@ -3440,8 +3760,13 @@
           <t>Câu trả lời trích dẫn Điều 25 của Nghị định 101/2024/NĐ-CP, là văn bản còn hiệu lực, liên quan đến việc xác định loại đất và thủ tục cấp đổi Giấy chứng nhận quyền sử dụng đất. Điều luật này bao phủ phần thủ tục và điều kiện để công nhận phần diện tích tăng thêm là đất trồng cây lâu năm. Tuy nhiên, câu trả lời chưa trích dẫn cụ thể nội dung của điều luật, nhưng đã giải thích rõ ràng về quy trình và điều kiện cần thiết.</t>
         </is>
       </c>
-    </row>
-    <row r="59">
+      <c r="I58" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="409.6" customHeight="1">
       <c r="A59" s="2" t="n">
         <v>58</v>
       </c>
@@ -3493,8 +3818,13 @@
           <t>Câu trả lời đã trích dẫn Luật Đất đai 2024 (Luật số 31/2024/QH15) và Nghị định 102/2024/NĐ-CP, cả hai đều còn hiệu lực. Luật Đất đai 2024 thay thế Luật Đất đai 2013, và Nghị định 102/2024/NĐ-CP thay thế các nghị định cũ liên quan đến thủ tục cấp Giấy chứng nhận quyền sử dụng đất. Câu trả lời đã bao phủ đầy đủ các khía cạnh về nguồn gốc đất, quá trình sử dụng đất, và yêu cầu bổ sung giấy tờ theo quy định hiện hành.</t>
         </is>
       </c>
-    </row>
-    <row r="60">
+      <c r="I59" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="160" customHeight="1">
       <c r="A60" s="2" t="n">
         <v>59</v>
       </c>
@@ -3535,8 +3865,13 @@
           <t>Câu trả lời đã trích dẫn Điều 564 Bộ luật Dân sự 2015, quy định về việc ủy quyền lại. Điều này còn hiệu lực và phù hợp với câu hỏi về việc ủy quyền lại trong giao dịch nhà đất. Điều luật này cho phép người được ủy quyền có thể ủy quyền lại nếu được sự đồng ý của người ủy quyền hoặc trong trường hợp bất khả kháng. Câu trả lời đã bao phủ đầy đủ vấn đề pháp lý liên quan đến việc ủy quyền lại.</t>
         </is>
       </c>
-    </row>
-    <row r="61">
+      <c r="I60" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="409.6" customHeight="1">
       <c r="A61" s="2" t="n">
         <v>60</v>
       </c>
@@ -3581,8 +3916,13 @@
           <t>Câu trả lời đã trích dẫn Điều 8 Thông tư 10/2024/TT-BTNMT và Điều 25 Nghị định 101/2024/NĐ-CP. Cả hai văn bản này đều còn hiệu lực và liên quan đến việc cấp Giấy chứng nhận quyền sử dụng đất lần đầu. Điều 8 Thông tư 10/2024/TT-BTNMT quy định về việc xác định loại đất theo hiện trạng sử dụng tại thời điểm đăng ký. Điều 25 Nghị định 101/2024/NĐ-CP quy định về việc cấp giấy chứng nhận cho đất có nguồn gốc lấn, chiếm nhưng hiện đang sử dụng vào mục đích nông nghiệp. Các điều luật này đã bao phủ phần lớn câu hỏi về điều kiện cấp giấy chứng nhận quyền sử dụng đất lần đầu cho đất nông nghiệp.</t>
         </is>
       </c>
-    </row>
-    <row r="62">
+      <c r="I61" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="409.6" customHeight="1">
       <c r="A62" s="2" t="n">
         <v>61</v>
       </c>
@@ -3628,8 +3968,13 @@
           <t>Câu trả lời đã trích dẫn Điều 3 và Điều 10 của Nghị định 123/2024/NĐ-CP, và Điều 139 của Luật Đất đai 2024 (Luật số 31/2024/QH15). Các điều luật này còn hiệu lực và phù hợp với tình huống hỏi về việc cấp Giấy chứng nhận quyền sử dụng đất lần đầu và xử phạt hành vi chuyển mục đích sử dụng đất. Điều 3 và 10 của Nghị định 123/2024/NĐ-CP đề cập đến thời hiệu xử phạt và mức phạt cho hành vi chuyển mục đích sử dụng đất. Điều 139 của Luật Đất đai 2024 liên quan đến việc công nhận quyền sử dụng đất trong trường hợp sử dụng đất không đúng mục đích nhưng ổn định và phù hợp quy hoạch. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý cần thiết cho câu hỏi.</t>
         </is>
       </c>
-    </row>
-    <row r="63">
+      <c r="I62" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="409.6" customHeight="1">
       <c r="A63" s="2" t="n">
         <v>62</v>
       </c>
@@ -3682,8 +4027,13 @@
           <t>Câu trả lời trích dẫn Điều 133 Luật Đất đai 2024 và Điều 41 Thông tư 10/2024/TT-BTNMT, nhưng không có nội dung cụ thể của các điều này trong câu trả lời. Ngoài ra, câu trả lời cũng trích dẫn Điều 43 và 33 của Luật Hôn nhân và gia đình 2014, nhưng không có nội dung cụ thể của các điều này trong câu trả lời. Điều 27 và 45 Luật Đất đai 2024 được trích dẫn nhưng không có nội dung cụ thể. Cần lưu ý rằng các điều luật này cần được trích dẫn cụ thể và đúng nội dung để đảm bảo tính chính xác và hiệu lực của câu trả lời.</t>
         </is>
       </c>
-    </row>
-    <row r="64">
+      <c r="I63" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="409.6" customHeight="1">
       <c r="A64" s="2" t="n">
         <v>63</v>
       </c>
@@ -3735,8 +4085,13 @@
           <t>Câu trả lời đã trích dẫn Điều 116 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là văn bản hiện hành và có hiệu lực. Điều luật này liên quan đến việc chuyển mục đích sử dụng đất từ đất nông nghiệp sang đất ở, phù hợp với câu hỏi của người dùng. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý liên quan đến việc chuyển mục đích sử dụng đất, bao gồm cả quy hoạch sử dụng đất và các điều kiện cụ thể tại địa phương.</t>
         </is>
       </c>
-    </row>
-    <row r="65">
+      <c r="I64" s="6" t="inlineStr">
+        <is>
+          <t>Loại 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="409.6" customHeight="1">
       <c r="A65" s="2" t="n">
         <v>64</v>
       </c>
@@ -3792,8 +4147,13 @@
           <t>Câu trả lời đã trích dẫn Điều 25 của Nghị định 101/2024/NĐ-CP và Điều 5, 9 của Nghị định 88/2024/NĐ-CP. Các điều luật này đều còn hiệu lực và liên quan đến việc công nhận đất ở và bồi thường khi thu hồi đất. Điều 25 của Nghị định 101/2024/NĐ-CP liên quan đến việc xác định diện tích đất ở khi có nhà xây dựng trước 01/7/2014. Điều 5 và 9 của Nghị định 88/2024/NĐ-CP liên quan đến bồi thường đất khi thu hồi. Các điều luật này đã bao phủ phần lớn câu hỏi về việc công nhận đất ở và bồi thường khi có quy hoạch, tuy nhiên, cần thêm thông tin cụ thể từ cơ quan chức năng để xác định chính xác trường hợp của người hỏi.</t>
         </is>
       </c>
-    </row>
-    <row r="66">
+      <c r="I65" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="395" customHeight="1">
       <c r="A66" s="2" t="n">
         <v>65</v>
       </c>
@@ -3838,8 +4198,13 @@
           <t>Câu trả lời trích dẫn Điều 6 của Luật Xử lý vi phạm hành chính 2012 (Luật số 15/2012/QH13) để giải thích về thời hiệu xử phạt vi phạm hành chính, điều này là đúng và còn hiệu lực. Tuy nhiên, câu trả lời không trích dẫn điều luật cụ thể từ Luật Đất đai 2024 hoặc các nghị định mới liên quan đến việc chuyển đổi mục đích sử dụng đất, mà chỉ đề cập đến Nghị định 123/2024/NĐ-CP mà không giải thích rõ nội dung điều luật này. Do đó, tiêu chí trích dẫn điều luật bị đánh giá là false vì thiếu sự bao phủ đầy đủ và chính xác của các điều luật liên quan đến vấn đề chuyển đổi mục đích sử dụng đất.</t>
         </is>
       </c>
-    </row>
-    <row r="67">
+      <c r="I66" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="409.6" customHeight="1">
       <c r="A67" s="2" t="n">
         <v>66</v>
       </c>
@@ -3892,8 +4257,13 @@
           <t>Câu trả lời có đề cập đến Điều 45 của Luật Đất đai 2024 (Luật số 31/2024/QH15), tuy nhiên không có nội dung cụ thể nào từ điều luật này được trích dẫn. Điều này làm cho việc đánh giá tính đúng đắn và hiệu lực của điều luật không thể thực hiện được. Ngoài ra, không có điều luật nào khác được trích dẫn để hỗ trợ cho các luận điểm trong câu trả lời. Do đó, tiêu chí trích dẫn điều luật bị đánh giá là false.</t>
         </is>
       </c>
-    </row>
-    <row r="68">
+      <c r="I67" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="409.6" customHeight="1">
       <c r="A68" s="2" t="n">
         <v>67</v>
       </c>
@@ -3941,8 +4311,13 @@
           <t>Câu trả lời trích dẫn Khoản 2 Điều 89 Luật Xây dựng 2014 (Luật số 50/2014/QH13) để giải thích về việc sửa chữa nhà mà không cần giấy phép xây dựng. Tuy nhiên, Luật Xây dựng 2014 đã bị thay thế bởi Luật Xây dựng 2020 (Luật số 62/2020/QH14), có hiệu lực từ 01/01/2021. Do đó, việc trích dẫn Luật Xây dựng 2014 là không còn hiệu lực. Câu trả lời đã bao phủ phần giải thích về việc sửa chữa nhà trong tình huống đất đang tranh chấp, nhưng sử dụng điều luật hết hiệu lực.</t>
         </is>
       </c>
-    </row>
-    <row r="69">
+      <c r="I68" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="409.6" customHeight="1">
       <c r="A69" s="2" t="n">
         <v>68</v>
       </c>
@@ -3998,8 +4373,13 @@
           <t>Câu trả lời đã trích dẫn Điều 152 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là văn bản hiện hành và có hiệu lực từ 01/08/2024. Điều luật này liên quan đến việc thu hồi Giấy chứng nhận quyền sử dụng đất trong trường hợp cấp sai đối tượng, không đủ điều kiện cấp hoặc không đúng nguồn gốc. Điều luật này bao phủ phần yêu cầu hủy hoặc thu hồi Giấy chứng nhận đã cấp trái pháp luật. Tuy nhiên, câu trả lời chưa trích dẫn cụ thể các điều luật liên quan đến quy trình khởi kiện hoặc tố giác tại cơ quan công an, nhưng đã hướng dẫn chi tiết các bước cần thực hiện trong tình huống này.</t>
         </is>
       </c>
-    </row>
-    <row r="70">
+      <c r="I69" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="409.6" customHeight="1">
       <c r="A70" s="2" t="n">
         <v>69</v>
       </c>
@@ -4050,8 +4430,13 @@
           <t>Câu trả lời đã trích dẫn Điều 235 và 236 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là văn bản hiện hành và có hiệu lực từ 01/08/2024. Điều 235 quy định về thủ tục hòa giải tranh chấp đất đai tại UBND cấp xã, là bước bắt buộc trước khi khởi kiện tại Tòa án. Điều 236 quy định về thẩm quyền giải quyết tranh chấp đất đai khi có Giấy chứng nhận quyền sử dụng đất. Các điều luật này bao phủ đầy đủ vấn đề pháp lý liên quan đến tranh chấp đất đai và thủ tục giải quyết tranh chấp.</t>
         </is>
       </c>
-    </row>
-    <row r="71">
+      <c r="I70" s="6" t="inlineStr">
+        <is>
+          <t>Loại 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="395" customHeight="1">
       <c r="A71" s="2" t="n">
         <v>70</v>
       </c>
@@ -4097,8 +4482,13 @@
           <t>Câu trả lời đã trích dẫn các điều luật từ Bộ luật Dân sự 2015, bao gồm Điều 351 về vi phạm nghĩa vụ dân sự, Điều 418 về thỏa thuận phạt vi phạm và Điều 328 về trách nhiệm trả lại cọc. Các điều luật này đều còn hiệu lực và phù hợp với tình huống tranh chấp hợp đồng đặt cọc và chuyển mục đích sử dụng đất. Tuy nhiên, câu trả lời chưa đề cập đến các quy định cụ thể về chuyển mục đích sử dụng đất theo Luật Đất đai 2024, nhưng điều này không ảnh hưởng lớn đến việc giải quyết tranh chấp hợp đồng dân sự.</t>
         </is>
       </c>
-    </row>
-    <row r="72">
+      <c r="I71" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="409.6" customHeight="1">
       <c r="A72" s="2" t="n">
         <v>71</v>
       </c>
@@ -4158,8 +4548,13 @@
           <t>Câu trả lời trích dẫn Điều 138 Luật Đất đai 2024 và Điều 7 Luật Khiếu nại 2011. Tuy nhiên, không có nội dung cụ thể của các điều luật này được trích dẫn trong câu trả lời. Điều 138 Luật Đất đai 2024 có thể liên quan đến việc cấp Giấy chứng nhận quyền sử dụng đất, nhưng không có nội dung cụ thể nào được đưa ra để chứng minh điều này. Điều 7 Luật Khiếu nại 2011 liên quan đến quyền khiếu nại, nhưng cũng không có nội dung cụ thể nào được trích dẫn. Do đó, tiêu chí trích dẫn điều luật bị đánh giá là false do thiếu nội dung cụ thể và không có căn cứ rõ ràng từ các điều luật được trích dẫn.</t>
         </is>
       </c>
-    </row>
-    <row r="73">
+      <c r="I72" s="6" t="inlineStr">
+        <is>
+          <t>Loại 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="380" customHeight="1">
       <c r="A73" s="2" t="n">
         <v>72</v>
       </c>
@@ -4203,8 +4598,13 @@
           <t>Câu trả lời đã trích dẫn các điều luật từ Luật Đất đai 2024 (Luật số 31/2024/QH15), bao gồm Điều 76 về quyền sử dụng đất khi có quy hoạch nhưng chưa có kế hoạch sử dụng đất hằng năm, Điều 95 về điều kiện bồi thường khi thu hồi đất, và Điều 111 về bồi thường tái định cư. Các điều luật này đều còn hiệu lực và phù hợp với tình huống người hỏi. Câu trả lời đã bao phủ đầy đủ các khía cạnh liên quan đến việc bồi thường khi đất nằm trong quy hoạch và điều kiện để được bồi thường hoặc tái định cư.</t>
         </is>
       </c>
-    </row>
-    <row r="74">
+      <c r="I73" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="409.6" customHeight="1">
       <c r="A74" s="2" t="n">
         <v>73</v>
       </c>
@@ -4259,8 +4659,13 @@
           <t>Câu trả lời có trích dẫn Điều 138 của Luật Đất đai 2024 (Luật số 31/2024/QH15), tuy nhiên không có nội dung cụ thể của điều luật này được nêu ra trong câu trả lời. Điều này làm cho việc đánh giá tính đúng đắn và hiệu lực của điều luật trở nên khó khăn. Ngoài ra, câu trả lời không trích dẫn các điều luật cụ thể liên quan đến việc cấp Giấy chứng nhận quyền sử dụng đất trong trường hợp không có giấy tờ hợp lệ, điều này có thể làm giảm mức độ bao phủ của câu trả lời đối với vấn đề pháp lý được hỏi.</t>
         </is>
       </c>
-    </row>
-    <row r="75">
+      <c r="I74" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="409.6" customHeight="1">
       <c r="A75" s="2" t="n">
         <v>74</v>
       </c>
@@ -4317,8 +4722,13 @@
 Các điều luật trích dẫn đã bao phủ đầy đủ các khía cạnh cần thiết để giải quyết vấn đề của người hỏi, bao gồm xác định ranh giới đất, quyền lối đi, thủ tục tặng cho và giải quyết tranh chấp.</t>
         </is>
       </c>
-    </row>
-    <row r="76">
+      <c r="I75" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="409.6" customHeight="1">
       <c r="A76" s="2" t="n">
         <v>75</v>
       </c>
@@ -4364,8 +4774,13 @@
           <t>Câu trả lời đã trích dẫn Điều 141 của Luật Đất đai 2024 (Luật số 31/2024/QH15) và Điều 10 của Nghị quyết 254/2025/QH15. Điều 141 cho phép xác định lại diện tích đất ở đối với thửa đất có vườn, ao/đất thổ cư đã được cấp giấy chứng nhận trước ngày 01/7/2004 khi người sử dụng đất có nhu cầu, nếu có giấy tờ về quyền sử dụng đất theo luật định. Điều này còn hiệu lực và phù hợp với tình huống của người hỏi. Điều 10 của Nghị quyết 254/2025/QH15 liên quan đến chính sách thu tiền sử dụng đất trong một số trường hợp, cũng còn hiệu lực và có liên quan đến việc chuyển mục đích sử dụng đất. Cả hai điều luật đã bao phủ đầy đủ vấn đề pháp lý mà người hỏi quan tâm.</t>
         </is>
       </c>
-    </row>
-    <row r="77">
+      <c r="I76" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="409.6" customHeight="1">
       <c r="A77" s="2" t="n">
         <v>76</v>
       </c>
@@ -4422,8 +4837,13 @@
           <t>Câu trả lời đã trích dẫn Điều 137 của Luật Đất đai 2024, điều này liên quan đến việc cấp Giấy chứng nhận quyền sử dụng đất cho các trường hợp có giấy tờ về quyền sử dụng đất từ chế độ cũ, như Bằng khoán điền thổ. Điều này còn hiệu lực và phù hợp với tình huống. Ngoài ra, Điều 651 Bộ luật Dân sự 2015 cũng được trích dẫn đúng để giải thích về quyền thừa kế, điều này cũng còn hiệu lực và phù hợp với tình huống thừa kế đất đai. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý cần thiết cho việc cấp sổ đỏ và thừa kế.</t>
         </is>
       </c>
-    </row>
-    <row r="78">
+      <c r="I77" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="288" customHeight="1">
       <c r="A78" s="2" t="n">
         <v>77</v>
       </c>
@@ -4467,8 +4887,13 @@
           <t>Câu trả lời trích dẫn Điều 35 của Luật Hôn nhân và gia đình 2014, điều này còn hiệu lực và đúng với việc xác định quyền sở hữu tài sản chung của vợ chồng. Tuy nhiên, trích dẫn Điều 27 của Luật Đất đai 2024 là không chính xác vì không có điều luật nào như vậy trong Luật Đất đai 2024. Do đó, tiêu chí trích dẫn điều luật bị đánh giá là false.</t>
         </is>
       </c>
-    </row>
-    <row r="79">
+      <c r="I78" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="409.6" customHeight="1">
       <c r="A79" s="2" t="n">
         <v>78</v>
       </c>
@@ -4517,8 +4942,13 @@
           <t>Câu trả lời trích dẫn Điều 27 và 45 của Luật Đất đai 2024 (Luật số 31/2024/QH15). Tuy nhiên, không có thông tin chi tiết về nội dung của các điều luật này trong câu trả lời, và không có xác nhận về tính hiệu lực của các điều luật này. Ngoài ra, không có điều luật cụ thể nào được trích dẫn để giải quyết vấn đề về đất chung nhiều chủ hoặc việc chuyển đổi mục đích sử dụng đất. Do đó, tiêu chí trích dẫn điều luật bị đánh giá là không đạt.</t>
         </is>
       </c>
-    </row>
-    <row r="80">
+      <c r="I79" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="272" customHeight="1">
       <c r="A80" s="2" t="n">
         <v>79</v>
       </c>
@@ -4561,8 +4991,13 @@
           <t>Câu trả lời đã trích dẫn Điều 116 và Điều 121 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là văn bản hiện hành và có hiệu lực từ 01/08/2024. Điều 116 quy định về chuyển mục đích sử dụng đất, và Điều 121 quy định về quy hoạch, kế hoạch sử dụng đất. Các điều luật này phù hợp với tình huống người dùng hỏi về việc xác định vị trí đất thổ cư và chuyển mục đích sử dụng đất. Tuy nhiên, câu trả lời chưa trích dẫn cụ thể nội dung của các điều luật này, nhưng đã bao phủ được phần lớn vấn đề pháp lý liên quan đến việc xác định vị trí đất thổ cư và chuyển mục đích sử dụng đất.</t>
         </is>
       </c>
-    </row>
-    <row r="81">
+      <c r="I80" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="208" customHeight="1">
       <c r="A81" s="2" t="n">
         <v>80</v>
       </c>
@@ -4604,8 +5039,13 @@
           <t>Câu trả lời trích dẫn Điều 152 của Luật Đất đai 2024 (Luật số 31/2024/QH15), điều này còn hiệu lực và phù hợp với tình huống đính chính Giấy chứng nhận quyền sử dụng đất do sai sót trong đo đạc. Điều luật này bao phủ phần yêu cầu đính chính sổ đỏ khi có sai sót nhỏ trong đo đạc, tuy nhiên không đi sâu vào chi tiết quy trình cụ thể, nhưng đã nêu rõ các bước cần thiết như nộp hồ sơ và đo đạc lại.</t>
         </is>
       </c>
-    </row>
-    <row r="82">
+      <c r="I81" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="256" customHeight="1">
       <c r="A82" s="2" t="n">
         <v>81</v>
       </c>
@@ -4647,8 +5087,13 @@
           <t>Câu trả lời đã trích dẫn các điều luật từ Bộ luật Dân sự 2015, bao gồm Điều 58, 59, 60, 609 và 651. Các điều luật này đều còn hiệu lực và liên quan đến vấn đề giám hộ, quản lý tài sản của người mất năng lực hành vi dân sự, và quy định về thừa kế. Điều 58, 59, 60 quy định về quyền và nghĩa vụ của người giám hộ, cấm người giám hộ thực hiện giao dịch với chính mình. Điều 609 và 651 quy định về thừa kế, chỉ ra rằng việc chia thừa kế chỉ thực hiện sau khi người để lại di sản qua đời. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý liên quan đến việc chuyển nhượng quyền sử dụng đất trong trường hợp này.</t>
         </is>
       </c>
-    </row>
-    <row r="83">
+      <c r="I82" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="409.6" customHeight="1">
       <c r="A83" s="2" t="n">
         <v>82</v>
       </c>
@@ -4695,8 +5140,13 @@
           <t>Câu trả lời đã trích dẫn Điều 13 của Thông tư 26/2024/TT-BTNMT và Điều 220 của Luật Đất đai 2024 (Luật số 31/2024/QH15), cả hai đều còn hiệu lực và liên quan đến vấn đề đo đạc, xác định ranh giới đất và điều kiện tách thửa. Điều 13 Thông tư 26/2024/TT-BTNMT hướng dẫn về việc đo đạc, xác định ranh giới đất và cần có sự thỏa thuận của các bên liên quan. Điều 220 Luật Đất đai 2024 quy định về điều kiện tách thửa, bao gồm việc đất không có tranh chấp và đáp ứng các điều kiện về diện tích tối thiểu theo quy định của địa phương. Các điều luật này đã bao phủ đầy đủ vấn đề người dùng hỏi về việc xử lý chồng ranh và điều kiện tách thửa.</t>
         </is>
       </c>
-    </row>
-    <row r="84">
+      <c r="I83" s="6" t="inlineStr">
+        <is>
+          <t>Loại 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="409.6" customHeight="1">
       <c r="A84" s="2" t="n">
         <v>83</v>
       </c>
@@ -4744,8 +5194,13 @@
           <t>Câu trả lời có trích dẫn Điều 140 của Luật Đất đai 2024 (Luật số 31/2024/QH15), tuy nhiên không có nội dung cụ thể của điều luật này được nêu ra trong câu trả lời. Điều này làm cho việc đánh giá tính đúng đắn và hiệu lực của điều luật không thể thực hiện được. Ngoài ra, câu trả lời đã bao phủ các vấn đề liên quan đến việc cấp sổ đỏ từ giấy tờ viết tay, điều kiện cấp sổ, và các yếu tố cần kiểm tra như quy hoạch, tranh chấp, nhưng không có điều luật cụ thể nào được trích dẫn để hỗ trợ các luận điểm này.</t>
         </is>
       </c>
-    </row>
-    <row r="85">
+      <c r="I84" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="409.6" customHeight="1">
       <c r="A85" s="2" t="n">
         <v>84</v>
       </c>
@@ -4793,8 +5248,13 @@
           <t>Câu trả lời đã trích dẫn Điều 220 của Luật Đất đai 2024 (Luật số 31/2024/QH15), điều này còn hiệu lực và liên quan đến việc tách thửa đất. Điều luật này quy định về điều kiện tách thửa, bao gồm diện tích tối thiểu do UBND tỉnh quy định. Câu trả lời đã bao phủ đầy đủ các khía cạnh cần thiết để giải quyết vấn đề tách thửa đất nuôi trồng thủy sản, bao gồm điều kiện diện tích tối thiểu, các phương án xử lý khi không đủ điều kiện tách thửa, và các yếu tố pháp lý liên quan khác.</t>
         </is>
       </c>
-    </row>
-    <row r="86">
+      <c r="I85" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="409.6" customHeight="1">
       <c r="A86" s="2" t="n">
         <v>85</v>
       </c>
@@ -4843,8 +5303,13 @@
           <t>Câu trả lời trích dẫn Điều 138 của Luật Đất đai 2024 (Luật số 31/2024/QH15), điều này liên quan đến việc cấp Giấy chứng nhận quyền sử dụng đất cho người đang sử dụng đất không có giấy tờ. Điều luật này còn hiệu lực và phù hợp với tình huống người dùng hỏi về việc xin cấp sổ đỏ cho đất đã có nhà ở nhưng hiện tại nhà đã sập. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý cần thiết để giải quyết vấn đề của người dùng.</t>
         </is>
       </c>
-    </row>
-    <row r="87">
+      <c r="I86" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="256" customHeight="1">
       <c r="A87" s="2" t="n">
         <v>86</v>
       </c>
@@ -4887,8 +5352,13 @@
           <t>Câu trả lời trích dẫn Điều 45 của Luật Đất đai 2024 (Luật số 31/2024/QH15), điều này còn hiệu lực và đúng với tình huống. Điều luật này quy định về các điều kiện để thực hiện giao dịch chuyển nhượng quyền sử dụng đất, bao gồm việc đất không tranh chấp, không bị kê biên, còn thời hạn sử dụng, và đã hoàn thành nghĩa vụ tài chính. Câu trả lời đã bao phủ đầy đủ các điều kiện cần thiết để chuyển nhượng đất trong trường hợp đất nằm trong quy hoạch nhưng chưa có thông báo thu hồi.</t>
         </is>
       </c>
-    </row>
-    <row r="88">
+      <c r="I87" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="409.6" customHeight="1">
       <c r="A88" s="2" t="n">
         <v>87</v>
       </c>
@@ -4941,8 +5411,13 @@
 Các điều luật trích dẫn đã bao phủ đầy đủ các khía cạnh pháp lý cần thiết cho việc tặng cho quyền sử dụng đất cho con chưa thành niên, bao gồm cả thủ tục và miễn thuế.</t>
         </is>
       </c>
-    </row>
-    <row r="89">
+      <c r="I88" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="380" customHeight="1">
       <c r="A89" s="2" t="n">
         <v>88</v>
       </c>
@@ -4986,8 +5461,13 @@
           <t>Câu trả lời đã trích dẫn Điều 220 của Luật Đất đai 2024 (Luật số 31/2024/QH15), quy định về điều kiện tách thửa, bao gồm việc đất phải có Giấy chứng nhận, không tranh chấp, không bị kê biên, và thửa đất sau tách phải đạt diện tích tối thiểu do UBND tỉnh quy định. Điều luật này còn hiệu lực và phù hợp với vấn đề tách thửa mà người dùng hỏi. Tuy nhiên, câu trả lời cũng lưu ý rằng cần kiểm tra quyết định tách thửa của UBND tỉnh nơi có đất để biết rõ diện tích tối thiểu và điều kiện cụ thể tại địa phương, điều này chưa được bao phủ bởi điều luật trích dẫn.</t>
         </is>
       </c>
-    </row>
-    <row r="90">
+      <c r="I89" s="6" t="inlineStr">
+        <is>
+          <t>Loại 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="409.6" customHeight="1">
       <c r="A90" s="2" t="n">
         <v>89</v>
       </c>
@@ -5041,8 +5521,13 @@
           <t>Câu trả lời trích dẫn Điều 45 của Luật Đất đai 2024 và Điều 328 của Bộ luật Dân sự 2015. Tuy nhiên, không có nội dung cụ thể nào từ Điều 45 của Luật Đất đai 2024 được trích dẫn hoặc giải thích rõ ràng trong câu trả lời. Điều 328 của Bộ luật Dân sự 2015 liên quan đến quy định về đặt cọc, nhưng không có nội dung cụ thể nào từ điều này được trích dẫn hoặc giải thích rõ ràng trong câu trả lời. Do đó, mặc dù các điều luật được đề cập có thể tồn tại và còn hiệu lực, nhưng việc trích dẫn không rõ ràng và không đầy đủ nội dung cụ thể từ các điều luật này khiến tiêu chí trích dẫn điều luật bị đánh giá là không đạt.</t>
         </is>
       </c>
-    </row>
-    <row r="91">
+      <c r="I90" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="409.6" customHeight="1">
       <c r="A91" s="2" t="n">
         <v>90</v>
       </c>
@@ -5089,8 +5574,13 @@
           <t>Câu trả lời trích dẫn Điều 24 Luật Hộ tịch 2014 và Điều 24 Nghị định 123/2015/NĐ-CP. Tuy nhiên, cả hai văn bản này đều đã hết hiệu lực và bị thay thế bởi các văn bản mới. Luật Hộ tịch 2014 đã bị thay thế bởi Luật Hộ tịch 2024, và Nghị định 123/2015/NĐ-CP đã bị thay thế bởi các nghị định mới. Do đó, việc trích dẫn này không còn hiệu lực hiện hành.</t>
         </is>
       </c>
-    </row>
-    <row r="92">
+      <c r="I91" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="409.6" customHeight="1">
       <c r="A92" s="2" t="n">
         <v>91</v>
       </c>
@@ -5142,8 +5632,13 @@
           <t>Câu trả lời có trích dẫn Điều 220 của Luật Đất đai 2024, tuy nhiên không có nội dung cụ thể của điều luật này để xác định tính chính xác và hiệu lực. Ngoài ra, câu trả lời cũng đề cập đến Điều 7 của Luật Khiếu nại 2011, điều này là đúng và còn hiệu lực. Tuy nhiên, không có trích dẫn cụ thể từ Luật Đất đai 2024 để xác định rõ ràng việc tách thửa có bị cấm hay không dựa trên nguồn gốc đất. Cần có thêm thông tin chi tiết về quy định của Luật Đất đai 2024 và các văn bản hướng dẫn liên quan để đánh giá đầy đủ.</t>
         </is>
       </c>
-    </row>
-    <row r="93">
+      <c r="I92" s="6" t="inlineStr">
+        <is>
+          <t>Loại 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="256" customHeight="1">
       <c r="A93" s="2" t="n">
         <v>92</v>
       </c>
@@ -5186,8 +5681,13 @@
           <t>Câu trả lời đã trích dẫn Điều 116 và 121 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là văn bản hiện hành và có hiệu lực. Điều 116 quy định về điều kiện chuyển mục đích sử dụng đất, và Điều 121 quy định về thủ tục chuyển mục đích sử dụng đất. Cả hai điều này đều liên quan và cần thiết để giải quyết vấn đề người dùng hỏi về việc chuyển đổi mục đích sử dụng đất từ đất nông nghiệp sang đất ở. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý cần thiết cho tình huống này.</t>
         </is>
       </c>
-    </row>
-    <row r="94">
+      <c r="I93" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="409.6" customHeight="1">
       <c r="A94" s="2" t="n">
         <v>93</v>
       </c>
@@ -5236,8 +5736,13 @@
           <t>Câu trả lời trích dẫn Luật Đất đai 2024 (Luật số 31/2024/QH15) và Điều 11 Nghị quyết 254/2025/QH15. Tuy nhiên, Nghị quyết 254/2025/QH15 không tồn tại, do đó việc trích dẫn này là sai. Luật Đất đai 2024 là văn bản còn hiệu lực và phù hợp với tình huống, nhưng không có điều luật cụ thể nào được trích dẫn từ văn bản này để giải quyết vấn đề của người hỏi. Do đó, tiêu chí trích dẫn điều luật bị đánh giá là false.</t>
         </is>
       </c>
-    </row>
-    <row r="95">
+      <c r="I94" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="409.6" customHeight="1">
       <c r="A95" s="2" t="n">
         <v>94</v>
       </c>
@@ -5283,8 +5788,13 @@
           <t>Câu trả lời đã trích dẫn Điều 47 Nghị định 102/2024/NĐ-CP, quy định về việc giao đất nhỏ hẹp xen kẹt cho người sử dụng đất liền kề. Nghị định này còn hiệu lực và phù hợp với tình huống hỏi về việc mua phần đất nhỏ hẹp không thuộc về ai để gộp vào sổ đỏ. Điều luật đã bao phủ phần chính của câu hỏi về thủ tục và điều kiện để có thể hợp thửa phần đất này.</t>
         </is>
       </c>
-    </row>
-    <row r="96">
+      <c r="I95" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="409.6" customHeight="1">
       <c r="A96" s="2" t="n">
         <v>95</v>
       </c>
@@ -5331,8 +5841,13 @@
           <t>Câu trả lời trích dẫn Điều 254 Bộ luật Dân sự 2015 về quyền lối đi qua, điều này còn hiệu lực và phù hợp với vấn đề lối đi chung. Tuy nhiên, câu trả lời trích dẫn Điều 27 Luật Đất đai 2024, nhưng không có nội dung cụ thể của điều này trong câu trả lời, và không có thông tin về việc điều này có liên quan trực tiếp đến việc hiến đất làm đường. Ngoài ra, không có điều luật cụ thể nào từ Luật Đất đai 2024 được trích dẫn để giải thích về việc hiến đất làm đường. Do đó, tiêu chí trích dẫn điều luật bị đánh giá là false.</t>
         </is>
       </c>
-    </row>
-    <row r="97">
+      <c r="I96" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="409.6" customHeight="1">
       <c r="A97" s="2" t="n">
         <v>96</v>
       </c>
@@ -5383,8 +5898,13 @@
           <t>Câu trả lời trích dẫn Điều 33 và 35 của Luật Hôn nhân và gia đình 2014, và Điều 68 của Bộ luật Dân sự 2015, đều còn hiệu lực và đúng với tình huống về tài sản chung và biệt tích. Tuy nhiên, câu trả lời trích dẫn Điều 135 của Luật Đất đai 2024, nhưng không có nội dung cụ thể của điều luật này trong câu trả lời, và không rõ ràng về tính hiệu lực của điều luật này trong bối cảnh câu hỏi. Do đó, tiêu chí trích dẫn điều luật bị đánh giá là false.</t>
         </is>
       </c>
-    </row>
-    <row r="98">
+      <c r="I97" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="409.6" customHeight="1">
       <c r="A98" s="2" t="n">
         <v>97</v>
       </c>
@@ -5432,8 +5952,13 @@
           <t>Câu trả lời đã trích dẫn Điều 3 của Luật Thuế sử dụng đất phi nông nghiệp (Luật số 48/2010/QH12) và Điều 220 của Luật Đất đai 2024 (Luật số 31/2024/QH15). Cả hai điều luật này đều còn hiệu lực và phù hợp với tình huống: Điều 3 Luật Thuế sử dụng đất phi nông nghiệp quy định về nghĩa vụ nộp thuế của người sử dụng đất, và Điều 220 Luật Đất đai 2024 quy định về điều kiện tách thửa. Các điều luật này đã bao phủ đầy đủ vấn đề về nghĩa vụ thuế và thủ tục tách thửa, sang tên.</t>
         </is>
       </c>
-    </row>
-    <row r="99">
+      <c r="I98" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="409.6" customHeight="1">
       <c r="A99" s="2" t="n">
         <v>98</v>
       </c>
@@ -5483,8 +6008,13 @@
           <t>Câu trả lời đã trích dẫn Điều 91 và Điều 96 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là văn bản hiện hành và có hiệu lực từ 01/08/2024. Điều 91 quy định về nguyên tắc bồi thường khi Nhà nước thu hồi đất, trong đó có việc bồi thường bằng tiền hoặc đất khác nếu có nhu cầu và điều kiện. Điều 96 quy định về các khoản bồi thường và hỗ trợ khác như cây trồng, vật nuôi, hỗ trợ ổn định đời sống và chuyển đổi nghề. Các điều luật này đã bao phủ đầy đủ các khía cạnh liên quan đến bồi thường đất nông nghiệp khi bị thu hồi, bao gồm cả việc xác định giá đất và các khoản hỗ trợ bổ sung.</t>
         </is>
       </c>
-    </row>
-    <row r="100">
+      <c r="I99" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="409.6" customHeight="1">
       <c r="A100" s="2" t="n">
         <v>99</v>
       </c>
@@ -5536,8 +6066,13 @@
           <t>Câu trả lời có trích dẫn Điều 27 và Điều 45 của Luật Đất đai 2024, tuy nhiên không có nội dung cụ thể của các điều luật này trong câu trả lời. Ngoài ra, Điều 225 Bộ luật Dân sự 2015 được trích dẫn đúng và còn hiệu lực, nhưng không có nội dung cụ thể được nêu ra. Câu trả lời đã bao phủ phần lớn vấn đề pháp lý liên quan đến quyền sử dụng đất và việc xây dựng trái phép, nhưng không có điều luật cụ thể nào được trích dẫn để giải thích rõ ràng về quyền và nghĩa vụ của các bên trong tình huống này.</t>
         </is>
       </c>
-    </row>
-    <row r="101">
+      <c r="I100" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="409.6" customHeight="1">
       <c r="A101" s="2" t="n">
         <v>100</v>
       </c>
@@ -5592,8 +6127,13 @@
           <t>Câu trả lời đã trích dẫn Điều 138 của Luật Đất đai 2024 và Điều 11 của Nghị định 103/2024/NĐ-CP. Cả hai văn bản này đều còn hiệu lực và phù hợp với tình huống cấp sổ đỏ lần đầu cho đất sử dụng trước năm 1980. Điều 138 Luật Đất đai 2024 quy định về điều kiện cấp sổ đỏ cho đất không có giấy tờ nhưng sử dụng ổn định, không tranh chấp. Điều 11 Nghị định 103/2024/NĐ-CP quy định về mức thu tiền sử dụng đất khi công nhận đất ở trong hạn mức và vượt hạn mức. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý liên quan đến việc cấp sổ đỏ và nghĩa vụ tài chính.</t>
         </is>
       </c>
-    </row>
-    <row r="102">
+      <c r="I101" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="395" customHeight="1">
       <c r="A102" s="2" t="n">
         <v>101</v>
       </c>
@@ -5645,8 +6185,13 @@
           <t>Câu trả lời trích dẫn Điều 220 của Luật Đất đai 2024 (Luật số 31/2024/QH15), tuy nhiên không có nội dung cụ thể của điều luật này trong câu trả lời. Điều này làm cho việc xác định tính đúng đắn và hiệu lực của điều luật không thể thực hiện được. Câu trả lời đã bao phủ phần lớn các yếu tố cần thiết để tách thửa, nhưng không có điều luật cụ thể nào được trích dẫn để hỗ trợ cho các yêu cầu về diện tích tối thiểu, kích thước cạnh tối thiểu, và các yêu cầu khác liên quan đến quy hoạch và hạ tầng.</t>
         </is>
       </c>
-    </row>
-    <row r="103">
+      <c r="I102" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="409.6" customHeight="1">
       <c r="A103" s="2" t="n">
         <v>102</v>
       </c>
@@ -5692,8 +6237,13 @@
           <t>Câu trả lời đã trích dẫn Điều 121 và 133 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là văn bản hiện hành, để giải thích về việc chuyển mục đích sử dụng đất và thủ tục thừa kế quyền sử dụng đất. Điều 121 quy định về việc chuyển mục đích sử dụng đất, trong đó có việc chuyển từ đất nông nghiệp sang đất ở, cần phải xin phép cơ quan có thẩm quyền. Điều 133 quy định về thủ tục thừa kế quyền sử dụng đất, không yêu cầu bắt buộc phải chuyển mục đích sử dụng đất trước khi thực hiện thừa kế. Câu trả lời cũng đề cập đến chi phí chuyển đổi mục đích sử dụng đất theo Nghị quyết 254/2025/QH15, mặc dù nghị quyết này chưa có hiệu lực nhưng không ảnh hưởng đến tính đúng đắn của câu trả lời trong bối cảnh hiện tại.</t>
         </is>
       </c>
-    </row>
-    <row r="104">
+      <c r="I103" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="304" customHeight="1">
       <c r="A104" s="2" t="n">
         <v>103</v>
       </c>
@@ -5740,8 +6290,13 @@
           <t>Câu trả lời trích dẫn Điều 43 và 44 của Luật Hôn nhân và gia đình 2014 (Luật số 52/2014/QH13), quy định về tài sản riêng của vợ, chồng. Tuy nhiên, các điều luật này vẫn còn hiệu lực và đúng với tình huống hỏi về tài sản riêng trong hôn nhân. Tuy nhiên, câu trả lời không trích dẫn điều luật nào từ Luật Đất đai 2024 hoặc các nghị định mới liên quan đến việc chuyển nhượng hoặc thế chấp quyền sử dụng đất, do đó không đáp ứng đầy đủ tiêu chí trích dẫn điều luật.</t>
         </is>
       </c>
-    </row>
-    <row r="105">
+      <c r="I104" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="409.6" customHeight="1">
       <c r="A105" s="2" t="n">
         <v>104</v>
       </c>
@@ -5790,8 +6345,13 @@
           <t>Câu trả lời đã trích dẫn các điều luật từ Luật Đất đai 2024 (Điều 95, 102, 108, 111) và Nghị định 88/2024/NĐ-CP, đều là các văn bản còn hiệu lực và phù hợp với tình huống thu hồi đất và tái định cư. Điều 95 đề cập đến điều kiện cấp Giấy chứng nhận quyền sử dụng đất, Điều 102 và 108 liên quan đến bồi thường khi thu hồi đất, và Điều 111 về tái định cư. Các điều luật này đã bao phủ đầy đủ các khía cạnh của câu hỏi về bồi thường và tái định cư khi thu hồi đất.</t>
         </is>
       </c>
-    </row>
-    <row r="106">
+      <c r="I105" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="409.6" customHeight="1">
       <c r="A106" s="2" t="n">
         <v>105</v>
       </c>
@@ -5840,8 +6400,13 @@
           <t>Câu trả lời đã trích dẫn các điều luật từ Nghị định 88/2024/NĐ-CP và Luật Đất đai 2024, là các văn bản còn hiệu lực hiện hành. Điều 11 Nghị định 88/2024/NĐ-CP quy định về việc bồi thường bằng đất ở hoặc nhà ở tái định cư khi diện tích đất còn lại nhỏ hơn diện tích tối thiểu và không còn đất ở khác. Điều 160 Luật Đất đai 2024 quy định về giá bồi thường đất. Các điều luật này đã bao phủ vấn đề về điều kiện tái định cư và giá bồi thường, nhưng chưa đề cập chi tiết về quy định diện tích tối thiểu cụ thể của từng địa phương.</t>
         </is>
       </c>
-    </row>
-    <row r="107">
+      <c r="I106" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="409.6" customHeight="1">
       <c r="A107" s="2" t="n">
         <v>106</v>
       </c>
@@ -5891,8 +6456,13 @@
           <t>Câu trả lời có trích dẫn Điều 3 và Điều 9 của Luật Đất đai 2024 (Luật số 31/2024/QH15). Tuy nhiên, không có nội dung cụ thể nào từ các điều luật này được nêu ra trong câu trả lời, và việc trích dẫn này không rõ ràng, không cung cấp thông tin cụ thể về nội dung điều luật liên quan đến vấn đề cấp sổ đỏ và việc xây dựng nhà trên đất. Do đó, tiêu chí trích dẫn điều luật bị đánh giá là không đạt yêu cầu.</t>
         </is>
       </c>
-    </row>
-    <row r="108">
+      <c r="I107" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="409.6" customHeight="1">
       <c r="A108" s="2" t="n">
         <v>107</v>
       </c>
@@ -5941,8 +6511,13 @@
           <t>Câu trả lời có trích dẫn Điều 459 Bộ luật Dân sự 2015 và Điều 45 Luật Đất đai 2024. Tuy nhiên, Điều 459 Bộ luật Dân sự 2015 không được trích dẫn cụ thể nội dung và không rõ ràng về việc áp dụng trong tình huống này. Điều 45 Luật Đất đai 2024 được trích dẫn nhưng không có nội dung cụ thể và không rõ ràng về việc áp dụng trong tình huống này. Cần lưu ý rằng việc trích dẫn điều luật cần cụ thể và rõ ràng hơn để người đọc hiểu rõ hơn về quyền và nghĩa vụ của mình trong tình huống này.</t>
         </is>
       </c>
-    </row>
-    <row r="109">
+      <c r="I108" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="380" customHeight="1">
       <c r="A109" s="2" t="n">
         <v>108</v>
       </c>
@@ -5987,8 +6562,13 @@
           <t>Câu trả lời đã trích dẫn Điều 152 của Luật Đất đai 2024 (Luật số 31/2024/QH15), điều này còn hiệu lực và phù hợp với việc chỉnh lý giấy chứng nhận quyền sử dụng đất khi có sai sót. Ngoài ra, câu trả lời cũng đề cập đến Điều 7 của Luật Khiếu nại 2011 (Luật số 02/2011/QH13), điều này cũng còn hiệu lực và liên quan đến quyền khiếu nại của người dân khi không đồng ý với quyết định hành chính. Các điều luật này đã bao phủ đầy đủ vấn đề pháp lý mà người dùng gặp phải.</t>
         </is>
       </c>
-    </row>
-    <row r="110">
+      <c r="I109" s="6" t="inlineStr">
+        <is>
+          <t>Loại 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="409.6" customHeight="1">
       <c r="A110" s="2" t="n">
         <v>109</v>
       </c>
@@ -6042,8 +6622,13 @@
           <t>Câu trả lời trích dẫn Điều 61 Nghị định 253/2026/NĐ-CP, Điều 67 Thông tư 89/2026/TT-BTC và Điều 45 Luật Đất đai 2024. Tuy nhiên, các văn bản này không tồn tại hoặc không có hiệu lực tại thời điểm hiện tại (2023). Do đó, tiêu chí trích dẫn điều luật bị đánh giá là false. Câu trả lời đã bao phủ các bước thực hiện thủ tục tặng cho đất giữa các thành viên gia đình và các lưu ý về thuế, lệ phí, nhưng không có điều luật cụ thể nào được trích dẫn đúng và còn hiệu lực để hỗ trợ cho các bước này.</t>
         </is>
       </c>
-    </row>
-    <row r="111">
+      <c r="I110" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="409.6" customHeight="1">
       <c r="A111" s="2" t="n">
         <v>110</v>
       </c>
@@ -6095,8 +6680,13 @@
           <t>Câu trả lời đã trích dẫn Điều 81 và Điều 237 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là văn bản hiện hành và có hiệu lực từ 01/08/2024. Điều 81 quy định về việc thu hồi đất do vi phạm pháp luật về đất đai, trong đó có trường hợp dự án chậm tiến độ. Điều 237 quy định về quyền khiếu nại quyết định thu hồi đất. Các điều luật này đã bao phủ vấn đề pháp lý về thu hồi đất do vi phạm tiến độ và quyền khiếu nại của gia đình đối với quyết định thu hồi.</t>
         </is>
       </c>
-    </row>
-    <row r="112">
+      <c r="I111" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="409.6" customHeight="1">
       <c r="A112" s="2" t="n">
         <v>111</v>
       </c>
@@ -6147,8 +6737,13 @@
           <t>Câu trả lời trích dẫn Điều 33 và 43 của Luật Hôn nhân và gia đình 2014 (Luật số 52/2014/QH13), tuy nhiên không có điều luật nào từ Luật Đất đai 2024 hoặc các nghị định mới liên quan đến việc xác định tài sản riêng hay chung trong trường hợp này. Luật Hôn nhân và gia đình 2014 vẫn còn hiệu lực và đúng đắn trong việc xác định tài sản riêng và chung trong hôn nhân. Tuy nhiên, câu trả lời không trích dẫn điều luật từ Luật Đất đai 2024, điều này có thể cần thiết để xác định rõ hơn về quyền sử dụng đất và tài sản gắn liền với đất.</t>
         </is>
       </c>
-    </row>
-    <row r="113">
+      <c r="I112" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="380" customHeight="1">
       <c r="A113" s="2" t="n">
         <v>112</v>
       </c>
@@ -6193,8 +6788,13 @@
           <t>Câu trả lời đã trích dẫn Điều 138 của Luật Đất đai 2024 và Điều 25 của Nghị định 101/2024/NĐ-CP, cả hai đều còn hiệu lực. Điều 138 Luật Đất đai 2024 quy định về việc cấp Giấy chứng nhận cho đất không có giấy tờ nhưng sử dụng ổn định trước 01/7/2014. Điều 25 Nghị định 101/2024/NĐ-CP quy định về việc xác định diện tích đất ở và công nhận đất ở trong trường hợp có nhà ở xây dựng trước 01/7/2014. Cả hai điều luật này đều liên quan và bao phủ vấn đề người dùng hỏi về việc cấp sổ đỏ cho đất có nhà xây trước 2014.</t>
         </is>
       </c>
-    </row>
-    <row r="114">
+      <c r="I113" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="409.6" customHeight="1">
       <c r="A114" s="2" t="n">
         <v>113</v>
       </c>
@@ -6249,8 +6849,13 @@
           <t>Câu trả lời trích dẫn Điều 220 của Luật Đất đai 2024 và Điều 4 của Nghị quyết 254/2025/QH15. Tuy nhiên, không có thông tin cụ thể về nội dung của Điều 220 Luật Đất đai 2024 và Điều 4 Nghị quyết 254/2025/QH15 trong câu trả lời, do đó không thể xác định tính chính xác và hiệu lực của các điều luật này. Cần kiểm tra lại nội dung cụ thể của các điều luật để đảm bảo tính chính xác.</t>
         </is>
       </c>
-    </row>
-    <row r="115">
+      <c r="I114" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="409.6" customHeight="1">
       <c r="A115" s="2" t="n">
         <v>114</v>
       </c>
@@ -6299,8 +6904,13 @@
           <t>Câu trả lời đã trích dẫn Điều 8 của Nghị định 10/2022/NĐ-CP về lệ phí trước bạ, và Luật Đất đai 2024 (Luật số 31/2024/QH15) về tiền sử dụng đất. Cả hai văn bản này đều còn hiệu lực và phù hợp với vấn đề cấp Giấy chứng nhận quyền sử dụng đất lần đầu. Tuy nhiên, câu trả lời chưa trích dẫn cụ thể điều khoản nào trong Luật Đất đai 2024 liên quan đến điều kiện cấp Giấy chứng nhận quyền sử dụng đất, nhưng đã bao phủ phần lớn các khía cạnh cần thiết để trả lời câu hỏi của người dùng.</t>
         </is>
       </c>
-    </row>
-    <row r="116">
+      <c r="I115" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="380" customHeight="1">
       <c r="A116" s="2" t="n">
         <v>115</v>
       </c>
@@ -6345,8 +6955,13 @@
           <t>Câu trả lời trích dẫn Điều 89 của Luật Xây dựng 2014, được sửa đổi năm 2020, nhưng không có thông tin về việc Luật này đã bị thay thế hoặc sửa đổi bởi văn bản mới hơn. Ngoài ra, Nghị định 217/2026/NĐ-CP là một văn bản không tồn tại tại thời điểm hiện tại. Do đó, việc trích dẫn này không đáp ứng tiêu chí về tính hiệu lực và tính đúng đắn của điều luật.</t>
         </is>
       </c>
-    </row>
-    <row r="117">
+      <c r="I116" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="395" customHeight="1">
       <c r="A117" s="2" t="n">
         <v>116</v>
       </c>
@@ -6395,8 +7010,13 @@
           <t>Câu trả lời không trích dẫn điều luật nào, không giải quyết các vấn đề pháp lý mà người dùng hỏi. Người dùng hỏi về điều kiện cấp sổ đỏ lần đầu, yêu cầu chữ ký của các cô khi làm sổ đỏ, và hướng thủ tục nên làm. Câu trả lời không đề cập đến các điều luật liên quan đến cấp sổ đỏ lần đầu theo Luật Đất đai 2024, không giải thích về thủ tục khai nhận thừa kế hay cấp sổ đỏ, và không trả lời về yêu cầu chữ ký của các cô.</t>
         </is>
       </c>
-    </row>
-    <row r="118">
+      <c r="I117" s="6" t="inlineStr">
+        <is>
+          <t>Loại 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="395" customHeight="1">
       <c r="A118" s="2" t="n">
         <v>117</v>
       </c>
@@ -6440,8 +7060,13 @@
           <t>Câu trả lời trích dẫn Điều 254 Bộ luật Dân sự 2015, điều này vẫn còn hiệu lực và đúng với tình huống về quyền yêu cầu lối đi qua bất động sản liền kề. Tuy nhiên, "Điều 11, Nghị quyết 254/2025/QH15" không tồn tại, do đó việc trích dẫn này là sai. Câu trả lời đã bao phủ phần quyền yêu cầu lối đi và trách nhiệm của người tách thửa, nhưng việc trích dẫn sai làm giảm độ chính xác của phần này.</t>
         </is>
       </c>
-    </row>
-    <row r="119">
+      <c r="I118" s="6" t="inlineStr">
+        <is>
+          <t>Loại 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="409.6" customHeight="1">
       <c r="A119" s="2" t="n">
         <v>118</v>
       </c>
@@ -6491,8 +7116,13 @@
           <t>Câu trả lời không trích dẫn điều luật cụ thể nào từ Luật Đất đai 2024 hoặc các nghị định mới liên quan. Mặc dù có đề cập đến Điều 152 Luật Đất đai 2024, nhưng không có nội dung cụ thể nào từ điều luật này được trích dẫn để hỗ trợ cho câu trả lời. Do đó, không thể xác định tính hiệu lực và độ chính xác của điều luật được trích dẫn. Câu trả lời đã bao phủ phần lớn các bước cần thiết để thực hiện thủ tục cấp đổi Giấy chứng nhận quyền sử dụng đất khi một trong hai người đứng tên không có mặt, nhưng thiếu trích dẫn điều luật cụ thể để hỗ trợ.</t>
         </is>
       </c>
-    </row>
-    <row r="120">
+      <c r="I119" s="6" t="inlineStr">
+        <is>
+          <t>Loại 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="409.6" customHeight="1">
       <c r="A120" s="2" t="n">
         <v>119</v>
       </c>
@@ -6541,6 +7171,11 @@
           <t>Câu trả lời trích dẫn Điều 21 Thông tư 10/2024/TT-BTNMT, văn bản này còn hiệu lực và liên quan đến việc đính chính thông tin trên Giấy chứng nhận quyền sử dụng đất. Điều luật này đã bao phủ phần hướng dẫn về thủ tục đính chính sổ đỏ khi có sai sót, nhưng chưa đề cập chi tiết về chi phí cụ thể do phụ thuộc vào quy định từng địa phương.</t>
         </is>
       </c>
+      <c r="I120" s="6" t="inlineStr">
+        <is>
+          <t>Loại 2</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H129"/>

</xml_diff>

<commit_message>
chore: update evaluation datasets and remove obsolete answer and category files
</commit_message>
<xml_diff>
--- a/emlaw_crawler/answer_dat_dai_evaluated_gpt4o.xlsx
+++ b/emlaw_crawler/answer_dat_dai_evaluated_gpt4o.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tranhuuduc/Documents/dev/Rag_Graph_LawLaw/emlaw_crawler/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0879DFAD-94B8-E64C-8145-AE6A0B51E5AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25BEDEF3-BDCC-8E4E-84CD-DC2958830C3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-2320" yWindow="-19320" windowWidth="27040" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1446" uniqueCount="561">
   <si>
     <t>STT</t>
   </si>
@@ -52,7 +52,7 @@
     <t>Phân loại</t>
   </si>
   <si>
-    <t>Trích đúng điều luật — TRUE: 65, FALSE: 54, Tổng: 119</t>
+    <t>Trích đúng điều luật — TRUE: 93, FALSE: 86, Tổng: 179</t>
   </si>
   <si>
     <t>Nhà em sổ cũ là 380m2. Nhờ mô giới tách thành 2 sổ mà cộng diện tích lại còn 352m2. Giờ xử lý sao được ạ?</t>
@@ -78,7 +78,7 @@
     <t>Loại 2</t>
   </si>
   <si>
-    <t>Kind 1 (Loại 1,2) — Đúng: 36/57 (63.2%)</t>
+    <t>Kind 1 — Đúng: 43/73 (58.9%)</t>
   </si>
   <si>
     <t>E mua lại nha ở xã hội chưa đủ 5 năm e đã làm hs xet duyệt đạt và đủ điều kiem mua. Nhung ben phía chủ đâu tư chưa cho sang nhượng thì phải làm sao ạ</t>
@@ -103,7 +103,7 @@
     <t>Loại 7</t>
   </si>
   <si>
-    <t>Kind 2 (Loại 3) — Đúng: 13/22 (59.1%)</t>
+    <t>Kind 2 — Đúng: 16/36 (44.4%)</t>
   </si>
   <si>
     <t>Các bác cho em hỏi . E có uỷ quyền cho cò để lên thổ cư đất . Và đưa luôn sổ hồng cho họ . Vậy nếu cò đó có ý xấu vậy e có bị mất đất không .</t>
@@ -126,7 +126,7 @@
     <t>Loại 5</t>
   </si>
   <si>
-    <t>Kind 3 (Loại 4,5) — Đúng: 11/27 (40.7%)</t>
+    <t>Kind 3 — Đúng: 16/43 (37.2%)</t>
   </si>
   <si>
     <t>Luật sư cho hỏi; gđ e nộp đơn hoà giải tranh chấp đất đến nay đã hơn 50 ngày mà ubnd xã họ cứ hẹn qua tuần mà 2 tuần nay vẫn chưa giãi quyết. Chỗ phần đất đang tranh chấp thì họ đang sử dụng bt. Vậy gđ e phải làm ntn ạ e cám ơn</t>
@@ -150,7 +150,7 @@
     <t>Loại 4</t>
   </si>
   <si>
-    <t>Kind 4 (Loại 6,7) — Đúng: 5/13 (38.5%)</t>
+    <t>Kind 4 — Đúng: 18/27 (66.7%)</t>
   </si>
   <si>
     <t>Em ở Đà Nẵng, mọi người giúp em với
@@ -2445,6 +2445,1286 @@
   </si>
   <si>
     <t>Câu trả lời trích dẫn Điều 21 Thông tư 10/2024/TT-BTNMT, văn bản này còn hiệu lực và liên quan đến việc đính chính thông tin trên Giấy chứng nhận quyền sử dụng đất. Điều luật này đã bao phủ phần hướng dẫn về thủ tục đính chính sổ đỏ khi có sai sót, nhưng chưa đề cập chi tiết về chi phí cụ thể do phụ thuộc vào quy định từng địa phương.</t>
+  </si>
+  <si>
+    <t>Trước đây Ông em có mua cho Bố em 1 mảnh đất, thời điểm đó chỉ có phiếu thu tiền , chưa có sổ đỏ. Ở quê thì mọi người cũng nhiều người cũng chưa có sổ như thế. Sau này lúc Ông e mất, các cô các Bác đã ký giấy từ chối nhận quyền thừa kế và để mảnh đất đó cho Bố em. Gia đình em đã mang giấy tờ đi nộp để làm Sổ đỏ, tuy nhiên giấy tờ đã bị thất lạc, do có xáo trộn lãnh đạo địa chính lúc ấy. Bây giờ nhà em muốn làm sổ đỏ thì phải làm như thế nào ạ? giấy tờ gốc hiện tại nhà em k còn, chỉ còn bản hình ảnh thôi ạ</t>
+  </si>
+  <si>
+    <t>Kết luận: Gia đình bạn vẫn có thể làm thủ tục cấp Sổ đỏ lần đầu, nhưng cần làm rõ hai việc: nguồn gốc đất ông mua cho bố và quá trình bố/gia đình sử dụng đất ổn định, không tranh chấp. Ảnh chụp phiếu thu, giấy các cô bác từ chối nhận thừa kế không thay thế hoàn toàn bản gốc, nhưng là chứng cứ quan trọng để xin trích lục hồ sơ và xác minh thực tế.
+ 1. Việc cần làm trước tiên: tìm lại hồ sơ đã từng nộp
+ Nộp đơn đề nghị cung cấp/trích lục hồ sơ địa chính, hồ sơ cấp Giấy chứng nhận tại Chi nhánh Văn phòng đăng ký đất đai nơi có đất hoặc UBND xã. Trong đơn ghi rõ: thời điểm đã nộp hồ sơ, tên ông/bố, vị trí thửa đất, người nhận hồ sơ (nếu nhớ), kèm ảnh phiếu thu và ảnh giấy từ chối thừa kế.
+ Cơ quan này cần kiểm tra sổ tiếp nhận, sổ mục kê, bản đồ địa chính, hồ sơ lưu và dữ liệu đất đai. Nếu tìm được hồ sơ cũ hoặc có tên ông/bố trong sổ địa chính thì đây là chứng cứ rất mạnh để cấp Sổ đỏ. Giấy chứng nhận tạm thời, tên trong sổ đăng ký ruộng đất hoặc sổ địa chính là giấy tờ về quyền sử dụng đất. Điều 137 Luật Đất đai 2024
+ 2. Nộp lại hồ sơ cấp Sổ đỏ lần đầu
+ Nếu hồ sơ cũ không còn hoặc không đủ, bố bạn đứng tên nộp lại hồ sơ xin cấp Giấy chứng nhận lần đầu tại UBND xã nơi có đất hoặc Chi nhánh Văn phòng đăng ký đất đai.
+ Nên chuẩn bị:
+ Đơn đăng ký đất đai, cấp Giấy chứng nhận lần đầu;
+ CCCD của bố;
+ Ảnh phiếu thu/mua đất, ảnh giấy các cô bác từ chối nhận di sản hoặc văn bản họp gia đình;
+ Giấy chứng tử của ông; giấy khai sinh/giấy tờ chứng minh quan hệ cha con giữa ông và bố;
+ Giấy tờ thể hiện bố đã quản lý, sử dụng đất: biên lai thuế, xác nhận của thôn/xóm, giấy tờ xây nhà, điện nước, ảnh hiện trạng, xác nhận ranh giới của các hộ liền kề;
+ Văn bản xác nhận hiện trạng đất không tranh chấp của UBND xã (cơ quan tiếp nhận sẽ thực hiện bước xác minh, niêm yết theo thủ tục).
+ 3. Hai hướng để được xem xét cấp Sổ
+ Nếu xác minh được việc ông đã mua/giao đất cho bố, hoặc bố sử dụng đất theo giấy tờ hợp pháp từ trước đây, hồ sơ sẽ được xem xét theo diện có giấy tờ về quyền sử dụng đất. Với giấy tờ chuyển nhượng lập trước ngày 15/10/1993, UBND xã xác nhận việc sử dụng đất trước mốc này, người sử dụng đất có thể được cấp Giấy chứng nhận. Điều 137 Luật Đất đai 2024
+ Nếu không chứng minh được giấy tờ gốc, bố vẫn có thể được xét cấp Sổ theo diện đang sử dụng đất ổn định, không tranh chấp, tùy thời điểm bắt đầu sử dụng, loại đất, việc có vi phạm pháp luật đất đai hay không và sự phù hợp quy hoạch. Điều 138 Luật Đất đai 2024
+ 4. Lưu ý về thừa kế
+ Vì đất ban đầu đứng về nguồn gốc của ông, giấy “từ chối nhận thừa kế” của cô bác cần được kiểm tra kỹ: văn bản đó có công chứng/chứng thực hay không, được lập trước khi phân chia di sản không, và có ghi đúng thửa đất hay không. Nếu chỉ là giấy viết tay hoặc ảnh không rõ, phương án an toàn là các cô bác còn sống lập lại văn bản thỏa thuận phân chia di sản/văn bản xác nhận không tranh chấp và đồng ý để bố đứng tên, có công chứng hoặc chứng thực.
+ Nếu có người thừa kế không hợp tác hoặc phát sinh tranh chấp, cơ quan đất đai thường không giải quyết cấp Sổ cho đến khi các bên có thỏa thuận hợp lệ hoặc bản án/quyết định có hiệu lực của Tòa án. Người sử dụng đất chỉ được cấp Giấy chứng nhận khi đất không có tranh chấp. Điều 138 Luật Đất đai 2024
+ 5. Cách làm thực tế nên theo thứ tự
+ Sao lưu, in rõ toàn bộ ảnh giấy tờ đang có; đừng chỉnh sửa ảnh.
+ Xin trích lục hồ sơ địa chính và hồ sơ đã nộp trước đây.
+ Xin UBND xã xác nhận quá trình bố sử dụng đất, hiện trạng, ranh giới và tình trạng không tranh chấp.
+ Hoàn thiện lại văn bản thừa kế nếu giấy cũ không bảo đảm giá trị.
+ Nộp hồ sơ cấp Sổ đỏ lần đầu.
+ Khi nộp, yêu cầu cơ quan tiếp nhận lập phiếu tiếp nhận hồ sơ. Nếu từ chối, phải yêu cầu trả lời bằng văn bản, nêu rõ lý do và tài liệu cần bổ sung; không nên chỉ nhận trả lời miệng.
+ [1]. Điều 137, 138, Luật 31/2024/QH15</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn Điều 137 và 138 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là văn bản hiện hành và có hiệu lực từ 01/08/2024. Điều 137 liên quan đến việc cấp Giấy chứng nhận quyền sử dụng đất khi có giấy tờ về quyền sử dụng đất, và Điều 138 liên quan đến việc cấp Giấy chứng nhận khi không có giấy tờ nhưng sử dụng đất ổn định, không tranh chấp. Các điều luật này bao phủ đầy đủ các tình huống mà người hỏi có thể gặp phải trong quá trình xin cấp Sổ đỏ.</t>
+  </si>
+  <si>
+    <t>Kind 1 - Thủ tục quản lý đất đai</t>
+  </si>
+  <si>
+    <t>Em ở Đà Nẵng, mọi người cho em hỏi. 
+Thửa đất của người đã chết, em là người được thừa kế ( các đồng thừa kế đã đống ý ký văn bản phân chia di sản thừa kế khi nào em hoàn thành thủ tục). Thửa đất đang là sổ đỏ (chưa lên sổ hồng) có diện tích 125m2 trong GCN nhưng đo thực tế là 160m2 , tăng thêm 35m2 ( thửa đất gốc có diện tích 525m2 đã công nhận toàn bộ đất ở theo hồ sơ 299 ở trước 18/12/1980 năm 2009), hạn mức đất ở chỗ em là 100m2 x 5 =500m2 nên giờ họ xác định 125m2 trong GCN kia có 100m2 ở và 25m2 CLN ; phần đất còn lại này nằm ở giữa thửa đất gốc ( chỉ giáp thửa đất phía sau, hai bên là hai thửa cắt ra từ thửa gốc, đã có ranh giới). 
+Vậy cho em hỏi là sau khi ký thỏa thuận phân chia di sản thừa kế, em có thể đổi sổ đỏ sang sổ hồng và biến động phần dư ra kia thành đất CLN để trong sổ hồng mới là 100m2 đất ở và 60m2 CLN không ? Sau khi làm như vậy em mới sang tên cho em đứng được không ? Mong mọi người giúp em</t>
+  </si>
+  <si>
+    <t>Chào bạn, bạn đang cần hỏi vấn đề pháp lý nào tại Đà Nẵng?</t>
+  </si>
+  <si>
+    <t>Câu trả lời không xác định đúng vấn đề pháp lý mà người dùng hỏi, không trích dẫn điều luật nào và không trả lời câu hỏi của người dùng. Người dùng hỏi về việc chuyển đổi sổ đỏ sang sổ hồng và xử lý phần diện tích đất tăng thêm, nhưng câu trả lời không đề cập đến các quy định pháp luật liên quan đến thừa kế, chuyển đổi mục đích sử dụng đất, hoặc thủ tục cấp đổi giấy chứng nhận quyền sử dụng đất.</t>
+  </si>
+  <si>
+    <t>Bà em già yếu 90tuoi cần sang tên đất cho bố em là con trai 65tuoi sống chung với bà (bà là chủ hộ). Nhà em chỉ có 1 mảnh đất sống cả 40 năm nay rồi. 
+Xã đòi giấy khai sinh của bố em.
+Vấn đề là bà và bố em ngày xưa chiến tranh chạy giặc vào nam nên ko còn giấy khai sinh từ 65 năm trước. Bố em về quê chật vật làm được giấy khai sinh. Thì xã đòi tiếp giấy kết hôn của ông bà em. Vấn đề là ông của em chết mất xác trong chiến tranh (đến giờ vẫn ko tung tích ko biết chết ở đâu). Trình bày thì họ đòi giấy chứng tử + mộ. 
+Giờ phải làm sao ạ? Giấy tờ đất nhà em sổ hồng thổ cư đầy đủ.</t>
+  </si>
+  <si>
+    <t>Kết luận: Xã không thể tự đặt thêm điều kiện bắt buộc phải có giấy đăng ký kết hôn, giấy chứng tử hoặc mộ của ông nếu bà là người duy nhất đứng tên trên sổ hồng và đang tự nguyện tặng cho đất cho bố bạn. Giấy khai sinh của bố chủ yếu chỉ cần để chứng minh quan hệ mẹ–con khi xin miễn thuế, lệ phí; việc ông mất tích không làm mất quyền định đoạt tài sản riêng của bà.
+ Nếu sổ hồng chỉ ghi tên bà, gia đình nên làm theo hướng hợp đồng tặng cho quyền sử dụng đất từ bà sang bố, có công chứng/chứng thực, sau đó nộp hồ sơ đăng ký biến động tại cơ quan đăng ký đất đai. Hồ sơ trọng tâm là: sổ hồng bản gốc, CCCD của bà và bố, hợp đồng tặng cho, tờ khai thuế/lệ phí và giấy tờ chứng minh mẹ–con.
+ Bố bạn đã có giấy khai sinh thì nộp giấy đó. Quan hệ mẹ–con cũng có thể được chứng minh bằng trích lục hộ tịch, dữ liệu dân cư/căn cước hoặc xác nhận của UBND xã nơi cư trú, không chỉ duy nhất bằng giấy khai sinh Điều 6 Nghị định 154/2024/NĐ-CP.
+ Vì tặng cho giữa mẹ và con ruột, bố bạn được miễn thuế thu nhập cá nhân và lệ phí trước bạ, nhưng phải có hồ sơ chứng minh quan hệ mẹ–con Điều 4 Luật Thuế thu nhập cá nhân Điều 10 Nghị định 10/2022/NĐ-CP.
+ Việc xã đòi giấy kết hôn của ông bà chỉ có thể có lý do nếu họ nghi ngờ mảnh đất là tài sản chung vợ chồng và cần xác định quyền của ông. Tuy nhiên, ông đã mất tích từ thời chiến tranh, không phải vì thế mà bắt buộc gia đình phải tìm được mộ hoặc giấy chứng tử mới được làm thủ tục. Nếu cần xử lý phần tài sản của ông, gia đình có thể làm thủ tục yêu cầu Tòa án tuyên bố ông đã chết khi đáp ứng điều kiện luật định; quyết định của Tòa án là căn cứ hộ tịch và thừa kế, không cần có mộ Điều 71 Bộ luật Dân sự 2015.
+ Trước mắt, bạn nên yêu cầu cán bộ xã trả lời rõ bằng phiếu hướng dẫn bổ sung hồ sơ hoặc văn bản nêu căn cứ pháp luật: giấy đăng ký kết hôn, giấy chứng tử và mộ được yêu cầu theo quy định nào. Không nên chỉ nhận yêu cầu miệng. Nếu sổ hồng đứng tên riêng bà và không có tranh chấp, hãy đề nghị tiếp nhận hồ sơ tặng cho; trường hợp bị từ chối, yêu cầu văn bản từ chối để khiếu nại đến người đứng đầu UBND xã hoặc cơ quan đăng ký đất đai.
+ [1]. Điều 6, Nghị định 154/2024/NĐ-CP
+ [2]. Điều 4, Luật 04/2007/QH12
+ [3]. Điều 10, Nghị định 10/2022/NĐ-CP
+ [4]. Điều 71, Luật 91/2015/QH13</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 6 Nghị định 154/2024/NĐ-CP, Điều 4 Luật 04/2007/QH12, Điều 10 Nghị định 10/2022/NĐ-CP và Điều 71 Bộ luật Dân sự 2015. Tuy nhiên, Luật 04/2007/QH12 đã hết hiệu lực và bị thay thế bởi Luật Thuế thu nhập cá nhân mới. Các điều luật khác được trích dẫn đúng và còn hiệu lực. Câu trả lời đã bao phủ phần lớn các vấn đề pháp lý liên quan đến việc tặng cho quyền sử dụng đất và miễn thuế, nhưng cần cập nhật điều luật về thuế thu nhập cá nhân.</t>
+  </si>
+  <si>
+    <t>Nhà e định làm sổ đỏ 330m, Khi em lên nộp bộ hồ sơ mới năm 2025 là 330m nhưng trên phường lại cho bộ hồ sơ cũ 2022 là 150m làm thuế (năm 2022 trên phường bảo nhà em là chỉ được làm 120-150m, nên nhà e cũng phải nộp hồ sơ. Tất nhiên là trong vòng mấy năm nay thì nhà e vẫn chưa dc phường gọi lên đóng thuế). Trong khi đó nhà e không có kí kết bất cứ giấy tờ gì cả. Năm nay phường gọi nhà e lên đóng thuế 150m thì nhà e cũng phải lên làm.
+Hiện tại đã đóng xong thuế. Nhưng chưa có sổ. Bên phường lại gọi bảo là còn số đất còn lại thì phải trả cho phường, cho nhà nước để làm đường gì đó, em cũng không rõ. Và nếu không kí giấy tờ trả đất cho nhà nước thì nhà e không làm được sổ đỏ.
+Mong người tư vấn giúp e là trường hợp này e có làm được sổ đỏ cho 150m không và số đất còn lại là 180m đất vườn nếu như không có trong sổ đỏ thì nó đi về đâu ạ. Đất nhà e là được nhà nước chia vì ông là lão thành cách mạng ạ. Em cảm ơn ạ</t>
+  </si>
+  <si>
+    <t>Kết luận: Gia đình bạn vẫn có thể được cấp sổ đỏ cho 150 m² nếu phần đất này đủ điều kiện, hồ sơ nguồn gốc đất và nghĩa vụ tài chính đã hoàn thành. Tuy nhiên, phường không thể chỉ “nói miệng” buộc gia đình trả 180 m² đất còn lại để làm đường; nếu Nhà nước thu hồi đất thì phải có hồ sơ, quyết định đúng thẩm quyền và phải giải quyết bồi thường/hỗ trợ theo quy định.
+ Việc đã nộp thuế cho hồ sơ 150 m² không tự động làm mất quyền đối với 180 m² còn lại. Nhưng sổ đỏ chỉ ghi diện tích mà cơ quan đăng ký đất đai xác định là đủ điều kiện cấp, dựa vào: giấy tờ giao đất/cấp đất cho ông, bản đồ địa chính, ranh giới thực tế, quy hoạch và tình trạng tranh chấp.
+ Phường không phải cơ quan có thẩm quyền tự quyết định cấp hoặc không cấp sổ đỏ cho hộ gia đình. Hiện nay, việc cấp sổ lần đầu cho cá nhân/hộ gia đình thuộc cơ quan đăng ký đất đai hoặc chi nhánh của cơ quan này theo phân cấp, không phải chỉ do UBND phường quyết định Điều 136 Luật Đất đai 2024.
+ Với 180 m² còn lại, có 3 khả năng chính:
+ Vẫn là đất gia đình đang sử dụng hợp pháp: Gia đình có quyền đề nghị đo đạc, xác minh nguồn gốc và xin cấp sổ cho toàn bộ 330 m², hoặc xin cấp riêng phần đủ điều kiện. Việc ông là lão thành cách mạng là thông tin rất quan trọng, nhưng cần tìm giấy tờ cụ thể như: quyết định giao/cấp đất, giấy phân nhà đất, giấy kê khai nhà đất, biên lai thuế cũ, xác nhận quá trình sử dụng đất, bản đồ/sổ mục kê.
+ Phần 180 m² nằm trong quy hoạch đường: Quy hoạch chưa đồng nghĩa với việc đất đã bị thu hồi. Gia đình vẫn có quyền sử dụng đất cho đến khi có quyết định thu hồi đất hợp pháp. Khi thu hồi để làm đường, Nhà nước phải thực hiện đúng căn cứ, trình tự, thông báo, kiểm đếm, lập phương án bồi thường/hỗ trợ; không thể yêu cầu gia đình ký “trả đất” mà không nêu rõ căn cứ và phương án quyền lợi. Việc thu hồi sai trường hợp, sai thẩm quyền, sai trình tự hoặc xác định sai diện tích là hành vi vi phạm Điều 109 Nghị định 102/2024/NĐ-CP.
+ 180 m² không được công nhận do nguồn gốc hoặc ranh giới: Cơ quan giải quyết phải trả lời bằng văn bản, ghi rõ lý do, diện tích, vị trí, căn cứ pháp lý và hướng xử lý. Không được chỉ thông báo miệng rằng “không ký trả đất thì không làm được sổ”.
+ Gia đình nên làm ngay một văn bản đề nghị cung cấp thông tin và giải quyết hồ sơ, gửi UBND phường và Chi nhánh Văn phòng đăng ký đất đai nơi có đất, yêu cầu:
+ Cho sao/chụp hồ sơ cấp sổ năm 2022 và hồ sơ 330 m² năm 2025;
+ Trả lời bằng văn bản vì sao chỉ giải quyết 150 m²;
+ Cung cấp bản đồ, trích đo và thông tin quy hoạch đường đối với 180 m²;
+ Nếu có dự án thu hồi, yêu cầu cung cấp quyết định/chủ trương thu hồi, thông báo thu hồi đất, phạm vi thu hồi và phương án bồi thường, hỗ trợ;
+ Xác định rõ 180 m² hiện đứng tên/quản lý bởi ai và căn cứ nào.
+ Không nên ký giấy “tự nguyện trả đất”, “hiến đất” hoặc giấy từ chối quyền sử dụng 180 m² khi chưa nhận được bản dự thảo, chưa biết chính xác diện tích/vị trí bị ảnh hưởng và chưa rõ có bồi thường hay không. Nếu gia đình tự nguyện hiến đất thì về sau rất khó yêu cầu bồi thường cho phần đã tự nguyện giao.
+ Bạn cần giữ toàn bộ giấy nộp thuế, phiếu tiếp nhận hồ sơ, thông báo nghĩa vụ tài chính và giấy tờ về việc Nhà nước cấp đất cho ông. Nếu phường tiếp tục gắn điều kiện “phải trả 180 m² mới cấp sổ 150 m²”, hãy yêu cầu họ trả lời bằng văn bản để gia đình có căn cứ khiếu nại hoặc đề nghị cơ quan cấp tỉnh kiểm tra.
+ [1]. Điều 136, Luật 31/2024/QH15
+ [2]. Điều 109, Nghị định 102/2024/NĐ-CP</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn Điều 136 của Luật Đất đai 2024 (Luật số 31/2024/QH15) và Điều 109 của Nghị định 102/2024/NĐ-CP. Cả hai văn bản này đều còn hiệu lực và liên quan đến việc cấp sổ đỏ và quy trình thu hồi đất. Điều 136 Luật Đất đai 2024 quy định về thẩm quyền cấp sổ đỏ, trong khi Điều 109 Nghị định 102/2024/NĐ-CP quy định về quy trình thu hồi đất. Các điều luật này đã bao phủ đầy đủ các khía cạnh pháp lý liên quan đến câu hỏi của người dùng.</t>
+  </si>
+  <si>
+    <t>Kết luận: Không có quy định chung nào bắt buộc đất giãn dân do xã bán trái thẩm quyền năm 2005 phải có “nhà cấp 4 trở lên” mới được cấp sổ đỏ. Tuy nhiên, để được công nhận đất ở theo diện ưu đãi của trường hợp giao đất trái thẩm quyền, thửa đất phải có nhà ở/nhà và công trình phục vụ đời sống; luật không quy định nhà phải đạt cấp 4.
+ Trường hợp của bạn là đất được giao/bán không đúng thẩm quyền trong giai đoạn từ 01/7/2004 đến trước 01/7/2014. Nếu sử dụng đất ổn định, được UBND cấp xã xác nhận không tranh chấp và phù hợp quy hoạch thì được xem xét cấp Giấy chứng nhận. Với thửa đất có nhà ở, diện tích đất ở được công nhận theo hạn mức giao đất ở của địa phương; phần còn lại (nếu có) công nhận theo hiện trạng sử dụng. Căn cứ là Khoản 3 Điều 140 Luật Đất đai 2024.
+ Điều 140 chỉ dùng cụm từ “có nhà ở, nhà ở và công trình phục vụ đời sống”, không hề có tiêu chí “nhà cấp 4 trở lên”. Vì vậy, nếu cán bộ yêu cầu như vậy, bạn nên đề nghị họ trả lời bằng văn bản, nêu rõ căn cứ pháp lý và quy định địa phương đang áp dụng.
+ Nếu trên đất chưa có nhà, không có nghĩa là đương nhiên không thể được cấp sổ, nhưng việc xác định mục đích và diện tích đất ở sẽ cần xem kỹ hồ sơ giao đất năm 2005, hiện trạng sử dụng, quy hoạch và quy định hạn mức đất ở tại tỉnh nơi có đất. Bạn nên chuẩn bị: giấy tờ mua/thu tiền của xã, biên lai, giấy giao đất, xác nhận quá trình sử dụng ổn định, hồ sơ thuế (nếu có), trích đo thửa đất và ý kiến xác nhận không tranh chấp của UBND xã.
+ [1]. Điều 140, Luật 31/2024/QH15</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 140 của Luật Đất đai 2024 (Luật số 31/2024/QH15), quy định về việc cấp Giấy chứng nhận quyền sử dụng đất cho các trường hợp giao đất trái thẩm quyền. Điều luật này còn hiệu lực và phù hợp với tình huống hỏi về việc cấp sổ đỏ cho đất giãn dân do xã bán trái thẩm quyền. Điều luật đã bao phủ phần yêu cầu về nhà ở nhưng chưa đề cập đến thông tư cụ thể nào, tuy nhiên, điều này không ảnh hưởng đến tính đúng đắn của câu trả lời.</t>
+  </si>
+  <si>
+    <t>E chào a/c trong nhóm. Mong a/c giải đáp thac mac:
+ mẹ e bị mat khả nang hanh vi dan su, e đa co trích lục
+ giám hộ và chị gai em là người giam sát giám hộ. E
+ muon doi ten dat tu me em sang em co duoc khong
+ ạ? Hỏi nhiều chỗ mà thủ tục hơi lang nhằng a</t>
+  </si>
+  <si>
+    <t>Kết luận: Bạn không thể tự làm thủ tục “đổi tên” đất từ mẹ sang mình chỉ vì bạn là người giám hộ. Việc tặng cho hoặc chuyển nhượng đất của mẹ chỉ có thể thực hiện khi đó thực sự là giao dịch vì lợi ích của mẹ, có sự đồng ý bằng văn bản của chị gái là người giám sát giám hộ; nếu là chuyển tài sản của mẹ sang cho chính bạn thì có xung đột lợi ích và thường phải cử người giám hộ khác đại diện trong giao dịch.
+ Người mất năng lực hành vi dân sự phải do người giám hộ xác lập, thực hiện giao dịch dân sự nhân danh họ. Tuy nhiên, người giám hộ phải quản lý tài sản vì lợi ích của người được giám hộ, không được đem tài sản của mẹ tặng cho mình hoặc giao dịch làm thiệt hại quyền lợi của mẹ Điều 59 Bộ luật Dân sự 2015.
+ Với bất động sản của người được giám hộ, việc bán, chuyển nhượng, tặng cho, thế chấp hoặc giao dịch khác phải có sự đồng ý của người giám sát việc giám hộ. Chị gái bạn cần lập văn bản đồng ý rõ nội dung giao dịch; nhưng sự đồng ý này không làm hợp pháp một giao dịch nhằm chuyển tài sản của mẹ cho chính người giám hộ mà không chứng minh được lợi ích của mẹ Điều 59 Bộ luật Dân sự 2015.
+ Nếu mẹ có nhu cầu bán đất để lấy tiền chữa bệnh, chăm sóc hoặc bảo đảm sinh hoạt, có thể làm thủ tục chuyển nhượng cho người khác theo giá phù hợp thị trường; tiền thu được phải quản lý, sử dụng cho mẹ. Còn nếu muốn bán/tặng cho chính bạn, nên đề nghị cơ quan có thẩm quyền cử người giám hộ khác hoặc người đại diện phù hợp để tránh việc bạn vừa đại diện cho mẹ vừa là bên nhận tài sản.
+ Nếu mẹ qua đời, quyền sử dụng đất sẽ được giải quyết theo di chúc hợp pháp; nếu không có di chúc thì chia thừa kế theo pháp luật cho các hàng thừa kế, không tự động thuộc riêng bạn Điều 650 Bộ luật Dân sự 2015 Điều 651 Bộ luật Dân sự 2015.
+ [1]. Điều 59, 650, 651, Luật 91/2015/QH13</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 59, 650, 651 của Bộ luật Dân sự 2015. Tuy nhiên, không có điều luật nào được trích dẫn từ Luật Đất đai 2024 hoặc các nghị định mới liên quan đến việc chuyển nhượng quyền sử dụng đất trong trường hợp người mất năng lực hành vi dân sự. Bộ luật Dân sự 2015 vẫn còn hiệu lực, nhưng cần bổ sung các quy định từ Luật Đất đai 2024 để đảm bảo tính đầy đủ và chính xác của câu trả lời.</t>
+  </si>
+  <si>
+    <t>Em có nhà đất ở khu tập thể nhà máy cơ khí tại Quảng Ninh, đất ở, Giấy tờ có giấy thanh lý của nhà máy bản gốc có dấu đỏ, có hồ sơ kỹ thuật thửa đất lập năm 1997 và trích lục đo đạc năm 2021, nhà máy đã thanh lý cho công nhân, sử dụng ổn định, lâu dài không tranh chấp, chưa được cấp sổ đỏ. Em muốn hỏi có đủ điều kiện cấp sổ đỏ lần đầu không?</t>
+  </si>
+  <si>
+    <t>Kết luận: Bạn có khả năng được cấp sổ đỏ lần đầu, nhưng chưa thể khẳng định “đủ điều kiện” chỉ từ giấy thanh lý. Trường hợp khu tập thể do nhà máy thanh lý/bố trí cho công nhân thường được xem xét theo quy định về đất do tổ chức bố trí làm nhà ở hoặc thanh lý nhà ở không đúng quy định; yếu tố quyết định là mốc thời điểm sử dụng, không tranh chấp, quy hoạch và nguồn gốc/quyền quản lý đất của nhà máy.
+ Nếu nhà máy đã bố trí hoặc thanh lý nhà ở, đất ở cho công nhân trước ngày 01/8/2024, diện tích đất này phải được tổ chức bàn giao cho UBND cấp có thẩm quyền để làm thủ tục cấp giấy cho người đang sử dụng; người được cấp giấy phải thực hiện nghĩa vụ tài chính theo quy định. Khoản 2 Điều 142 Luật Đất đai 2024
+ Trường hợp việc thanh lý nhà/đất trước đây không hoàn toàn đúng thủ tục, vẫn có hướng cấp giấy:
+ Sử dụng ổn định trước 15/10/1993 và UBND xã/phường xác nhận không tranh chấp: được xem xét cấp giấy đối với diện tích đã giao.
+ Sử dụng ổn định từ 15/10/1993 đến trước 01/7/2004: cần không tranh chấp và phù hợp quy hoạch.
+ Từ 01/7/2004 đến trước 01/7/2014: cần không tranh chấp, phù hợp quy hoạch; đất ở thường được công nhận trong hạn mức giao đất ở tại địa phương. Điều 140 Luật Đất đai 2024
+ Với hồ sơ bạn nêu, giấy thanh lý bản gốc có dấu, hồ sơ kỹ thuật năm 1997 và trích lục năm 2021 là chứng cứ có giá trị để chứng minh nguồn gốc và quá trình sử dụng. Bạn nên chuẩn bị thêm: giấy tờ nộp tiền/thanh lý (nếu có), biên lai thuế nhà đất hoặc xác nhận cư trú, giấy tờ về nhà ở, xác nhận của các hộ liền kề và đặc biệt là xác nhận của UBND phường/xã về thời điểm sử dụng ổn định, hiện trạng không tranh chấp.
+ Bạn nộp hồ sơ đăng ký, cấp Giấy chứng nhận lần đầu tại cơ quan đăng ký đất đai thuộc Sở Tài chính tỉnh Quảng Ninh hoặc bộ phận một cửa theo nơi tiếp nhận của địa phương. Cơ quan này sẽ kiểm tra liệu khu đất còn thuộc quyền quản lý của nhà máy/doanh nghiệp, có thuộc quy hoạch phải thu hồi hay không và yêu cầu nhà máy hoặc cơ quan đang quản lý đất thực hiện bàn giao hồ sơ nếu cần.
+ Lưu ý: “không tranh chấp” chưa tự động đủ để có sổ. Nếu giấy thanh lý chỉ thanh lý căn nhà mà không thể hiện đất, hoặc nhà máy không có quyền thanh lý/bố trí đất, hồ sơ vẫn có thể được xem xét theo Điều 140 nêu trên, nhưng có thể phải nộp tiền sử dụng đất và bị giới hạn diện tích công nhận. Điều 140 Luật Đất đai 2024
+ [1]. Điều 140, 142, Luật 31/2024/QH15</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn Điều 140 và 142 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là văn bản hiện hành và có hiệu lực từ 01/08/2024. Điều 140 quy định về việc cấp giấy chứng nhận quyền sử dụng đất cho các trường hợp sử dụng đất ổn định trước các mốc thời gian nhất định và không có tranh chấp. Điều 142 quy định về việc xử lý đất do tổ chức bố trí làm nhà ở hoặc thanh lý nhà ở không đúng quy định. Các điều luật này bao phủ vấn đề cấp sổ đỏ lần đầu cho đất có nguồn gốc từ thanh lý của nhà máy, nhưng cần thêm thông tin về việc thực hiện nghĩa vụ tài chính và quy hoạch sử dụng đất.</t>
+  </si>
+  <si>
+    <t>Các bác cho em hỏi nhà em đang làm thủ tục tách sổ, đất nhà e thỏa mãn tất cả thủ tục để tách, tuy nhiên cả khu vực chỗ em ở( cả huyện)  tọa độ giữa các nhà bị hay lệch khoang 50 cm, vậy việc tách sổ có bị ảnh hưởng gì không ạ? đo thực tế đất đủ diện tích trên sổ không tranh chấp, đất nhà em sử dụng và được cấp sổ lâu năm rồi. Cảm ơn các bác.</t>
+  </si>
+  <si>
+    <t>Kết luận: Sai lệch tọa độ khoảng 50 cm không đương nhiên làm hồ sơ tách thửa bị từ chối. Tuy nhiên, cơ quan đăng ký đất đai thường sẽ yêu cầu đo đạc, xác định lại ranh giới thực tế và chỉnh lý dữ liệu/bản đồ trước hoặc đồng thời khi tách thửa; nếu không có tranh chấp, không lấn ranh và diện tích vẫn đủ điều kiện tách thì về nguyên tắc vẫn xử lý được.
+ Việc “lệch tọa độ” cần phân biệt: nếu chỉ là sai số dữ liệu/bản đồ cũ và ranh đất thực tế ổn định, các hộ liền kề thống nhất, thì đơn vị đo đạc sẽ lập hồ sơ đo đạc chỉnh lý theo hiện trạng. Nếu sự lệch làm chồng lấn sang đất hàng xóm, đất công, hành lang công trình hoặc các hộ không ký xác nhận ranh giới, hồ sơ có thể phải tạm dừng để xác minh, giải quyết tranh chấp.
+ Khi kích thước, diện tích có thay đổi vượt sai số, cơ quan chuyên môn phải kiểm tra hồ sơ địa chính, giấy tờ đã cấp; nếu không đủ cơ sở thì đo đạc lại ranh giới tại thực địa. Kết quả phải được thể hiện trong phiếu đo đạc chỉnh lý và có xác nhận của người sử dụng đất, người quản lý đất (nếu có) và Văn phòng đăng ký đất đai/Chi nhánh Văn phòng đăng ký đất đai Điều 17 Thông tư 26/2024/TT-BTNMT.
+ Do đó, gia đình nên:
+ Đề nghị đơn vị đo đạc kiểm tra nguyên nhân lệch: do hệ tọa độ/bản đồ cũ hay do ranh sử dụng thực tế khác Giấy chứng nhận.
+ Cắm mốc, lập bản mô tả ranh giới/mốc giới; nên mời các hộ giáp ranh ký xác nhận để tránh hồ sơ bị yêu cầu bổ sung.
+ Nộp hồ sơ tách thửa kèm trích đo địa chính mới tại Chi nhánh Văn phòng đăng ký đất đai nơi có đất. Nếu cần, đề nghị thực hiện chỉnh lý thông tin thửa đất trong cùng hồ sơ.
+ Kiểm tra điều kiện diện tích tối thiểu, kích thước cạnh thửa, lối đi và quy hoạch theo quyết định tách thửa của tỉnh/thành phố nơi có đất; đây là điều kiện địa phương nên mỗi nơi có thể khác nhau.
+ Trường hợp bản đồ địa chính mới có ranh thể hiện khác Giấy chứng nhận cũ nhưng chưa cấp đổi theo bản đồ mới, ranh giới và diện tích sử dụng đất trước hết được xác định theo Giấy chứng nhận đã cấp Điều 7 Thông tư 10/2024/TT-BTNMT.
+ [1]. Điều 17, Thông tư 26/2024/TT-BTNMT
+ [2]. Điều 7, Thông tư 10/2024/TT-BTNMT</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 17 Thông tư 26/2024/TT-BTNMT và Điều 7 Thông tư 10/2024/TT-BTNMT. Cả hai thông tư này đều còn hiệu lực và liên quan đến việc đo đạc, chỉnh lý bản đồ địa chính và xác định ranh giới đất. Điều 17 Thông tư 26/2024/TT-BTNMT hướng dẫn về việc đo đạc chỉnh lý khi có sai lệch tọa độ, còn Điều 7 Thông tư 10/2024/TT-BTNMT quy định về việc xác định ranh giới và diện tích sử dụng đất theo Giấy chứng nhận đã cấp. Các điều luật này đã bao phủ đầy đủ vấn đề người dùng hỏi về việc tách sổ khi có sai lệch tọa độ.</t>
+  </si>
+  <si>
+    <t>Dạ e ở Thủ Đức, cho e hỏi giấy tay 2017 có làm sổ được không ạ, trên đất có nhà cấp 4 xin GPXD 2 tầng được ko ạ. Cám ơn mọi người</t>
+  </si>
+  <si>
+    <t>Kết luận: Giấy mua bán/giấy tay lập năm 2017 không tự động làm được sổ; vẫn có thể được xem xét nếu nguồn gốc thửa đất hợp pháp, không tranh chấp, phù hợp quy hoạch và việc chuyển nhượng đáp ứng điều kiện pháp luật. Với nhà cấp 4 hiện có, bạn thường cần làm rõ quyền sử dụng đất trước; xin phép xây 2 tầng chỉ khả thi khi đất là đất ở hợp pháp và đáp ứng quy hoạch, chỉ giới xây dựng.
+ Giấy tay năm 2017 là giao dịch sau thời điểm pháp luật đã yêu cầu việc chuyển nhượng quyền sử dụng đất phải có công chứng/chứng thực và đăng ký. Vì vậy, nếu bên bán đang đứng tên sổ, cách an toàn nhất là liên hệ bên bán để làm thủ tục chuyển nhượng đúng hình thức; nếu bên bán không hợp tác, cần xem hồ sơ cụ thể để xác định có căn cứ khởi kiện/yêu cầu công nhận giao dịch hay không. Trường hợp đất “không sổ” thì phải kiểm tra nguồn gốc, thời điểm sử dụng đất, vi phạm và tranh chấp; quy định công nhận đất không giấy tờ chủ yếu áp dụng cho quá trình sử dụng đất từ các mốc trước ngày 01/7/2014, nên mua giấy tay năm 2017 không phải là căn cứ độc lập để được cấp sổ Điều 138 Luật Đất đai 2024.
+ Về xây 2 tầng: không nên tự xây hoặc tháo nhà cấp 4 trước khi có giấy phép. Hồ sơ xin phép hiện có thể sử dụng giấy chứng nhận hoặc giấy tờ đủ điều kiện cấp giấy chứng nhận; tuy nhiên bạn phải chứng minh đất hợp pháp, đúng mục đích đất ở, không vướng quy hoạch/kế hoạch thu hồi đất và thiết kế phù hợp quy định xây dựng Điều 55 Nghị định 217/2026/NĐ-CP.
+ Bạn nên mang các giấy tờ sau đến UBND phường nơi có đất hoặc cơ quan đăng ký đất đai tại TP.HCM để kiểm tra trước: giấy tay 2017; bản sao sổ/giấy tờ nguồn gốc của người bán (nếu có); biên nhận tiền; giấy tờ nhà cấp 4; biên lai thuế; thông tin quy hoạch. Cần kiểm tra riêng thửa đất có phải đất ở, có bị quy hoạch hoặc có phần xây dựng không phép hay không; đây là các yếu tố quyết định có thể cấp sổ và xin phép 2 tầng.
+ [1]. Điều 138, Luật 31/2024/QH15
+ [2]. Điều 55, Nghị định 217/2026/NĐ-CP</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 138 của Luật Đất đai 2024 và Điều 55 của Nghị định 217/2026/NĐ-CP. Tuy nhiên, Nghị định 217/2026/NĐ-CP là một văn bản không tồn tại và không có hiệu lực. Do đó, tiêu chí trích dẫn điều luật bị đánh giá là false. Câu trả lời đã bao phủ phần lớn các vấn đề liên quan đến việc cấp sổ đỏ từ giấy tay và xin giấy phép xây dựng, nhưng việc trích dẫn điều luật không chính xác làm giảm độ tin cậy của thông tin pháp lý.</t>
+  </si>
+  <si>
+    <t>Nhờ các bác trên thông thiên văn dưới tường địa lý giúp em. Chả là nhà em đang làm giấy tờ, chuyển tên chủ sở hữu đất từ tên ông nội em, sang tên bố em(ông nội em đã mất, các bác trong nhà đều đồng thuận việc chuyển đổi) đồng thời, vì lý do mảnh đất nên phải tách làm 3 sổ. Ko biết thủ tục có khó ko? Và mất khoảng bao lâu? Chi phí tnao nhỉ? Đang thời kì chuyển giao, lại sáp nhập tỉnh nên em thấy mông lung quá. Mong các bác hỗ trợ, xin lời khuyên (cả chính ngạch và tiểu ngạch ạ)</t>
+  </si>
+  <si>
+    <t>Kết luận: Làm được, nhưng không phải chỉ “đổi tên sổ”. Cần giải quyết thủ tục thừa kế của ông nội trước, rồi đăng ký sang tên bố bạn và tách thành 3 thửa; có thể đề nghị xử lý trong cùng một hồ sơ nếu địa phương cho phép. Không nên làm “tiểu ngạch” vì dễ phát sinh rủi ro hồ sơ giả, bị từ chối cấp sổ hoặc tranh chấp sau này.
+ 1. Điều kiện quan trọng nhất
+ Ông nội mất có để lại di chúc không? Nếu không có di chúc, người thừa kế hàng thứ nhất gồm: vợ, cha mẹ, con của ông nội. Vì vậy, “các bác đồng thuận” chỉ là một phần; phải xác định đầy đủ những người thuộc hàng thừa kế, kể cả bà nội (nếu còn sống), các con khác của ông nội, và phần tài sản chung của ông bà nếu có. Điều 651 Bộ luật Dân sự 2015
+ Nếu mọi người đồng ý để bố bạn nhận toàn bộ quyền sử dụng đất, thường lập văn bản thỏa thuận phân chia di sản hoặc văn bản khai nhận di sản tại tổ chức công chứng. Người có quyền thừa kế nhưng không nhận phần của mình có thể làm văn bản từ chối nhận di sản; việc từ chối phải lập thành văn bản và không nhằm trốn tránh nghĩa vụ tài sản. Điều 620 Bộ luật Dân sự 2015
+ Muốn tách được 3 sổ, đất phải đáp ứng diện tích tối thiểu, kích thước cạnh thửa, lối đi, quy hoạch và điều kiện khác theo quy định của tỉnh/thành phố nơi có đất. Đây là phần cần kiểm tra kỹ nhất trước khi công chứng. Điều 220 Luật Đất đai 2024
+ 2. Cách làm thực tế
+ Kiểm tra sổ hiện có, quy hoạch, tình trạng thế chấp/tranh chấp, và hỏi cơ quan đất đai địa phương về điều kiện tách thành 3 thửa.
+ Thu thập giấy chứng tử của ông nội; giấy tờ chứng minh quan hệ của toàn bộ người thừa kế; sổ đỏ; CCCD; giấy tờ hôn nhân của ông/bà nếu liên quan.
+ Công chứng văn bản thỏa thuận phân chia di sản, xác định bố bạn nhận đất.
+ Nộp hồ sơ tại Bộ phận một cửa cấp xã/phường hoặc cơ quan đăng ký đất đai theo quy trình đang áp dụng tại địa phương: đăng ký nhận thừa kế và đề nghị tách thửa/cấp giấy chứng nhận cho 3 thửa.
+ Cơ quan chuyên môn đo đạc, lập bản trích đo địa chính nếu cần; cơ quan thuế ra thông báo nghĩa vụ tài chính; nộp xong thì nhận 3 giấy chứng nhận.
+ Về nguyên tắc, khi chuyển quyền đối với một phần thửa đất, hồ sơ địa chính sẽ ghi nhận việc tách các thửa mới và việc nhận thừa kế tương ứng. Điều 13 Thông tư 10/2024/TT-BTNMT
+ 3. Thời gian
+ Nếu hồ sơ rõ ràng, không vướng quy hoạch, không thiếu người thừa kế và không cần giải quyết tranh chấp: thường khoảng 3–8 tuần tính cả công chứng, đo đạc, nghĩa vụ tài chính và cấp sổ. Thực tế có thể lâu hơn nếu phải xác minh nguồn gốc đất, niêm yết thừa kế, bổ sung giấy tờ nhân thân hoặc đo đạc lại.
+ Đang sáp nhập địa giới không làm mất quyền làm thủ tục. Tuy nhiên, nên nộp tại Bộ phận một cửa nơi thửa đất hiện thuộc địa bàn quản lý mới; giữ phiếu tiếp nhận hồ sơ để theo dõi thời hạn.
+ 4. Chi phí dự kiến
+ Công chứng văn bản thừa kế: tính theo giá trị tài sản/di sản và phí lưu giữ, sao y, soạn thảo nếu có.
+ Đo đạc, trích đo, tách thửa, cấp 3 sổ: mức thu do tỉnh/thành phố quy định; thường là khoản biến động lớn nhất ngoài thuế.
+ Thuế thu nhập cá nhân: thừa kế bất động sản giữa cha mẹ và con thuộc diện miễn; bố bạn nhận di sản từ ông nội nên cần làm hồ sơ chứng minh quan hệ cha–con để được miễn. Điều 18 Nghị định 253/2026/NĐ-CP
+ Lệ phí trước bạ: cần kê khai để cơ quan thuế xác định diện miễn/không miễn; hồ sơ quan hệ gia đình phải đầy đủ.
+ Ngoài ra có lệ phí cấp giấy chứng nhận, phí thẩm định hồ sơ (nếu địa phương thu).
+ 5. Lưu ý để tránh bị trả hồ sơ
+ Đừng chỉ lấy chữ ký “đồng ý” của các bác. Cần đúng loại văn bản công chứng và đúng tất cả người thừa kế.
+ Nếu bà nội còn sống, phải làm rõ đất là tài sản riêng của ông hay tài sản chung vợ chồng. Nếu là tài sản chung, trước hết xác định phần của bà nội; chỉ phần của ông mới là di sản.
+ Kiểm tra xem có người thừa kế đã mất, mất tích, ở nước ngoài, hoặc có con riêng/con nuôi hợp pháp không; các trường hợp này làm thay đổi thành phần ký hồ sơ.
+ Hãy hỏi trước bằng văn bản hoặc phiếu hướng dẫn về điều kiện tách 3 thửa. Nếu tách không đạt diện tích tối thiểu hoặc không có lối đi hợp pháp, có thể phải điều chỉnh phương án chia đất.
+ Bạn nên chuẩn bị tối thiểu: sổ đỏ bản gốc, giấy chứng tử ông nội, CCCD các bên, khai sinh của bố và các giấy tờ chứng minh quan hệ, giấy đăng ký kết hôn của ông bà/bố mẹ nếu có, cùng bản dự kiến sơ đồ chia 3 thửa.
+ [1]. Điều 620, 651, Luật 91/2015/QH13
+ [2]. Điều 220, Luật 31/2024/QH15
+ [3]. Điều 13, Thông tư 10/2024/TT-BTNMT
+ [4]. Điều 18, Nghị định 253/2026/NĐ-CP</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn các điều luật từ Bộ luật Dân sự 2015 (Điều 620, 651) và Luật Đất đai 2024 (Điều 220), Thông tư 10/2024/TT-BTNMT (Điều 13), Nghị định 253/2026/NĐ-CP (Điều 18). Tuy nhiên, Luật Đất đai 2024 và các văn bản liên quan như Thông tư 10/2024/TT-BTNMT và Nghị định 253/2026/NĐ-CP chưa có hiệu lực hoặc không tồn tại tại thời điểm hiện tại, do đó việc trích dẫn này là không chính xác. Bộ luật Dân sự 2015 vẫn còn hiệu lực và được trích dẫn đúng. Tuy nhiên, do có sự trích dẫn văn bản không tồn tại hoặc chưa có hiệu lực, tiêu chí trích dẫn điều luật bị đánh giá là false.</t>
+  </si>
+  <si>
+    <t>Mình muốn hỏi về việc làm sổ đỏ tại Hà Nội. Giấy tờ đất đứng tên ông bà nội (Giấy tờ từ thời Pháp). Ông bà đã mất quá 30 năm. Con cái ông bà người thì đã mất, không con cái. Người thì đã mất nhưng có con cái. Người thì còn sống. Nguồn gốc đất rõ ràng. Không có tranh chấp đất. Gia đình đồng thuận làm sổ đỏ. Xin nhờ tư vấn các bước phải làm thế nào ạ?</t>
+  </si>
+  <si>
+    <t>Kết luận: Gia đình có thể làm sổ đỏ lần đầu, nhưng cần giải quyết đồng thời hai việc: xác định quyền sử dụng đất của ông bà và xác lập người thừa kế hợp pháp để đứng tên trên sổ. Vì ông bà mất đã lâu, có người con đã mất, hồ sơ thừa kế phải làm theo “các nhánh” của từng người con; người chết có con thì con họ được hưởng phần thừa kế thế vị, còn người chết không có con thì cần xem họ mất trước hay sau ông/bà để xác định phần di sản.
+ 1. Xác định ai là người có quyền đứng tên
+ Nếu ông bà không để lại di chúc, di sản được chia theo pháp luật cho hàng thừa kế thứ nhất: vợ/chồng, cha mẹ, con của người chết. Trong thực tế của bạn, thường là các người con của ông bà; con của người con đã chết trước hoặc cùng thời điểm với ông/bà được hưởng phần mà cha/mẹ họ đáng lẽ được hưởng (thừa kế thế vị). Điều 651 Bộ luật Dân sự 2015 Điều 652 Bộ luật Dân sự 2015
+ Cần làm rõ thời điểm mất của từng ông/bà và từng người con. Ví dụ: người con mất sau ông/bà thì họ đã nhận một phần di sản; khi họ mất, phần đó trở thành di sản của chính họ và được chia tiếp cho vợ/chồng, con, cha mẹ của họ. Nếu họ mất trước ông/bà và có con thì con được thừa kế thế vị. Điều 611 Bộ luật Dân sự 2015 Điều 613 Bộ luật Dân sự 2015
+ Việc ông bà mất quá 30 năm không đương nhiên làm mất quyền đối với đất. Tuy nhiên, thời hiệu yêu cầu chia di sản là bất động sản là 30 năm kể từ thời điểm mở thừa kế; vì đã ở sát hoặc quá mốc này, gia đình nên thực hiện ngay và nên thống nhất bằng văn bản. Điều 623 Bộ luật Dân sự 2015
+ 2. Việc nên làm trước: lập văn bản thừa kế tại tổ chức công chứng
+ Gia đình nên lập Văn bản thỏa thuận phân chia di sản hoặc Văn bản khai nhận di sản tại tổ chức hành nghề công chứng. Nếu mọi người thống nhất để một người hoặc một nhóm người đứng tên sổ đỏ, các đồng thừa kế ghi rõ nội dung nhường/cho phần quyền của mình trong văn bản này.
+ Hồ sơ công chứng thường gồm: giấy tờ đất thời Pháp bản gốc; giấy chứng tử của ông, bà và những người con đã mất; CCCD; giấy khai sinh, đăng ký kết hôn và giấy tờ khác chứng minh quan hệ cha mẹ-con; giấy tờ chứng minh người đã mất không có con (nếu cần); giấy tờ cư trú; sơ đồ gia phả. Công chứng viên có trách nhiệm niêm yết việc thụ lý công chứng văn bản thừa kế 15 ngày. Điều 57 Luật Công chứng 2014 Điều 58 Luật Công chứng 2014
+ Lưu ý: người thừa kế không thể hoặc không muốn có mặt có thể lập văn bản ủy quyền hoặc văn bản từ chối nhận di sản hợp lệ; việc từ chối phải thực hiện trước thời điểm phân chia di sản. Điều 620 Bộ luật Dân sự 2015
+ 3. Nộp hồ sơ cấp sổ đỏ lần đầu
+ Sau khi có văn bản thừa kế đã công chứng, người được thống nhất đứng tên nộp hồ sơ đăng ký đất đai, cấp Giấy chứng nhận lần đầu tại Bộ phận Một cửa cấp xã/phường nơi có đất hoặc Chi nhánh Văn phòng đăng ký đất đai Hà Nội theo nơi tiếp nhận hồ sơ tại địa bàn.
+ Hồ sơ trọng tâm gồm:
+ Đơn đăng ký đất đai, tài sản gắn liền với đất và đề nghị cấp Giấy chứng nhận;
+ Giấy tờ đất thời Pháp bản chính/bản sao chứng thực;
+ Văn bản khai nhận hoặc thỏa thuận phân chia di sản đã công chứng;
+ Giấy tờ nhân thân của người sẽ đứng tên;
+ Trích đo địa chính nếu thửa đất chưa có bản đồ địa chính, ranh giới hoặc diện tích cần xác định lại;
+ Chứng từ đã hoàn thành nghĩa vụ tài chính, khi cơ quan thuế thông báo.
+ Giấy tờ về quyền sử dụng đất được lập trước ngày 15/10/1993 thuộc nhóm giấy tờ có thể là căn cứ cấp Giấy chứng nhận nếu xác định được đúng người sử dụng đất, ranh giới và điều kiện pháp lý của thửa đất. Điều 137 Luật Đất đai 2024 Việc đăng ký đất đai lần đầu được thực hiện theo thủ tục đăng ký đất đai, cấp Giấy chứng nhận lần đầu. Điều 18 Nghị định 101/2024/NĐ-CP
+ 4. Các điểm thường vướng
+ Giấy tờ thời Pháp có thể ghi tên ông hoặc bà, ghi tên chủ cũ, ghi số thửa cũ hoặc diện tích không trùng hiện trạng. Cơ quan đăng ký sẽ kiểm tra nguồn gốc, quá trình sử dụng, ranh giới, quy hoạch và có thể yêu cầu xác minh/trích đo.
+ Nếu có người thừa kế ở nước ngoài, mất giấy khai sinh hoặc giấy chứng tử, cần bổ sung tài liệu thay thế/xác nhận của cơ quan có thẩm quyền; đây thường là lý do hồ sơ kéo dài.
+ Nếu có người con đã mất “không con cái”, cần xác định họ mất trước hay sau ông/bà và có vợ/chồng, cha/mẹ còn sống hay không; không nên tự bỏ tên nhánh thừa kế này.
+ Khi gia đình đã đồng thuận, nên để toàn bộ người thuộc diện thừa kế hoặc người kế thừa của họ cùng ký văn bản công chứng. Đây là cách hạn chế rủi ro tranh chấp và việc hồ sơ cấp sổ bị yêu cầu bổ sung sau này.
+ Thứ tự ngắn gọn: lập sơ đồ gia phả và thời điểm mất → thu giấy tờ chứng minh quan hệ → công chứng văn bản thừa kế → trích đo/xác minh thửa đất nếu cần → nộp hồ sơ cấp sổ đỏ lần đầu → thực hiện nghĩa vụ tài chính theo thông báo.
+ [1]. Điều 611, 613, 620, 623, 651, 652, Luật 91/2015/QH13
+ [2]. Điều 57, 58, Luật 53/2014/QH13
+ [3]. Điều 137, Luật 31/2024/QH15
+ [4]. Điều 18, Nghị định 101/2024/NĐ-CP</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn các điều luật từ Bộ luật Dân sự 2015 (Điều 611, 613, 620, 623, 651, 652) và Luật Công chứng 2014 (Điều 57, 58) là đúng và còn hiệu lực. Tuy nhiên, câu trả lời cũng trích dẫn Điều 137 của Luật Đất đai 2024 và Điều 18 của Nghị định 101/2024/NĐ-CP, nhưng không có thông tin cụ thể về nội dung của các điều luật này, do đó không thể xác định tính chính xác và hiệu lực của chúng. Ngoài ra, cần lưu ý rằng Luật Đất đai 2024 và các nghị định liên quan đã thay thế hoàn toàn Luật Đất đai 2013 và các nghị định cũ, nên việc trích dẫn cần phải chính xác và cụ thể hơn.</t>
+  </si>
+  <si>
+    <t>Ở thanh hoá nhờ các bác tư vấn giúp là nhà e có sổ đỏ bị cháy mất sổ đứng tên bố e giờ ông chết còn bà giờ làm ntn nhờ các bác tư vấn giúp</t>
+  </si>
+  <si>
+    <t>Kết luận: Gia đình không thể chỉ xin cấp lại sổ đỏ mang tên bố vì bố đã mất. Cần làm thủ tục xác lập quyền thừa kế đối với thửa đất trước, sau đó người được hưởng thừa kế làm thủ tục đăng ký sang tên và được cấp Giấy chứng nhận mới; việc sổ bị cháy cần khai báo rõ khi nộp hồ sơ.
+ Gia đình chuẩn bị: giấy chứng tử của bố; CCCD của mẹ và các con; giấy tờ chứng minh quan hệ (khai sinh, đăng ký kết hôn); bản photo/chụp sổ đỏ nếu còn; giấy tờ về việc cháy sổ (nếu có).
+ Nếu bố có di chúc hợp pháp thì làm theo di chúc. Nếu không có di chúc, hàng thừa kế thứ nhất gồm: vợ, cha mẹ đẻ/nuôi và các con đẻ/nuôi của bố; những người này hưởng phần bằng nhau. Vì vậy, các con không thể tự để một mình mẹ đứng tên nếu chưa có văn bản thỏa thuận/phân chia hoặc từ chối nhận di sản của những người thừa kế khác. Điều 651 Bộ luật Dân sự 2015
+ Các đồng thừa kế đến tổ chức công chứng tại Thanh Hóa lập “Văn bản khai nhận di sản” hoặc “Văn bản thỏa thuận phân chia di sản”. Nếu thống nhất để mẹ nhận toàn bộ đất, văn bản cần ghi rõ các người thừa kế tặng cho/thỏa thuận để mẹ nhận phần di sản đó. Thời hiệu yêu cầu chia di sản là bất động sản là 30 năm từ thời điểm bố mất. Điều 623 Bộ luật Dân sự 2015
+ Sau khi có văn bản công chứng, nộp hồ sơ đăng ký biến động/sang tên tại Bộ phận một cửa cấp xã hoặc Văn phòng đăng ký đất đai/chi nhánh Văn phòng đăng ký đất đai nơi có đất ở Thanh Hóa. Hồ sơ thường gồm: đơn đăng ký biến động; văn bản thừa kế đã công chứng; giấy chứng tử; giấy tờ nhân thân; sổ đỏ còn lại hoặc văn bản trình bày việc sổ bị cháy, mất.
+ Việc cấp lại/cấp mới giấy chứng nhận trong trường hợp giấy cũ bị mất, hư hỏng được thực hiện theo thủ tục đăng ký đất đai; cơ quan tiếp nhận sẽ hướng dẫn thêm việc niêm yết, xác minh nếu cần. Nghị định 101/2024/NĐ-CP
+ Lưu ý: Nếu sổ đỏ là tài sản chung của bố mẹ hình thành trong thời kỳ hôn nhân, trước hết xác định phần của mẹ trong khối tài sản chung; chỉ phần thuộc bố mới chia thừa kế. Điều 33 Luật Hôn nhân và gia đình 2014
+ [1]. Điều 623, 651, Luật 91/2015/QH13
+ [2]. Nghị định 101/2024/NĐ-CP
+ [3]. Điều 33, Luật 52/2014/QH13</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 651 và Điều 623 của Bộ luật Dân sự 2015, và Điều 33 của Luật Hôn nhân và gia đình 2014, tất cả đều còn hiệu lực và đúng với vấn đề thừa kế và tài sản chung. Tuy nhiên, câu trả lời cũng trích dẫn Nghị định 101/2024/NĐ-CP, là văn bản mới và đúng hiệu lực, nhưng không có thông tin cụ thể về nội dung điều khoản nào được áp dụng. Cần bổ sung chi tiết về điều khoản cụ thể trong Nghị định 101/2024/NĐ-CP để đánh giá mức độ bao phủ.</t>
+  </si>
+  <si>
+    <t>Nhờ các ac giúp ạ. Giờ e làm thừa kế , bố e mất rồi ko có giấy khai sinh , mà ra tư pháp xin họ bảo Ng mất rồi họ ko cấp lại.xin xác nhận bố e là con của ông bà nhưng cũng ko đc. Hó bảo phải bên vpcc về xác minh . Mà vpcc thì họ ko có trách nhiệm làm vc đấy. Vậy giờ e phải làm thế nào ạ</t>
+  </si>
+  <si>
+    <t>Kết luận: Cơ quan tư pháp không thể chỉ trả lời miệng “người đã mất thì không cấp lại”. Bạn cần yêu cầu họ tiếp nhận hồ sơ đăng ký lại khai sinh hoặc trả lời từ chối bằng văn bản; nếu không còn đủ căn cứ để đăng ký lại, con đường phù hợp là yêu cầu Tòa án xác định quan hệ cha, mẹ, con để làm thủ tục thừa kế.
+ Thử thủ tục đăng ký lại khai sinh của bố bạn trước.
+ Người yêu cầu có thể là người thân thích; việc đăng ký lại được thực hiện khi sổ hộ tịch và bản chính giấy khai sinh đều bị mất, đồng thời có giấy tờ/tài liệu chứng minh nội dung khai sinh. Việc bố đã mất không phải tự nó là lý do để từ chối nhận, xem xét hồ sơ. Điều 24 Luật Hộ tịch 2014 Điều 25 Luật Hộ tịch 2014 Điều 26 Luật Hộ tịch 2014
+ Hồ sơ nên kèm mọi tài liệu cũ có ghi tên ông bà là cha mẹ của bố bạn: CCCD/CMND cũ, sổ hộ khẩu, lý lịch Đảng/đoàn, hồ sơ đi học, hồ sơ cán bộ, hồ sơ quân đội, giấy đăng ký kết hôn, giấy chứng tử, giấy tờ đất, hồ sơ bảo hiểm, hồ sơ khám chữa bệnh, giấy khai sinh của các anh chị em ruột của bố… Bản sao trích lục hộ tịch cũng là giấy tờ hộ tịch có giá trị như bản chính. Điều 6 Luật Hộ tịch 2014
+ Nộp tại UBND cấp xã có thẩm quyền về hộ tịch nơi trước đây bố bạn đăng ký khai sinh hoặc nơi bố bạn cư trú trước khi mất. Khi nộp, đề nghị cán bộ lập giấy tiếp nhận; nếu từ chối, yêu cầu nêu rõ căn cứ và trả lời bằng văn bản để có cơ sở khiếu nại hoặc khởi kiện hành chính.
+ Nếu không thể đăng ký lại khai sinh: nộp đơn tại TAND khu vực nơi bố bạn cư trú cuối cùng/yêu cầu xác định bố bạn là con của ông bà. Đây là việc dân sự thuộc thẩm quyền giải quyết của Tòa án; quyết định có hiệu lực của Tòa là căn cứ rất mạnh để công chứng khai nhận hoặc thỏa thuận phân chia di sản. Điều 29 Bộ luật Tố tụng dân sự 2015 Điều 101 Luật Hôn nhân và Gia đình 2014
+ Kèm theo đơn: giấy chứng tử của bố; giấy tờ của bạn chứng minh bạn là con của bố; giấy tờ của ông bà; toàn bộ tài liệu gián tiếp nêu trên; bản tường trình của người thân, hàng xóm; và đề nghị Tòa thu thập hồ sơ lưu tại công an, trường học, cơ quan công tác, cơ quan lưu trữ. Nếu còn người thân ruột của bố, nên đề nghị họ ký xác nhận hoặc tham gia phiên họp.
+ Văn phòng công chứng không có nghĩa vụ tự đi “xác minh” thay gia đình. Công chứng viên được quyền yêu cầu bổ sung tài liệu, xác minh hoặc yêu cầu giám định khi thấy cần thiết, nhưng không thể thay Tòa án xác lập quan hệ cha mẹ con khi chứng cứ hộ tịch không còn. Điều 40 Luật Công chứng 2014 Điều 57 Luật Công chứng 2014
+ Lưu ý: nếu đang gần hết thời hiệu yêu cầu chia di sản thì cần nộp yêu cầu tại Tòa sớm. Thời hiệu yêu cầu chia di sản là 30 năm với bất động sản và 10 năm với động sản, tính từ thời điểm bố bạn mất. Điều 623 Bộ luật Dân sự 2015
+ [1]. Điều 6, 24, 25, 26, Luật 60/2014/QH13
+ [2]. Điều 29, Luật 92/2015/QH13
+ [3]. Điều 101, Luật 52/2014/QH13
+ [4]. Điều 40, 57, Luật 53/2014/QH13
+ [5]. Điều 623, Luật 91/2015/QH13</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn các điều luật từ Luật Hộ tịch 2014, Bộ luật Tố tụng dân sự 2015, Luật Hôn nhân và Gia đình 2014, Luật Công chứng 2014 và Bộ luật Dân sự 2015. Tuy nhiên, các văn bản này đã bị thay thế hoặc hết hiệu lực bởi các văn bản mới từ năm 2024. Do đó, việc trích dẫn các điều luật này là không còn hiệu lực hiện hành. Câu trả lời đã bao phủ vấn đề về thủ tục đăng ký lại khai sinh và xác định quan hệ cha mẹ con qua Tòa án, nhưng cần cập nhật điều luật mới để đảm bảo tính chính xác và hiệu lực.</t>
+  </si>
+  <si>
+    <t>Kết luận: Tầng hầm bạn mô tả có thể được ghi nhận là công trình xây dựng/tài sản gắn liền với đất khi xác minh hiện trạng, nhưng không tự động làm đất khai hoang đủ điều kiện cấp sổ đỏ lần đầu. Cơ quan có thẩm quyền sẽ xét riêng nguồn gốc, thời điểm sử dụng đất, quy hoạch, tranh chấp và việc xây dựng có hợp pháp hay không.
+ Tầng hầm có móng, dầm, cột, sàn bê tông, cầu thang, bể phốt là kết cấu kiên cố; nên đề nghị đoàn xác minh lập biên bản ghi rõ: diện tích, vị trí, kết cấu, mục đích sử dụng, thời điểm xây dựng thực tế từ năm 2013 và tình trạng đang tồn tại. Thông tin về nhà/công trình, nguồn gốc sử dụng đất, thời điểm sử dụng và tranh chấp là nội dung được kiểm tra khi đăng ký đất đai lần đầu Điều 11 Thông tư 10/2024/TT-BTNMT.
+ Tuy nhiên, để được cấp sổ, gia đình cần chứng minh việc sử dụng đất ổn định và không tranh chấp; đồng thời đất không thuộc trường hợp bị loại trừ như đất công, hành lang bảo vệ công trình, quy hoạch phải thu hồi hoặc khu vực không được công nhận. Nếu nguồn gốc thực tế bị xác định là lấn, chiếm nhưng đã sử dụng làm nhà ở trước 01/7/2014, không thuộc quy hoạch rừng đặc dụng/rừng phòng hộ hoặc công trình hạ tầng công cộng, vẫn có thể được xem xét cấp giấy và phải thực hiện nghĩa vụ tài chính Điều 139 Luật Đất đai 2024.
+ Lưu ý quan trọng: công trình xây năm 2013 không đồng nghĩa với “hợp lệ” về xây dựng. Nếu thời điểm đó công trình thuộc diện phải có giấy phép xây dựng nhưng không có giấy phép, tầng hầm có thể vẫn được ghi nhận hiện trạng, nhưng việc chứng nhận quyền sở hữu công trình hoặc xử lý vi phạm xây dựng sẽ được xem xét riêng.
+ Gia đình nên nộp/kèm: ảnh công trình qua các năm; xác nhận của người liền kề hoặc tổ dân phố; biên lai điện, nước, thuế; hồ sơ bản vẽ/biên bản xây dựng (nếu có); giấy tờ về việc khai hoang, giao đất hoặc xác nhận sử dụng đất của UBND xã. Khi biên bản xác minh ghi không đúng hiện trạng hoặc không ghi nhận tầng hầm, gia đình nên yêu cầu ghi ý kiến trực tiếp vào biên bản và giữ một bản/chụp lại.
+ [1]. Điều 11, Thông tư 10/2024/TT-BTNMT
+ [2]. Điều 139, Luật 31/2024/QH15</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn Điều 11 của Thông tư 10/2024/TT-BTNMT và Điều 139 của Luật Đất đai 2024 (Luật số 31/2024/QH15). Cả hai văn bản này đều còn hiệu lực và liên quan đến việc xác minh công trình xây dựng và điều kiện cấp sổ đỏ lần đầu cho đất khai hoang. Điều 11 Thông tư 10/2024/TT-BTNMT quy định về việc kiểm tra thông tin khi đăng ký đất đai lần đầu, bao gồm công trình xây dựng trên đất. Điều 139 Luật Đất đai 2024 quy định về việc cấp giấy chứng nhận quyền sử dụng đất cho đất có nguồn gốc lấn, chiếm nhưng đã sử dụng ổn định trước 01/7/2014. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý cần thiết cho câu hỏi của người dùng.</t>
+  </si>
+  <si>
+    <t>Mọi người cho em hỏi,em lam hồ so cap sổ
+ lần đầu, hạn nộp thuế nhà nước cho hạn là
+ trong vòng bao nhiêu ngày!</t>
+  </si>
+  <si>
+    <t>Kết luận: Khi làm sổ lần đầu, thời hạn nộp tiền không tính từ ngày nộp hồ sơ mà tính theo Thông báo nộp tiền của cơ quan thuế. Thông thường, khoản tiền sử dụng đất phải nộp sẽ có hạn theo pháp luật quản lý thuế; nếu được ghi nợ thì nộp theo thời hạn ghi nợ.
+ Đối với hộ gia đình, cá nhân được cấp Giấy chứng nhận lần đầu, thông báo thuế phải ghi rõ: thời hạn nộp khoản tiền sử dụng đất không được ghi nợ theo pháp luật quản lý thuế và thời hạn nộp khoản được ghi nợ (nếu có) Điều 22 Nghị định 103/2024/NĐ-CP.
+ Bạn nên xem chính xác dòng “thời hạn nộp tiền” trên thông báo của cơ quan thuế. Nộp quá hạn có thể bị tính tiền chậm nộp theo quy định thuế.
+ [1]. Điều 22, Nghị định 103/2024/NĐ-CP</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 22 của Nghị định 103/2024/NĐ-CP, là văn bản còn hiệu lực, quy định về thời hạn nộp tiền sử dụng đất khi cấp Giấy chứng nhận lần đầu. Điều luật này đã bao phủ phần chính của câu hỏi về thời hạn nộp thuế khi làm hồ sơ cấp sổ lần đầu. Tuy nhiên, câu trả lời không nêu rõ thời hạn cụ thể mà chỉ hướng dẫn người dùng kiểm tra thông báo của cơ quan thuế, điều này là hợp lý vì thời hạn cụ thể có thể khác nhau tùy trường hợp.</t>
+  </si>
+  <si>
+    <t>Gần đây mình có oàn thiện một hồ sơ về đất đai, và khi nộp thì có nộp bản chính giấy khai sinh. Mọi người cho mình hỏi là:
+ - Có bắt buộc nộp giấy khai sinh trong hồ sơ không?
+ - Nếu không thì liên hệ với cơ quan liên quan để xin rút bản chính, nộp bản sao ạ?
+ - Trong trường hợp không xin rút được thì xử lí như thế nào?</t>
+  </si>
+  <si>
+    <t>Kết luận: Không phải mọi hồ sơ đất đai đều bắt buộc nộp bản chính Giấy khai sinh. Bạn nên liên hệ ngay nơi đã tiếp nhận hồ sơ để đề nghị trả lại bản chính và thay bằng bản sao chứng thực hoặc bản sao kèm xuất trình bản chính đối chiếu, nếu thành phần hồ sơ không bắt buộc phải lưu bản chính.
+ Khi nộp trực tiếp hồ sơ đất đai, bạn có quyền chọn nộp bản sao và xuất trình bản chính để đối chiếu, hoặc nộp bản sao đã được chứng thực; không nhất thiết phải giao luôn bản chính cho cơ quan tiếp nhận. Khoản 2 Điều 12 Nghị định 102/2024/NĐ-CP
+ Bạn nên làm phiếu/đơn đề nghị rút lại bản chính Giấy khai sinh, ghi: họ tên, mã hồ sơ/ngày nộp, tên thủ tục đất đai, đề nghị nhận lại bản chính và nộp thay bằng bản sao chứng thực. Mang theo CCCD, phiếu tiếp nhận hồ sơ và bản sao chứng thực Giấy khai sinh đến Bộ phận Một cửa hoặc Văn phòng đăng ký đất đai nơi nhận hồ sơ.
+ Nếu cơ quan nói không thể trả, bạn hãy yêu cầu họ trả lời rõ bằng văn bản hoặc ghi trên phiếu hướng dẫn: Giấy khai sinh là thành phần hồ sơ nào và căn cứ nào buộc phải nộp bản chính. Trường hợp bản chính thực sự cần để giải quyết thủ tục, cơ quan phải bảo quản và hoàn trả theo quy trình khi không còn cần thiết; bạn nên giữ phiếu biên nhận thể hiện đã nộp bản chính.
+ Nếu bị thất lạc hoặc không thể lấy lại, bạn có thể xin bản sao trích lục khai sinh tại UBND cấp xã nơi đã đăng ký khai sinh trước đây hoặc bất kỳ UBND cấp xã có thẩm quyền khai thác dữ liệu hộ tịch. Bản sao trích lục hộ tịch có giá trị sử dụng thay cho bản chính trong giao dịch, trừ trường hợp pháp luật quy định khác. Điều 63 Luật Hộ tịch 2014
+ [1]. Điều 12, Nghị định 102/2024/NĐ-CP
+ [2]. Điều 63, Luật 60/2014/QH13</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 12 Nghị định 102/2024/NĐ-CP và Điều 63 Luật Hộ tịch 2014. Tuy nhiên, Nghị định 102/2024/NĐ-CP là văn bản mới và có thể chưa được phổ biến rộng rãi, cần kiểm tra lại tính chính xác của điều luật này. Điều 63 Luật Hộ tịch 2014 là đúng và còn hiệu lực, nhưng không trực tiếp liên quan đến việc nộp giấy khai sinh trong hồ sơ đất đai. Câu trả lời đã bao phủ phần lớn câu hỏi về việc xử lý khi đã nộp bản chính giấy khai sinh, nhưng cần kiểm tra lại điều luật cụ thể về việc nộp giấy khai sinh trong hồ sơ đất đai.</t>
+  </si>
+  <si>
+    <t>Em mới bán căn chung cư studio ( là tải sản duy nhất tính đến thời điểm hiện tại của hai vợ chồng). Khi bán là dc tư vấn là miễn thuế thu nhập cá nhân do là tai sản duy nhất. Tuy nhiên, cục thuế mới thông báo tụi e ko được miễn, do còn có tài sản thứ 2, là mảnh đất đã được tụi em bán cách đây 5 năm. Thuế yêu cầu phải về Văn phòng công chứng xin trích lục chứng minh hợp đồng mua bán của mảnh này.
+Cách đây 5 năm, Ông chủ Lý bán mảnh đất này có số thửa là 888-1, số tờ 2 cho vợ chồng em. Mảnh này là lô nhỏ tách ra từ thửa lớn của ông, khi bán có các con và vợ có đồng ý kí bán.
+Sau vài năm vợ chồng e bán lại thửa 888-1, tơ số 2 cho ông khách Lâm, thửa này sau khi bán thì đổi tên số thửa là 1012, số tờ 10.
+Thực chất 2 thửa này là 1. Em mua và bán lại khách khác thôi. Nhưng giờ thuế tra ra thửa 888-1 đầu tiên vẫn là sở hữu của chồng em. Nên ko dc giảm thuế TNCN khi bán căn chung cư . Họ yêu cầu xác minh Hợp đồng mua bán của thửa 888-1, chứng minh vc chỉ có tài sản duy nhất. Vợ chồng em làm sao chứng minh dc 2 mảnh này là 1 và đã bán đi rồi ạ.
+Đi văn phòng công chứng đã công chứng cho manh 888-1 thì chỉ chưng minh dc quyền nhận chuyển nhượng mảnh này.
+Đi vpcc đã công chứng manh 1012, thì chỉ trích lục dc dã bán mảnh 1012.
+Làm sao chứng minh vc e chỉ có tài sản duy nhất là căn chung cư hiện tại ạ?
+Em đang rất rối. Mong quy anh chị tư vấn giúp ạ</t>
+  </si>
+  <si>
+    <t>Kết luận: Nếu thửa 888-1 thực tế đã được chuyển nhượng cho ông Lâm và sau khi chỉnh lý địa chính được đổi thành thửa 1012, thì tại thời điểm bán căn studio vợ chồng bạn không còn quyền sử dụng thửa đất đó. Bạn cần chứng minh “chuỗi lịch sử biến động” giữa hai số thửa; giấy trích lục riêng từng hợp đồng công chứng thường chưa đủ.
+ Việc cần làm ngay
+ Đến Văn phòng đăng ký đất đai/Chi nhánh Văn phòng đăng ký đất đai nơi có đất, nộp đơn đề nghị:
+ cung cấp thông tin, trích lục hồ sơ địa chính;
+ xác nhận lịch sử biến động của thửa 888-1, tờ bản đồ 2 sang thửa 1012, tờ bản đồ 10;
+ xác nhận thửa 1012 là thửa đất được cấp đổi/chỉnh lý/đánh số lại từ thửa 888-1;
+ xác nhận việc đăng ký sang tên cho ông Lâm và tình trạng vợ chồng bạn đã không còn đứng tên trên thửa đất này.
+ Yêu cầu quan trọng nhất là văn bản xác nhận phải ghi rõ: “thửa 888-1 tờ bản đồ số 2 và thửa 1012 tờ bản đồ số 10 là cùng một vị trí/thửa đất sau khi đo đạc, chỉnh lý hoặc thay đổi số thửa, số tờ bản đồ”. Khi biên tập lại bản đồ địa chính, số thửa có thể được đánh lại và phải có bảng tham chiếu số thửa cũ – số thửa mới Điều 18 Thông tư 26/2024/TT-BTNMT.
+ Xin kèm các giấy tờ có thể hiện liên kết giữa hai thửa:
+ hồ sơ cấp Giấy chứng nhận hoặc hồ sơ đăng ký biến động khi sang tên ông Lâm;
+ trang biến động trên Giấy chứng nhận cũ (nếu còn);
+ trích đo địa chính, mảnh trích đo, sơ đồ thửa đất;
+ bảng đối chiếu số thửa cũ và số thửa mới;
+ văn bản trả lời chính thức của Văn phòng đăng ký đất đai.
+ Nộp cho cơ quan thuế một bộ giải trình gồm:
+ hợp đồng công chứng mua thửa 888-1;
+ hợp đồng công chứng bán cho ông Lâm (thửa 1012);
+ bản sao Giấy chứng nhận/sơ đồ thửa đất của các giao dịch nếu có;
+ đặc biệt là văn bản xác nhận lịch sử biến động của Văn phòng đăng ký đất đai;
+ đơn giải trình nêu rõ: thửa 1012 không phải tài sản thứ hai, mà là chính thửa 888-1 sau đổi số thửa/tờ bản đồ và đã bán từ 5 năm trước.
+ Theo quy định hiện hành, điều kiện miễn thuế là tại thời điểm chuyển nhượng căn studio, người chuyển nhượng chỉ có một nhà ở hoặc một thửa đất ở; đồng thời phải đáp ứng điều kiện thời gian sở hữu và chuyển nhượng toàn bộ nhà/đất đó Điều 19 Nghị định 253/2026/NĐ-CP. Vì vậy, trọng tâm không phải chứng minh vợ chồng bạn “chưa từng có đất”, mà chứng minh tại ngày ký bán căn studio, đất cũ đã không còn thuộc quyền sử dụng của vợ chồng bạn.
+ Mẫu nội dung đơn đề nghị xác nhận
+ Kính đề nghị Văn phòng đăng ký đất đai tra cứu, cung cấp trích lục hồ sơ địa chính và xác nhận lịch sử biến động đối với thửa đất số 888-1, tờ bản đồ số 2 và thửa đất số 1012, tờ bản đồ số 10.
+ Đề nghị xác nhận hai số thửa nêu trên có phải cùng một thửa đất/vị trí đất trước và sau khi đo đạc, chỉnh lý hoặc thay đổi số thửa, số tờ bản đồ hay không; thời điểm vợ chồng tôi chuyển nhượng quyền sử dụng đất cho ông Lâm; và tình trạng hiện nay vợ chồng tôi không còn đăng ký quyền sử dụng đất đối với thửa đất nêu trên.
+ Mục đích sử dụng: bổ sung hồ sơ giải trình miễn thuế thu nhập cá nhân khi chuyển nhượng nhà ở duy nhất.
+ Nếu cơ quan thuế chỉ thông báo miệng, bạn nên đề nghị họ lập thông báo/yêu cầu bổ sung hồ sơ bằng văn bản, để biết rõ thời hạn và nội dung phải chứng minh. Nộp bộ giải trình có phiếu tiếp nhận, yêu cầu cơ quan thuế trả lời bằng văn bản về việc chấp nhận hay không chấp nhận miễn thuế.
+ [1]. Điều 18, Thông tư 26/2024/TT-BTNMT
+ [2]. Điều 19, Nghị định 253/2026/NĐ-CP</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 18 Thông tư 26/2024/TT-BTNMT và Điều 19 Nghị định 253/2026/NĐ-CP. Tuy nhiên, cả hai văn bản này đều không tồn tại trong thực tế, do đó vi phạm tiêu chí về tính tồn tại và hiệu lực của điều luật. Câu trả lời đã bao phủ phần lớn vấn đề pháp lý liên quan đến việc chứng minh tài sản duy nhất để được miễn thuế thu nhập cá nhân, nhưng việc trích dẫn điều luật không chính xác làm giảm độ tin cậy của câu trả lời.</t>
+  </si>
+  <si>
+    <t>Kind 2 - Quyền, nghĩa vụ và việc sử dụng đất</t>
+  </si>
+  <si>
+    <t>Anh chị cho em hỏi là Nghị quyết số 254/2025/QH15 của Quốc hội,trong đó có việc giảm 70% tiền SDĐ khi chuyển mục đích lần đầu có thật hay ko? Em nộp hs đề nghị được chuyển mục đích từ tháng 10 năm 2025 và nay đã có thông báo nộp tiền SDĐ nhưng chưa được giảm trong văn bản thông báo thì giờ em phải làm ntn? Nhờ mn hiểu biết hướng dẫn giúp ạ. Em xin cảm ơn</t>
+  </si>
+  <si>
+    <t>Kết luận: Có. Nghị quyết 254/2025/QH15 có quy định ưu đãi khi chuyển lần đầu từ đất vườn, ao hoặc đất nông nghiệp trong cùng thửa có đất ở sang đất ở; nhưng không phải “giảm 70%” cho mọi trường hợp. Với diện tích trong hạn mức đất ở, bạn chỉ nộp 30% phần chênh lệch, tức giảm tương đương 70% phần chênh lệch.
+ Nghị quyết có hiệu lực từ 01/01/2026. Người đã được quyết định cho phép chuyển mục đích trong giai đoạn 01/8/2024 đến trước 01/01/2026, nếu chưa nộp tiền theo thông báo thuế,</t>
+  </si>
+  <si>
+    <t>Câu trả lời không trích dẫn điều luật cụ thể nào từ Nghị quyết 254/2025/QH15. Ngoài ra, thông tin về việc "giảm 70%" không được xác nhận rõ ràng và không có căn cứ pháp lý cụ thể nào được nêu ra. Câu trả lời cũng không cung cấp hướng dẫn cụ thể cho người dùng về cách xử lý tình huống hiện tại của họ.</t>
+  </si>
+  <si>
+    <t>Cho e hỏi nếu đất đồng sở hữu nhưng chưa xác định diênn tích của từng cá nhân trong đó thì bây giờ cần phải làm gì ạ?</t>
+  </si>
+  <si>
+    <t>Kết luận: Nếu đất đang đồng sở hữu mà chưa xác định phần diện tích của từng người, trước hết các đồng sở hữu nên lập văn bản thỏa thuận phân chia quyền sử dụng đất. Nếu không thể thỏa thuận, một hoặc nhiều người có thể yêu cầu Tòa án chia tài sản chung.
+ Việc chia chỉ thực hiện được khi thửa đất đáp ứng điều kiện tách thửa theo quy định địa phương và phù hợp quy hoạch. Các bên nên thống nhất rõ: mỗi người nhận vị trí nào, diện tích bao nhiêu m², lối đi chung (nếu có), chi phí đo đạc và nghĩa vụ thuế/phí.
+ Sau khi thỏa thuận, thực hiện theo trình tự:
+ Thuê đo đạc, lập bản vẽ hiện trạng và phương án chia thửa.
+ Lập văn bản phân chia có công chứng/chứng thực.
+ Nộp hồ sơ đăng ký biến động, tách thửa và cấp Giấy chứng nhận riêng tại cơ quan đăng ký đất đai cấp tỉnh/xã theo cơ chế tiếp nhận hồ sơ hiện hành.
+ Nhận sổ riêng cho từng người nếu đủ điều kiện.
+ Khi chưa chia, Giấy chứng nhận phải ghi đầy đủ tên các người có chung quyền sử dụng đất; nếu cử một người đại diện đứng tên thì phải có văn bản thỏa thuận đại diện. Điều 12 Thông tư 10/2024/TT-BTNMT
+ Lưu ý: Một người không được tự ý bán, tặng cho, thế chấp “phần đất của mình” khi phần đó chưa được xác định; việc định đoạt quyền sử dụng đất chung cần sự đồng ý của các đồng sở hữu, trừ trường hợp có thỏa thuận hoặc bản án khác. Điều 218 Bộ luật Dân sự 2015
+ Nếu bạn cho biết đất ở tỉnh/thành nào, tổng diện tích, loại đất và hiện có sổ chung hay chưa, có thể xác định cụ thể có đủ điều kiện tách thửa hay không.
+ [1]. Điều 12, Thông tư 10/2024/TT-BTNMT</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 12 Thông tư 10/2024/TT-BTNMT và Điều 218 Bộ luật Dân sự 2015. Tuy nhiên, Thông tư 10/2024/TT-BTNMT không tồn tại, do đó vi phạm tiêu chí về trích dẫn điều luật. Điều 218 Bộ luật Dân sự 2015 là đúng và còn hiệu lực, nhưng không đủ để bao quát toàn bộ vấn đề về đồng sở hữu đất đai và tách thửa.</t>
+  </si>
+  <si>
+    <t>Anh chị luật sư cho e hỏi chút. E ở HN, mảnh đất nhà e được cấp sổ năm 2004 diện tích là 900m². Trong sổ có ghi đất sử dụng 250m² T (lâu dài) và 650m² vườn. 
+ Nhưng diện tích thực tế hiện tại khoảng 1300m². Đất nhà e có 2 mặt giáp suối.
+ Giờ bố mẹ e muốn cho tặng cho 2 con thì thủ tục như thế nào và trường hợp đất thực tế nhiều hơn so với sổ thì xử lý như thế nào ạ. Anh chị tư vấn giúp em.
+ E cảm ơn ạ !</t>
+  </si>
+  <si>
+    <t>Kết luận: Bố mẹ bạn chỉ nên làm thủ tục tặng cho sau khi đo đạc, xác định rõ phần đất thực tế tăng thêm 400 m² có thuộc quyền sử dụng hợp pháp hay không. Phần 900 m² đã ghi trên sổ có thể tặng cho nếu đủ điều kiện; còn 400 m² chênh lệch không tự động được công nhận và không nên đưa vào hợp đồng tặng cho khi chưa được cơ quan đăng ký đất đai xác nhận.
+ 1. Xử lý diện tích thực tế 1.300 m²
+ Sổ năm 2004 đang xác nhận tổng diện tích 900 m² gồm 250 m² đất ở/lâu dài và 650 m² đất vườn. Việc thực tế đang sử dụng khoảng 1.300 m² cần đo đạc địa chính chính thức, xác định ranh giới với các hộ liền kề và đặc biệt là mốc hành lang, đất công ven suối.
+ Nếu 400 m² tăng thêm chỉ là sai số đo đạc, ranh giới sử dụng ổn định, không tranh chấp, không lấn đất công/hành lang suối: gia đình có thể đề nghị đăng ký biến động hoặc cấp đổi sổ theo số liệu đo đạc thực tế.
+ Nếu phần tăng thêm là đất ven suối, đất do Nhà nước quản lý, đất thuộc hành lang bảo vệ nguồn nước hoặc có dấu hiệu lấn chiếm: không được công nhận để tặng cho; có thể phải trả lại phần đất đó.
+ “Giáp suối” không đồng nghĩa toàn bộ đất gia đình đang dùng là hợp pháp. Cần kiểm tra chỉ giới hành lang bảo vệ nguồn nước và hồ sơ địa chính tại địa phương trước.
+ Người sử dụng đất chỉ được tặng cho khi có Giấy chứng nhận, đất không tranh chấp, không bị kê biên, còn thời hạn sử dụng và không bị áp dụng biện pháp khẩn cấp tạm thời Điều 45 Luật Đất đai 2024.
+ 2. Tặng cho hai người con: cần tách thửa hay không?
+ Nếu bố mẹ muốn mỗi người con đứng tên một phần đất riêng: phải làm thủ tục tách thửa trước hoặc tách thửa đồng thời với thủ tục tặng cho. Diện tích, kích thước từng thửa sau tách phải đáp ứng quy định đang áp dụng tại Hà Nội; phần đất ở và đất vườn cần được thể hiện rõ theo từng thửa.
+ Nếu bố mẹ muốn hai con cùng đứng tên chung toàn bộ thửa đất: không nhất thiết tách thửa; có thể lập hợp đồng tặng cho quyền sử dụng đất cho hai người con theo tỷ lệ cụ thể, ví dụ mỗi người 1/2.
+ Do đất có hai loại mục đích sử dụng, khi chia nên xác định rõ: mỗi con được nhận bao nhiêu m² đất ở và bao nhiêu m² đất vườn. Không nên tự ghi toàn bộ diện tích là đất ở vì đất vườn không tự chuyển thành đất ở.
+ 3. Trình tự nên thực hiện
+ Liên hệ Văn phòng đăng ký đất đai/chi nhánh nơi có đất để đề nghị trích đo địa chính, kiểm tra ranh giới, diện tích chênh lệch và tình trạng đất ven suối.
+ Nếu đủ điều kiện, làm thủ tục cấp đổi/chỉnh lý Giấy chứng nhận theo kết quả đo đạc; nếu muốn chia riêng thì lập hồ sơ tách thửa.
+ Sau khi diện tích hợp pháp được xác định, bố mẹ và các con lập hợp đồng tặng cho tại tổ chức công chứng.
+ Nộp hồ sơ đăng ký biến động sang tên tại cơ quan đăng ký đất đai. Hồ sơ cơ bản gồm: sổ gốc, hợp đồng tặng cho đã công chứng, giấy tờ nhân thân, giấy tờ chứng minh quan hệ cha mẹ–con và hồ sơ tách thửa nếu có.
+ 4. Thuế, phí
+ Tặng cho quyền sử dụng đất giữa cha mẹ và con thuộc trường hợp được miễn thuế thu nhập cá nhân và miễn lệ phí trước bạ, nếu hồ sơ chứng minh đúng quan hệ cha mẹ–con. Gia đình vẫn có thể phải nộp phí đo đạc, phí thẩm định, phí cấp/cấp đổi sổ và nghĩa vụ tài chính nếu được công nhận thêm diện tích đất ngoài sổ.
+ Lưu ý quan trọng: Không ký hợp đồng tặng cho theo diện tích “khoảng 1.300 m²” khi sổ mới ghi 900 m². Hợp đồng chỉ nên ghi theo diện tích hợp pháp trên Giấy chứng nhận hoặc theo hồ sơ đo đạc đã được cơ quan có thẩm quyền chấp nhận.
+ [1]. Điều 45, Luật 31/2024/QH15</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn Điều 45 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là văn bản hiện hành và có hiệu lực từ 01/08/2024. Điều luật này quy định về điều kiện để người sử dụng đất có thể thực hiện quyền tặng cho quyền sử dụng đất, bao gồm việc đất phải có Giấy chứng nhận, không tranh chấp, không bị kê biên, còn thời hạn sử dụng và không bị áp dụng biện pháp khẩn cấp tạm thời. Câu trả lời đã bao phủ đầy đủ các khía cạnh của câu hỏi, bao gồm xử lý diện tích đất thực tế lớn hơn so với sổ và thủ tục tặng cho quyền sử dụng đất.</t>
+  </si>
+  <si>
+    <t>NN giao đất cho TC kinh tế, nham bố trí
+ nhà ở cho cán bộ, nviên trong đơn vị. Cán
+ bộ nviên có được bán lại cho người ngoài
+ đvị k ?</t>
+  </si>
+  <si>
+    <t>Kết luận: Không thể khẳng định cán bộ, nhân viên được tự bán nhà/đất cho người ngoài đơn vị. Việc bán chỉ hợp pháp khi người đó đã được Nhà nước hoặc tổ chức giao/bán hợp pháp và đã có quyền sở hữu nhà, quyền sử dụng đất riêng; đồng thời không bị hạn chế chuyển nhượng theo quyết định giao đất, hồ sơ dự án hoặc loại nhà ở.
+ Nếu đất được Nhà nước giao trực tiếp cho tổ chức kinh tế để bố trí chỗ ở nội bộ, thì tổ chức là bên có quyền đối với đất. Cán bộ, nhân viên chỉ được bố trí ở, thuê hoặc thuê mua thường chưa đương nhiên có quyền bán cho người khác. Người tự ý bán khi chưa được cấp Giấy chứng nhận hoặc chưa được tổ chức chuyển quyền hợp pháp thì giao dịch có nguy cơ vô hiệu.
+ Chỉ có thể bán ra ngoài đơn vị khi, tối thiểu:
+ Người bán đã đứng tên Giấy chứng nhận đối với nhà ở/quyền sử dụng đất hoặc đủ điều kiện được cấp Giấy chứng nhận;
+ Nhà, đất không có tranh chấp, không bị kê biên, còn thời hạn sử dụng và không thuộc trường hợp pháp luật cấm/chưa cho chuyển nhượng;
+ Việc bán phù hợp với quy định của dự án và văn bản giao đất; nếu là nhà ở xã hội, nhà công vụ, nhà thuộc tài sản công hoặc nhà được ưu đãi thì có hạn chế riêng;
+ Hợp đồng chuyển nhượng được công chứng/chứng thực theo quy định và đăng ký biến động. Điều 45 Luật Đất đai 2024 Điều 164 Luật Nhà ở 2023
+ Cần phân biệt: nếu đây là nhà công vụ hoặc nhà do cơ quan/đơn vị bố trí để ở trong thời gian công tác thì không được mua bán như tài sản riêng. Điều 32 Luật Nhà ở 2023
+ Bạn nên kiểm tra 3 giấy tờ: quyết định Nhà nước giao đất cho tổ chức, hợp đồng/quyết định phân nhà cho cán bộ nhân viên, và Giấy chứng nhận của căn nhà/đất. Chỉ cần một trong các giấy tờ này ghi “không được chuyển nhượng”, “chỉ để bố trí nội bộ”, hoặc chưa tách/cấp sổ riêng thì không nên giao dịch với người ngoài đơn vị.
+ [1]. Điều 45, Luật 31/2024/QH15
+ [2]. Điều 32, 164, Luật 27/2023/QH15</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 45 Luật Đất đai 2024 và Điều 32, 164 Luật Nhà ở 2023. Tuy nhiên, không có nội dung cụ thể của các điều luật này được nêu ra trong câu trả lời, và không có thông tin nào xác nhận rằng các điều luật này có liên quan trực tiếp đến vấn đề chuyển nhượng nhà ở cho cán bộ, nhân viên trong tổ chức kinh tế. Do đó, không thể xác nhận tính đúng đắn và hiệu lực của các điều luật được trích dẫn.</t>
+  </si>
+  <si>
+    <t>Mọi người cho e tham khảo với ạ: chồng e được hợp đồng uỷ quyền toàn phần sổ đỏ của chính và theo e biết thì chồng e giờ không đứng tên sổ đất đó được vì là người được uỷ quyền đúng không các ơi.
+ Và nếu giờ chồng e cho e đứng tên có được không ạ và phải làm bước nào cho hợp lí , mong mọi người tham vấn giúp em với ạ. E cám mn nhiều ❤️</t>
+  </si>
+  <si>
+    <t>Kết luận: Chồng bạn không thể dùng giấy ủy quyền để tự chuyển sổ đất từ chủ đất sang chính tên chồng bạn. Tuy nhiên, chồng bạn có thể đại diện chủ đất để ký hợp đồng chuyển nhượng hoặc tặng cho cho bạn, nếu giấy ủy quyền còn hiệu lực và ghi rõ quyền định đoạt/chuyển nhượng/tặng cho; việc này cần bảo đảm không trái phạm vi ủy quyền và ý chí của chủ đất.
+ Người được ủy quyền là người đại diện cho chủ đất, không phải là chủ sở hữu đất. Vì vậy, chồng bạn không được xác lập giao dịch mà bên chuyển là chủ đất (do chồng đại diện) và bên nhận lại chính là chồng bạn; đây là giao dịch với chính mình, có nguy cơ vô hiệu nếu không có sự đồng ý/ủy quyền hợp lệ từ chủ đất. Điều 141 Bộ luật Dân sự 2015
+ Nếu chuyển sang tên bạn, chồng bạn là người đại diện bên chuyển, còn bạn là bên nhận nên về nguyên tắc không phải giao dịch “với chính mình”. Nhưng cần kiểm tra kỹ giấy ủy quyền có cho phép chồng bạn: ký hợp đồng chuyển nhượng/tặng cho; nộp hồ sơ; kê khai và nộp thuế, phí; làm thủ tục sang tên hay không. Nếu giấy chỉ ghi “quản lý”, “làm thủ tục hành chính” thì chưa đủ để bán/tặng cho.
+ Cách an toàn nhất là để chủ đất trực tiếp ký hợp đồng tặng cho/chuyển nhượng cho bạn tại tổ chức công chứng. Nếu chủ đất không thể ký, nên lập lại văn bản ủy quyền công chứng, ghi rõ chồng bạn được ký hợp đồng chuyển nhượng hoặc tặng cho quyền sử dụng đất cho bạn, giá trị giao dịch (nếu mua bán), quyền nộp hồ sơ và nhận kết quả.
+ Đất phải có Giấy chứng nhận, không tranh chấp, không bị kê biên, còn thời hạn sử dụng và không bị áp dụng biện pháp khẩn cấp tạm thời mới đủ điều kiện chuyển nhượng/tặng cho. Điều 45 Luật Đất đai 2024 Hợp đồng chuyển nhượng hoặc tặng cho quyền sử dụng đất phải được công chứng hoặc chứng thực. Điều 27 Luật Đất đai 2024
+ Lưu ý thêm: nếu bạn và chồng đã kết hôn, đất đứng tên riêng bạn nhưng tiền mua là tài sản chung vợ chồng thì vẫn có thể phát sinh tranh chấp về tài sản chung. Nếu muốn là tài sản riêng của bạn, nên chọn hình thức tặng cho riêng bạn và ghi rõ trong hợp đồng: “tặng cho riêng bà…; không nhập vào tài sản chung vợ chồng”.
+ [1]. Điều 141, Luật 91/2015/QH13
+ [2]. Điều 27, 45, Luật 31/2024/QH15</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn Điều 141 Bộ luật Dân sự 2015 về quyền và nghĩa vụ của người được ủy quyền, điều này còn hiệu lực và phù hợp với tình huống. Ngoài ra, câu trả lời cũng trích dẫn Điều 27 và 45 của Luật Đất đai 2024 (Luật số 31/2024/QH15), đây là luật mới có hiệu lực từ 01/08/2024, thay thế Luật Đất đai 2013. Điều 27 quy định về công chứng, chứng thực hợp đồng chuyển nhượng hoặc tặng cho quyền sử dụng đất, và Điều 45 quy định về điều kiện chuyển nhượng, tặng cho quyền sử dụng đất. Các điều luật này đều còn hiệu lực và phù hợp với vấn đề pháp lý được hỏi.</t>
+  </si>
+  <si>
+    <t>Em muốn hỏi vấn đề như sau ạ:
+ Sổ đỏ đứng tên 2 người đồng sở hữu.Nhưng hiện tại muốn bán mảnh đất.Nhưng vì lý do địa lý đi làm xa.Đã làm hợp đồng uỷ quyền lại có công chứng của văn phòng công chứng giao toàn quyền cho người còn lại quyết định mọi thủ tục liên quan.
+ Nhưng vẫn không thực hiện được là sao ạ</t>
+  </si>
+  <si>
+    <t>Kết luận: Có hợp đồng ủy quyền công chứng chưa chắc người được ủy quyền đã tự ký bán đất được. Văn phòng công chứng thường từ chối nếu văn bản ủy quyền không ghi thật rõ quyền ký hợp đồng chuyển nhượng, nhận tiền, nộp hồ sơ sang tên; hoặc nếu đất là tài sản chung vợ chồng, quyền ủy quyền đã hết/hủy, hay có dấu hiệu rủi ro giao dịch.
+ Với đất đứng tên 2 đồng sở hữu, việc bán phải có sự đồng ý của cả hai. Người ở xa có thể ủy quyền, nhưng người được ủy quyền chỉ được thực hiện đúng phạm vi đã ghi trong giấy ủy quyền; giao dịch vượt phạm vi này không ràng buộc người ủy quyền, trừ trường hợp được chấp nhận sau đó Điều 141 Bộ luật Dân sự 2015.
+ Bạn kiểm tra hợp đồng ủy quyền có các nội dung cụ thể như sau không:
+ Quyền “thay mặt ký hợp đồng chuyển nhượng quyền sử dụng đất/quyền sở hữu nhà ở” với bên mua;
+ Thông tin chính xác thửa đất, số Giấy chứng nhận;
+ Quyền thỏa thuận giá, phương thức thanh toán, ký hồ sơ công chứng, hồ sơ thuế và sang tên;
+ Quyền nhận tiền chuyển nhượng hoặc chỉ định tiền phải chuyển thẳng vào tài khoản của người ủy quyền;
+ Thời hạn ủy quyền còn hiệu lực.
+ Hợp đồng ủy quyền về nguyên tắc là sự thỏa thuận để bên được ủy quyền thực hiện công việc nhân danh bên ủy quyền; nếu không ghi thời hạn thì thường có hiệu lực 01 năm kể từ ngày xác lập Điều 562 Bộ luật Dân sự 2015 Điều 563 Bộ luật Dân sự 2015. Việc ủy quyền có thể chấm dứt khi hết hạn, công việc hoàn thành, một bên đơn phương chấm dứt, hoặc người ủy quyền/người được ủy quyền chết, mất năng lực hành vi dân sự... Điều 569 Bộ luật Dân sự 2015.
+ Ngoài ra, nếu một hoặc cả hai phần đất là tài sản chung vợ chồng, dù sổ chỉ ghi tên một người, công chứng viên có thể yêu cầu vợ/chồng cùng ký hoặc có văn bản xác nhận/ủy quyền hợp lệ. Việc định đoạt bất động sản là tài sản chung phải có sự thỏa thuận bằng văn bản của vợ chồng Điều 35 Luật Hôn nhân và gia đình 2014.
+ Cách xử lý thực tế: mang bản gốc giấy ủy quyền đến đúng văn phòng công chứng đang từ chối và yêu cầu họ nêu rõ lý do từ chối bằng văn bản. Nếu lý do là thiếu phạm vi ủy quyền, người ở xa cần lập lại hoặc bổ sung ủy quyền tại tổ chức công chứng nơi mình đang có mặt; không nhất thiết phải về nơi có đất. Văn bản mới nên ghi đúng các quyền nêu trên, đặc biệt là quyền ký hợp đồng chuyển nhượng.
+ [1]. Điều 141, 562, 563, 569, Luật 91/2015/QH13
+ [2]. Điều 35, Luật 52/2014/QH13</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn các điều luật từ Bộ luật Dân sự 2015 (Điều 141, 562, 563, 569) và Luật Hôn nhân và gia đình 2014 (Điều 35). Tuy nhiên, các điều luật này đã bị thay thế bởi các quy định mới trong Bộ luật Dân sự 2024 và Luật Hôn nhân và gia đình 2024. Do đó, việc trích dẫn các điều luật này là không còn hiệu lực. Câu trả lời đã bao phủ vấn đề về ủy quyền và các điều kiện cần thiết trong hợp đồng ủy quyền, nhưng cần cập nhật điều luật mới để đảm bảo tính chính xác và hiệu lực pháp lý.</t>
+  </si>
+  <si>
+    <t>Kính nhờ Quý Luật Sư cùng Quý cao nhận chỉ giáo giúp trường hợp sau:
++ Chồng sn 1972,
++ Vợ SN 1971,
++ Kết hôn 1997,
++ Sinh con trai sn 1998;
++ Năm 2000 người chồng bỏ đi biệt tăm, còn vợ một mình nuôi con nhỏ tới nay;
++ Năm 2023 Vợ mua được căn nhà riêng!
++ Vậy bây giờ năm 2026 người vợ muốn bán nhà chính tự họ làm việc và dành dụm tích góp tiền của để mua nhà và nay muốn chứng minh tài sản riêng của người vợ để chứng thực được tự do bán căn nhà này để thanh toán các công nợ vay mượn người khác thì phải làm như thế nào mới hợp pháp và đúng chuẩn pháp lý chuyển nhượng cho người khác!
+Xin mọi người chỉ giáo giúp ạ!
+Chân thành cám ơn mọi người!
+Trân trọng!</t>
+  </si>
+  <si>
+    <t>Kết luận: Căn nhà mua năm 2023, khi vợ chồng chưa ly hôn, về nguyên tắc vẫn bị suy đoán là tài sản chung vợ chồng, dù người chồng đã bỏ đi từ năm 2000. Người vợ không nên tự bán một mình nếu chưa có căn cứ pháp lý xác lập nhà là tài sản riêng hoặc quyền sở hữu riêng; cách an toàn nhất là yêu cầu Tòa án giải quyết tình trạng hôn nhân và tài sản.
+ Việc chồng không còn chung sống, không chu cấp, vợ tự nuôi con và tự tích góp tiền mua nhà là chứng cứ rất quan trọng. Tuy nhiên, tài sản hình thành trong thời kỳ hôn nhân thường được coi là tài sản chung, trừ khi vợ chứng minh đó là tài sản riêng; khi không chứng minh được nguồn gốc thì pháp luật cũng coi là tài sản chung. Điều 33 Luật Hôn nhân và gia đình 2014
+ Tài sản riêng có thể là tài sản mỗi người có trước hôn nhân; được thừa kế riêng, tặng cho riêng; hoặc tài sản hình thành từ tài sản riêng. Người nào cho rằng nhà là tài sản riêng thì có nghĩa vụ đưa ra chứng cứ chứng minh. Điều 43 Luật Hôn nhân và gia đình 2014 Điều 44 Luật Hôn nhân và gia đình 2014
+ Hướng xử lý phù hợp:
+ Nếu còn liên lạc được với chồng:
+ Hai người có thể lập văn bản thỏa thuận xác nhận căn nhà là tài sản riêng của vợ hoặc thỏa thuận chia tài sản chung trong thời kỳ hôn nhân. Văn bản liên quan đến bất động sản phải được công chứng theo quy định. Sau đó đăng ký biến động để ghi nhận quyền sở hữu riêng của vợ trước khi bán. Điều 38 Luật Hôn nhân và gia đình 2014 Điều 47 Luật Hôn nhân và gia đình 2014
+ Nếu chồng biệt tích, không rõ còn sống hay ở đâu:
+ Không thể chỉ làm “giấy cam kết tài sản riêng” tại văn phòng công chứng để tự bán nhà, vì công chứng viên thường sẽ yêu cầu chữ ký/chấp thuận của chồng hoặc bản án, quyết định của Tòa án. Việc tự bán có thể bị tranh chấp, yêu cầu hủy giao dịch sau này.
+ Người vợ cần thu thập chứng cứ chồng vắng mặt liên tục: xác nhận của Công an/UBND cấp xã nơi cư trú cuối cùng, xác nhận tổ dân phố, lời khai người thân, tài liệu tìm kiếm, tin nhắn hoặc giấy tờ khác. Nếu chồng đã biệt tích từ năm 2000 và không có tin tức xác thực, có thể yêu cầu Tòa án tuyên bố chồng mất tích; điều kiện là đã biệt tích 02 năm liền trở lên dù đã áp dụng đầy đủ biện pháp thông báo, tìm kiếm. Điều 68 Bộ luật Dân sự 2015
+ Sau khi có quyết định tuyên bố mất tích:
+ Người vợ có thể yêu cầu Tòa án cho ly hôn với người chồng bị tuyên bố mất tích. Khi ly hôn, đề nghị Tòa án giải quyết luôn căn nhà: công nhận là tài sản riêng nếu chứng minh được toàn bộ nguồn tiền riêng, hoặc chia tài sản chung và giao nhà cho vợ sở hữu theo phần Tòa án xác định. Khoản 2 Điều 56 Luật Hôn nhân và gia đình 2014 Điều 59 Luật Hôn nhân và gia đình 2014
+ Hồ sơ chứng minh nguồn tiền mua nhà nên chuẩn bị gồm: hợp đồng mua bán/chuyển nhượng năm 2023; giấy chứng nhận; sao kê ngân hàng; giấy nhận tiền bán tài sản riêng (nếu có); chứng cứ thu nhập, kinh doanh, vay tiền; giấy vay và chứng từ trả nợ; xác nhận chồng không chung sống, không đóng góp; chứng cứ vợ một mình nuôi con, quản lý tài sản từ năm 2000.
+ Lưu ý quan trọng: Việc căn nhà đứng tên một mình người vợ chưa đủ để khẳng định đó là tài sản riêng. Với nhà là tài sản chung, việc bán phải có sự thỏa thuận bằng văn bản của cả vợ và chồng; nếu không, giao dịch có rủi ro rất lớn cho cả người bán và người mua. Điều 35 Luật Hôn nhân và gia đình 2014
+ Khi đã có bản án/quyết định có hiệu lực xác định nhà thuộc riêng vợ hoặc giao toàn bộ nhà cho vợ, người vợ mang giấy tờ đó cùng giấy chứng nhận nhà đất, giấy tờ nhân thân đến tổ chức công chứng để ký hợp đồng chuyển nhượng; sau đó người mua làm thủ tục đăng ký sang tên theo quy định đất đai.
+ [1]. Điều 33, 35, 38, 43, 44, 47, 56, 59, Luật 52/2014/QH13
+ [2]. Điều 68, Luật 91/2015/QH13</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn các điều luật từ Luật Hôn nhân và gia đình 2014 và Bộ luật Dân sự 2015. Tuy nhiên, Luật Hôn nhân và gia đình 2014 vẫn còn hiệu lực, nhưng các điều luật này không trực tiếp giải quyết vấn đề tài sản riêng trong trường hợp cụ thể này. Câu trả lời đã bao phủ phần lớn các khía cạnh pháp lý liên quan đến việc xác định tài sản riêng và thủ tục cần thiết khi người chồng biệt tích, nhưng không cập nhật các quy định mới nhất nếu có thay đổi sau năm 2023.</t>
+  </si>
+  <si>
+    <t>Mình rất mong cộng đồng giúp đỡ và giải đáp giùm mình. Cụ thể: Khoảng năm 2000, ba mình có mua đất hơn 300m^2 (thuộc đất trồng cây lâu năm) thuộc sổ chung từ chủ đất A, có xác nhận vi bằng. Năm 2018, người chủ này đã mất và theo mình biết, chủ A còn có những người con chưa được ủy quyền thừa kế đất ở trên. Bây giờ ba mình mong muốn làm sổ để chuyển nhượng quyền sử dụng đất cho các con thì làm như thế nào?!</t>
+  </si>
+  <si>
+    <t>Kết luận: Ba bạn chưa thể tự làm sổ riêng hoặc chuyển nhượng phần hơn 300 m² chỉ dựa vào vi bằng và việc đang đứng chung trên sổ của ông A. Vì ông A đã mất, trước hết cần xác định giao dịch năm 2000 có chứng cứ gì, những người thừa kế của ông A phải hoàn tất thủ tục thừa kế; sau đó họ mới có thể cùng ba bạn ký thủ tục hợp thức hóa, tách thửa và sang tên nếu đất đủ điều kiện.
+ Vi bằng chỉ là tài liệu ghi nhận sự kiện, hành vi hoặc việc giao nhận tiền/giấy tờ (nếu có); không tự thay thế hợp đồng chuyển nhượng quyền sử dụng đất được công chứng hoặc chứng thực. Hợp đồng chuyển nhượng đất của cá nhân về nguyên tắc phải công chứng/chứng thực Điều 27 Luật Đất đai 2024.
+ 1. Việc cần làm đầu tiên: xác minh hồ sơ
+ Cần thu thập: vi bằng bản gốc, giấy tay mua bán (nếu có), chứng cứ trả tiền, giấy giao đất, người làm chứng, biên lai thuế, xác nhận quản lý/sử dụng ổn định, ảnh hiện trạng và bản gốc Giấy chứng nhận đang mang tên ông A.
+ Đồng thời kiểm tra: diện tích 300 m² nằm ở vị trí nào trên thửa đất chung; có đang tranh chấp/quy hoạch/kê biên không; đất có đủ diện tích tối thiểu để tách thửa theo quy định nơi có đất không. Vì bạn chưa nêu tỉnh/thành phố nên chưa thể kết luận diện tích này có tách được hay không.
+ 2. Người thừa kế của ông A phải tham gia
+ Khi ông A mất, quyền sử dụng đất đứng tên ông A trở thành di sản. Những người thừa kế hợp pháp của ông A cần lập văn bản khai nhận hoặc thỏa thuận phân chia di sản tại tổ chức công chứng; nếu không có di chúc thì xác định theo hàng thừa kế thứ nhất gồm vợ/chồng, cha mẹ, con của ông A Điều 651 Bộ luật Dân sự 2015.
+ Sau đó có hai hướng:
+ Hướng thuận lợi nhất: toàn bộ người thừa kế thừa nhận việc ông A đã bán phần đất này cho ba bạn, cùng ký văn bản thỏa thuận và hợp đồng chuyển nhượng/công nhận giao dịch tại tổ chức công chứng. Sau đó thực hiện tách thửa, đăng ký biến động và cấp Giấy chứng nhận cho ba bạn.
+ Nếu có người không hợp tác hoặc tranh chấp: ba bạn cần khởi kiện tại Tòa án yêu cầu công nhận giao dịch/chuyển quyền hoặc giải quyết tranh chấp quyền sử dụng đất. Vi bằng, giấy giao nhận tiền, quá trình sử dụng đất công khai ổn định là chứng cứ quan trọng, nhưng không bảo đảm chắc chắn Tòa sẽ công nhận vì còn phụ thuộc nội dung giấy tờ, thời điểm giao dịch, việc giao đất thực tế và ý kiến các thừa kế.
+ 3. Tách thửa rồi mới sang tên riêng
+ Chỉ khi người có quyền hợp pháp đối với thửa đất ký hồ sơ chuyển nhượng và thửa đất đủ điều kiện tách, ba bạn mới có thể được cấp sổ riêng cho phần hơn 300 m². Điều kiện cơ bản để chuyển nhượng gồm: có Giấy chứng nhận, đất không tranh chấp, không bị kê biên, còn thời hạn sử dụng và không bị áp dụng biện pháp khẩn cấp tạm thời Điều 45 Luật Đất đai 2024.
+ Do đất là đất trồng cây lâu năm, nếu ba bạn hoặc các con muốn xây nhà thì phải kiểm tra quy hoạch và làm thủ tục chuyển mục đích sử dụng đất trước hoặc đồng thời theo quy định; không nên tự xây khi đất vẫn là đất nông nghiệp.
+ 4. Ba bạn có thể chuyển cho các con khi nào?
+ An toàn nhất là: hoàn tất sổ riêng đứng tên ba bạn trước, rồi ba bạn lập hợp đồng tặng cho hoặc chuyển nhượng cho các con, có công chứng/chứng thực và đăng ký sang tên. Không nên “bán tiếp” bằng giấy tay/vi bằng khi ba bạn chưa có sổ riêng, vì sẽ làm chuỗi giấy tờ phức tạp và tăng nguy cơ tranh chấp.
+ Nếu các con là người dự kiến nhận đất, có thể cân nhắc để toàn bộ người thừa kế ông A chuyển nhượng trực tiếp cho các con, nhưng chỉ nên làm khi tất cả người thừa kế đã thống nhất rõ ràng và cơ quan đăng ký đất đai chấp nhận hồ sơ.
+ [1]. Điều 27, 45, Luật 31/2024/QH15
+ [2]. Điều 651, Luật 91/2015/QH13</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn Điều 27 và Điều 45 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là văn bản còn hiệu lực, liên quan đến việc công chứng/chứng thực hợp đồng chuyển nhượng quyền sử dụng đất và điều kiện chuyển nhượng. Ngoài ra, Điều 651 của Bộ luật Dân sự 2015 (Luật số 91/2015/QH13) cũng được trích dẫn, quy định về hàng thừa kế, là văn bản còn hiệu lực. Các điều luật này đã bao phủ các vấn đề về thủ tục thừa kế, chuyển nhượng và tách thửa đất, tuy nhiên chưa đề cập cụ thể đến quy định về diện tích tối thiểu để tách thửa theo từng địa phương.</t>
+  </si>
+  <si>
+    <t>Anh chị cho hỏi: anh chị cho tặng em dâu đất thì phải nộp thuế thu nhập cá nhân không. Vì chồng của em dâu không ở nhà nên phait cho riêng em dâu</t>
+  </si>
+  <si>
+    <t>Kết luận: Có. Anh/chị chồng tặng cho đất riêng cho em dâu không thuộc diện miễn thuế thu nhập cá nhân, dù chồng của em dâu vắng mặt hoặc không đứng tên nhận tặng cho. Em dâu là người nhận quà tặng sẽ phải nộp thuế thu nhập cá nhân.
+Pháp luật chỉ miễn thuế khi tặng cho bất động sản giữa các quan hệ như vợ chồng; cha mẹ chồng với con dâu; hoặc anh, chị, em ruột. “Anh/chị chồng” với “em dâu” không phải là anh, chị, em ruột và không nằm trong danh sách được miễn. Khoản 1 Điều 4 Luật Thuế thu nhập cá nhân 2025 Khoản 1 Điều 18 Nghị định 253/2026/NĐ-CP
+Thuế phải nộp là 10% phần giá trị quyền sử dụng đất được tặng cho vượt 20 triệu đồng trong mỗi lần nhận. Khoản 1 và khoản 2 Điều 18 Luật Thuế thu nhập cá nhân 2025
+Ngoài thuế thu nhập cá nhân, em dâu thường còn phải nộp lệ phí trước bạ 0,5%; quan hệ anh/chị chồng – em dâu cũng không thuộc diện miễn lệ phí trước bạ. Việc chồng vắng mặt không làm phát sinh miễn thuế; nếu tặng cho riêng em dâu thì hợp đồng và giấy chứng nhận sẽ ghi người nhận là em dâu.
+[1]. Điều 4, 18, Luật 109/2025/QH15
+[2]. Điều 18, Nghị định 253/2026/NĐ-CP</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Luật Thuế thu nhập cá nhân 2025 và Nghị định 253/2026/NĐ-CP, tuy nhiên các văn bản này chưa có hiệu lực tại thời điểm hiện tại (tháng 10/2023). Do đó, việc trích dẫn này không đúng với tình hình pháp lý hiện hành. Câu trả lời đã xác định đúng vấn đề pháp lý về việc tặng cho đất giữa anh/chị chồng và em dâu không thuộc diện miễn thuế thu nhập cá nhân và lệ phí trước bạ, nhưng cần căn cứ vào các văn bản pháp luật hiện hành tại thời điểm hiện tại.</t>
+  </si>
+  <si>
+    <t>Mình sắp đc tặng 700met đất thổ cư từ Sổ 3000met tách thửa ra. Giờ có bị giảm thổ cư ko vậy a/c?
+Sổ mình 2004 cln, đã nộp tiền chuyển mục đích năm 2011 lên 1500 met thổ cư , ở bình dương</t>
+  </si>
+  <si>
+    <t>Kết luận: Việc tách 700 m² ra từ sổ 3.000 m² không tự làm giảm diện tích đất ở (thổ cư) đã được công nhận 1.500 m² năm 2011. Khi tách, cơ quan đăng ký sẽ phân bổ 1.500 m² đất ở đó vào các thửa mới theo hồ sơ tách/tặng cho; phần còn lại vẫn là đất CLN.
+Ví dụ, nếu tách cho bạn 700 m² và hồ sơ xác định toàn bộ 700 m² này nằm trong phần đất ở, sổ mới của bạn sẽ ghi 700 m² đất ở; sổ còn lại ghi 800 m² đất ở và phần đất CLN còn lại. Không có quy định tự động “cắt giảm” đất ở chỉ vì tách thửa.
+Tuy nhiên, cần kiểm tra 3 điểm trước khi làm:
+Trên Giấy chứng nhận hiện tại phải thể hiện rõ 1.500 m² đất ở và 1.500 m² CLN; đối chiếu sơ đồ để xác định vị trí 700 m² định tách có nằm trong phần đất ở hay không.
+Thửa sau tách phải đáp ứng diện tích tối thiểu, kích thước cạnh và lối đi theo quy định địa phương; đồng thời đất phải có sổ, không tranh chấp, không bị kê biên và còn thời hạn sử dụng. Điều 220 Luật Đất đai 2024
+Nếu 700 m² có lẫn đất CLN thì sổ mới sẽ ghi cả hai loại đất theo diện tích thực tế; muốn toàn bộ là đất ở thì chỉ thực hiện được nếu phần đất đó đã là đất ở hoặc được cơ quan có thẩm quyền cho phép chuyển mục đích trước/tại thời điểm giải quyết hồ sơ.
+Nên yêu cầu văn phòng công chứng và đơn vị đo đạc ghi rõ trong hợp đồng, trích đo: “Tặng cho quyền sử dụng 700 m² đất ở thuộc thửa…”, nếu đúng thực tế theo sổ và sơ đồ. Đừng chỉ ghi chung “700 m² đất”, vì có thể dẫn đến sổ mới bị ghi cả đất CLN.
+[1]. Điều 220, Luật 31/2024/QH15</t>
+  </si>
+  <si>
+    <t>Câu trả lời có trích dẫn Điều 220 của Luật Đất đai 2024 (Luật số 31/2024/QH15), nhưng không nêu rõ nội dung của điều luật này, do đó không thể xác định tính đúng đắn và liên quan của điều luật được trích dẫn. Ngoài ra, câu trả lời không trích dẫn đầy đủ các điều luật cần thiết để giải quyết vấn đề về tách thửa và chuyển mục đích sử dụng đất, chẳng hạn như các quy định về diện tích tối thiểu tách thửa, quy định về chuyển mục đích sử dụng đất từ đất CLN sang đất ở.</t>
+  </si>
+  <si>
+    <t>Thời điểm 2002 nhà e có xây dựng 1 căn
+ nhà trên đất nông nghiệp. Đến nay e đi
+ chuyển đổi mục đích sử dụng đất thì có bị
+ xử phạt vphc về việc xây dựng nhà trái
+ phép trên đất NN k ạ.</t>
+  </si>
+  <si>
+    <t>Kết luận: Thông thường, bạn không còn bị phạt tiền về việc tự chuyển đất nông nghiệp sang đất ở từ năm 2002, vì thời hiệu xử phạt vi phạm hành chính về đất đai là 2 năm. Tuy nhiên, việc có được cho chuyển mục đích và có phải xử lý phần nhà xây trên đất nông nghiệp hay không còn phụ thuộc hiện trạng, quy hoạch và hồ sơ đất.
+Hành vi xây nhà trên đất nông nghiệp thường bị xem là đã tự chuyển mục đích sử dụng đất. Thời hiệu phạt đối với vi phạm đất đai là 2 năm; với hành vi đã kết thúc thì tính từ ngày chấm dứt hành vi. Nhà đã xây xong từ năm 2002, không cải tạo/mở rộng vi phạm thêm thì về nguyên tắc đã hết thời hiệu phạt tiền. Điều 6 Luật Xử lý vi phạm hành chính 2012 Điều 3 Nghị định 123/2024/NĐ-CP
+Dù hết thời hiệu phạt, cơ quan có thẩm quyền vẫn sẽ xem đất có phù hợp quy hoạch, có đủ điều kiện chuyển mục đích hay không. Nếu được chấp thuận, bạn phải nộp tiền sử dụng đất theo thông báo; nhà xây từ trước không đương nhiên làm đất trở thành đất ở. Việc tự ý chuyển đất nông nghiệp sang đất ở là hành vi bị xử lý theo quy định đất đai hiện hành. Điều 10 Nghị định 123/2024/NĐ-CP
+Bạn nên nộp hồ sơ xin chuyển mục đích tại cơ quan quản lý đất đai cấp xã/tỉnh nơi có đất, kèm sổ đỏ và thông tin hiện trạng nhà. Không nên tự tháo dỡ hoặc tự sửa chữa, xây thêm nhà trước khi có ý kiến bằng văn bản của cơ quan có thẩm quyền.
+[1]. Điều 6, Luật 15/2012/QH13
+[2]. Điều 3, 10, Nghị định 123/2024/NĐ-CP</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 6 của Luật Xử lý vi phạm hành chính 2012 (Luật số 15/2012/QH13) và Điều 3, 10 của Nghị định 123/2024/NĐ-CP. Tuy nhiên, Luật Xử lý vi phạm hành chính 2012 vẫn còn hiệu lực, nhưng Nghị định 123/2024/NĐ-CP không tồn tại. Do đó, việc trích dẫn Nghị định này là sai và không có căn cứ pháp lý. Câu trả lời đã bao phủ phần thời hiệu xử phạt vi phạm hành chính và quy trình chuyển đổi mục đích sử dụng đất, nhưng trích dẫn điều luật không chính xác.</t>
+  </si>
+  <si>
+    <t>Dạ mọi người cho em hỏi, ngày mai e sẽ lên chi cục thuế quận 12 để tính lại tiền sử dụng đất, (240 mét vuông) giấy thông báo từ năm 2016 là 144 triệu nhưng chưa đóng tới bây giờ, theo em tìm hiểu thì sẽ có 2 hướng: 
+ - đóng tiền nộp chậm thì tầm 300-400tr
+ - tính theo giá mới thì lên tới 2 tỷ 5
+ Cả nhà em đang rất hoang mang vì nếu lên tới 2 tỷ 5 thì là phải bán đất thôi ạ 🙁</t>
+  </si>
+  <si>
+    <t>Kết luận: Không nên mặc định rằng gia đình phải chọn giữa “nộp chậm 300–400 triệu” và “tính lại theo giá mới 2,5 tỷ”. Nếu thông báo năm 2016 được ban hành đúng, chưa bị cơ quan thuế/đất đai thu hồi hoặc điều chỉnh, nguyên tắc là vẫn nộp theo số tiền đã thông báo và tiền chậm nộp; không tự động áp giá đất hiện nay.
+Bạn cần mang theo thông báo nghĩa vụ tài chính năm 2016, sổ đỏ, hồ sơ xin chuyển mục đích và các chứng từ đã nộp (nếu có) để đề nghị cơ quan thuế trả lời bằng văn bản 3 nội dung:
+Thông báo 144 triệu năm 2016 hiện còn hiệu lực hay đã bị hủy/điều chỉnh? Nếu còn hiệu lực, đề nghị in bảng tính số tiền gốc và tiền chậm nộp đến ngày dự kiến nộp.
+Nếu cơ quan nói phải tính lại theo giá hiện nay, yêu cầu nêu rõ quyết định/văn bản nào hủy thông báo năm 2016 và căn cứ pháp lý để xác định lại nghĩa vụ. Chỉ nói miệng “phải theo giá mới” thì chưa đủ để gia đình quyết định.
+Kiểm tra xem gia đình có thuộc trường hợp được ghi nợ tiền sử dụng đất theo chính sách tại thời điểm được cấp sổ/chuyển mục đích hay không. Nếu trước đây đã có hồ sơ ghi nợ hợp lệ thì cách tính sẽ khác; không phải trường hợp nào chậm đóng cũng được áp dụng.
+Tiền chậm nộp thuế và các khoản thu khác thuộc ngân sách nhà nước thường được tính theo tỷ lệ 0,03%/ngày trên số tiền chậm nộp, nhưng phải xác định đúng thời điểm bắt đầu tính, các lần thay đổi chính sách và tình trạng pháp lý của thông báo cũ. Điều 59 Luật Quản lý thuế 2019
+Bạn cũng nên lưu ý: “Chi cục Thuế quận 12” là cách gọi trước đây; hiện cơ quan thuế tổ chức theo mô hình mới. Tuy nhiên, hồ sơ nghĩa vụ tài chính đất đai vẫn cần được cơ quan thuế có thẩm quyền tra cứu, đối chiếu với cơ quan quản lý đất đai. Không nên nộp tiền hoặc ký đề nghị “xác định lại nghĩa vụ theo giá hiện hành” trước khi nhận được bảng tính và căn cứ bằng văn bản.
+[1]. Điều 59, Luật 38/2019/QH14</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 59 của Luật Quản lý thuế 2019 (Luật số 38/2019/QH14), điều này liên quan đến việc tính tiền chậm nộp thuế. Tuy nhiên, câu trả lời không trích dẫn các điều luật liên quan đến việc xác định nghĩa vụ tài chính về đất đai, như Luật Đất đai 2024 và các nghị định mới liên quan. Do đó, mặc dù điều luật trích dẫn còn hiệu lực, nhưng chưa bao phủ đầy đủ các khía cạnh pháp lý cần thiết cho tình huống này.</t>
+  </si>
+  <si>
+    <t>Các anh chị bạn bè trong nhóm cho em hỏi 1 việc thế này.Sổ đỏ nhà e được cấp năm 2000 do bố em là thương binh hạng 2/4 , ngày trước được miễn tiền thuế đất phi nông nghiệp nhưng bây giờ theo luật đất đai 2024 bên thuế bảo chỉ được giảm 50% tiền thuế đất phi nông nghiệp .Nhưng do trước được miễn nên nhà em cũng không để ý đi kê khai thuế nên bây giờ bên thuế họ truy thu thuế và phạt nộp chậm từ năm 2000 có đúng không ạ.E xin cảm ơn!</t>
+  </si>
+  <si>
+    <t>Kết luận: Việc giảm còn 50% thuế là có cơ sở nếu bố bạn là thương binh hạng 2/4. Nhưng cơ quan thuế không thể “phạt” gia đình từ năm 2000; cần phân biệt giữa truy thu số thuế còn thiếu và tiền chậm nộp, đồng thời kiểm tra thời kỳ thuế và việc gia đình đã từng được xác nhận miễn thuế hay chưa.
+Thuế sử dụng đất phi nông nghiệp chỉ áp dụng từ ngày 01/01/2012; vì vậy không có căn cứ truy thu loại thuế này từ năm 2000 đến hết năm 2011. Thương binh hạng 1/4 được miễn; thương binh hạng 2/4 được giảm 50% số thuế phải nộp đối với đất ở trong hạn mức. Điều 9 Luật Thuế sử dụng đất phi nông nghiệp 2010 Điều 10 Luật Thuế sử dụng đất phi nông nghiệp 2010
+Nếu gia đình không kê khai hoặc chưa được cơ quan thuế ra quyết định miễn/giảm đúng hồ sơ, cơ quan thuế có thể xác định lại số thuế còn thiếu từ các năm thuộc thời kỳ áp dụng thuế. Tuy nhiên, gia đình nên nộp ngay hồ sơ chứng minh bố là thương binh hạng 2/4 để yêu cầu tính giảm 50% cho các năm đủ điều kiện; không chấp nhận cách tính toàn bộ 100% nếu đối tượng và đất đáp ứng điều kiện giảm.
+Về “phạt”: phạt vi phạm thủ tục thuế có thời hiệu 2 năm, nên không thể nay ra quyết định phạt cho hành vi không kê khai từ các năm quá xa. Điều 8 Nghị định 125/2020/NĐ-CP Còn tiền chậm nộp là khoản khác với tiền phạt; cơ quan thuế cần xuất bảng tính riêng, nêu rõ từng năm thuế, số thuế sau giảm, ngày tính chậm nộp và căn cứ tính.
+Bạn nên đề nghị cơ quan thuế cung cấp bằng văn bản: (1) bảng truy thu từng năm, chỉ từ năm 2012; (2) quyết định hoặc căn cứ áp dụng giảm 50%; (3) bảng tiền chậm nộp tách riêng; (4) căn cứ vì sao trước đây gia đình được miễn nhưng nay chỉ giảm. Mang theo giấy chứng nhận thương binh, sổ đỏ, thông báo/biên lai thuế cũ và giấy tờ từng thể hiện việc miễn thuế (nếu có).
+[1]. Điều 9, 10, Luật 48/2010/QH12
+[2]. Điều 8, Nghị định 125/2020/NĐ-CP</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 9, 10 của Luật Thuế sử dụng đất phi nông nghiệp 2010 (Luật 48/2010/QH12) và Điều 8 của Nghị định 125/2020/NĐ-CP. Các điều luật này đều còn hiệu lực và đúng với vấn đề miễn giảm thuế cho thương binh và xử lý vi phạm thủ tục thuế. Tuy nhiên, câu trả lời không trích dẫn điều luật nào từ Luật Đất đai 2024 hoặc các nghị định mới liên quan đến việc miễn giảm thuế đất phi nông nghiệp theo quy định mới nhất, do đó không đáp ứng đầy đủ yêu cầu về trích dẫn điều luật hiện hành.</t>
+  </si>
+  <si>
+    <t>Năm 2022, Em có mua 1 miếng đất, trên đất có trồng cây cao su đã già. Nhưng em ở xa không trực tiếp quản lý, chỉ cho thuê, khoảng năm 2023 thì nhà hàng xóm đã cắt cây caosu tự múc mương lấn chiếm qua 2000m2 để trồng cây, sự việc chỉ được phát hiện khi gần đây em có nhu cầu vay vốn, cần có trích lục mới nên đã gọi địa chính vào đo. Theo sổ cũ thì đất của em là 1.5320m2, bản đồ vệ tinh thì đất của em diện tích 1.5490m2 và  dài xuống dưới chỗ mà bị lấn chiếm  (gần khớp với sổ, chỉ chênh &gt;100m2 do lệch bờ mương xung quanh) , nhưng nhà ông A cứ khẳng định ông đã cho người múc lại mương trồng cây, đó là đất của ông. Khi em hỏi sổ thì ông nói ông chưa có sổ/chưa đo.
+Vậy bây giờ em cần làm gì để đòi lại được đất ạ? Nếu như đất của ông A bao gồm cả phần 2000m2 kia thì không lẽ trước đây địa chính đã đo sai đất cho em hay sao ạ.</t>
+  </si>
+  <si>
+    <t>Kết luận: Bạn nên yêu cầu UBND xã/phường nơi có đất hòa giải tranh chấp ranh giới, đồng thời đề nghị đo đạc hiện trạng và xác định ranh theo hồ sơ địa chính. Không tự chặt cây, phá mương hay lấy lại đất bằng cách cưỡng ép; nếu hòa giải không thành, bạn có thể khởi kiện yêu cầu ông A trả lại diện tích đã lấn chiếm.
+Diện tích trên sổ ghi “1.5320 m²” thường được hiểu là 15.320 m², không phải 1.532 m². Việc bản đồ vệ tinh thể hiện khoảng 15.490 m² không phải căn cứ pháp lý để xác định ranh; ranh giới được xác định chủ yếu theo Giấy chứng nhận, bản đồ/sổ mục kê, mốc giới và kết quả đo đạc hồ sơ địa chính.
+Bạn cần thực hiện theo thứ tự:
+Thu thập: sổ đỏ, hợp đồng mua bán năm 2022, trích lục/bản đồ địa chính, hồ sơ kỹ thuật thửa đất khi cấp sổ, ảnh hiện trạng, ảnh cây cao su/mương cũ, hợp đồng cho thuê và lời làm chứng của người thuê hoặc hàng xóm.
+Làm đơn yêu cầu UBND xã/phường tổ chức hòa giải tranh chấp đất đai; đề nghị mời cơ quan chuyên môn đo đạc, đối chiếu tọa độ và ranh trên hồ sơ địa chính.
+Nếu hòa giải không thành, nộp đơn khởi kiện tại TAND khu vực nơi có đất, yêu cầu: xác định ranh giới; buộc ông A trả lại phần đất lấn chiếm; tháo dỡ/cải tạo trả lại hiện trạng nếu cần; bồi thường thiệt hại do chặt cây cao su, chiếm dụng đất và chi phí đo đạc hợp lý.
+Hòa giải tranh chấp đất đai tại UBND cấp xã là thủ tục bắt buộc trước khi khởi kiện tranh chấp về quyền sử dụng đất. Điều 235 Luật Đất đai 2024 Sau hòa giải không thành, người có Giấy chứng nhận được lựa chọn khởi kiện tại Tòa án. Điều 236 Luật Đất đai 2024
+Ông A nói “chưa có sổ, chưa đo” không tự làm phát sinh quyền đối với 2.000 m² đất. Ngược lại, sổ đỏ của bạn là chứng cứ rất mạnh; nhưng cần đo chồng ghép tọa độ hồ sơ với thực địa để kết luận chính xác phần nào thuộc sổ của bạn. Nếu hồ sơ đo đạc cũ thực sự sai, cơ quan đăng ký đất đai phải xem xét, xử lý theo hồ sơ nguồn gốc và quy định về đính chính/cấp đổi; ông A cũng không vì thế mà được tự ý múc mương, trồng cây trên phần đất đang tranh chấp.
+[1]. Điều 235, 236, Luật 31/2024/QH15</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn Điều 235 và 236 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là các điều luật còn hiệu lực và liên quan đến thủ tục hòa giải tranh chấp đất đai và quyền khởi kiện tại Tòa án sau khi hòa giải không thành. Điều luật này bao phủ phần yêu cầu hòa giải và khởi kiện, nhưng chưa đề cập cụ thể đến việc xử lý nếu hồ sơ đo đạc cũ sai sót.</t>
+  </si>
+  <si>
+    <t>Kind 3 - Tranh chấp và các tình huống pháp lý cụ thể</t>
+  </si>
+  <si>
+    <t>Cho tôi hỏi là, tôi có sang tên một mảnh đất, và có làm hợp đồng giấy tay, mà lúc làm hợp đồng giấy tay đó, chỉ ghi bên bán, mà không ghi tên bên mua, mà cũng không có mặt người mua tại đó, mà nhờ trưởng ấp viết tên chứ không ký thì theo anh/ chị ở đây là hợp đông này có hiệu lực không?
+Dù tôi có bảo răng căn cứ theo hợp đông mà giải quyêt thì họ cứ khăng khăng tôi phải trả cọc 1 đên 2 cho họ, họ còn đòi kiện tôi ra tòà nữa. Mà bản gốc họ giữ, tôi chỉ giữ hình ảnh, thì liệu nếu họ viết thêm gì vào bản gốc thì có sao không? Và họ không ghi tôi đã nhận cọc hay gì mà họ chỉ ghi tôi đã nhận tiền chuyến nhượng, và tôi không có kí tên cọc nào cả, chỉ kí tên phần tiền chuyển nhượng, nhưng không ghi rõ ai đưa tiền cho tôi, chỉ có trưởng ấp kí chứng kiến. Tôi xin cảm ơn!</t>
+  </si>
+  <si>
+    <t>Kết luận: Giấy viết tay chỉ ghi bên bán, không xác định bên mua, người mua không ký/không tham gia, lại không có chữ ký của bạn ở phần nhận cọc thì rất khó được coi là hợp đồng chuyển nhượng hoặc thỏa thuận đặt cọc có hiệu lực. Bên kia muốn đòi “phạt cọc gấp 1–2 lần” phải chứng minh có giao kết đặt cọc, bạn đã nhận cọc và có thỏa thuận phạt cọc.
+Hợp đồng phải xác định được các bên, có sự tự nguyện thỏa thuận và nội dung giao dịch. Hợp đồng chuyển nhượng quyền sử dụng đất còn phải được công chứng hoặc chứng thực, trừ trường hợp pháp luật có quy định khác; giấy tay thường không đủ điều kiện để sang tên. Điều 117 Bộ luật Dân sự 2015 Khoản 3 Điều 27 Luật Đất đai 2024
+Về đặt cọc, chỉ khi có chứng cứ bạn nhận một khoản tiền để bảo đảm việc giao kết/thực hiện hợp đồng thì mới áp dụng quy định về cọc. Nếu bên nhận cọc từ chối giao kết thì phải trả cọc và một khoản tương đương, trừ khi hai bên có thỏa thuận khác. Tuy nhiên, không có chữ ký của bạn tại phần nhận cọc, không ghi số tiền cọc, không nêu người giao tiền thì bên yêu cầu phải tự chứng minh các sự kiện này. Điều 328 Bộ luật Dân sự 2015
+Chữ ký “chứng kiến” của trưởng ấp không thay thế chữ ký/xác nhận ý chí của bên mua, không tự làm giấy tay thành hợp đồng chuyển nhượng đất hợp lệ. Trưởng ấp cũng không có thẩm quyền công chứng, chứng thực hợp đồng chuyển nhượng quyền sử dụng đất. Khoản 3 Điều 27 Luật Đất đai 2024
+Về bản gốc: ảnh chụp là chứng cứ điện tử/tài liệu tham khảo, nhưng bạn nên sao lưu ảnh gốc, tin nhắn, ghi âm, người làm chứng, chứng từ chuyển khoản và mọi trao đổi cho thấy nội dung thực tế. Nếu họ sửa/chèn thêm nội dung sau khi bạn ký, bạn có quyền yêu cầu Tòa án buộc xuất trình bản gốc, trưng cầu giám định mực, nét chữ, thời điểm lập tài liệu; phần bị thêm/sửa không thể dùng làm căn cứ ràng buộc bạn nếu không chứng minh được bạn đã chấp thuận.
+Nếu họ khởi kiện, bạn cần nộp bản tự khai/ý kiến phản đối, nêu rõ: không có thỏa thuận đặt cọc; không nhận cọc; giấy không xác định bên mua; bạn không ký vào nội dung cọc; yêu cầu họ xuất trình bản gốc và chứng minh việc giao tiền. Tuyệt đối không ký thêm giấy “xác nhận nợ cọc”, “cam kết hoàn cọc” nếu nội dung không đúng sự thật.
+[1]. Điều 117, 328, Luật 91/2015/QH13
+[2]. Điều 27, Luật 31/2024/QH15</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn Điều 117 và 328 của Bộ luật Dân sự 2015, đây là các điều luật còn hiệu lực và phù hợp với vấn đề hợp đồng và đặt cọc. Tuy nhiên, câu trả lời cũng trích dẫn Khoản 3 Điều 27 Luật Đất đai 2024, nhưng không có điều luật nào như vậy trong Luật Đất đai 2024. Do đó, việc trích dẫn này là không chính xác và không tồn tại. Điều này dẫn đến việc đánh giá tiêu chí trích dẫn điều luật là false.</t>
+  </si>
+  <si>
+    <t>Chuyện tế nhị nên e xin phép ẩn danh
+ Câu chuyện của e bắt đầu ngày 24/11, em có cọc mua 1 căn chung cư của chị gái chồng vs giá trị 5 tỉ. E và bạn có chung nhau, e 200tr, ban 500tr, do lúc đó c ý cần 700tr để giải quyết việc nên c ý bảo cọc 700tr. Thời hạn cọc là 1 tháng từ 24/11 tới 24/12. Tới ngày 12/12 do công việc của e có phát sinh, e ko bán dc lô đất của mình nên e có gọi cho c thì c báo là c trả lại cọc, có 3 người cùng nghe
+ Tới ngày 24/12 bạn e cần tiền vào 1 lô đất khác thì e có gọi điện trc xin lại phần cọc của bạn m thì c hẹn 12 qua nhà c
+ Tới tối 11/12 gọi điện thì c bảo bh bán dc thì trả cọc và phải phạt cọc, ý c nói là 200tr. Trong khi chung cư đó c đã bán dc 10 ngày rồi, đang trong tg nhận cọc của ngta vẫn bán đúng 5 tỉ
+ Bạn e có quan điểm rõ ràng là e có lỗi nên phạt cọc thì phạt vc nhà e phải chịu nhưng chị vẫn đòi phạt
+ Nói thêm là nhà c ck e rất giàu, luôn bảo rằng làm cái này cái kia hàng trăm tỉ. CE cũng đang rất hòa thuận, ck c ý bận công việc nên làm việc j từ cái nhỏ nhất là trông con cho c ý nấu cơm cũng là ck m sang trông hộ 
+ Vậy xin hỏi nếu trong trường hợp c ck e ko trả cọc e có quyền kiện ra toà ko? Và e có cơ hội lấy lại tiền của m trong trường hợp này ko?</t>
+  </si>
+  <si>
+    <t>Kết luận: Bạn có quyền khởi kiện để đòi lại khoản 700 triệu đồng; khả năng lấy lại tiền phụ thuộc chủ yếu vào nội dung giấy cọc, chứng cứ giao tiền và việc hai bên đã thỏa thuận hủy/trả cọc ngày 12/12. Việc bên bán đã bán căn hộ cho người khác trong thời hạn đặt cọc là tình tiết có lợi cho bạn, vì có thể thể hiện họ không tiếp tục dành căn hộ để giao dịch với bạn.
+Nếu giấy cọc quy định thời hạn đến 24/12 nhưng không có thỏa thuận gia hạn, mà ngày 12/12 chị gái chồng đã nói “trả lại cọc” và có 3 người nghe, bạn cần giữ tin nhắn, lịch sử cuộc gọi, ghi âm hợp pháp (nếu có) và thông tin 3 người làm chứng. Đây là căn cứ để lập luận hai bên đã chấm dứt thỏa thuận cọc theo thống nhất, nên bên bán phải hoàn lại đủ 700 triệu; không có cơ sở giữ lại 200 triệu sau đó.
+Trường hợp Tòa xác định bạn vi phạm nghĩa vụ mua căn hộ và không có thỏa thuận hủy cọc, bên nhận cọc có thể được giữ cọc. Tuy nhiên, họ không đương nhiên được giữ thêm tiền ngoài 700 triệu, trừ khi có thỏa thuận phạt vi phạm/bồi thường riêng và chứng minh được căn cứ. Ngược lại, nếu bên nhận cọc từ chối bán hoặc đã bán cho người khác làm giao dịch không thể thực hiện, bạn có thể yêu cầu hoàn cọc và khoản tương đương giá trị cọc, trừ khi giấy cọc có thỏa thuận khác. Điều 328 Bộ luật Dân sự 2015
+Việc bạn và bạn bè cùng góp tiền là quan hệ nội bộ giữa hai người; khi khởi kiện, người đứng tên bên đặt cọc hoặc người trực tiếp giao tiền nên là nguyên đơn. Nếu giấy cọc ghi cả hai người, hai người cùng khởi kiện; nếu chỉ ghi bạn nhưng bạn của bạn chuyển khoản/giao tiền trực tiếp, cần đưa bạn ấy vào tham gia tố tụng hoặc có giấy xác nhận nguồn tiền để tránh tranh chấp sau này.
+Nên làm ngay:
+Gửi văn bản/tin nhắn yêu cầu hoàn trả 700 triệu, nêu rõ thời hạn thanh toán (ví dụ 7 ngày), số tài khoản nhận tiền và căn cứ: đã thống nhất trả cọc ngày 12/12; căn hộ đã bán cho người khác.
+Sao lưu giấy cọc, chứng từ chuyển 700 triệu, tin nhắn, cuộc gọi, thông tin người làm chứng; ghi nhận thông tin về việc căn hộ đã bán, ngày nhận cọc của người mới.
+Hết thời hạn mà không trả, nộp đơn khởi kiện tại TAND khu vực nơi bị đơn cư trú; yêu cầu trả tiền cọc, lãi do chậm trả và, nếu có đủ căn cứ, yêu cầu phạt cọc. Nghĩa vụ chậm trả tiền phải chịu lãi theo thỏa thuận hoặc theo luật. Điều 357 Bộ luật Dân sự 2015 Điều 468 Bộ luật Dân sự 2015
+Không nên tự ý đăng tải thông tin, gây sức ép công khai hoặc giữ giấy tờ/tài sản của họ để trừ nợ. Tranh chấp trong phạm vi gia đình vẫn giải quyết theo chứng cứ và thỏa thuận cọc.
+[1]. Điều 328, 357, 468, Luật 91/2015/QH13</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 328, 357, 468 của Bộ luật Dân sự 2015 (Luật 91/2015/QH13), các điều luật này vẫn còn hiệu lực và phù hợp với tình huống đặt cọc và tranh chấp hợp đồng. Tuy nhiên, câu trả lời không trích dẫn điều luật nào từ Luật Đất đai 2024 hoặc các nghị định mới liên quan, nếu có, để làm rõ thêm về quyền lợi và nghĩa vụ trong giao dịch bất động sản. Điều này có thể làm giảm mức độ bao phủ của câu trả lời đối với toàn bộ vấn đề pháp lý liên quan.</t>
+  </si>
+  <si>
+    <t>Trước đây cha mẹ tôi đi khai hoang một khu đất, lúc đó là đất trống, đồng không mông quạnh, không phải đất do ông bà để lại. Cha mẹ tôi bao đất, sử dụng ổn định, làm nhà ở và có xin phép địa phương thời điểm đó.
+ Hiện nay trong khuôn viên đất gia đình tôi đang ở có khoảng gần 1.000 m² đất chưa có bất kỳ giấy tờ nào, phần đất này đang thể hiện trên hồ sơ địa phương mang tên chú ruột tôi. Lý do là trước đây anh em tôi không ở nhà nên cha tôi nhờ chú đứng tên giúp cho dễ làm thủ tục giấy tờ, chứ thực tế gia đình tôi là người khai hoang và sử dụng đất từ đầu đến nay.
+ Nay gia đình tôi muốn làm hồ sơ xin cấp giấy chứng nhận (làm bìa) cho phần đất còn lại nên đề nghị chú tôi ký giấy ủy quyền hoặc xác nhận, nhưng chú tôi không đồng ý ký, gây tranh chấp.
+ Xin hỏi trong trường hợp đất khai hoang, sử dụng ổn định lâu dài như vậy thì gia đình tôi có hướng giải quyết pháp lý nào không? Cần làm những thủ tục gì để bảo vệ quyền lợi?</t>
+  </si>
+  <si>
+    <t>Kết luận: Gia đình bạn vẫn có hướng bảo vệ quyền lợi, nhưng không thể làm sổ trực tiếp khi phần đất đang đứng tên chú trên hồ sơ địa chính và chú không hợp tác. Trước hết phải giải quyết tranh chấp, chứng minh việc chú chỉ “đứng tên hộ”; nếu hòa giải không thành thì khởi kiện yêu cầu xác định quyền sử dụng đất thuộc cha mẹ/gia đình bạn.
+1. Việc cần làm ngay
+Nộp đơn yêu cầu hòa giải tranh chấp đất đai tại UBND xã/phường nơi có đất. Trong đơn nêu rõ: nguồn gốc cha mẹ khai hoang; quá trình sử dụng liên tục, làm nhà, thực hiện nghĩa vụ; việc nhờ chú đứng tên chỉ là nhờ thủ tục; yêu cầu công nhận quyền sử dụng gần 1.000 m² cho gia đình và đề nghị chú phối hợp ký hồ sơ.
+UBND cấp xã phải xác minh nguồn gốc, quá trình sử dụng, thu thập tài liệu và tổ chức hòa giải; thời hạn là không quá 30 ngày. Đây là thủ tục bắt buộc trước khi khởi kiện tranh chấp đất đai. Điều 235 Luật Đất đai 2024 Điều 105 Nghị định 102/2024/NĐ-CP
+2. Chứng cứ gia đình cần tập hợp
+Cần xin sao lục hồ sơ địa chính thể hiện việc chú đứng tên: đơn đăng ký, kê khai, biên bản xét duyệt, bản đồ, sổ mục kê, căn cứ ghi tên chú. Đồng thời chuẩn bị chứng cứ cha mẹ mới là người sử dụng thực tế: giấy xin phép địa phương trước đây, biên lai thuế, điện nước, hộ khẩu, ảnh nhà ở qua các thời kỳ, giấy tờ xây dựng, xác nhận hàng xóm/người cao tuổi, nhân chứng biết việc khai hoang và việc nhờ đứng tên.
+Nếu có tin nhắn, ghi âm, giấy viết tay hoặc người làm chứng xác nhận chú từng thừa nhận đứng tên giúp thì đây là chứng cứ đặc biệt quan trọng. Không nên chỉ dựa vào việc gia đình ở lâu, vì hồ sơ địa chính đang mang tên chú sẽ là chứng cứ bất lợi cần được giải thích bằng tài liệu cụ thể.
+3. Nếu hòa giải không thành
+Gia đình khởi kiện tại TAND khu vực nơi có đất, yêu cầu: xác định quyền sử dụng đất thuộc cha mẹ/gia đình bạn; hủy hoặc điều chỉnh thông tin địa chính ghi tên chú nếu việc ghi tên không đúng; buộc chú thực hiện thủ tục trả lại quyền sử dụng đất hoặc chấm dứt việc cản trở cấp sổ. Người có Giấy chứng nhận hoặc giấy tờ về quyền sử dụng đất có quyền khởi kiện tại Tòa; với vụ việc của bạn, Tòa sẽ xem xét toàn bộ chứng cứ về nguồn gốc và quá trình sử dụng thực tế. Điều 236 Luật Đất đai 2024
+Sau khi có biên bản hòa giải thành có chữ ký của chú, hoặc bản án/quyết định có hiệu lực của Tòa, gia đình mới làm thủ tục đăng ký, cấp Giấy chứng nhận theo kết quả đó. Trường hợp đất thực tế chưa có giấy tờ về quyền sử dụng đất, điều kiện cấp sổ còn được đối chiếu theo thời điểm bắt đầu sử dụng, việc sử dụng ổn định, không tranh chấp và điều kiện tại Điều 138 Luật Đất đai 2024.
+Lưu ý: không tự làm giấy “xác nhận đất của cha mẹ” giả chữ ký chú, không tự chuyển nhượng/cầm cố phần đất đang tranh chấp. Nếu chú có ý định bán hoặc chuyển dịch quyền đối với đất, bạn nên nộp đơn hòa giải sớm và thông báo bằng văn bản cho cơ quan đăng ký đất đai về tình trạng tranh chấp.
+[1]. Điều 138, 235, 236, Luật 31/2024/QH15
+[2]. Điều 105, Nghị định 102/2024/NĐ-CP</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn các điều luật từ Luật Đất đai 2024 và Nghị định 102/2024/NĐ-CP, cụ thể là Điều 235, 236 của Luật Đất đai 2024 và Điều 105 của Nghị định 102/2024/NĐ-CP. Các điều luật này còn hiệu lực và phù hợp với tình huống tranh chấp đất đai, thủ tục hòa giải, và khởi kiện để xác định quyền sử dụng đất. Tuy nhiên, câu trả lời chưa đề cập chi tiết đến Điều 138 Luật Đất đai 2024 về điều kiện cấp Giấy chứng nhận quyền sử dụng đất, nhưng đã bao phủ phần lớn các bước cần thiết để giải quyết tranh chấp và bảo vệ quyền lợi của gia đình người hỏi.</t>
+  </si>
+  <si>
+    <t>Mình ở đồng Nai, năm 2018 mình có mua nền đất 100m2 bằng vi bằng. Lúc đó chủ đất phân nền ra bán, đường đi nội bộ. Lúc mua chủ nói hiện đang làm hồ sơ hiến đường sau này sẽ tãch sổ và lên thổ cư riêng từng sổ ( chi phí tách sổ lên thổ cư người mua phải chịu) nhưng đã nhiều năm trôi qua nhưng chủ không tách sổ được chỉ nói là chưa tách được. Vì thế nên mình cũng không xây dựng được do xã không cho. Giờ mình có khởi kiện ra tòa để toà tuyên công nhận hđ mua bán được không cả nhà( tiền mình đã trả hết) hay mình yêu cầu tuyên vô hiệu ah, mong mọi người tư vấn</t>
+  </si>
+  <si>
+    <t>Kết luận: Bạn có thể khởi kiện, nhưng khả năng yêu cầu Tòa “công nhận hợp đồng mua bán và buộc tách sổ riêng” là thấp nếu đất vẫn là một thửa lớn, chưa đủ điều kiện tách thửa/chuyển mục đích và giao dịch chỉ lập bằng vi bằng. Hướng thực tế hơn là yêu cầu Tòa tuyên giao dịch vô hiệu, buộc chủ đất hoàn trả toàn bộ tiền đã nhận, lãi chậm trả và bồi thường thiệt hại nếu chứng minh được lỗi của họ.
+Vi bằng chỉ ghi nhận sự kiện giao nhận tiền, giao giấy tờ hoặc lời trình bày tại thời điểm lập; không thay thế hợp đồng chuyển nhượng đất đã công chứng/chứng thực và không làm bạn tự động có quyền sử dụng nền 100 m². Hợp đồng chuyển nhượng quyền sử dụng đất phải được công chứng hoặc chứng thực, trừ trường hợp luật có quy định khác. Khoản 3 Điều 27 Luật Đất đai 2024
+Để chuyển nhượng được một phần thửa đất, phần đất đó phải có thể tách thành thửa riêng theo quy định, có lối đi hợp pháp, phù hợp quy hoạch và đủ điều kiện đăng ký. Nếu chủ đất không tách được do phân lô trái quy định hoặc không đủ điều kiện chuyển mục đích lên đất ở, Tòa thường không thể “hợp thức hóa” bằng cách công nhận cho bạn một nền riêng.
+Giao dịch vi phạm điều kiện về hình thức có thể bị vô hiệu; khi giao dịch vô hiệu, các bên hoàn trả cho nhau những gì đã nhận. Bên có lỗi gây thiệt hại phải bồi thường. Điều 117 Bộ luật Dân sự 2015 Điều 129 Bộ luật Dân sự 2015 Điều 131 Bộ luật Dân sự 2015
+Bạn nên khởi kiện tại TAND khu vực nơi có đất, yêu cầu chính:
+Tuyên giao dịch chuyển nhượng nền đất 100 m² vô hiệu;
+Buộc chủ đất trả lại toàn bộ số tiền bạn đã thanh toán;
+Yêu cầu lãi do chậm trả tiền và bồi thường chi phí hợp lý nếu có chứng cứ;
+Yêu cầu áp dụng biện pháp khẩn cấp tạm thời nếu có nguy cơ chủ đất chuyển nhượng, thế chấp cả thửa đất.
+Hồ sơ nên có: vi bằng, giấy tay/phiếu thu, sao kê chuyển khoản, tin nhắn cam kết tách sổ/chuyển thổ cư, quảng cáo bán nền, người làm chứng, giấy tờ về thửa đất gốc và văn bản/xác nhận của xã về việc không được xây dựng. Đừng tiếp tục nộp thêm tiền “phí tách sổ” khi chủ đất chưa chứng minh được khả năng tách thửa bằng văn bản của cơ quan có thẩm quyền.
+[1]. Điều 27, Luật 31/2024/QH15
+[2]. Điều 117, 129, 131, Luật 91/2015/QH13</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 27 Luật Đất đai 2024 và các điều 117, 129, 131 của Bộ luật Dân sự 2015. Tuy nhiên, Điều 27 Luật Đất đai 2024 không tồn tại hoặc không liên quan đến nội dung câu hỏi. Các điều của Bộ luật Dân sự 2015 là đúng và còn hiệu lực, nhưng không có điều luật nào từ Luật Đất đai 2024 được trích dẫn đúng và có hiệu lực. Câu trả lời đã bao phủ phần về giao dịch vi bằng và khả năng khởi kiện, nhưng thiếu điều luật cụ thể từ Luật Đất đai 2024 về điều kiện tách thửa và chuyển mục đích sử dụng đất.</t>
+  </si>
+  <si>
+    <t>Em chào mọi người ạ,dạ em muốn mọi người tư vấn giúp em ạ,câu chuyện của em như sau: Mẹ chồng em có viết giấy ủy quyền thừa kế tài sản và đất ở cho chồng em trước khi anh lấy vợ,( Bố chồng em đã mất) Và cách đây mấy năm mẹ chồng em có nói với với ace trong nhà là mẹ em muốn làm sổ đỏ sang tên cho chồng em,trong ace trong nhà có 1 người không ký để làm sổ đỏ cho chồng em (Trong khi đó người anh đó đã được bm em chia đất cho ạ,và diện tích đất còn nhiều hơn của chồng em).Mọi người tư vấn giúp em trường hợp của chồng em bây giờ phải như thế nào mới sang tên được ạ?Em cảm ơn ạ.</t>
+  </si>
+  <si>
+    <t>Kết luận: Chồng bạn chỉ có thể sang tên toàn bộ đất khi xác định đúng nguồn gốc đất và có giấy tờ thừa kế hợp lệ. Giấy “ủy quyền thừa kế” của mẹ chồng không tự làm chồng bạn thành chủ đất; nếu đó thực chất là di chúc hợp pháp thì phải làm thủ tục khai nhận/phân chia di sản, còn nếu đất vẫn là tài sản của mẹ thì mẹ cần tặng cho hoặc chuyển nhượng.
+1. Cần phân biệt 2 trường hợp
+Đất là tài sản riêng của mẹ chồng hoặc phần đất mẹ đang sở hữu: mẹ có quyền lập hợp đồng tặng cho chồng bạn tại tổ chức công chứng. Khi đó, anh/chị/em của chồng bạn không có quyền “ký hay không ký” để ngăn việc mẹ tặng cho tài sản riêng của mình. Sau công chứng, nộp hồ sơ đăng ký biến động sang tên.
+Đất là tài sản chung của bố mẹ hoặc là di sản của bố chồng: phần của bố phải chia thừa kế. Nếu bố mất không để lại di chúc, mẹ, các con và cha mẹ của bố (nếu còn sống tại thời điểm bố mất) thuộc hàng thừa kế thứ nhất và được hưởng phần bằng nhau. Vì vậy, một người anh không đồng ý thì không thể lập văn bản phân chia di sản để sang toàn bộ đất cho chồng bạn. Điều 651 Bộ luật Dân sự 2015
+2. “Ủy quyền thừa kế” cần kiểm tra lại
+Pháp luật không có hình thức độc lập gọi là “ủy quyền thừa kế”. Cần xem bản gốc là: di chúc, giấy ủy quyền, giấy cho tặng hay giấy cam kết.
+Nếu là di chúc của mẹ, chỉ phát sinh hiệu lực từ khi mẹ qua đời; trước đó mẹ vẫn có quyền sửa, thay thế hoặc hủy di chúc. Di chúc phải bảo đảm người lập minh mẫn, tự nguyện và nội dung/hình thức hợp pháp. Điều 630 Bộ luật Dân sự 2015 Điều 640 Bộ luật Dân sự 2015
+Nếu là giấy ủy quyền, giấy này chỉ cho phép chồng bạn thay mẹ thực hiện một công việc trong phạm vi ủy quyền; không phải là việc chuyển quyền sở hữu đất. Đặc biệt, nếu mẹ mất thì về nguyên tắc việc ủy quyền chấm dứt. Điều 422 Bộ luật Dân sự 2015
+3. Hướng xử lý phù hợp
+Kiểm tra sổ đỏ hiện đang đứng tên ai; thời điểm cấp sổ; đất có phải tài sản chung bố mẹ không; bố mất năm nào và có di chúc hay không.
+Nếu mẹ là chủ sử dụng hợp pháp đối với phần đất định cho: làm hợp đồng tặng cho quyền sử dụng đất có công chứng, rồi sang tên.
+Nếu phải chia di sản của bố: các đồng thừa kế cùng lập văn bản thỏa thuận phân chia di sản tại công chứng. Nếu người anh không ký, gia đình có thể hòa giải; không được thì chồng bạn hoặc mẹ chồng khởi kiện yêu cầu Tòa án chia di sản thừa kế. Văn bản phân chia di sản đã công chứng là căn cứ đăng ký sang tên đất. Điều 59 Luật Công chứng 2024
+Lưu ý, nếu người anh đã từng được bố mẹ cho đất riêng thì điều đó không tự làm mất quyền thừa kế của anh ấy đối với phần di sản của bố, trừ khi có văn bản từ chối nhận di sản hợp lệ hoặc có thỏa thuận phân chia trước đó.
+[1]. Điều 422, 630, 640, 651, Luật 91/2015/QH13
+[2]. Điều 59, Luật 46/2024/QH15</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn các điều luật từ Bộ luật Dân sự 2015 (Điều 422, 630, 640, 651) và Luật Công chứng 2024 (Điều 59). Tuy nhiên, Luật Đất đai 2013 đã bị thay thế bởi Luật Đất đai 2024, và các nghị định cũ cũng đã bị thay thế. Do đó, việc trích dẫn các điều luật từ văn bản cũ không còn hiệu lực là không chính xác. Cần cập nhật các điều luật từ Luật Đất đai 2024 và các nghị định mới để đảm bảo tính hiệu lực.</t>
+  </si>
+  <si>
+    <t>Công ty mình thuê đất của X30- BCA xây dựng nhà xưởng 5300m2. Nhưng khi dịch đến thì BCA mượn làm bệnh viện dã chiến. Đến nay là 5 năm nhưng chưa trả lại nhà xưởng, cũng k trả lại tiền cọc cho doanh nghiệp, thậm chí sang nhà kho cũng k được. Ép bên mình phải thanh lý hợp đồng rồi sẽ trình bộ phương án giải quyết sau. Đây là biên làm việc gần nhất mình xin được chia sẻ để anh chị nắm thông tin cụ thể ạ.</t>
+  </si>
+  <si>
+    <t>Kết luận: Doanh nghiệp không nên ký thanh lý hợp đồng vô điều kiện khi chưa nhận lại tiền cọc, tiền thuê đã trả trước và thỏa thuận rõ số tiền bồi hoàn. Việc bên cho thuê/BCA sử dụng nhà xưởng làm bệnh viện dã chiến không tự xóa nghĩa vụ hoàn trả tài sản bảo đảm và giải quyết hậu quả do không bàn giao được mặt bằng theo hợp đồng.
+Trước hết, cần xác định đúng chủ thể ký hợp đồng: X30/BCA hay đơn vị, doanh nghiệp được BCA ủy quyền. Gửi văn bản yêu cầu bên ký hợp đồng trong thời hạn cụ thể (7–15 ngày): bàn giao lại mặt bằng; hoàn trả cọc; hoàn tiền thuê thời gian không sử dụng được; thanh toán lãi chậm trả và bồi thường thiệt hại nếu hợp đồng hoặc chứng cứ cho phép.
+Không nên ký văn bản có các cụm như “hai bên đã thanh toán xong”, “không còn khiếu nại”, “tự nguyện thanh lý”, hoặc “sẽ trình phương án giải quyết sau”, nếu chưa ghi rõ: số tiền cọc, tiền thuê, thời hạn thanh toán, lãi chậm trả, người có thẩm quyền ký và chế tài nếu không thực hiện. Thỏa thuận hợp đồng hợp pháp có hiệu lực bắt buộc đối với các bên; bên vi phạm nghĩa vụ phải chịu trách nhiệm dân sự. Điều 385 Bộ luật Dân sự 2015 Điều 351 Bộ luật Dân sự 2015
+Nếu việc sử dụng làm bệnh viện dã chiến được coi là sự kiện bất khả kháng, bên thuê vẫn phải xem xét điều khoản về bất khả kháng và thông báo; điều này không mặc nhiên cho phép họ giữ cọc vô thời hạn. Nếu hợp đồng bị chấm dứt hoặc không thể tiếp tục thực hiện, các bên vẫn phải hoàn trả những gì đã nhận, trừ phần nghĩa vụ/thiệt hại được thỏa thuận hoặc pháp luật quy định khác. Điều 351 Bộ luật Dân sự 2015 Điều 420 Bộ luật Dân sự 2015
+Do bên liên quan là cơ quan/đơn vị thuộc BCA, cần tránh đối đầu trực tiếp. Doanh nghiệp nên gửi công văn qua đường văn thư, yêu cầu trả lời bằng văn bản; giữ toàn bộ hợp đồng, phụ lục, biên bản bàn giao, chứng từ cọc/thanh toán, các văn bản về việc trưng dụng/mượn nhà xưởng và biên bản làm việc gần nhất. Nếu không giải quyết, thực hiện cơ chế giải quyết tranh chấp ghi trong hợp đồng (thương lượng, trọng tài hoặc Tòa án); đồng thời đề nghị cơ quan cấp trên có thẩm quyền kiểm tra trách nhiệm của đơn vị ký hợp đồng.
+Lãi do chậm trả tiền được xác định theo thỏa thuận; nếu không có thỏa thuận thì áp dụng theo quy định pháp luật. Điều 357 Bộ luật Dân sự 2015 Điều 468 Bộ luật Dân sự 2015
+[1]. Điều 351, 357, 385, 420, 468, Luật 91/2015/QH13</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn các điều luật từ Bộ luật Dân sự 2015 (Luật số 91/2015/QH13), bao gồm: 
+- Điều 351: Trách nhiệm dân sự do vi phạm nghĩa vụ.
+- Điều 357: Lãi do chậm trả tiền.
+- Điều 385: Hợp đồng dân sự.
+- Điều 420: Thực hiện hợp đồng khi hoàn cảnh thay đổi cơ bản.
+- Điều 468: Lãi suất.
+Các điều luật này đều còn hiệu lực và phù hợp với tình huống tranh chấp hợp đồng thuê đất và việc sử dụng tài sản không đúng mục đích ban đầu. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý liên quan đến việc xử lý hợp đồng, trách nhiệm hoàn trả tài sản và tiền cọc, cũng như các biện pháp giải quyết tranh chấp.</t>
+  </si>
+  <si>
+    <t>Nha hang xom muc đat tu 2013 xuong 5 met lam đất
+ nhà em sut lun xuống gần đến móng nhà, nut tưong
+ nhe den nay 2024nha em muon giai quyet: hang xom
+ phải xây kè để giữ nguyên hiện trạng đất cho nhà e .
+ Mong các luật sư tư vấn cho em ạ</t>
+  </si>
+  <si>
+    <t>Kết luận: Gia đình bạn có thể yêu cầu hàng xóm chấm dứt việc gây sạt lở, xây kè hoặc thực hiện biện pháp kỹ thuật bảo đảm an toàn; nếu họ không hợp tác, có thể yêu cầu UBND xã/phường lập biên bản, hòa giải và khởi kiện yêu cầu khắc phục, bồi thường. Tuy nhiên, do việc múc đất xảy ra từ năm 2013, cần có kết luận hiện trạng để chứng minh sụt lún/nứt nhà hiện nay là hậu quả của việc đó.
+Chủ sở hữu khi đào, hạ thấp nền đất phải bảo đảm không xâm phạm quyền, lợi ích hợp pháp của bất động sản liền kề. Người gây thiệt hại do hành vi xâm phạm tài sản của người khác phải bồi thường; việc bồi thường có thể bao gồm chi phí khảo sát, gia cố/kè, sửa chữa nhà và thiệt hại thực tế khác có chứng từ. Điều 174 Bộ luật Dân sự 2015 Điều 584 Bộ luật Dân sự 2015 Điều 589 Bộ luật Dân sự 2015
+Bạn nên làm ngay:
+Chụp ảnh, quay video vết nứt, vị trí sụt lún; ghi nhận ngày tháng và mời hàng xóm chứng kiến.
+Gửi đơn UBND xã/phường đề nghị kiểm tra hiện trạng, lập biên bản, hòa giải; đề nghị yêu cầu bên hàng xóm tạm ngừng đào/múc thêm nếu còn diễn ra.
+Thuê đơn vị có chuyên môn khảo sát kết cấu/địa chất để kết luận nguyên nhân, mức độ nguy hiểm và giải pháp kè. Đây là chứng cứ quan trọng nhất khi yêu cầu họ chịu chi phí.
+Gửi văn bản yêu cầu hàng xóm xây kè theo phương án kỹ thuật hoặc thanh toán chi phí để gia đình thực hiện. Không tự ý xây kè lấn sang đất họ.
+Nếu hòa giải không thành, khởi kiện tại TAND khu vực nơi có bất động sản, yêu cầu: buộc thực hiện biện pháp chống sạt lở/xây kè; bồi thường chi phí khắc phục và sửa nhà; chịu chi phí giám định, đo đạc hợp lý. Thời hiệu khởi kiện bồi thường thiệt hại là 3 năm kể từ ngày bạn biết hoặc phải biết quyền lợi của mình bị xâm phạm; do đó cần giải thích rõ thời điểm vết nứt, sụt lún hoặc mức nguy hiểm thực tế mới phát hiện/phát sinh, không nên để kéo dài thêm. Điều 588 Bộ luật Dân sự 2015
+Nếu nhà có dấu hiệu nguy hiểm như lún nhanh, nứt dầm/cột, nghiêng tường, hãy báo ngay UBND xã/phường và cơ quan quản lý xây dựng để kiểm tra an toàn; ưu tiên di dời người khỏi khu vực có nguy cơ sập.
+[1]. Điều 174, 584, 588, 589, Luật 91/2015/QH13</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn các điều luật từ Bộ luật Dân sự 2015, bao gồm Điều 174 (quy định về trách nhiệm của chủ sở hữu khi đào, hạ thấp nền đất), Điều 584 (trách nhiệm bồi thường thiệt hại ngoài hợp đồng), Điều 588 (thời hiệu khởi kiện về bồi thường thiệt hại), và Điều 589 (các khoản bồi thường thiệt hại). Các điều luật này đều còn hiệu lực và phù hợp với tình huống pháp lý mà người dùng hỏi, bao gồm việc yêu cầu bồi thường và biện pháp khắc phục hậu quả do hành vi của hàng xóm gây ra.</t>
+  </si>
+  <si>
+    <t>Chào anh chị, đất của em sau khi mua lại thì lúc làm hồ sơ lên thổ cư phát hiện bị sai vị trí trên sổ với thực tế, thực tế em mua miếng đất trống, nhưng trên sổ thì lại là đất bên hàng xóm, đã xây nền làm nhà tiền chế, em thoả thuận vs hàng xóm sẽ bán lại đất cho hàng xóm, nhưng khi làm hồ sơ sang tên cán bộ nói phải đăng kí đo đạc, cho em hỏi, sau khi đo đạc thì phải cấp lại sổ mới rồi mới bán được hay sao ạ, em định chỉ ranh khi đo cho địa chính đúng với miếng đất trên bản vẽ sổ đỏ luôn cho tiện, mà đất đó thì đã xây nền nhưng lại là đất trồng cây lâu năm. 
+Xin anh chị có kinh nghiệm, kiến thức tư vấn giúp em ạ.</t>
+  </si>
+  <si>
+    <t>Kết luận: Không nên “chỉ ranh” theo ý muốn để hợp thức hóa miếng đất khác với vị trí pháp lý đang ghi trên sổ. Trước hết cần đo đạc, xác định nguyên nhân sai lệch và làm thủ tục đính chính/cấp đổi Giấy chứng nhận (hoặc xử lý lại hồ sơ cấp sổ nếu sai nghiêm trọng); sau khi thông tin thửa đất được xác định đúng thì mới nên chuyển nhượng cho hàng xóm.
+ Việc cán bộ yêu cầu đo đạc là hợp lý. Đo đạc nhằm xác định chính xác: thửa đất trên sổ nằm ở đâu, ranh giới thực tế ra sao, diện tích có chênh lệch không, ai đang sử dụng và có chồng lấn với đất hàng xóm hay không. Bản đồ địa chính có thể được chỉnh lý khi cơ quan quản lý hoặc người dân phát hiện sai sót, sai khác về thông tin/rải ranh thửa đất. Điều 6 Nghị định 101/2024/NĐ-CP
+ Bạn không nên ký xác nhận ranh giới sai với thực tế chỉ để bản vẽ “khớp sổ đỏ”. Nếu biết đất trên sổ không phải đất mình đang mua/đang sử dụng mà vẫn kê khai khác thực tế, giao dịch sau này rất dễ bị tranh chấp, bị từ chối đăng ký sang tên; trường hợp khai báo không trung thực làm sai lệch hồ sơ đất đai còn có thể bị xử phạt và buộc làm lại thủ tục. Điều 27 Nghị định 123/2024/NĐ-CP
+ Về cách xử lý, thường có 2 khả năng:
+ Sổ của bạn cấp đúng thửa đất nhưng bản đồ, mốc giới hoặc thông tin trên sổ ghi sai vị trí: đo đạc xong, Văn phòng đăng ký đất đai sẽ kiểm tra và thực hiện đính chính/cấp đổi Giấy chứng nhận để thể hiện đúng thửa đất. Khi sổ mới hoặc trang chỉnh lý đã đúng, bạn ký hợp đồng chuyển nhượng cho hàng xóm.
+ Bạn thực tế mua một thửa khác với thửa ghi trong hợp đồng/sổ: đây không đơn thuần là “đính chính vị trí”. Cần xem lại hợp đồng mua bán trước đây, hồ sơ giao đất/cấp sổ và sự thống nhất của người bán cũ, các chủ đất liên quan. Có thể phải hủy/chỉnh sửa giao dịch cũ hoặc lập giao dịch chuyển quyền đúng đối tượng, chứ không thể tự đổi ranh để lấy thửa đất khác.
+ Mảnh đất hàng xóm đã xây nền, nhà tiền chế nhưng trên giấy là đất trồng cây lâu năm: việc xây dựng nhà có thể là sử dụng đất không đúng mục đích nếu chưa được cơ quan có thẩm quyền cho phép chuyển sang đất ở. Việc chuyển nhượng quyền sử dụng đất vẫn có thể được xem xét nếu đủ điều kiện, nhưng bên mua sẽ nhận đất theo mục đích đất trồng cây lâu năm, không mặc nhiên thành đất ở; thủ tục xin chuyển mục đích và nghĩa vụ tài chính là việc riêng sau đó.
+ Bạn nên làm theo thứ tự: đề nghị đo đạc; yêu cầu Văn phòng đăng ký đất đai trả lời bằng văn bản về nguyên nhân sai vị trí; chỉ ký xác nhận mốc ranh đúng thực tế; hoàn tất đính chính/cấp đổi hoặc xử lý giao dịch cũ; sau đó mới công chứng và đăng ký sang tên. Khi đi làm, mang theo sổ gốc, hợp đồng mua đất, sơ đồ thửa đất, giấy tờ của người bán cũ (nếu có) và văn bản thỏa thuận với hàng xóm.
+ [1]. Điều 6, Nghị định 101/2024/NĐ-CP
+ [2]. Điều 27, Nghị định 123/2024/NĐ-CP</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn Điều 6 của Nghị định 101/2024/NĐ-CP và Điều 27 của Nghị định 123/2024/NĐ-CP. Cả hai điều luật này đều còn hiệu lực và liên quan đến vấn đề đo đạc, chỉnh lý bản đồ địa chính và xử lý sai sót trong hồ sơ đất đai. Điều 6 của Nghị định 101/2024/NĐ-CP liên quan đến việc đo đạc, chỉnh lý bản đồ địa chính khi có sai sót. Điều 27 của Nghị định 123/2024/NĐ-CP liên quan đến việc xử lý sai sót trong hồ sơ đất đai và các biện pháp xử lý khi có sai phạm. Các điều luật này đã bao phủ đầy đủ các khía cạnh cần thiết để giải quyết vấn đề mà người hỏi gặp phải.</t>
+  </si>
+  <si>
+    <t>Nhà em mua đất 200m2 đất không thể tách đôi hay chia Diện tích nhỏ hơn. 
+Hiện có nhà ở bên cạnh đã xây nhà kiên cố cạnh phần đất nhà em. Trước đó nhà đó tự dưng bảo với gia đình em do địa chính cũ đo tọa độ bằng tay nên hiện nay số đo bằng máy khác với số đo bằng tay trước đây cho nên đuôi nhà đó bị xây lệch sang đất nhà em, muốn mua lại chỗ phần xây lấn sang. Nhưng do S đất không thể tách nên nhà đó lại tìm phương án khác…
+Gia đình đó do vợ 2 muốn sang tên sổ Hồng đứng cả tên vợ 2 nên muốn nhà e kí giáp danh để sang tên. Tuy nhiên nhà đó bảo mời bên đo đạc đến đo(không có mặt gia đình em) lại bảo lại không bị sang đất nhà em và đưa tờ giấy ép nhà e kí giáp danh gấp.‼️ 
+Ace hiểu luật cho e hỏi nếu nhà e mời bên đo đạc ở VPCC đến đo, sau đó nên làm gì để chứng minh nhà đó xây nhà không bị xây lấn sang nhà em và tránh rắc rối về sau thì có nên cắm mốc k ạ?</t>
+  </si>
+  <si>
+    <t>Kết luận: Chưa nên ký bất kỳ giấy “giáp ranh” nào nếu gia đình chưa trực tiếp tham gia đo đạc và chưa đối chiếu được ranh đất với hồ sơ địa chính/sổ hồng. Bạn nên đo đạc lại bởi đơn vị có chức năng, lập biên bản ranh giới có chữ ký các bên và cắm mốc bền vững; nếu phát hiện nhà bên cạnh lấn đất thì yêu cầu họ xử lý trước khi ký.
+ Việc đo đạc phải có gia đình bạn tham gia. Ranh giới thửa đất không chỉ dựa vào lời nói hay một lần đo riêng của hàng xóm; cần đối chiếu Giấy chứng nhận, trích lục/trích đo địa chính và hiện trạng. Khi đo, đơn vị đo đạc phải phối hợp với các chủ đất liền kề để chỉ ranh, đánh dấu các đỉnh thửa tại thực địa hoặc đóng cọc theo kết quả xác định ranh giới. Điều 13 Thông tư 26/2024/TT-BTNMT Điều 15 Thông tư 26/2024/TT-BTNMT
+ Không ký “giáp ranh” gấp hoặc ký khống. Chữ ký của bạn có thể bị dùng làm căn cứ rằng gia đình đã xác nhận ranh hiện tại là đúng, từ đó gây bất lợi nếu sau này phát hiện phần móng, tường hoặc đuôi nhà đã lấn sang đất. Việc họ sang tên sổ hồng cho vợ hai là giao dịch nội bộ của họ; gia đình bạn chỉ cần ký khi văn bản thực sự xác định đúng ranh giới với đất nhà bạn.
+ Cách làm an toàn:
+ Gửi văn bản hoặc tin nhắn rõ ràng: “Gia đình chỉ ký xác nhận sau khi cùng tham gia đo đạc, được cung cấp bản trích đo và kiểm tra thực địa.”
+ Thuê đơn vị đo đạc có tư cách hoạt động đo đạc bản đồ; yêu cầu lập bản trích đo địa chính/bản mô tả ranh giới, mốc giới, bảng tọa độ các điểm góc thửa.
+ Mời hàng xóm, đại diện UBND xã/phường hoặc cơ quan quản lý đất đai địa phương cùng chứng kiến nếu đang có dấu hiệu tranh chấp.
+ Khi ranh đã thống nhất, nên cắm mốc tại các điểm góc thửa bằng mốc bê tông/đinh sắt phù hợp hiện trạng; chụp ảnh, quay video, ghi nhận tọa độ và lập biên bản. Không tự ý cắm mốc lấn sang phần đất đang tranh chấp.
+ Chỉ ký khi giấy ghi đúng: số thửa, tờ bản đồ, diện tích, sơ đồ ranh, tọa độ mốc; và thêm câu: “Việc ký xác nhận chỉ xác nhận ranh giới theo bản trích đo kèm theo, không xác nhận quyền sở hữu công trình xây dựng nếu có dấu hiệu lấn chiếm.”
+ Nếu kết quả đo cho thấy có lấn đất: không ký xác nhận ranh theo hiện trạng công trình. Yêu cầu hàng xóm cùng lập biên bản, thỏa thuận phương án trả lại đất/tháo dỡ phần lấn chiếm hoặc nhận chuyển nhượng phần đất lấn chiếm nếu pháp luật và điều kiện tách thửa cho phép. Khi không tự thỏa thuận được, gửi đơn đề nghị hòa giải tranh chấp đất đai tại UBND xã/phường nơi có đất trước khi khởi kiện. Luật Đất đai 2024
+ Lưu ý: Văn phòng công chứng không phải cơ quan xác định chính thức ranh giới đất; họ có thể hỗ trợ chứng thực/chứng kiến theo</t>
+  </si>
+  <si>
+    <t>Câu trả lời có trích dẫn Điều 13 và Điều 15 của Thông tư 26/2024/TT-BTNMT. Tuy nhiên, Thông tư này không tồn tại hoặc không có hiệu lực hiện hành. Ngoài ra, không có điều luật nào từ Luật Đất đai 2024 được trích dẫn cụ thể. Do đó, tiêu chí trích dẫn điều luật bị đánh giá là không đúng.</t>
+  </si>
+  <si>
+    <t>Cho minh hỏi .năm 1997 anh rể minh có cho vk ck mình một mảnh đật và vk ck mình đã xây dựng nhà ở từ năm 1997 đến hiện tại bây giờ và kèm theo giấy viết tay của 2vk ck anh rể cho vk ck mình .nhưng giờ anh rể minh làm đơn ra tòa đòi lại. Mình xin chân thành gủi đến cồng động mạng cho mình lời ý kiến chân thâ</t>
+  </si>
+  <si>
+    <t>Kết luận: Anh rể không đương nhiên lấy lại được đất chỉ vì đã làm đơn kiện. Giấy viết tay, việc vợ chồng bạn đã xây nhà và ở công khai, ổn định từ năm 1997 là chứng cứ rất quan trọng để Tòa án xem xét việc anh rể đã cho đất hay chỉ cho ở nhờ.
+ Nếu giấy viết tay thể hiện rõ anh rể và vợ đã “cho/tặng” thửa đất cho vợ chồng bạn, có chữ ký; việc giao đất đã thực hiện, gia đình bạn quản lý và xây nhà suốt gần 30 năm mà họ không phản đối, thì bạn có cơ sở yêu cầu Tòa công nhận giao dịch tặng cho/chuyển quyền và bảo vệ quyền sử dụng thực tế. Tuy vậy, nếu đất khi cho chưa có sổ đỏ hoặc giấy cho chỉ ghi mơ hồ là “cho ở”, vụ việc sẽ cần xem kỹ chứng cứ.
+ Bạn cần nộp cho Tòa án:
+ Bản gốc giấy viết tay cho đất; đề nghị giám định chữ ký nếu bên kia phủ nhận.
+ Chứng cứ xây nhà từ năm 1997: biên lai vật liệu, ảnh, xác nhận hàng xóm, giấy phép/xác nhận xây dựng nếu có.
+ Hồ sơ cư trú, hóa đơn điện nước, thuế nhà đất, xác nhận sử dụng đất ổn định.
+ Người làm chứng biết việc cho đất, việc bạn xây nhà và anh rể không phản đối.
+ Giấy tờ về nguồn gốc đất, sổ đỏ (nếu anh rể đang đứng tên), sơ đồ hoặc đo đạc thực tế.
+ Về nguyên tắc, hợp đồng tặng cho bất động sản phải được lập theo hình thức luật định và quyền đối với bất động sản thường phát sinh khi đăng ký. Nhưng với giao dịch rất cũ đã thực hiện trên thực tế, Tòa án sẽ đánh giá toàn bộ quá trình giao đất, nhận đất, xây nhà, quản lý công khai và ý chí thực sự của các bên, không chỉ nhìn vào việc giấy tay chưa công chứng. Điều 459 Bộ luật Dân sự 2015
+ Tranh chấp quyền sử dụng đất thường không bị áp dụng thời hiệu khởi kiện; vì vậy, việc đã qua từ năm 1997 không tự động làm anh rể mất quyền kiện, nhưng thời gian sử dụng ổn định kéo dài lại là chứng cứ có lợi rất lớn cho phía bạn. Điều 155 Bộ luật Dân sự 2015
+ Nếu anh rể kiện đòi đất, vợ chồng bạn cần gửi văn bản ý kiến cho Tòa, nêu rõ: đất là tài sản đã được cho; đã giao và nhận từ năm 1997; gia đình đã đầu tư xây nhà, quản lý liên tục, công khai; yêu cầu Tòa bác yêu cầu đòi đất hoặc công nhận quyền sử dụng đất/giao dịch cho đất. Không nên tự ý ký giấy “trả đất”, “thừa nhận ở nhờ” hoặc hòa giải theo nội dung bất lợi khi chưa hiểu rõ.
+ Ngay cả trường hợp Tòa không công nhận việc cho đất vì vướng hình thức, việc nhà được xây từ lâu và có sự biết, không phản đối của anh rể có thể làm phát sinh yêu cầu xem xét giá trị căn nhà, chi phí đầu tư và lỗi của các bên khi giải quyết hậu quả giao dịch.
+ [1]. Điều 155, 459, Luật 91/2015/QH13</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 155 và 459 của Bộ luật Dân sự 2015 (Luật 91/2015/QH13), tuy nhiên, không có điều luật nào từ Luật Đất đai 2024 hoặc các nghị định mới liên quan đến việc tặng cho đất đai. Bộ luật Dân sự 2015 vẫn còn hiệu lực, nhưng cần bổ sung các quy định từ Luật Đất đai 2024 để đảm bảo tính đầy đủ và cập nhật của câu trả lời.</t>
+  </si>
+  <si>
+    <t>Luật sư cho em hỏi đất của cha ông để lại nhưng năm 1995 sổ quy chủ và sổ đỏ đứng tên bố mẹ em và 5 người con ong bà ở cùng vườn nhưng hộ khẩu khác hơn 10 năm sau ông đã mất bà nội kêu bác và bố về làm giấy thỏa thuận trong giấy ghi bà lấy lại 200 m2 làm nơi thờ cúng còn nữa bà cho bố em và bố và bác kí rồi bà điểm chỉ đến ub xã xác nhận và 2 người làm chứng mà mẹ em và mấy người con ko nhất trí vậy xin hỏi bản thỏa thuận này có hợp pháp ko ạ hay để lâu dài có phức tạp ko ạ nhờ luật sư tư vấn gúp</t>
+  </si>
+  <si>
+    <t>Kết luận: Nếu Giấy chứng nhận năm 1995 ghi tên bố mẹ bạn và 5 người con cùng có quyền sử dụng thửa đất, thì bà nội không thể tự quyết định “lấy lại” hoặc cho bố bạn 200 m² chỉ bằng giấy có chữ ký của bà, bố và bác. Văn bản đó có nguy cơ không có hiệu lực đối với phần quyền sử dụng đất của mẹ bạn và các người con không ký/không ủy quyền; để lâu sẽ rất dễ phát sinh tranh chấp thừa kế, chia đất và sang tên.
+ Cần phân biệt hai khả năng:
+ 200 m² đã thuộc quyền sử dụng chung của những người đứng tên sổ đỏ năm 1995: Mọi việc tặng cho, chia, chuyển quyền hoặc dành riêng phần đất này phải có sự tham gia của tất cả người có quyền trên sổ đỏ, hoặc có văn bản ủy quyền hợp lệ. Với đất chung không thể chia theo phần, các thành viên phải cùng thực hiện quyền hoặc ủy quyền cho đại diện thực hiện. Điều 27 Luật Đất đai 2024
+ 200 m² thực tế vẫn là tài sản riêng của bà nội, chưa từng được đưa vào diện tích cấp cho bố mẹ và các con: bà có thể định đoạt phần đất của mình. Tuy nhiên, phải xác định bằng sổ đỏ, hồ sơ địa chính, nguồn gốc đất và ranh giới; không thể chỉ dựa vào lời nói “đất cha ông để lại”.
+ Giấy “thỏa thuận” có UBND xã xác nhận và người làm chứng chưa chắc là hợp đồng chuyển quyền đất hợp lệ. Cần xem UBND xã xác nhận nội dung gì: chỉ xác nhận chữ ký, hay chứng thực hợp đồng/giao dịch. Đồng thời, giao dịch chuyển quyền sử dụng đất thông thường phải được công chứng hoặc chứng thực và phải đăng ký biến động thì mới đủ điều kiện làm thủ tục thay đổi trên sổ đỏ. Điều 27 Luật Đất đai 2024
+ Việc mẹ và các con không đồng ý là rất quan trọng nếu họ là người cùng đứng tên hoặc có quyền đối với đất. Họ không bị mất quyền chỉ vì không ký giấy; bố bạn cũng không thể tự ký thay phần quyền của vợ và con, trừ khi có ủy quyền hợp pháp.
+ Nên làm ngay:
+ Giữ bản gốc/ảnh chụp sổ đỏ năm 1995 và giấy thỏa thuận;
+ Xin trích lục hồ sơ cấp sổ, bản đồ/thửa đất tại cơ quan đăng ký đất đai để xác định chính xác 200 m² nằm trong diện tích của ai;
+ Không ký tiếp giấy tách thửa, sang tên, chỉnh lý sổ đỏ khi chưa thống nhất;
+ Nếu cần giữ nơi thờ cúng, nên lập thỏa thuận mới có đầy đủ người có quyền ký, xác định rõ vị trí, diện tích 200 m², quyền quản lý, người sử dụng và việc không được tự ý chuyển nhượng.
+ Bạn cần kiểm tra đúng dòng “Người sử dụng đất” trên sổ đỏ năm 1995: ghi tên từng người, ghi “hộ ông/bà”, hay chỉ ghi tên bố/mẹ. Chi tiết này quyết định ai phải ký và bà nội còn quyền với phần đất đó hay không.
+ [1]. Điều 27, Luật 31/2024/QH15</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 27 của Luật Đất đai 2024 (Luật số 31/2024/QH15), tuy nhiên, nội dung của Điều 27 không được mô tả rõ ràng và không có sự xác nhận về tính hiệu lực của điều luật này trong ngữ cảnh cụ thể. Ngoài ra, câu trả lời không trích dẫn đầy đủ các điều luật liên quan đến việc chuyển nhượng quyền sử dụng đất, thừa kế và các quy định về công chứng, chứng thực giao dịch đất đai. Do đó, tiêu chí trích dẫn điều luật bị đánh giá là không đạt.</t>
+  </si>
+  <si>
+    <t>Xin các anh/chị tư vấn giúp.
+ Em có mua 1 miếng đất trong đó có 400m2 thổ cư, đã hoàn tất các thủ tục công chứng chuyển nhượng, chuyển khoản đầy đủ tiền mua đất + tiền cò. Tới bước nộp hồ sơ vào phòng TN thì mới phát hiện đất lệch diện tích, khi gọi địa chính vào đo thì lại phát hiện có tranh chấp với hàng xóm, cun thể là hàng xóm lấn đất diện tích rất nhiều.
+ Em không thể nhận chuyển nhượng được, đã trao đổi lại với chủ cũ trả lại bớt tiền đúng với diện tích bị mất, nhưng chủ cũ cho rằng đã là hợp đồng rồi thì không trả lại, còn họ sẽ hỗ trợ đòi lại đất vì đất đó là của họ.
+ Hợp đồng của em bị dính điều khoản phải đóng tất cả các khoản thuế bao gồm cả thuế thu nhập của bên bán, thuế đất hàng năm.
+ Tuy nhiên em vẫn chưa nhận được chuyển nhượng, chưa được bàn giao đủ đất (vẫn giữ nguyên hiện trạng) thì các nghĩa vụ này do bên nào chịu trách nhiệm ạ? Và mình cần làm gì để ép chủ cũ phải có trách nhiệm sớm đòi lại đất cho mình ạ</t>
+  </si>
+  <si>
+    <t>Kết luận: Bạn chưa nên nộp thêm tiền thuế, phí hoặc nhận đất theo hiện trạng thiếu diện tích. Bên bán phải chịu trách nhiệm giao đúng thửa đất, đúng ranh giới và diện tích đã cam kết; nếu không khắc phục được trong thời hạn hợp lý, bạn có quyền yêu cầu giảm giá tương ứng hoặc hủy hợp đồng, đòi lại tiền đã thanh toán và bồi thường thiệt hại (nếu có căn cứ).
+ 1. Về diện tích đất bị thiếu và đất đang tranh chấp
+ Việc công chứng hợp đồng không có nghĩa là bên bán được miễn nghĩa vụ giao đất đúng thỏa thuận. Bạn cần đối chiếu kỹ: hợp đồng công chứng, Giấy chứng nhận, trích lục/trích đo địa chính và biên bản đo thực tế để xác định thiếu bao nhiêu m², thiếu phần nào, có thuộc đúng thửa đã mua không.
+ Nếu hàng xóm đang lấn chiếm phần đất thuộc quyền sử dụng hợp pháp của bên bán, bên bán phải chủ động giải quyết tranh chấp và bàn giao cho bạn đủ đất. Bạn không bắt buộc nhận phần đất thiếu rồi tự đi kiện hàng xóm, trừ khi hai bên có thỏa thuận mới rõ ràng về việc này. Bên chuyển nhượng cũng phải bảo đảm điều kiện chuyển nhượng, trong đó quyền sử dụng đất không bị kê biên và còn trong thời hạn sử dụng; việc có tranh chấp thực tế là rủi ro pháp lý nghiêm trọng đối với giao dịch Điều 45 Luật Đất đai 2024.
+ Bạn có thể chọn một trong các hướng:
+ Yêu cầu bên bán giải quyết tranh chấp, hoàn trả đủ phần đất và hoàn tất bàn giao trong một thời hạn cụ thể;
+ Thỏa thuận giảm giá/hoàn tiền theo diện tích thực tế bị thiếu, lập phụ lục hợp đồng và xác định rõ ranh giới, diện tích chuyển nhượng thực nhận;
+ Nếu bên bán không giao được đủ đất hoặc không xử lý tranh chấp đúng hạn: yêu cầu hủy/chấm dứt hợp đồng, hoàn trả toàn bộ tiền mua đất, tiền thuế/phí bạn đã nộp thay (nếu có), lãi chậm trả và thiệt hại thực tế.
+ 2. Thuế, phí và nghĩa vụ tài chính
+ Về quan hệ với cơ quan thuế, thuế thu nhập cá nhân từ chuyển nhượng bất động sản là thu nhập của người bán. Tuy nhiên, các bên được thỏa thuận người mua nộp thay. Vì hợp đồng của bạn ghi bạn chịu cả thuế thu nhập cá nhân của bên bán, cơ quan thuế có thể căn cứ thỏa thuận đó khi kê khai; nhưng đây chỉ là phân chia chi phí giữa hai bên, không làm mất quyền yêu cầu hoàn lại nếu giao dịch bị hủy do lỗi hoặc do bên bán không giao đúng đất.
+ Thuế sử dụng đất phi nông nghiệp hằng năm về nguyên tắc gắn với người có quyền sử dụng đất. Khi bạn chưa đăng ký sang tên và chưa được giao đủ đất, bên bán vẫn là người đứng tên trên Giấy chứng nhận; bạn không nên tự nộp khoản này nếu chưa có thỏa thuận rõ về thời điểm bạn nhận bàn giao và nhận nghĩa vụ. Thuế thu nhập cá nhân đối với chuyển nhượng quyền sử dụng đất tính theo giá chuyển nhượng, thuế suất 2% Điều 29 Luật Thuế thu nhập cá nhân.
+ Đặc biệt, nếu hồ sơ sang tên chưa hoàn tất do đất tranh chấp hoặc không khớp hiện trạng, bạn nên yêu cầu cơ quan tiếp nhận hồ sơ trả lời bằng văn bản về lý do tạm dừng/trả hồ sơ; không ký thêm giấy tờ xác nhận đã nhận đủ đất hoặc nhận bàn giao hiện trạng.
+ 3. Việc nên làm ngay
+ Gửi bên bán một văn bản yêu cầu thực hiện hợp đồng, bằng thư bảo đảm hoặc vi bằng/thừa phát lại nếu cần. Nêu rõ: diện tích thiếu, vị trí tranh chấp, tài liệu đo đạc kèm theo, thời hạn yêu cầu bên bán xử lý và bàn giao đủ đất (ví dụ 15–30 ngày).
+ Trong văn bản, ghi rõ nếu quá hạn bạn sẽ lựa chọn: giảm giá và hoàn tiền phần thiếu; hoặc yêu cầu Tòa án hủy hợp đồng, buộc hoàn trả tiền, lãi và bồi thường. Không nên chỉ trao đổi bằng điện thoại hay tin nhắn không đầy đủ.
+ Đề nghị UBND cấp xã tổ chức hòa giải tranh chấp ranh giới/lấn chiếm giữa bên bán và hàng xóm. Tranh chấp đất đai phải được hòa giải tại UBND cấp xã trước khi khởi kiện theo thủ tục tranh chấp đất đai Điều 235 Luật Đất đai 2024. Bạn nên yêu cầu bên bán đứng đơn hoặc cùng ký đơn, vì hiện bên bán vẫn là người đứng tên quyền sử dụng đất.
+ Nếu bên bán không hợp tác, bạn có thể khởi kiện tại Tòa án yêu cầu buộc thực hiện đúng hợp đồng hoặc hủy hợp đồng và hoàn tiền. Khi khởi kiện, có thể đề nghị Tòa áp dụng biện pháp khẩn cấp tạm thời để ngăn bên bán chuyển nhượng, thế chấp hoặc định đoạt thửa đất trong thời gian giải quyết.
+ 4. Lưu ý về tiền “cò”
+ Khoản tiền môi giới chỉ đòi lại được tùy theo thỏa thuận với môi giới và lỗi của họ. Nếu môi giới biết hoặc phải biết tình trạng lấn chiếm, diện tích không đúng nhưng vẫn cung cấp thông tin sai, cam kết sai hoặc che giấu thông tin để bạn giao kết, bạn có cơ sở yêu cầu hoàn tiền môi giới và bồi thường thiệt hại. Giữ toàn bộ tin nhắn quảng cáo, giấy giới thiệu, ghi âm, phiếu thu và chứng từ chuyển khoản.
+ Bạn nên giữ: hợp đồng công chứng; Giấy chứng nhận; biên bản đo đạc; ảnh/video mốc giới; hồ sơ bị từ chối/tạm dừng sang tên; toàn bộ chứng từ thanh toán; trao đổi với bên bán và môi giới. Đây là chứng cứ quan trọng nhất để buộc bên bán chịu trách nhiệm.
+ [1]. Điều 45, 235, Luật 31/2024/QH15
+ [2]. Điều 29, Luật 04/2007/QH12</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 45 và 235 của Luật Đất đai 2024 (Luật số 31/2024/QH15) và Điều 29 của Luật Thuế thu nhập cá nhân 2007 (Luật số 04/2007/QH12). Tuy nhiên, không có điều luật nào trong Luật Đất đai 2024 có số điều 45 và 235, do đó việc trích dẫn này là không chính xác và không tồn tại. Điều 29 của Luật Thuế thu nhập cá nhân 2007 vẫn còn hiệu lực và đúng với nội dung về thuế suất 2% cho chuyển nhượng quyền sử dụng đất. Tuy nhiên, việc trích dẫn điều luật về thuế không bao phủ toàn bộ vấn đề pháp lý của câu hỏi, đặc biệt là về tranh chấp đất đai và trách nhiệm của bên bán.</t>
+  </si>
+  <si>
+    <t>Em muốn hỏi về vấn đề lấn chiếm đất công hẽm công cộng. Công trình xây dựng lấn chiếm trái phép đã hơn 5 năm mà uỷ ban địa phương vẫn chưa giải quyết thoả đáng và công trình đó hiện tại xuống cấp sắt thép trên cao hơn chục mét có dấu hiệu rơi sang nhà em. Gần đây em cũng đã tiếp tục gửi đơn xin uỷ ban giải quyết sớm nhưng uỷ ban đến nay đã hơn 4 tháng vẫn chưa trà lời văn bản cho em. Mong quý anh chị tư vấn giúp em. Em ở Vĩnh Long ạ</t>
+  </si>
+  <si>
+    <t>Kết luận: Bạn nên tách vụ việc thành 2 hướng xử lý đồng thời: (1) yêu cầu xử lý khẩn cấp nguy cơ sắt thép/vật liệu rơi gây tai nạn; (2) khiếu nại việc cơ quan có thẩm quyền chậm hoặc không giải quyết đơn về hành vi lấn chiếm hẻm công cộng. Việc công trình tồn tại hơn 5 năm không làm hợp thức hóa hành vi lấn chiếm đất công hoặc phần lối đi công cộng.
+ 1. Việc cần làm ngay để bảo vệ an toàn
+ Gửi ngay một đơn có tiêu đề: “Đơn đề nghị kiểm tra, áp dụng biện pháp khẩn cấp bảo đảm an toàn công trình” đến UBND phường/xã nơi có công trình, đồng gửi UBND tỉnh Vĩnh Long, cơ quan quản lý xây dựng cấp tỉnh và Công an phường/xã.
+ Nêu rõ: vị trí công trình; sắt thép ở độ cao hơn 10m đang xuống cấp, có nguy cơ rơi vào nhà/người; yêu cầu lập biên bản hiện trạng, khoanh vùng nguy hiểm, buộc chủ công trình che chắn/tháo dỡ phần nguy hiểm và trả lời bằng văn bản. Kèm ảnh, video có ngày giờ, bản sao các đơn cũ và giấy tiếp nhận/bằng chứng đã gửi đơn.
+ Nếu có dấu hiệu sắt thép sắp rơi hoặc đang gây nguy hiểm tức thời, gọi 113 hoặc 114, đồng thời báo chính quyền địa phương để lập biên bản. Không tự ý trèo lên, tháo dỡ hoặc tác động vào công trình vì có thể nguy hiểm và phát sinh tranh chấp.
+ Chủ sở hữu hoặc người quản lý công trình có nghĩa vụ bảo đảm an toàn cho người, tài sản và công trình lân cận; nếu gây thiệt hại thì phải bồi thường. Điều 605 Bộ luật Dân sự 2015
+ 2. Về lấn chiếm hẻm công cộng
+ Hẻm ở Vĩnh Long được xác định là đường hoặc lối đi công cộng đã hoàn chỉnh hạ tầng và đưa vào sử dụng; vì vậy, cần xác minh cụ thể phần bị xây lấn có thuộc đất giao thông/lối đi công cộng theo hồ sơ địa chính, quy hoạch hoặc quản lý thực tế hay không. Điều 2 Nghị quyết 39/2025/NQ-HĐND
+ Trong đơn, bạn không nên chỉ ghi chung là “đất công”. Hãy yêu cầu cơ quan nhà nước: xác minh mốc giới; cung cấp thông tin thửa đất/quy hoạch; xác định phần diện tích hẻm bị chiếm; kiểm tra giấy phép xây dựng (nếu có); xử lý hành vi xây dựng/lấn chiếm trái phép và khôi phục lối đi công cộng nếu có vi phạm.
+ 3. Việc UBND chưa trả lời hơn 4 tháng
+ Nếu đơn của bạn là khiếu nại về hành vi hành chính hoặc việc không thực hiện nhiệm vụ của cơ quan/người có thẩm quyền, thời hạn giải quyết lần đầu thông thường là 30 ngày; vụ việc phức tạp có thể tối đa 45 ngày, không tính thời gian xác minh ở vùng sâu, vùng xa theo luật. Điều 28 Luật Khiếu nại 2011
+ Khi hết thời hạn mà không được giải quyết, bạn có quyền khiếu nại lần hai đến cấp trên trực tiếp của người có thẩm quyền giải quyết lần đầu, hoặc khởi kiện vụ án hành chính tại Tòa án. Điều 33 Luật Khiếu nại 2011
+ Bạn nên gửi Đơn khiếu nại về việc không giải quyết/giải quyết chậm đơn đến Chủ tịch UBND cấp trên trực tiếp, kèm toàn bộ chứng cứ nộp đơn trước đây. Yêu cầu nêu rõ: buộc trả lời bằng văn bản; kiểm tra trách nhiệm người tiếp nhận, xử lý; tổ chức kiểm tra hiện trường khẩn cấp do nguy cơ mất an toàn.
+ 4. Hồ sơ nên chuẩn bị
+ Ảnh/video toàn cảnh hẻm, phần lấn chiếm và sắt thép xuống cấp; nên quay từ vị trí nhà bạn để thể hiện nguy cơ rơi sang nhà.
+ Đơn cũ, biên nhận, phiếu chuyển đơn, tin nhắn/email hoặc giấy báo phát bưu điện.
+ Bản đồ, trích lục, giấy tờ nhà đất của bạn (nếu có); chữ ký/xác nhận của các hộ dân cùng bị ảnh hưởng.
+ Nhật ký theo ngày về thời điểm phát hiện nguy hiểm, đã báo ai và phản hồi nhận được.
+ Khi nộp đơn, hãy yêu cầu đóng dấu nhận trên bản lưu; nếu gửi bưu điện thì gửi bảo đảm và giữ phiếu gửi. Trọng tâm trước mắt là buộc cơ quan kiểm tra, ngăn nguy cơ tai nạn; việc xử lý dứt điểm phần lấn chiếm sẽ cần dựa trên kết quả xác minh đất đai, lộ giới và giấy phép xây dựng.
+ [1]. Điều 28, 33, Luật 02/2011/QH13</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 605 Bộ luật Dân sự 2015 và Điều 28, 33 Luật Khiếu nại 2011. Các điều luật này vẫn còn hiệu lực và phù hợp với vấn đề an toàn công trình và khiếu nại hành chính. Tuy nhiên, câu trả lời không trích dẫn điều luật cụ thể về lấn chiếm đất công cộng, và không cập nhật theo Luật Đất đai 2024 và các nghị định mới liên quan. Do đó, tiêu chí trích dẫn điều luật bị đánh giá là false.</t>
+  </si>
+  <si>
+    <t>Nhà em có cho người thuê đất sau đó họ tự dựng xưởng lên . Hết hạn hợp đồng họ ko chuyển đi . Rất láo toét, đã thuê 10 năm. Sau đó nhà em bị thu hồi đất , nhà nước đền bù tiền xưởng, nhà em đã nhận tiền , nhưng người thuê bảo đó là tiền xưởng của họ . Họ gửi đơn kiện nhà em là tội chiếm đoạt tài sản . Vậy có phải là hình sự ko ạ . Nhà em mà bị thua kiện thì có thiệt hại gì không ạ ! Được 200 nhà em đã trả 150 mà nó còn không chịu . Cuối cùng nó đã chịu cầm 150 triệu còn xin 10 tháng tiền thuê chỗ . Khi công an vào cuộc . Đúng loại bẩn bựa.</t>
+  </si>
+  <si>
+    <t>Kết luận: Theo thông tin bạn nêu, đây trước hết là tranh chấp dân sự về quyền sở hữu nhà xưởng và tiền bồi thường, chưa thể coi là tội “chiếm đoạt tài sản” chỉ vì gia đình bạn đã nhận tiền bồi thường. Muốn xử lý hình sự, cơ quan điều tra phải chứng minh gia đình bạn có thủ đoạn gian dối hoặc ý thức chiếm giữ trái pháp luật tài sản chắc chắn thuộc người thuê; việc hai bên còn tranh cãi ai là chủ xưởng thường là dấu hiệu của tranh chấp dân sự.
+ Người thuê tự dựng xưởng trên đất thuê không đồng nghĩa họ đương nhiên được nhận toàn bộ tiền bồi thường. Cần xem rất kỹ: hợp đồng thuê đất; điều khoản về việc xây xưởng, xử lý xưởng khi hết hạn thuê; biên bản bàn giao/hoàn trả đất; hồ sơ kiểm đếm, phương án bồi thường và quyết định phê duyệt bồi thường của cơ quan có thẩm quyền.
+ Nếu phương án bồi thường ghi gia đình bạn là người được nhận tiền, gia đình nhận theo quyết định đó thì đây là căn cứ rất quan trọng để bảo vệ mình. Nếu người thuê cho rằng tiền xưởng thuộc họ, họ cần khởi kiện dân sự để yêu cầu chia/hoàn trả tiền; không thể chỉ gửi đơn tố giác là gia đình bạn tự động thành bị can.
+ Tội lừa đảo chỉ đặt ra khi có hành vi dùng thủ đoạn gian dối để chiếm đoạt tài sản; tội lạm dụng tín nhiệm đòi hỏi có việc nhận tài sản hợp pháp rồi dùng thủ đoạn, bỏ trốn hoặc dù có khả năng mà cố tình không trả nhằm chiếm đoạt. Các dấu hiệu này phải được chứng minh cụ thể, không được suy diễn từ một tranh chấp hợp đồng thuê và bồi thường đất đai. Điều 174 Bộ luật Hình sự 2015 Điều 175 Bộ luật Hình sự 2015
+ Việc gia đình đã trả 150 triệu đồng và người thuê đã nhận khoản này, kèm thỏa thuận hỗ trợ 10 tháng tiền thuê chỗ, là tình tiết có lợi. Nếu có giấy nhận tiền, biên bản hòa giải, tin nhắn hoặc ghi âm thể hiện họ đồng ý nhận để giải quyết vụ việc, cần giữ thật kỹ. Tuy nhiên, nếu giấy tờ có ghi “tạm nhận”, “không từ bỏ quyền khởi kiện” hoặc chưa phải thỏa thuận chấm dứt toàn bộ tranh chấp thì họ vẫn có thể kiện dân sự.
+ Nếu gia đình “thua kiện” dân sự, rủi ro chính thường là:
+ Phải trả thêm phần tiền bồi thường xưởng mà Tòa xác định thuộc người thuê;
+ Có thể phải trả lãi chậm trả tính từ khi bị yêu cầu hợp lệ hoặc từ thời điểm bản án có hiệu lực;
+ Chịu án phí dân sự tương ứng phần nghĩa vụ bị buộc trả;
+ Nếu đã có thỏa thuận 150 triệu là khoản thanh toán cuối cùng, số này phải được tính trừ khi xác định nghĩa vụ còn lại.
+ Gia đình nên chuẩn bị ngay: hợp đồng thuê và phụ lục; giấy tờ chứng minh ngày hết hạn thuê và yêu cầu họ trả đất; hồ sơ thu hồi đất, kiểm đếm, phương án/ quyết định bồi thường; chứng cứ xưởng được xây khi nào, bằng tiền ai, có được chủ đất cho phép không; chứng từ trả 150 triệu; văn bản hoặc chứng cứ về hỗ trợ 10 tháng thuê chỗ.
+ Khi làm việc với công an, gia đình nên trình bày nhất quán: tiền được nhận theo hồ sơ bồi thường của Nhà nước; quyền sở hữu xưởng đang có tranh chấp; gia đình không gian dối, không bỏ trốn, đã thiện chí chi trả/hỗ trợ. Đề nghị cơ quan tiếp nhận xác định đây là tranh chấp dân sự nếu không có chứng cứ về hành vi chiếm đoạt. Không nên ký giấy thừa nhận “chiếm đoạt” hoặc cam kết trả thêm tiền khi chưa đối chiếu toàn bộ hồ sơ.
+ [1]. Điều 174, 175, Luật 100/2015/QH13</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 174 và 175 của Bộ luật Hình sự 2015 (Luật 100/2015/QH13) về tội lừa đảo chiếm đoạt tài sản và tội lạm dụng tín nhiệm chiếm đoạt tài sản. Tuy nhiên, không có điều luật nào từ Luật Đất đai 2024 hoặc các nghị định mới liên quan đến bồi thường khi thu hồi đất được trích dẫn. Do đó, việc trích dẫn điều luật không đầy đủ và không cập nhật theo luật hiện hành.</t>
+  </si>
+  <si>
+    <t>Em đang gặp một tình huống mong muốn các anh chị tư vấn giúp em.
+ Hôm trước em có cọc tiền 100tr mua 1 mảnh đất có nhà bên trên đất ( hợp đồng cọc viết tay có môi giới làm chứng). Đến khi đo đạc lại thì diện tích đất lớn hơn diện tích sổ 5 m2, và không biết 5m2 thừa ở đâu ra vì chủ hiện tại cũng mua qua vài đời chủ rồi.
+ Thấy vậy chủ hiện tại đòi tăng giá và nếu không đồng ý sẽ trả lại tiền cọc và có ý không bồi thường cọc. ( trong hợp đồng cọc có ghi nếu chủ không bán sẽ phải đền cọc 300tr).
+ Vài ngày nữa là đến hẹn công chứng mua bán nên em chưa biết sử lý trường hợp này sao.
+ Do là có bán số lượng vàng trước đó để chuẩn bị tiền, nay vàng lên tính ra mất 50tr mà không mua được đất nên cảm thấy khá buồn.
+ Mong các anh chị tư vấn giúp em xử lý thế nào ạ.</t>
+  </si>
+  <si>
+    <t>Kết luận: Nếu giấy đặt cọc ghi rõ bên bán không bán phải “đền cọc 300 triệu đồng”, việc bên bán tự tăng giá rồi từ chối bán theo giá đã thỏa thuận có dấu hiệu vi phạm cam kết đặt cọc. Bạn có quyền yêu cầu họ tiếp tục ký hợp đồng theo giá cũ hoặc khởi kiện yêu cầu trả khoản phạt cọc 300 triệu đồng; không nên nhận lại 100 triệu rồi ký giấy xác nhận đã giải quyết xong nếu chưa đồng ý.
+ Diện tích đo thực tế lớn hơn sổ 5 m² không tự động là lý do hợp pháp để bên bán đơn phương nâng giá. Khi công chứng chuyển nhượng, quyền sử dụng đất được chuyển giao theo diện tích, ranh giới và thông tin trên Giấy chứng nhận; 5 m² chênh lệch phải được làm rõ bằng đo đạc, hồ sơ địa chính trước khi giao dịch. Nếu phần này chưa có giấy tờ, không chắc thuộc quyền sử dụng hợp pháp của bên bán thì bạn càng không nên chấp nhận trả thêm tiền.
+ Theo quy định về đặt cọc, nếu bên nhận cọc từ chối giao kết/thực hiện hợp đồng thì phải trả lại tiền cọc và trả thêm một khoản tương đương giá trị cọc, trừ khi các bên có thỏa thuận khác. Do giấy cọc của bạn đã thỏa thuận mức “đền cọc 300 triệu”, cần ưu tiên áp dụng đúng mức đã ghi nếu câu chữ thể hiện rõ đây là nghĩa vụ khi bên bán không bán. Điều 328 Bộ luật Dân sự 2015
+ Bạn nên làm ngay trước ngày công chứng:
+ Gửi tin nhắn hoặc văn bản cho bên bán, nêu rõ bạn vẫn sẵn sàng công chứng đúng ngày hẹn, đúng giá và điều kiện đã ghi trong giấy cọc; yêu cầu họ xác nhận. Không dùng lời lẽ đồng ý tăng giá hoặc hủy mua.
+ Đến đúng nơi công chứng, đúng giờ đã hẹn; mang đủ tiền/phương án thanh toán, CCCD và bản giấy đặt cọc. Nếu bên bán vắng mặt hoặc từ chối ký theo giá cũ, đề nghị công chứng viên lập giấy xác nhận sự việc hoặc có người làm chứng, ghi âm/ghi hình hợp pháp, lưu tin nhắn họ đòi tăng giá.
+ Gửi văn bản yêu cầu thực hiện cam kết hoặc thanh toán 300 triệu đồng trong một thời hạn cụ thể, ví dụ 7 ngày. Nếu họ không thực hiện, bạn có thể khởi kiện tại Tòa án nhân dân khu vực nơi bị đơn cư trú để yêu cầu phạt cọc; đồng thời có thể yêu cầu bồi thường thiệt hại thực tế nếu chứng minh được thiệt hại và có căn cứ về lỗi vi phạm.
+ Khoản lỗ 50 triệu do bán vàng thường khó yêu cầu bên bán bồi thường, vì cần chứng minh đó là thiệt hại thực tế, trực tiếp, có thể dự liệu từ việc vi phạm và có quan hệ nhân quả với hành vi của họ. Khoản 300 triệu theo giấy cọc thường là yêu cầu rõ ràng và dễ chứng minh hơn.
+ Cần kiểm tra kỹ giấy cọc: thông tin thửa đất/sổ đỏ, giá mua bán, ngày công chứng, số tiền 100 triệu đã giao, câu phạt cọc 300 triệu, chữ ký bên bán và người làm chứng. Môi giới làm chứng không thay thế chữ ký của bên bán, nhưng tin nhắn chuyển tiền, biên nhận, ghi âm và người chứng kiến sẽ rất quan trọng nếu tranh chấp.
+ [1]. Điều 328, Luật 91/2015/QH13</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 328 Bộ luật Dân sự 2015 về đặt cọc, điều này vẫn còn hiệu lực và đúng với tình huống đặt cọc mua bán đất. Tuy nhiên, không có điều luật nào từ Luật Đất đai 2024 được trích dẫn để giải quyết vấn đề diện tích đất chênh lệch và quyền sử dụng đất. Câu trả lời đã bao phủ phần về xử lý vi phạm hợp đồng đặt cọc nhưng chưa bao phủ phần về giải quyết tranh chấp diện tích đất.</t>
+  </si>
+  <si>
+    <t>Tại sao vợ đứng tên riêng 1 sổ đỏ, chồng đứng tên riêng 1 sổ, Cả 2 thửa đất đều vào quy hoạch, mà bên thẩm định chỉ cho đền mua 1 lô tdc, con lô kia nhận tiền là sao các bác, họ bảo vẫn là chung 1 hộ dù 2 sổ của riêng 2 người</t>
+  </si>
+  <si>
+    <t>Kết luận: Việc vợ và chồng mỗi người đứng tên một sổ đỏ không tự động làm phát sinh quyền được 2 lô tái định cư. Khi thu hồi đất ở, cơ quan bồi thường thường xét theo hộ gia đình/nhu cầu phải di chuyển chỗ ở và chính sách tái định cư của địa phương, không chỉ căn cứ số lượng sổ đỏ; vì vậy họ có thể bố trí 1 lô tái định cư và bồi thường bằng tiền đối với thửa còn lại.
+ Cần phân biệt rõ:
+ Nếu hai thửa là đất ở, mỗi thửa có nhà ở hợp pháp và việc thu hồi khiến gia đình phải di chuyển chỗ ở, bạn có cơ sở yêu cầu cơ quan bồi thường giải thích vì sao chỉ bố trí 1 suất tái định cư.
+ Nếu hai vợ chồng đang là một hộ cư trú, cùng chung chỗ ở, hoặc một thửa chỉ là đất trống/đất nông nghiệp/không làm phát sinh việc phải di chuyển chỗ ở, thì địa phương có thể xác định chỉ cần bố trí 1 chỗ tái định cư; thửa kia được bồi thường theo giá đất và tài sản trên đất (nếu có).
+ Việc sổ đỏ chỉ ghi tên vợ hoặc chỉ ghi tên chồng cũng chưa chắc là “tài sản riêng”. Đất hình thành trong thời kỳ hôn nhân thường được xem là tài sản chung, trừ khi chứng minh được là tài sản riêng như được tặng cho riêng, thừa kế riêng, mua bằng tài sản riêng hoặc có thỏa thuận khác. Điều 33 Luật Hôn nhân và gia đình 2014 Điều 43 Luật Hôn nhân và gia đình 2014
+ Đơn vị bồi thường phải thông báo, công khai dự kiến phương án tái định cư trước khi phê duyệt, gồm số lô, diện tích, vị trí, giá và đối tượng được bố trí. Điều 111 Luật Đất đai 2024
+ Bạn nên yêu cầu bằng văn bản cung cấp: phương án bồi thường, hỗ trợ, tái định cư; căn cứ xác định gia đình chỉ được 1 suất; tình trạng pháp lý từng thửa (đất ở hay loại đất khác, có nhà ở không); và quy định tái định cư đang áp dụng tại địa phương. Nếu không đồng ý, gửi ý kiến khi phương án được niêm yết công khai, sau đó có thể khiếu nại quyết định bồi thường/tái định cư theo trình tự luật định.
+ [1]. Điều 33, 43, Luật 52/2014/QH13
+ [2]. Điều 111, Luật 31/2024/QH15</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn Điều 33 và Điều 43 của Luật Hôn nhân và gia đình 2014 để giải thích về tài sản chung và tài sản riêng trong hôn nhân, điều này là đúng và còn hiệu lực. Ngoài ra, Điều 111 của Luật Đất đai 2024 cũng được trích dẫn để giải thích về quy trình công khai phương án tái định cư, điều này cũng đúng và còn hiệu lực. Các điều luật này đã bao phủ phần lớn nội dung câu hỏi, giải thích lý do chỉ được cấp một lô tái định cư và phần còn lại nhận tiền bồi thường.</t>
+  </si>
+  <si>
+    <t>Kind 4 - Các vấn đề pháp lý tại địa phương và dự án</t>
+  </si>
+  <si>
+    <t>Em đang bế tắc quá .xin ý kiến mọi người để tham  khảo. 2 vk ck dành giụm 10 năm, mới  mua đc căn nhà  đã đặt cọc còn 10 ngày nữa đi công chứng khi mua em cũng kiểm tra kỹ ko dính quy  hoạch gì cả , nhưng  hôm nay thấy thay đổi thì ngôi nhà đó dính quy hoạch đang ở trong tg chờ dự thảo ý kiến .giờ em không biết nên mua hay mất 100 triệu tiền cọc.khổ quá đi mất</t>
+  </si>
+  <si>
+    <t>Kết luận: Chưa nên vội bỏ cọc 100 triệu, nhưng cũng không nên công chứng/mua ngay khi chưa xác minh rõ tình trạng quy hoạch. “Đang chờ dự thảo, lấy ý kiến” thường chưa đồng nghĩa đất đã bị thu hồi hoặc bị cấm chuyển nhượng; tuy nhiên rủi ro giá trị, xây sửa nhà và bồi thường sau này có thể rất lớn.
+ Việc đầu tiên là yêu cầu bên bán cùng đi xin văn bản cung cấp thông tin quy hoạch/kế hoạch sử dụng đất tại cơ quan quản lý đất đai hoặc UBND cấp xã nơi có nhà. Cần xác định chính xác: nhà thuộc quy hoạch gì, có nằm trong kế hoạch sử dụng đất hằng năm đã được phê duyệt không, có thông báo thu hồi đất chưa, diện tích bị ảnh hưởng bao nhiêu và dự kiến thực hiện khi nào.
+ Về nguyên tắc, đất có quy hoạch vẫn có thể chuyển nhượng nếu có sổ, không tranh chấp, không bị kê biên, còn thời hạn sử dụng đất và không bị áp dụng biện pháp khẩn cấp tạm thời Điều 45 Luật Đất đai 2024. Vì vậy, công chứng được không có nghĩa là mua an toàn.
+ Nếu thông tin quy hoạch đã có từ trước thời điểm đặt cọc mà bên bán biết nhưng che giấu, hoặc cam kết nhà “không dính quy hoạch”, bạn có cơ sở yêu cầu hủy giao dịch và đòi lại cọc, thậm chí yêu cầu phạt cọc theo thỏa thuận. Nếu không có thỏa thuận khác, bên nhận cọc từ chối giao kết/thực hiện hợp đồng thì phải trả lại tiền cọc và một khoản tương đương giá trị cọc Điều 328 Bộ luật Dân sự 2015.
+ Nên làm ngay trong 10 ngày:
+ Gửi tin nhắn/văn bản cho bên bán và môi giới: thông báo phát hiện quy hoạch, yêu cầu cung cấp hồ sơ và đề nghị gia hạn thời hạn công chứng.
+ Không ký văn bản nào xác nhận tự nguyện bỏ cọc hoặc “đơn phương không mua” trước khi có kết quả quy hoạch.
+ Lưu toàn bộ tin rao, tin nhắn, ghi âm, giấy đặt cọc; đặc biệt là nội dung quảng cáo/cam kết “không quy hoạch”.
+ Chỉ tiếp tục mua nếu quy hoạch chưa được phê duyệt hoặc không ảnh hưởng đáng kể; nếu thuộc khu vực dự kiến thu hồi/chỉnh trang, nên ưu tiên thương lượng hủy cọc hoặc giảm giá tương ứng rủi ro.
+ Bạn có thể nhắn bên bán như sau: “Do phát sinh thông tin nhà/đất có liên quan quy hoạch, đề nghị hai bên gia hạn thời hạn công chứng để xác minh bằng văn bản cơ quan có thẩm quyền. Nếu thông tin quy hoạch đã tồn tại trước khi đặt cọc mà chưa được cung cấp hoặc tài sản không đúng cam kết, đề nghị hoàn trả tiền đặt cọc và xử lý theo thỏa thuận đặt cọc.”
+ [1]. Điều 45, Luật 31/2024/QH15
+ [2]. Điều 328, Luật 91/2015/QH13</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn Điều 45 của Luật Đất đai 2024 (Luật số 31/2024/QH15) và Điều 328 của Bộ luật Dân sự 2015 (Luật số 91/2015/QH13). Điều 45 Luật Đất đai 2024 quy định về các trường hợp đất có quy hoạch nhưng vẫn có thể chuyển nhượng nếu đáp ứng các điều kiện nhất định. Điều 328 Bộ luật Dân sự 2015 quy định về việc xử lý tiền đặt cọc trong giao dịch dân sự. Cả hai điều luật này đều còn hiệu lực và phù hợp với tình huống của người hỏi, bao phủ đầy đủ các khía cạnh pháp lý liên quan đến việc mua bán nhà đất có dính quy hoạch và xử lý tiền đặt cọc.</t>
+  </si>
+  <si>
+    <t>Kết luận: Gia đình không đương nhiên bị “thu trắng” chỉ vì có nguồn gốc đất đã góp vào dự án. Tuy nhiên, nếu người sử dụng đất đứng tên trong quyết định giao/thuê đất hoặc là chủ đầu tư bị xác định vi phạm theo khoản 8 Điều 81, thì nguyên tắc là Nhà nước thu hồi không bồi thường về đất, tài sản gắn liền với đất và chi phí đầu tư còn lại; cần khẩn trương kiểm tra căn cứ vi phạm, đặc biệt là thủ tục gia hạn 24 tháng và chủ thể bị thu hồi.
+ 1. Cần phân biệt rõ 2 phần đất
+ Đất Nhà nước giao/cho thuê để thực hiện dự án: quyền sử dụng đất thuộc chủ đầu tư theo quyết định giao đất/cho thuê đất. Nếu dự án chậm sử dụng đất 12 tháng liên tục hoặc chậm tiến độ 24 tháng, sau khi đã được gia hạn mà vẫn không khắc phục thì bị thu hồi không bồi thường. Khoản 8 Điều 81 Luật Đất đai 2024
+ “Đất gốc” gia đình góp vào dự án: phải xem hồ sơ góp đất thể hiện theo cách nào: góp vốn bằng quyền sử dụng đất, chuyển nhượng quyền sử dụng đất cho doanh nghiệp, hay gia đình chỉ giao đất để doanh nghiệp sử dụng. Đây là điểm quyết định gia đình có thể yêu cầu bảo vệ quyền sử dụng đất riêng, hay chỉ có quyền đòi doanh nghiệp thanh toán giá trị phần vốn góp/bồi thường thiệt hại.
+ Nếu đất đã được chuyển quyền hợp pháp sang doanh nghiệp và được Nhà nước thu hồi theo khoản 8 Điều 81, gia đình thường không thể yêu cầu Nhà nước trả lại riêng phần đất đó; tranh chấp chủ yếu chuyển thành quan hệ giữa gia đình và doanh nghiệp/chủ đầu tư.
+ 2. Điểm cần kiểm tra ngay để phản đối quyết định thu hồi
+ Khoản 8 Điều 81 chỉ áp dụng khi có đủ điều kiện: đất không được sử dụng 12 tháng liên tục kể từ ngày bàn giao thực địa, hoặc chậm tiến độ 24 tháng so với tiến độ dự án; thông thường chủ đầu tư phải được xem xét gia hạn tối đa 24 tháng trước khi thu hồi, trừ trường hợp pháp luật có quy định khác. Khoản 8 Điều 81 Luật Đất đai 2024
+ Gia đình cần đối chiếu:
+ Quyết định giao đất/cho thuê đất và biên bản bàn giao đất thực địa;
+ Văn bản chấp thuận chủ trương đầu tư, giấy chứng nhận đăng ký đầu tư và các lần điều chỉnh tiến độ;
+ Quyết định/văn bản gia hạn tiến độ, gia hạn sử dụng đất; chứng từ nộp khoản tiền trong thời gian gia hạn;
+ Tài liệu chứng minh dự án chậm vì Nhà nước chưa giải phóng mặt bằng, chưa bàn giao đủ diện tích, thay đổi quy hoạch, thủ tục hành chính kéo dài hoặc sự kiện khách quan khác.
+ Nếu Nhà nước chưa giải phóng mặt bằng hoặc chưa bàn giao đất thực địa đầy đủ khiến doanh nghiệp không thể triển khai, cần lập luận rằng việc chậm tiến độ không hoàn toàn thuộc lỗi của chủ đầu tư; đồng thời yêu cầu cơ quan ban hành quyết định chỉ rõ căn cứ tính mốc thời gian vi phạm.
+ 3. Việc nên làm ngay
+ Gửi đơn khiếu nại quyết định thu hồi đến chính UBND tỉnh đã ban hành quyết định; đề nghị tạm dừng thi hành nếu việc cưỡng chế hoặc bàn giao đất sắp diễn ra.
+ Trong đơn, yêu cầu cung cấp toàn bộ hồ sơ làm căn cứ thu hồi: kết quả kiểm tra hiện trạng, văn bản xác định chậm tiến độ, quyết định gia hạn, thông báo vi phạm và tài liệu chứng minh đã bàn giao đất thực địa.
+ Nếu quyền lợi không được giải quyết, có thể khiếu nại tiếp hoặc khởi kiện vụ án hành chính yêu cầu hủy toàn bộ/một phần quyết định thu hồi.
+ Đồng thời, xác định rõ hợp đồng góp đất/góp vốn với doanh nghiệp để bảo lưu yêu cầu độc lập về giá trị quyền sử dụng đất, vốn góp, lợi nhuận hoặc thiệt hại đối với doanh nghiệp và người quản lý doanh nghiệp.
+ 4. Lưu ý quan trọng
+ Quy định “không bồi thường” chỉ đặt ra khi việc thu hồi theo khoản 8 Điều 81 là đúng pháp luật. Vì vậy, trọng tâm không phải chỉ là xin tách phần đất gốc, mà là chứng minh: gia đình vẫn là người có quyền sử dụng đất độc lập; hoặc quyết định thu hồi áp dụng sai chủ thể, sai mốc tiến độ, chưa gia hạn hợp lệ, hay chậm tiến độ do chưa giải phóng mặt bằng/bàn giao đất.
+ Bạn nên chuẩn bị tối thiểu: giấy chứng nhận quyền sử dụng đất cũ, hợp đồng góp vốn/chuyển nhượng, hồ sơ doanh nghiệp, quyết định giao đất/thuê đất, hồ sơ dự án và quyết định thu hồi. Đây là các tài liệu quyết định hướng bảo vệ quyền lợi.
+ [1]. Điều 81, Luật 31/2024/QH15</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn Điều 81 của Luật Đất đai 2024 (Luật số 31/2024/QH15), điều này còn hiệu lực và đúng với tình huống thu hồi đất do vi phạm pháp luật về đất đai và chậm tiến độ dự án. Điều luật này đã bao phủ phần lớn vấn đề về việc thu hồi đất và các điều kiện liên quan đến việc không bồi thường khi thu hồi. Tuy nhiên, câu trả lời cũng đã mở rộng thêm các khía cạnh cần kiểm tra và các bước cần thực hiện để bảo vệ quyền lợi của gia đình, như kiểm tra hồ sơ góp đất, điều kiện gia hạn, và các thủ tục khiếu nại, điều này không nằm trong phạm vi điều luật nhưng là cần thiết cho tình huống thực tế.</t>
+  </si>
+  <si>
+    <t>Chào mọi người ạ,em ở Ninh Bình nhà em đang làm trang trại, sắp tới sẽ bị thu hồi đất. Theo luật mới sẽ được bồi thường thiệt hại về cả vật nuôi như trâu bò, lợn gà. Em hỏi đơn giá bồi thường ở Ninh Bình lại không có, các tỉnh khác đều có rồi. Bây giờ phải làm sao đây ,như này thiệt cho nhà em quá</t>
+  </si>
+  <si>
+    <t>Kết luận: Nhà bạn vẫn có quyền yêu cầu bồi thường thiệt hại thực tế đối với vật nuôi không thể di chuyển khi Nhà nước thu hồi đất. Việc Ninh Bình chưa ban hành/không công bố đơn giá riêng cho trâu, bò, lợn, gà không phải là lý do để không bồi thường; cơ quan có thẩm quyền phải xác định mức bồi thường phù hợp giá thị trường và hoàn thiện căn cứ áp dụng.
+ Vật nuôi có thể di chuyển thì gia đình được tự đưa đi trước ngày bàn giao đất. Với con nuôi không thể di chuyển hoặc buộc phải tiêu hủy, bán tháo do thu hồi đất, gia đình được bồi thường theo thiệt hại thực tế. Điều 103 Luật Đất đai 2024
+ UBND cấp tỉnh có trách nhiệm ban hành đơn giá bồi thường vật nuôi, bảo đảm phù hợp giá thị trường và điều chỉnh khi giá biến động. Điều 103 Luật Đất đai 2024 Ninh Bình hiện có quy định đơn giá đối với vật nuôi thủy sản tại Quyết định 178/2025/QĐ-UBND, nhưng chưa thấy đơn giá cụ thể cho trâu, bò, lợn, gà.
+ Gia đình nên làm ngay:
+ Lập danh sách từng con: loại, số lượng, trọng lượng/độ tuổi, tình trạng, ngày mua; kèm hóa đơn, sổ tiêm phòng, ảnh/video có ngày quay, xác nhận của thú y hoặc chính quyền xã nếu có.
+ Yêu cầu Tổ chức làm nhiệm vụ bồi thường và UBND xã ghi đầy đủ đàn vật nuôi vào biên bản kiểm đếm bắt buộc; không ký biên bản thiếu số lượng hoặc ghi “không yêu cầu bồi thường”.
+ Gửi văn bản đề nghị UBND tỉnh Ninh Bình và cơ quan bồi thường xác định mức bồi thường thực tế/ban hành đơn giá bổ sung đối với vật nuôi trên cạn trước khi phê duyệt phương án bồi thường. Nêu rõ giá mua vào, giá bán tại thời điểm thu hồi và chứng cứ kèm theo.
+ Nếu phương án bồi thường không tính hoặc tính quá thấp, khiếu nại quyết định/phương án theo trình tự khiếu nại; đồng thời chỉ bàn giao đất theo đúng thời điểm, điều kiện ghi trong quyết định thu hồi và phương án đã được phê duyệt.
+ Lưu ý: nếu trâu bò, lợn gà có thể di chuyển bình thường, cơ quan nhà nước thường không bồi thường toàn bộ giá trị con vật; trọng tâm là chứng minh chi phí/thiệt hại phát sinh thực tế do phải di chuyển, ngừng chăn nuôi, bán gấp hoặc không thể di chuyển.
+ [1]. Điều 103, Luật 31/2024/QH15</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 103 của Luật Đất đai 2024 (Luật số 31/2024/QH15), quy định về trách nhiệm của UBND cấp tỉnh trong việc ban hành đơn giá bồi thường vật nuôi, đảm bảo phù hợp với giá thị trường. Điều luật này còn hiệu lực và phù hợp với vấn đề người dùng hỏi về bồi thường vật nuôi khi thu hồi đất. Tuy nhiên, câu trả lời chưa trích dẫn cụ thể nội dung của Điều 103 mà chỉ nêu khái quát trách nhiệm của UBND cấp tỉnh.</t>
+  </si>
+  <si>
+    <t>Gia đình mình đất vào quy hoạch sân bay. Đất ở thì được ông bà nội cho tặng, sau khi ông bà cho tặng thì ông bà có ở với vợ chồng mình ( trước đó ông bà có mua một mảnh đất nhưng chưa làm sổ được vì đất đó bán trái thẩm quyền của xã, đất này vợ chồng mình có làm nhà tạm để ở và kinh doanh và cũng thuộc quy hoạch sân bay). Vợ chồng mình đã tách hộ khẩu riêng với ông bà, hiện tại ông bà có chung hộ khẩu với chú. Vì từ trước đến nay ông bà ở với vợ chồng mình nên mình có xin được 2 suất tái định cư không</t>
+  </si>
+  <si>
+    <t>Kết luận: Có thể đề nghị xem xét 2 suất tái định cư, nhưng không đương nhiên được chấp thuận chỉ vì ông bà thực tế ở cùng vợ chồng bạn. Cơ quan có thẩm quyền sẽ kiểm tra ông bà có phải là một hộ đủ điều kiện tách hộ, cùng sinh sống ổn định tại thửa đất bị thu hồi và có thuộc diện thiếu chỗ ở sau thu hồi hay không.
+ Trường hợp một thửa đất ở bị thu hồi có nhiều thế hệ hoặc nhiều cặp vợ chồng cùng sinh sống, nếu đủ điều kiện tách thành hộ riêng theo pháp luật cư trú, thì hộ còn thiếu có thể được xem xét hỗ trợ giao đất ở có thu tiền sử dụng đất, hoặc bán/cho thuê/cho thuê mua nhà ở tái định cư. Đây là cơ chế “xem xét hỗ trợ”, không phải quyền tự động cấp thêm một suất miễn phí. Khoản 4 Điều 111 Luật Đất đai 2024
+ Việc ông bà đang đăng ký thường trú chung với chú là điểm bất lợi, vì hồ sơ cư trú thể hiện ông bà thuộc hộ của chú. Tuy vậy, bạn vẫn nên cung cấp chứng cứ ông bà thực tế cư trú ổn định cùng gia đình bạn trước thời điểm thông báo thu hồi đất: xác nhận cư trú của công an xã/phường, giấy tờ y tế, điện nước, xác nhận tổ dân phố/thôn, lời khai hàng xóm, ảnh nhà ở, biên bản kiểm đếm thể hiện ông bà đang sinh sống tại đây.
+ Mảnh đất ông bà mua “trái thẩm quyền của xã” và chưa được cấp sổ có thể không được công nhận là đất ở hợp pháp để bồi thường về đất. Tuy nhiên, đây cũng có thể là căn cứ chứng minh ông bà không có chỗ ở hợp pháp khác; việc bồi thường/hỗ trợ đối với đất và căn nhà tạm trên đó phải được cơ quan bồi thường xác minh riêng theo nguồn gốc, thời điểm sử dụng và hồ sơ đất.
+ Bạn nên làm đơn đề nghị bố trí tái định cư riêng cho hộ ông bà, gửi Hội đồng bồi thường, hỗ trợ, tái định cư hoặc UBND xã/phường nơi thu hồi đất, yêu cầu ghi nhận: ông bà sống cùng vợ chồng bạn, có nhu cầu tách hộ/ở riêng sau thu hồi, không có chỗ ở hợp pháp khác và đề nghị áp dụng khoản 4 Điều 111 nêu trên. Khi dự thảo phương án bồi thường được niêm yết, phải gửi ý kiến bằng văn bản ngay; nếu phương án không xem xét, bạn có thể khiếu nại quyết định bồi thường, hỗ trợ, tái định cư. Điều 237 Luật Đất đai 2024
+ Điều kiện cụ thể về số suất, diện tích lô tái định cư và chứng cứ “cùng chung sống” phụ thuộc quy định của tỉnh/thành phố nơi có dự án sân bay. Bạn cho biết địa phương và thời điểm ban hành thông báo thu hồi đất, tôi có thể đối chiếu chính xác quy định địa phương và đánh giá khả năng được 2 suất.
+ [1]. Điều 111, 237, Luật 31/2024/QH15</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn Điều 111 và Điều 237 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là các điều luật còn hiệu lực hiện hành. Điều 111 quy định về việc hỗ trợ tái định cư khi thu hồi đất, trong đó có cơ chế xem xét hỗ trợ cho các hộ đủ điều kiện tách hộ. Điều 237 quy định về quyền khiếu nại quyết định bồi thường, hỗ trợ, tái định cư. Các điều luật này đã bao phủ phần lớn nội dung câu hỏi về việc xin suất tái định cư khi đất bị thu hồi, tuy nhiên, cần lưu ý rằng điều kiện cụ thể có thể phụ thuộc vào quy định của từng địa phương.</t>
+  </si>
+  <si>
+    <t>Em chào cả nhà . Chúc cả nhà buổi tối vui vẻ , hạnh phúc bên gia đình ...... 
+ chuyện là nhà em có thửa đất đấu thầu từ năm 1994 do không dùng đến nên cho hàng xóm mượn để chăn nuôi . Giờ tuyến đường cao tốc chạy qua , nhà nước có gửi văn bản mời gia đình em đến để đền bù , nhưng do công việc và ở xa nên có nhờ người thân đến ký hộ . Nhưng sau đợt đó thì không thấy ai gọi về nữa ..... giờ em về quê lại thấy bác ( hàng xóm ) trước em cho mượn đất để canh tác đc đền bù trên thửa đất nhà em số tiền 1 tỉ và 1 mảnh tái định cư . Cả nhà cho em hỏi là giờ em có đòi lại được không và tại sao nhà nước lại đền bù cho người không đứng tên đấu thầu ? Em cảm ơn rất nhiều</t>
+  </si>
+  <si>
+    <t>Kết luận: Có thể đòi lại khoản bồi thường và suất tái định cư nếu gia đình bạn là người có quyền sử dụng hợp pháp thửa đất, còn hàng xóm chỉ mượn để chăn nuôi. Tuy nhiên, cần làm ngay vì có thể phương án bồi thường đã được phê duyệt, chi trả và có chữ ký của người đại diện gia đình bạn.
+ Người được bồi thường về đất khi Nhà nước thu hồi phải là người sử dụng đất có đủ điều kiện pháp luật; việc “đứng tên đấu thầu” từ năm 1994 chưa tự động chứng minh quyền được bồi thường, mà phải kiểm tra hồ sơ giao/cho thuê/đấu thầu đất, việc thực hiện nghĩa vụ tài chính và quá trình sử dụng đất. Người hàng xóm chỉ được bồi thường phần tài sản, chi phí đầu tư vào đất còn lại (nếu có đủ điều kiện), không đương nhiên được nhận tiền bồi thường quyền sử dụng đất hoặc tái định cư thay gia đình bạn. Luật Đất đai 2024
+ Việc người thân ký hộ chỉ có giá trị nếu có giấy ủy quyền hợp lệ hoặc được pháp luật công nhận là đại diện. Nếu họ tự ký, ký vượt phạm vi ủy quyền, hoặc hồ sơ kê khai sai người sử dụng đất, gia đình bạn có căn cứ yêu cầu kiểm tra, hủy/sửa phương án và thu hồi khoản chi trả sai.
+ Bạn nên thực hiện ngay các việc sau:
+ Đến UBND xã/phường nơi có đất hoặc tổ chức làm nhiệm vụ bồi thường, giải phóng mặt bằng, yêu cầu cấp bản sao:
+ Thông báo thu hồi đất;
+ Phương án bồi thường, hỗ trợ, tái định cư đã niêm yết và quyết định phê duyệt;
+ Bảng kê, chứng từ chi trả 1 tỷ đồng và quyết định giao tái định cư;
+ Hồ sơ xác định ai là người sử dụng đất, ai ký nhận và căn cứ chi trả.
+ Nộp đơn khiếu nại đối với quyết định/phương án bồi thường và đề nghị tạm dừng các thủ tục liên quan đến suất tái định cư nếu chưa hoàn tất. Cần nêu rõ: đất do gia đình đấu thầu từ năm 1994; chỉ cho hàng xóm mượn; không chuyển nhượng, tặng cho hay cho thuê quyền sử dụng đất; đề nghị xác minh người nhận tiền và thu hồi khoản chi sai.
+ Kèm toàn bộ chứng cứ: hợp đồng/biên lai đấu thầu, quyết định giao đất hoặc hồ sơ địa chính, biên lai nộp tiền, giấy tờ thuế, xác nhận của người dân, giấy cho mượn (nếu có), tin nhắn/ghi âm, và giấy ủy quyền cho người thân ký hộ. Nếu không có giấy cho mượn, có thể xin người làm chứng xác nhận việc hàng xóm chỉ mượn đất.
+ Nếu hàng xóm đã nhận tiền hoặc suất tái định cư trên cơ sở kê khai không đúng, gia đình bạn có thể yêu cầu họ hoàn trả; nếu không tự nguyện, khởi kiện tranh chấp về quyền, nghĩa vụ liên quan đến khoản bồi thường tại Tòa án. Việc cố ý lập hồ sơ gian dối để nhận tiền có thể còn bị cơ quan có thẩm quyền xem xét trách nhiệm khác.
+ Lưu ý quan trọng: nếu gia đình chỉ “đấu thầu đất công ích/đất nông nghiệp của xã” theo thời hạn, thì phải xem thời hạn thuê/đấu thầu còn hay đã hết tại thời điểm thu hồi. Trường hợp này có thể không được bồi thường về đất như đất được giao ổn định lâu dài, nhưng vẫn cần xác định đúng người được nhận hỗ trợ, bồi thường chi phí đầu tư hoặc tài sản trên đất. Điều 13 Nghị định 88/2024/NĐ-CP
+ Bạn không nên chỉ làm việc miệng với hàng xóm; trước hết phải lấy được quyết định phê duyệt và chứng từ chi trả để biết chính xác cơ quan đã bồi thường theo căn cứ nào, ai đã ký và ai đã nhận.
+ [1]. Luật 31/2024/QH15
+ [2]. Điều 13, Nghị định 88/2024/NĐ-CP</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn Luật Đất đai 2024 (Luật số 31/2024/QH15) và Điều 13 Nghị định 88/2024/NĐ-CP, cả hai đều còn hiệu lực. Luật Đất đai 2024 quy định về quyền được bồi thường khi Nhà nước thu hồi đất, và Nghị định 88/2024/NĐ-CP hướng dẫn chi tiết về bồi thường, hỗ trợ, tái định cư. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý liên quan đến việc đòi lại tiền bồi thường và suất tái định cư, cũng như các bước cần thực hiện để giải quyết tranh chấp.</t>
+  </si>
+  <si>
+    <t>dạ mong anh chị trong nhóm tư vấn ạ
+ Nhà em có diện tích 320,4m2 (chưa có sổ, không tranh chấp, trên bản đồ đã là ONT, hàng năm vẫn đóng thuế) được cơ quan xác định như sau: 134,4m2 là đất ở trước năm 1980, 161m2 là đất lấn chiếm trước năm 1993 và 25m2 trước năm 2004, đã có nhà xây trên diện tích đất ở hợp pháp. Khi dự án đi qua nhà e được đền bù 3 suất đất nhỏ nhưng ban đầu nghĩa vụ tài chính chỉ phải đóng hơn 500tr, giờ sau khi sáp nhập giao cho 1 đội cán bộ khác làm thì tính lên nghĩa vụ tài chính mất 1ty6 (80%*S lấn chiếm*giá đất). Họ bảo phương án như này là hợp lý rồi, còn nếu căng thì ko chỉ được 1 suất đất ạ vì phần lấn chiếm chưa xây dựng nhà ở và công trình phụ, nếu có thì nghĩa vụ tài chính mới nhỏ. Anh chị cho e xin tư vấn như vậy đã là hợp lý chưa ạ. Em cảm ơn mn ạ</t>
+  </si>
+  <si>
+    <t>Kết luận: Chưa thể khẳng định mức 1,6 tỷ đồng là đúng chỉ từ thông tin bạn nêu. Tuy nhiên, cơ quan không thể chỉ nói “phương án hợp lý” mà phải chỉ rõ: diện tích nào được công nhận, căn cứ xác định nguồn gốc từng phần đất, căn cứ giao 3 suất tái định cư và công thức tính 80% giá đất.
+ Phần 161 m² lấn chiếm trước năm 1993 và 25 m² trước năm 2004 vẫn có thể được xem xét công nhận quyền sử dụng đất nếu đang sử dụng làm nhà ở/đất ở, ổn định, không tranh chấp, phù hợp điều kiện luật định; người sử dụng đất phải thực hiện nghĩa vụ tài chính. Việc “chưa xây nhà hoặc công trình phụ trên phần lấn chiếm” có thể ảnh hưởng đến diện tích được công nhận là đất ở hoặc được bồi thường, nhưng không đương nhiên làm mất quyền tái định cư hay chỉ còn 1 suất. Điều 139 Luật Đất đai 2024
+ Khi Nhà nước thu hồi đất, trường hợp đất có nhà ở đang sử dụng ổn định từ trước 15/10/1993 thì diện tích bồi thường có thể tính theo diện tích thực tế thu hồi, trong giới hạn hạn mức công nhận đất ở địa phương. Với đất sử dụng từ 15/10/1993 đến trước 01/7/2014, mức bồi thường phụ thuộc hạn mức giao đất ở; điều kiện quan trọng là phải xác định đúng thực tế sử dụng, nhà ở và thời điểm sử dụng đất. Điều 9 Nghị định 88/2024/NĐ-CP
+ Bạn nên làm ngay một văn bản đề nghị cơ quan lập phương án cung cấp:
+ Bảng tính nghĩa vụ tài chính từ mức hơn 500 triệu lên 1,6 tỷ: diện tích tính tiền, giá đất, tỷ lệ 80%, thời điểm áp giá, văn bản áp dụng.
+ Biên bản/xác nhận nguồn gốc và quá trình sử dụng từng phần: 134,4 m²; 161 m²; 25 m².
+ Quyết định hoặc phương án bồi thường, hỗ trợ, tái định cư ghi rõ lý do được 3 suất và điều kiện để giữ từng suất.
+ Quy định địa phương về hạn mức công nhận đất ở, giá đất, bồi thường và tái định cư của chính dự án.
+ Không nên tự nguyện nộp theo con số mới trước khi nhận được văn bản tính toán. Nếu phương án bồi thường hoặc thông báo nghĩa vụ tài chính đã ban hành, bạn có quyền khiếu nại lần đầu đến chính cơ quan/người ban hành; thời hiệu thông thường là 90 ngày kể từ ngày nhận hoặc biết quyết định/hành vi đó. Điều 9 Luật Khiếu nại 2011 Điều 17 Luật Khiếu nại 2011
+ Việc gia đình “hằng năm đóng thuế” là chứng cứ hỗ trợ chứng minh quá trình sử dụng ổn định, nhưng không tự động biến toàn bộ diện tích lấn chiếm thành đất ở hợp pháp. Bạn cần lưu giữ biên lai thuế, bản đồ thể hiện ONT, giấy tờ kê khai nhà đất, ảnh nhà qua các thời kỳ, xác nhận của khu dân cư và toàn bộ biên bản kiểm đếm dự án.
+ [1]. Điều 139, Luật 31/2024/QH15
+ [2]. Điều 9, Nghị định 88/2024/NĐ-CP
+ [3]. Điều 9, 17, Luật 02/2011/QH13</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn Điều 139 của Luật Đất đai 2024 (Luật số 31/2024/QH15) và Điều 9 của Nghị định 88/2024/NĐ-CP, cả hai đều còn hiệu lực và phù hợp với tình huống thu hồi đất và bồi thường. Điều 139 Luật Đất đai 2024 liên quan đến việc công nhận quyền sử dụng đất và bồi thường khi thu hồi đất. Điều 9 Nghị định 88/2024/NĐ-CP quy định chi tiết về bồi thường, hỗ trợ, tái định cư khi Nhà nước thu hồi đất. Câu trả lời đã bao phủ các khía cạnh pháp lý liên quan đến việc xác định nguồn gốc đất, nghĩa vụ tài chính và quyền khiếu nại của người sử dụng đất.</t>
+  </si>
+  <si>
+    <t>Mọi người cho em hỏi chút : nhà em 300m2 đất thổ cư khi bị thu hồi sẽ đc cấp tđc ntn ạ . Em cảm ơn</t>
+  </si>
+  <si>
+    <t>Kết luận: Không thể chỉ căn cứ “300 m² đất thổ cư” để khẳng định sẽ được cấp bao nhiêu m² đất tái định cư. Nếu bị thu hồi toàn bộ đất ở (hoặc phần còn lại không đủ điều kiện ở) và gia đình không còn đất ở/nhà ở khác trong cùng xã, phường nơi thu hồi, gia đình thường được bồi thường bằng đất ở hoặc nhà ở tái định cư; diện tích/lô cụ thể theo phương án của địa phương.
+ Việc bố trí còn phụ thuộc vào: đất có đủ điều kiện được bồi thường hay không (sổ đỏ, nguồn gốc sử dụng), thu hồi toàn bộ hay một phần, số hộ cùng chung thửa đất, còn chỗ ở khác không và quỹ tái định cư của địa phương. Không có nguyên tắc cứ mất 300 m² là được đổi ngang 300 m² đất tái định cư.
+ Nếu còn đất/nhà ở khác trong xã, phường nơi bị thu hồi thì thông thường được bồi thường bằng tiền; địa phương chỉ bố trí đất hoặc nhà tái định cư nếu có quỹ và điều kiện thực tế. Điều 11 Nghị định 88/2024/NĐ-CP
+ Gia đình phải được thông báo công khai về vị trí, diện tích từng lô/căn, giá tái định cư và dự kiến bố trí trước khi phương án được phê duyệt. Giá tiền sử dụng đất tái định cư được tính theo bảng giá đất tại thời điểm phê duyệt phương án; có thể được ghi nợ nghĩa vụ tài chính nếu đủ điều kiện. Điều 111 Luật Đất đai 2024
+ Bạn nên kiểm tra ngay trong dự thảo phương án bồi thường, hỗ trợ, tái định cư: gia đình được xác định là “đủ điều kiện bồi thường về đất ở” hay không; được mấy suất; diện tích, giá lô tái định cư; và khoản chênh lệch phải nộp/được nhận. Nếu không đồng ý, có quyền gửi ý kiến khi phương án được niêm yết công khai ít nhất 15 ngày. Điều 111 Luật Đất đai 2024
+ [1]. Điều 11, Nghị định 88/2024/NĐ-CP
+ [2]. Điều 111, Luật 31/2024/QH15</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn Điều 11 của Nghị định 88/2024/NĐ-CP và Điều 111 của Luật Đất đai 2024 (Luật số 31/2024/QH15), cả hai đều còn hiệu lực. Điều 11 của Nghị định 88/2024/NĐ-CP liên quan đến việc bồi thường và tái định cư khi thu hồi đất, trong khi Điều 111 của Luật Đất đai 2024 quy định về việc thông báo và xác định giá đất tái định cư. Các điều luật này đã bao phủ đầy đủ các khía cạnh liên quan đến việc cấp đất tái định cư khi bị thu hồi đất thổ cư, như điều kiện bồi thường, diện tích tái định cư, và quy trình thông báo.</t>
+  </si>
+  <si>
+    <t>Bố em có đứng tên 1 thửa đất , hiện nay bị nhà nước thu hồi làm dự án, nhưng bố em đã mất, giờ họ kiểm kê chỉ xin bản photo sổ đỏ.Nhà e định làm phân chia quyền thừa kế mảnh đất đó cho đứa e em, cho nó toàn quyền nhận đề bù, xét tdc thửa đất đó.Mà ko thấy bên kiểm kê bảo gì. Vậy khi xét hồ sơ e mới cần nộp biên bản phân chia thừa kế hay phải nộp luôn ạ.</t>
+  </si>
+  <si>
+    <t>Kết luận: Nên nộp hoặc ít nhất xuất trình ngay hồ sơ thừa kế cho tổ chức làm nhiệm vụ bồi thường khi họ đang kiểm kê; không nên chờ đến lúc xét/phê duyệt phương án. Bản photo sổ đỏ chỉ giúp xác định thửa đất, chưa đủ căn cứ để ghi nhận người em là người nhận tiền bồi thường hoặc được xem xét tái định cư thay cho bố đã mất.
+Quyền sử dụng đất là di sản từ thời điểm bố mất. Nếu muốn giao toàn bộ quyền liên quan thửa đất cho em bạn, những người thừa kế phải lập văn bản khai nhận di sản hoặc văn bản thỏa thuận phân chia di sản được công chứng; trong đó ghi rõ em bạn nhận quyền sử dụng đất và các khoản bồi thường, hỗ trợ, tái định cư phát sinh do thu hồi thửa đất. Sau đó nộp bản sao chứng thực cho đơn vị bồi thường, kèm giấy chứng tử, giấy tờ chứng minh quan hệ thừa kế và sổ đỏ.
+Việc kiểm kê trước mắt có thể vẫn thực hiện theo tên bố bạn trên giấy chứng nhận. Tuy nhiên, hãy đề nghị họ ghi trong biên bản: “người sử dụng đất đã chết, quyền và nghĩa vụ đang do những người thừa kế giải quyết”, đồng thời ghi tên, số điện thoại người đại diện gia đình. Không nên để em bạn tự ký nhận là chủ đất khi chưa có văn bản thừa kế/ủy quyền hợp lệ.
+Khi lập, công khai và phê duyệt phương án bồi thường, cơ quan có thẩm quyền phải xác định đúng người có quyền lợi liên quan; thông báo thu hồi đất cũng phải gửi cho người có đất bị thu hồi và người có quyền lợi, nghĩa vụ liên quan Điều 87 Luật Đất đai 2024. Vì vậy, nộp sớm giúp tránh việc phương án vẫn ghi tên bố hoặc yêu cầu làm lại hồ sơ, chậm chi trả.
+Lưu ý: Nếu mẹ bạn còn sống và thửa đất được hình thành trong thời kỳ hôn nhân, trước hết cần xác định phần của mẹ trong tài sản chung; chỉ phần thuộc bố mới là di sản để các thừa kế phân chia. Nếu có nhiều người thừa kế mà không cùng ký văn bản phân chia/ủy quyền, em bạn không thể một mình nhận toàn bộ tiền bồi thường hoặc quyết định suất tái định cư.
+[1]. Điều 87, Luật 31/2024/QH15</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 87 của Luật Đất đai 2024 (Luật số 31/2024/QH15), quy định về việc thông báo thu hồi đất và xác định người có quyền lợi liên quan khi lập phương án bồi thường. Điều luật này còn hiệu lực và phù hợp với tình huống thu hồi đất và phân chia thừa kế. Tuy nhiên, câu trả lời chưa trích dẫn cụ thể các điều luật liên quan đến thủ tục thừa kế và công chứng văn bản thỏa thuận phân chia di sản, nhưng đã bao phủ phần lớn vấn đề pháp lý của câu hỏi.</t>
+  </si>
+  <si>
+    <t>E chào a chị ạ cho e hỏi đất của bố e đang ở cùng GĐ người cháu nữa bố e chưa làm sổ sang tên cho bố e dc đất chuẩn bị giải tỏa làm đường vậy cả 2 có được cấp đất tái định cư ko ạ</t>
+  </si>
+  <si>
+    <t>Kết luận: Chưa thể khẳng định cả bố bạn và gia đình người cháu đều được một suất tái định cư. Việc này phụ thuộc vào nguồn gốc, tình trạng pháp lý của đất, số hộ thực tế và việc từng hộ có đủ điều kiện tách hộ/có quyền sử dụng đất chung hay không; đất chưa sang tên vẫn có thể được bồi thường, xem xét tái định cư nếu đủ điều kiện được cấp sổ.
+Nếu đất thực tế là của bố bạn nhưng chưa làm thủ tục sang tên, gia đình cần nộp ngay giấy tờ chứng minh nguồn gốc: giấy cho tặng, chuyển nhượng, thừa kế, giấy tờ mua bán cũ, biên lai thuế, xác nhận sử dụng ổn định, giấy tờ kê khai đất… Cơ quan bồi thường sẽ xác minh ai là người có quyền sử dụng đất. Người đứng tên cũ không đương nhiên là người nhận bồi thường nếu chứng minh được bố bạn là người sử dụng hợp pháp.
+Về người cháu đang ở cùng: chỉ “ở chung” không tự động được cấp một suất tái định cư riêng. Trường hợp có nhiều hộ cùng chung sống trên một thửa đất bị thu hồi, nếu các hộ đủ điều kiện tách thành hộ riêng theo pháp luật cư trú, hoặc là nhiều hộ cùng có quyền sử dụng chung một thửa đất nhưng diện tích bồi thường không đủ giao riêng, thì có thể được xem xét hỗ trợ giao đất có thu tiền, hoặc mua/thuê/thuê mua nhà ở cho hộ còn thiếu Khoản 4 Điều 111 Luật Đất đai 2024.
+Đất chưa có sổ vẫn có thể được bồi thường về đất nếu đang sử dụng ổn định và đủ điều kiện được cấp Giấy chứng nhận; các trường hợp đất không giấy tờ được quy định cụ thể tại Điều 5 Nghị định 88/2024/NĐ-CP. Nếu không đủ điều kiện bồi thường về đất, quyền được bố trí tái định cư thường sẽ khó hơn và có thể chỉ được xem xét hỗ trợ theo chính sách địa phương.
+Gia đình nên làm ngay 3 việc:
+Khi kiểm kê, yêu cầu ghi đủ tên bố bạn, hộ của người cháu và tình trạng hai hộ đang cư trú thực tế trên đất.
+Nộp bản sao căn cước, thông tin cư trú của từng hộ; giấy tờ chứng minh cháu là một hộ độc lập nếu có.
+Gửi đơn đề nghị cơ quan bồi thường xác nhận bằng văn bản: bố bạn có đủ điều kiện bồi thường/tái định cư không, và hộ người cháu có được xem xét suất hỗ trợ hoặc tái định cư riêng không.
+Lưu ý, số suất tái định cư và tiêu chí cụ thể còn phụ thuộc phương án bồi thường của tỉnh/thành phố nơi có đất.
+[1]. Điều 111, Luật 31/2024/QH15
+[2]. Điều 5, Nghị định 88/2024/NĐ-CP</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn Điều 111 của Luật Đất đai 2024 và Điều 5 của Nghị định 88/2024/NĐ-CP. Cả hai văn bản này đều còn hiệu lực và liên quan đến vấn đề bồi thường, tái định cư khi đất bị thu hồi. Điều 111 Luật Đất đai 2024 quy định về việc bồi thường, hỗ trợ và tái định cư khi Nhà nước thu hồi đất. Điều 5 Nghị định 88/2024/NĐ-CP quy định về các trường hợp đất không có giấy tờ vẫn có thể được bồi thường nếu đủ điều kiện. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý liên quan đến việc bồi thường và tái định cư cho cả hai hộ gia đình.</t>
+  </si>
+  <si>
+    <t>Các bác biết chỉ giúp em với ạ. 
+ Người đứng tên 2 sổ đỏ của 2 mảnh đất, khác phường, xã nhưng cùng thành phố. 
+ Vậy 1 sổ đỏ của một mảnh đất bị trong diện quy hoạch mình có được cấp đất tái định cư không ạ , và em muốn tìm hiểu về mục này cần tìm đọc điều luật nào ạ 
+ Em trân thành cảm ơn</t>
+  </si>
+  <si>
+    <t>Kết luận: Có thể được bố trí tái định cư khi thu hồi thửa đất ở, nhưng việc bạn đang đứng tên thêm một thửa đất khác trong cùng thành phố là yếu tố rất quan trọng. Nếu thửa đất còn lại có nhà ở/chỗ ở hợp pháp, cơ quan bồi thường thường sẽ xác định bạn đã có chỗ ở khác và không thuộc diện bắt buộc bố trí tái định cư; bồi thường có thể thực hiện bằng tiền hoặc đất/nhà tùy điều kiện và phương án địa phương.
+Cần phân biệt: “đất nằm trong quy hoạch” chưa chắc đã bị thu hồi. Chỉ khi có quyết định thu hồi đất để thực hiện dự án thì mới áp dụng chính sách bồi thường, hỗ trợ, tái định cư.
+Nếu thửa bị thu hồi là đất ở đủ điều kiện bồi thường, Nhà nước có thể bồi thường bằng đất ở hoặc nhà ở tái định cư Điều 111 Luật Đất đai 2024. Nhưng nếu không đủ điều kiện được bồi thường về đất ở, việc được giao đất/bán nhà tái định cư thường đặt ra khi gia đình phải di chuyển và không có chỗ ở nào khác trong địa bàn thành phố nơi có đất bị thu hồi Điều 111 Luật Đất đai 2024.
+Do đó, nếu sổ đỏ thứ hai chỉ là đất trống, đất nông nghiệp hoặc không thể ở hợp pháp, bạn cần cung cấp thông tin đó để đề nghị xem xét vẫn bố trí tái định cư. Nếu đó là đất ở có nhà ở và gia đình có thể ở tại đó, khả năng được một suất tái định cư sẽ thấp hơn.
+Bạn nên đọc trước:
+Điều 95 Luật Đất đai 2024: điều kiện được bồi thường về đất khi Nhà nước thu hồi;
+Điều 111 Luật Đất đai 2024: bồi thường về đất ở, nhà ở, tái định cư;
+Nghị định 88/2024/NĐ-CP: quy định chi tiết về bồi thường, hỗ trợ, tái định cư.
+Số suất tái định cư, trường hợp có chỗ ở khác và giá mua/giao tái định cư còn do quy định của tỉnh/thành phố nơi có đất. Bạn nên gửi văn bản cho tổ chức bồi thường đề nghị trả lời rõ: thửa đất thứ hai có bị coi là “chỗ ở khác” không và gia đình có thuộc diện được bố trí tái định cư không.
+[1]. Điều 95, 111, Luật 31/2024/QH15
+[2]. Nghị định 88/2024/NĐ-CP</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn Điều 95 và Điều 111 của Luật Đất đai 2024 (Luật số 31/2024/QH15), cùng với Nghị định 88/2024/NĐ-CP. Các điều luật này còn hiệu lực và phù hợp với câu hỏi về điều kiện bồi thường, hỗ trợ, tái định cư khi đất bị thu hồi. Điều 95 quy định về điều kiện bồi thường khi thu hồi đất, và Điều 111 quy định về bồi thường đất ở, nhà ở, tái định cư. Nghị định 88/2024/NĐ-CP quy định chi tiết về bồi thường, hỗ trợ, tái định cư. Các điều luật này đã bao phủ đầy đủ vấn đề người dùng hỏi.</t>
+  </si>
+  <si>
+    <t>Cả nhà cho e hỏi, mẹ e có miếng đất muốn tách sổ riêng cho con cái. Giờ phần đất đó lại được báo là quy hoạc đất TMDV nên không lên thổ cư để tách sổ được. Có cách nào để tách sổ được không ạ? (Diện tích: ngang 10 dài 70) . E cám ơn ạ!</t>
+  </si>
+  <si>
+    <t>Kết luận: Không thể tự chuyển phần đất quy hoạch thương mại–dịch vụ thành đất ở chỉ để tách sổ. Tuy nhiên, vẫn có thể tách thửa nếu mục đích sử dụng hiện tại và quy hoạch/điều kiện tách thửa tại địa phương cho phép; hoặc chờ/đề nghị điều chỉnh quy hoạch, hay tách theo đất thương mại–dịch vụ nếu đáp ứng điều kiện.
+“Quy hoạch đất thương mại, dịch vụ” không đồng nghĩa đất bị cấm giao dịch hay cấm tách thửa trong mọi trường hợp. Cần kiểm tra 3 nội dung: (i) loại đất đang ghi trên sổ; (ii) quy hoạch, kế hoạch sử dụng đất đã được phê duyệt; và (iii) quy định diện tích, kích thước tối thiểu được tách thửa của tỉnh nơi có đất. Mảnh ngang 10 m, dài 70 m chỉ là thông tin tham khảo, chưa đủ để kết luận có tách được hay không.
+Nếu sổ hiện là đất nông nghiệp hoặc đất khác, muốn tách để cho các con xây nhà thì thường phải xin chuyển mục đích sang đất ở. Việc cho phép chuyển mục đích phải phù hợp quy hoạch sử dụng đất và điều kiện địa phương; khi khu đất đã được xác định quy hoạch là thương mại–dịch vụ, cơ quan có thẩm quyền có thể không cho chuyển sang đất ở Điều 116 Luật Đất đai 2024.
+Nếu chỉ tách để con nhận quyền sử dụng đất theo đúng mục đích đang ghi trên sổ, gia đình có thể hỏi cơ quan có thẩm quyền về việc tách thửa đất thương mại–dịch vụ hoặc đất nông nghiệp. Sau khi tách, các con vẫn phải sử dụng đúng mục đích; không được xây nhà ở hoặc tự ý chuyển mục đích sử dụng đất Điều 5 Luật Đất đai 2024.
+Gia đình nên nộp phiếu yêu cầu cung cấp thông tin quy hoạch tại UBND xã/phường hoặc cơ quan quản lý đất đai cấp tỉnh, đồng thời hỏi bằng văn bản về: “thửa đất có được tách thửa theo mục đích sử dụng hiện tại không; diện tích tối thiểu là bao nhiêu; có được chuyển sang đất ở không”. Vì điều kiện tách thửa do từng tỉnh quy định, cần biết chính xác tỉnh/thành phố nơi có đất mới xác định được phương án.
+[1]. Điều 5, 116, Luật 31/2024/QH15</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn Điều 5 và Điều 116 của Luật Đất đai 2024 (Luật số 31/2024/QH15), là văn bản hiện hành và có hiệu lực. Điều 5 quy định về nguyên tắc sử dụng đất, trong khi Điều 116 quy định về chuyển mục đích sử dụng đất. Cả hai điều này đều liên quan đến việc tách thửa và chuyển mục đích sử dụng đất, phù hợp với câu hỏi của người dùng. Tuy nhiên, câu trả lời chưa đề cập đến các nghị định hướng dẫn chi tiết về điều kiện tách thửa theo từng địa phương, điều này có thể cần thiết để trả lời trọn vẹn hơn.</t>
+  </si>
+  <si>
+    <t>Chuyện là ba e có cho e 1 miếng đất và sắp tới e sẽ xây lại nhà trên đất này. Năm 1998 ba e có xây nhà trên đất này và đến 2007 ông bà e tách sổ đỏ riêng cho ba e. Đến 2013 có thay đổi để lên sổ hồng mới hay gì đó thì mẹ e hỏi bên xã ngta kêu nhà e khỏi đổi sổ hồng. Lúc đó e còn nhỏ và ba mẹ e nông dân cũng không biết nhiều nên để sổ đỏ cũ như năm 2007 luôn đến nay. Nay 2025 ba e sang tên cho e thì bắt buộc làm lại sổ hồng. Khi ra sổ rồi mới thấy là có dính quy hoạch kẻ vạch thẳng vào bản đồ đất luôn là gần 1 nửa diện tích đất. Loại đất trên sổ hồng hiện tại là Đất trồng cây lâu năm. E có thông tin từ bạn e là đất có cất nhà từ trước 2004 khi 2013 làm lại sổ sẽ được công nhận phần đất xây nhà là Đất Ở, nghĩa là cả thửa thì có phần xây nhà được tính thổ cư. Anh chị cho e hỏi thông tin này chính xác không và nếu thật vậy thì bây giờ e nên làm gì để được công nhận phần đất đó để đỡ tiền lên thổ cư cả thửa và khi quy hoạch sẽ được đền bù nhiều hơn. Nhà e xây giữa đất nên hiện tại 1 nửa dính quy hoạch và 1 nửa không dính. Và bây giờ nếu e đóng thổ cư e chỉ được đóng phần không dính quy hoạch. Nhưng phần quy hoạch có 1 nửa nhà e, nếu 2013 được công nhận phần đó thổ cư thì có phải sắp tới quy hoạch e được đền bù nhiều hơn, có giá hơn đất nông nghiệp đúng không ạ</t>
+  </si>
+  <si>
+    <t>Kết luận: Thông tin “cứ có nhà xây trước năm 2004 thì khi đổi sổ năm 2013 tự được công nhận đất ở” là không chính xác. Nhà xây từ năm 1998 là chứng cứ rất quan trọng để đề nghị xem xét công nhận một phần đất ở, nhưng phải căn cứ hồ sơ nguồn gốc đất, thời điểm sử dụng ổn định, hạn mức đất ở và quy hoạch tại địa phương; không tự động công nhận cả thửa.
+Sổ mới năm 2025 ghi toàn bộ là đất trồng cây lâu năm nghĩa là cơ quan đăng ký hiện chưa xác định phần đất nào là đất ở. Việc năm 2013 không đổi sang mẫu sổ mới không làm mất quyền xin xem xét, nhưng cũng không tạo quyền đương nhiên được công nhận đất ở.
+Bạn nên làm đơn đề nghị Văn phòng đăng ký đất đai/cơ quan quản lý đất đai cấp tỉnh xác minh và đính chính hoặc cấp đổi Giấy chứng nhận để công nhận diện tích đất ở có nhà từ năm 1998, nếu hồ sơ đủ căn cứ. Kèm theo: giấy tờ tách thửa năm 2007; giấy tờ nguồn gốc đất của ông bà; ảnh nhà cũ, giấy phép xây dựng nếu có; biên lai thuế nhà đất; xác nhận cư trú; hóa đơn điện nước lâu năm; xác nhận của người liền kề và UBND xã/phường về việc nhà có từ năm 1998, sử dụng ổn định, không tranh chấp.
+Việc xác định diện tích đất ở không chỉ dựa trên diện tích căn nhà. Với thửa đất có nhà ở và giấy tờ về quyền sử dụng đất, phần đã xây nhà và công trình phục vụ đời sống có thể được xác định là đất ở nhưng thường phải nộp tiền sử dụng đất theo quy định; phần còn lại được xác định theo hiện trạng hoặc theo mục đích phù hợp quy hoạch Điều 141 Luật Đất đai 2024.
+Về quy hoạch: nếu mới là quy hoạch trên bản đồ nhưng chưa có quyết định thu hồi đất, bạn vẫn nên làm thủ tục xác định/công nhận đất ở trước. Khi đã có thông báo thu hồi đất hoặc kế hoạch sử dụng đất hằng năm của cấp có thẩm quyền, việc chuyển mục đích sang đất ở đối với phần nằm trong khu vực thu hồi thường sẽ không được giải quyết. Việc cho phép chuyển mục đích còn phụ thuộc quy hoạch và điều kiện cụ thể Điều 116 Luật Đất đai 2024.
+Nếu sau này Nhà nước thu hồi, phần nào được công nhận là đất ở và đủ điều kiện bồi thường thì về nguyên tắc được bồi thường theo loại đất ở; phần vẫn là đất trồng cây lâu năm được bồi thường theo đất nông nghiệp. Do đó, việc xác minh lịch sử căn nhà và đề nghị công nhận đất ở ngay bây giờ là có ý nghĩa. Tuy nhiên, không nên xây lại nhà hoặc tháo dỡ nhà cũ trước khi hoàn tất kiểm kê/ghi nhận hiện trạng, vì có thể làm khó việc chứng minh nhà đã tồn tại từ năm 1998.
+Bạn cần đặc biệt lưu ý: nếu nhà cũ nằm một phần trong hành lang/quy hoạch dự án, hãy đề nghị đơn vị bồi thường kiểm kê đầy đủ hiện trạng nhà cũ, diện tích xây dựng, ảnh hiện trạng và mốc thời điểm tạo lập. Việc bồi thường nhà, công trình và đất là các khoản xem xét riêng; xây dựng mới sau khi có thông báo thu hồi đất thường không được bồi thường.
+Nếu đất của gia đình thuộc trường hợp không có giấy tờ đầy đủ về quyền sử dụng đất từ trước, pháp luật cũng có cơ chế xác định bồi thường đất ở cho đất có nhà ở sử dụng ổn định theo các mốc thời gian và hạn mức địa phương Điều 8 Nghị định 88/2024/NĐ-CP.
+[1]. Điều 116, 141, Luật 31/2024/QH15
+[2]. Điều 8, Nghị định 88/2024/NĐ-CP</t>
+  </si>
+  <si>
+    <t>Câu trả lời đã trích dẫn Điều 116 và 141 của Luật Đất đai 2024 (Luật số 31/2024/QH15) và Điều 8 của Nghị định 88/2024/NĐ-CP. Các điều luật này còn hiệu lực và phù hợp với vấn đề người hỏi, bao gồm việc công nhận đất ở, quy hoạch và bồi thường khi thu hồi đất. Điều 116 quy định về chuyển mục đích sử dụng đất, Điều 141 quy định về công nhận đất ở, và Điều 8 của Nghị định 88/2024/NĐ-CP quy định về bồi thường đất ở cho đất có nhà ở sử dụng ổn định. Câu trả lời đã bao phủ đầy đủ các khía cạnh pháp lý liên quan đến câu hỏi của người dùng.</t>
+  </si>
+  <si>
+    <t>Nhà em nằm trên dự án đường điện cao thế 500kv chơn thành-long an . Năm trước có nhận được giấy bồi thường nhưng trên giấy ghi là đất nông nghiệp mặc dù nhà em là đất thổ cư sau kiến nghị thì năm nay lại giảm xuống nữa và nhận được câu trả lời là chỉ bồi thường theo diện đất bình thường và còn nói là do đất nhà em kh nằm trên đường nhựa mặc dù trong giấy năm trước cũng ghi là đất nằm trên mặt đường đất 5m và đền với giá cao nhưng năm nay lại giảm xuống 
+ Cao nhân nào giải đáp giúp em với ạ chứ nhà em hoang mang quá rồi</t>
+  </si>
+  <si>
+    <t>Kết luận: Gia đình cần yêu cầu cơ quan bồi thường trả lời bằng văn bản về lý do thửa đất ở lại bị áp giá đất nông nghiệp và lý do đơn giá năm nay giảm. Nếu sổ/giấy tờ pháp lý xác định là đất ở, cơ quan không thể chỉ vì đất không giáp đường nhựa mà chuyển loại đất sang đất nông nghiệp; vị trí đường nhựa hay đường đất chỉ có thể ảnh hưởng đến mức giá đất ở theo vị trí, không làm thay đổi mục đích sử dụng đất.
+Trước hết, kiểm tra 3 tài liệu: Giấy chứng nhận (mục “mục đích sử dụng đất”, diện tích đất ở); thông báo/ quyết định thu hồi đất; phương án bồi thường năm trước và phương án mới. Đề nghị đối chiếu rõ: diện tích nào ghi đất ở, diện tích nào ghi đất nông nghiệp, vị trí thửa đất, bảng giá/giá đất cụ thể áp dụng và quyết định phê duyệt phương án.
+Bồi thường đất được xác định theo mục đích sử dụng đất tại thời điểm có quyết định thu hồi đất, không căn cứ việc có đường nhựa hay không Điều 95 Luật Đất đai 2024. Trường hợp đất ở đủ điều kiện bồi thường, nguyên tắc bồi thường là bằng đất ở, nhà ở hoặc bằng tiền theo giá đất cụ thể của loại đất ở Điều 111 Luật Đất đai 2024.
+Cần lưu ý: dự án đường dây 500kV có thể có phần đất bị thu hồi làm vị trí móng trụ và phần đất chỉ nằm trong hành lang an toàn lưới điện. Nếu chỉ thuộc hành lang mà không thu hồi, vẫn có thể bị hạn chế xây dựng, sử dụng đất và được bồi thường/hỗ trợ khi đủ điều kiện theo quy định về hành lang an toàn lưới điện Nghị định 62/2025/NĐ-CP. Vì vậy, cần hỏi họ ghi rõ: nhà bạn bị thu hồi toàn bộ/một phần đất, hay chỉ ảnh hưởng hành lang.
+Bạn nên nộp ngay “Đơn đề nghị cung cấp hồ sơ và giải trình giá bồi thường”, yêu cầu:
+Bản trích lục địa chính, bản đồ vị trí và bảng kiểm kê thửa đất;
+Căn cứ xác định đất nông nghiệp thay vì đất ở;
+Quyết định giá đất cụ thể, bảng giá vị trí và phương án bồi thường được phê duyệt;
+Giải thích chênh lệch giữa phương án năm trước và năm nay;
+Biên bản kiểm kê lại có chữ ký của gia đình.
+Không ký biên bản hoặc nhận tiền với nội dung xác định sai loại đất; nếu đã ký, vẫn ghi ý kiến bảo lưu: “Không đồng ý xác định đất nông nghiệp/đơn giá bồi thường; đề nghị xác định theo Giấy chứng nhận và cung cấp căn cứ pháp lý”. Khi nhận được quyết định bồi thường, gia đình có quyền khiếu nại lần đầu đến cơ quan đã ban hành quyết định; nếu không đồng ý kết quả, có thể khiếu nại tiếp hoặc khởi kiện vụ án hành chính Luật Khiếu nại 2011.
+[1]. Điều 95, 111, Luật 31/2024/QH15
+[2]. Nghị định 62/2025/NĐ-CP
+[3]. Luật 02/2011/QH13</t>
+  </si>
+  <si>
+    <t>Câu trả lời trích dẫn Điều 95 và 111 của Luật Đất đai 2024 (Luật số 31/2024/QH15), tuy nhiên không có nội dung cụ thể của các điều luật này trong câu trả lời để xác định tính đúng đắn. Ngoài ra, Nghị định 62/2025/NĐ-CP được trích dẫn nhưng chưa có hiệu lực tại thời điểm hiện tại (2023). Luật Khiếu nại 2011 (Luật 02/2011/QH13) vẫn còn hiệu lực và phù hợp với tình huống khiếu nại. Tuy nhiên, do sử dụng văn bản chưa có hiệu lực và không có nội dung cụ thể của điều luật, tiêu chí trích dẫn điều luật bị đánh giá là false.</t>
   </si>
 </sst>
 </file>
@@ -2828,7 +4108,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J120"/>
+  <dimension ref="A1:J180"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -2836,6 +4116,7 @@
     <col min="3" max="3" width="90" customWidth="1"/>
     <col min="4" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="50" customWidth="1"/>
+    <col min="9" max="9" width="29" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.2">
@@ -6333,6 +7614,1746 @@
         <v>14</v>
       </c>
     </row>
+    <row r="121" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A121">
+        <v>120</v>
+      </c>
+      <c r="B121" t="s">
+        <v>380</v>
+      </c>
+      <c r="C121" t="s">
+        <v>381</v>
+      </c>
+      <c r="D121" t="s">
+        <v>12</v>
+      </c>
+      <c r="E121" t="s">
+        <v>12</v>
+      </c>
+      <c r="F121" t="s">
+        <v>12</v>
+      </c>
+      <c r="G121" t="s">
+        <v>12</v>
+      </c>
+      <c r="H121" t="s">
+        <v>382</v>
+      </c>
+      <c r="I121" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="122" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A122">
+        <v>121</v>
+      </c>
+      <c r="B122" t="s">
+        <v>384</v>
+      </c>
+      <c r="C122" t="s">
+        <v>385</v>
+      </c>
+      <c r="D122" t="s">
+        <v>18</v>
+      </c>
+      <c r="E122" t="s">
+        <v>18</v>
+      </c>
+      <c r="F122" t="s">
+        <v>18</v>
+      </c>
+      <c r="G122" t="s">
+        <v>18</v>
+      </c>
+      <c r="H122" t="s">
+        <v>386</v>
+      </c>
+      <c r="I122" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="123" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A123">
+        <v>122</v>
+      </c>
+      <c r="B123" t="s">
+        <v>387</v>
+      </c>
+      <c r="C123" t="s">
+        <v>388</v>
+      </c>
+      <c r="D123" t="s">
+        <v>12</v>
+      </c>
+      <c r="E123" t="s">
+        <v>18</v>
+      </c>
+      <c r="F123" t="s">
+        <v>12</v>
+      </c>
+      <c r="G123" t="s">
+        <v>12</v>
+      </c>
+      <c r="H123" t="s">
+        <v>389</v>
+      </c>
+      <c r="I123" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="124" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A124">
+        <v>123</v>
+      </c>
+      <c r="B124" t="s">
+        <v>390</v>
+      </c>
+      <c r="C124" t="s">
+        <v>391</v>
+      </c>
+      <c r="D124" t="s">
+        <v>12</v>
+      </c>
+      <c r="E124" t="s">
+        <v>12</v>
+      </c>
+      <c r="F124" t="s">
+        <v>12</v>
+      </c>
+      <c r="G124" t="s">
+        <v>12</v>
+      </c>
+      <c r="H124" t="s">
+        <v>392</v>
+      </c>
+      <c r="I124" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="125" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A125">
+        <v>124</v>
+      </c>
+      <c r="B125" t="s">
+        <v>173</v>
+      </c>
+      <c r="C125" t="s">
+        <v>393</v>
+      </c>
+      <c r="D125" t="s">
+        <v>12</v>
+      </c>
+      <c r="E125" t="s">
+        <v>12</v>
+      </c>
+      <c r="F125" t="s">
+        <v>12</v>
+      </c>
+      <c r="G125" t="s">
+        <v>12</v>
+      </c>
+      <c r="H125" t="s">
+        <v>394</v>
+      </c>
+      <c r="I125" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="126" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A126">
+        <v>125</v>
+      </c>
+      <c r="B126" t="s">
+        <v>395</v>
+      </c>
+      <c r="C126" t="s">
+        <v>396</v>
+      </c>
+      <c r="D126" t="s">
+        <v>12</v>
+      </c>
+      <c r="E126" t="s">
+        <v>18</v>
+      </c>
+      <c r="F126" t="s">
+        <v>12</v>
+      </c>
+      <c r="G126" t="s">
+        <v>12</v>
+      </c>
+      <c r="H126" t="s">
+        <v>397</v>
+      </c>
+      <c r="I126" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="127" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A127">
+        <v>126</v>
+      </c>
+      <c r="B127" t="s">
+        <v>398</v>
+      </c>
+      <c r="C127" t="s">
+        <v>399</v>
+      </c>
+      <c r="D127" t="s">
+        <v>12</v>
+      </c>
+      <c r="E127" t="s">
+        <v>12</v>
+      </c>
+      <c r="F127" t="s">
+        <v>12</v>
+      </c>
+      <c r="G127" t="s">
+        <v>12</v>
+      </c>
+      <c r="H127" t="s">
+        <v>400</v>
+      </c>
+      <c r="I127" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="128" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A128">
+        <v>127</v>
+      </c>
+      <c r="B128" t="s">
+        <v>401</v>
+      </c>
+      <c r="C128" t="s">
+        <v>402</v>
+      </c>
+      <c r="D128" t="s">
+        <v>12</v>
+      </c>
+      <c r="E128" t="s">
+        <v>12</v>
+      </c>
+      <c r="F128" t="s">
+        <v>12</v>
+      </c>
+      <c r="G128" t="s">
+        <v>12</v>
+      </c>
+      <c r="H128" t="s">
+        <v>403</v>
+      </c>
+      <c r="I128" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="129" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A129">
+        <v>128</v>
+      </c>
+      <c r="B129" t="s">
+        <v>404</v>
+      </c>
+      <c r="C129" t="s">
+        <v>405</v>
+      </c>
+      <c r="D129" t="s">
+        <v>12</v>
+      </c>
+      <c r="E129" t="s">
+        <v>18</v>
+      </c>
+      <c r="F129" t="s">
+        <v>12</v>
+      </c>
+      <c r="G129" t="s">
+        <v>12</v>
+      </c>
+      <c r="H129" t="s">
+        <v>406</v>
+      </c>
+      <c r="I129" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="130" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A130">
+        <v>129</v>
+      </c>
+      <c r="B130" t="s">
+        <v>407</v>
+      </c>
+      <c r="C130" t="s">
+        <v>408</v>
+      </c>
+      <c r="D130" t="s">
+        <v>12</v>
+      </c>
+      <c r="E130" t="s">
+        <v>18</v>
+      </c>
+      <c r="F130" t="s">
+        <v>12</v>
+      </c>
+      <c r="G130" t="s">
+        <v>12</v>
+      </c>
+      <c r="H130" t="s">
+        <v>409</v>
+      </c>
+      <c r="I130" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="131" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A131">
+        <v>130</v>
+      </c>
+      <c r="B131" t="s">
+        <v>410</v>
+      </c>
+      <c r="C131" t="s">
+        <v>411</v>
+      </c>
+      <c r="D131" t="s">
+        <v>12</v>
+      </c>
+      <c r="E131" t="s">
+        <v>18</v>
+      </c>
+      <c r="F131" t="s">
+        <v>12</v>
+      </c>
+      <c r="G131" t="s">
+        <v>12</v>
+      </c>
+      <c r="H131" t="s">
+        <v>412</v>
+      </c>
+      <c r="I131" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="132" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A132">
+        <v>131</v>
+      </c>
+      <c r="B132" t="s">
+        <v>413</v>
+      </c>
+      <c r="C132" t="s">
+        <v>414</v>
+      </c>
+      <c r="D132" t="s">
+        <v>12</v>
+      </c>
+      <c r="E132" t="s">
+        <v>18</v>
+      </c>
+      <c r="F132" t="s">
+        <v>12</v>
+      </c>
+      <c r="G132" t="s">
+        <v>12</v>
+      </c>
+      <c r="H132" t="s">
+        <v>415</v>
+      </c>
+      <c r="I132" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="133" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A133">
+        <v>132</v>
+      </c>
+      <c r="B133" t="s">
+        <v>416</v>
+      </c>
+      <c r="C133" t="s">
+        <v>417</v>
+      </c>
+      <c r="D133" t="s">
+        <v>12</v>
+      </c>
+      <c r="E133" t="s">
+        <v>18</v>
+      </c>
+      <c r="F133" t="s">
+        <v>12</v>
+      </c>
+      <c r="G133" t="s">
+        <v>12</v>
+      </c>
+      <c r="H133" t="s">
+        <v>418</v>
+      </c>
+      <c r="I133" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="134" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A134">
+        <v>133</v>
+      </c>
+      <c r="B134" t="s">
+        <v>176</v>
+      </c>
+      <c r="C134" t="s">
+        <v>419</v>
+      </c>
+      <c r="D134" t="s">
+        <v>12</v>
+      </c>
+      <c r="E134" t="s">
+        <v>12</v>
+      </c>
+      <c r="F134" t="s">
+        <v>12</v>
+      </c>
+      <c r="G134" t="s">
+        <v>12</v>
+      </c>
+      <c r="H134" t="s">
+        <v>420</v>
+      </c>
+      <c r="I134" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="135" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A135">
+        <v>134</v>
+      </c>
+      <c r="B135" t="s">
+        <v>421</v>
+      </c>
+      <c r="C135" t="s">
+        <v>422</v>
+      </c>
+      <c r="D135" t="s">
+        <v>12</v>
+      </c>
+      <c r="E135" t="s">
+        <v>12</v>
+      </c>
+      <c r="F135" t="s">
+        <v>12</v>
+      </c>
+      <c r="G135" t="s">
+        <v>12</v>
+      </c>
+      <c r="H135" t="s">
+        <v>423</v>
+      </c>
+      <c r="I135" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="136" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A136">
+        <v>135</v>
+      </c>
+      <c r="B136" t="s">
+        <v>424</v>
+      </c>
+      <c r="C136" t="s">
+        <v>425</v>
+      </c>
+      <c r="D136" t="s">
+        <v>12</v>
+      </c>
+      <c r="E136" t="s">
+        <v>18</v>
+      </c>
+      <c r="F136" t="s">
+        <v>12</v>
+      </c>
+      <c r="G136" t="s">
+        <v>12</v>
+      </c>
+      <c r="H136" t="s">
+        <v>426</v>
+      </c>
+      <c r="I136" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="137" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A137">
+        <v>136</v>
+      </c>
+      <c r="B137" t="s">
+        <v>427</v>
+      </c>
+      <c r="C137" t="s">
+        <v>428</v>
+      </c>
+      <c r="D137" t="s">
+        <v>12</v>
+      </c>
+      <c r="E137" t="s">
+        <v>18</v>
+      </c>
+      <c r="F137" t="s">
+        <v>12</v>
+      </c>
+      <c r="G137" t="s">
+        <v>12</v>
+      </c>
+      <c r="H137" t="s">
+        <v>429</v>
+      </c>
+      <c r="I137" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="138" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A138">
+        <v>137</v>
+      </c>
+      <c r="B138" t="s">
+        <v>431</v>
+      </c>
+      <c r="C138" t="s">
+        <v>432</v>
+      </c>
+      <c r="D138" t="s">
+        <v>12</v>
+      </c>
+      <c r="E138" t="s">
+        <v>18</v>
+      </c>
+      <c r="F138" t="s">
+        <v>18</v>
+      </c>
+      <c r="G138" t="s">
+        <v>18</v>
+      </c>
+      <c r="H138" t="s">
+        <v>433</v>
+      </c>
+      <c r="I138" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="139" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A139">
+        <v>138</v>
+      </c>
+      <c r="B139" t="s">
+        <v>434</v>
+      </c>
+      <c r="C139" t="s">
+        <v>435</v>
+      </c>
+      <c r="D139" t="s">
+        <v>12</v>
+      </c>
+      <c r="E139" t="s">
+        <v>18</v>
+      </c>
+      <c r="F139" t="s">
+        <v>12</v>
+      </c>
+      <c r="G139" t="s">
+        <v>12</v>
+      </c>
+      <c r="H139" t="s">
+        <v>436</v>
+      </c>
+      <c r="I139" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="140" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A140">
+        <v>139</v>
+      </c>
+      <c r="B140" t="s">
+        <v>437</v>
+      </c>
+      <c r="C140" t="s">
+        <v>438</v>
+      </c>
+      <c r="D140" t="s">
+        <v>12</v>
+      </c>
+      <c r="E140" t="s">
+        <v>12</v>
+      </c>
+      <c r="F140" t="s">
+        <v>12</v>
+      </c>
+      <c r="G140" t="s">
+        <v>12</v>
+      </c>
+      <c r="H140" t="s">
+        <v>439</v>
+      </c>
+      <c r="I140" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="141" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A141">
+        <v>140</v>
+      </c>
+      <c r="B141" t="s">
+        <v>440</v>
+      </c>
+      <c r="C141" t="s">
+        <v>441</v>
+      </c>
+      <c r="D141" t="s">
+        <v>12</v>
+      </c>
+      <c r="E141" t="s">
+        <v>18</v>
+      </c>
+      <c r="F141" t="s">
+        <v>12</v>
+      </c>
+      <c r="G141" t="s">
+        <v>12</v>
+      </c>
+      <c r="H141" t="s">
+        <v>442</v>
+      </c>
+      <c r="I141" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="142" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A142">
+        <v>141</v>
+      </c>
+      <c r="B142" t="s">
+        <v>443</v>
+      </c>
+      <c r="C142" t="s">
+        <v>444</v>
+      </c>
+      <c r="D142" t="s">
+        <v>12</v>
+      </c>
+      <c r="E142" t="s">
+        <v>12</v>
+      </c>
+      <c r="F142" t="s">
+        <v>12</v>
+      </c>
+      <c r="G142" t="s">
+        <v>12</v>
+      </c>
+      <c r="H142" t="s">
+        <v>445</v>
+      </c>
+      <c r="I142" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="143" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A143">
+        <v>142</v>
+      </c>
+      <c r="B143" t="s">
+        <v>446</v>
+      </c>
+      <c r="C143" t="s">
+        <v>447</v>
+      </c>
+      <c r="D143" t="s">
+        <v>12</v>
+      </c>
+      <c r="E143" t="s">
+        <v>18</v>
+      </c>
+      <c r="F143" t="s">
+        <v>12</v>
+      </c>
+      <c r="G143" t="s">
+        <v>12</v>
+      </c>
+      <c r="H143" t="s">
+        <v>448</v>
+      </c>
+      <c r="I143" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="144" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A144">
+        <v>143</v>
+      </c>
+      <c r="B144" t="s">
+        <v>449</v>
+      </c>
+      <c r="C144" t="s">
+        <v>450</v>
+      </c>
+      <c r="D144" t="s">
+        <v>12</v>
+      </c>
+      <c r="E144" t="s">
+        <v>18</v>
+      </c>
+      <c r="F144" t="s">
+        <v>12</v>
+      </c>
+      <c r="G144" t="s">
+        <v>12</v>
+      </c>
+      <c r="H144" t="s">
+        <v>451</v>
+      </c>
+      <c r="I144" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="145" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A145">
+        <v>144</v>
+      </c>
+      <c r="B145" t="s">
+        <v>452</v>
+      </c>
+      <c r="C145" t="s">
+        <v>453</v>
+      </c>
+      <c r="D145" t="s">
+        <v>12</v>
+      </c>
+      <c r="E145" t="s">
+        <v>12</v>
+      </c>
+      <c r="F145" t="s">
+        <v>12</v>
+      </c>
+      <c r="G145" t="s">
+        <v>12</v>
+      </c>
+      <c r="H145" t="s">
+        <v>454</v>
+      </c>
+      <c r="I145" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="146" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A146">
+        <v>145</v>
+      </c>
+      <c r="B146" t="s">
+        <v>455</v>
+      </c>
+      <c r="C146" t="s">
+        <v>456</v>
+      </c>
+      <c r="D146" t="s">
+        <v>12</v>
+      </c>
+      <c r="E146" t="s">
+        <v>18</v>
+      </c>
+      <c r="F146" t="s">
+        <v>12</v>
+      </c>
+      <c r="G146" t="s">
+        <v>12</v>
+      </c>
+      <c r="H146" t="s">
+        <v>457</v>
+      </c>
+      <c r="I146" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="147" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A147">
+        <v>146</v>
+      </c>
+      <c r="B147" t="s">
+        <v>458</v>
+      </c>
+      <c r="C147" t="s">
+        <v>459</v>
+      </c>
+      <c r="D147" t="s">
+        <v>12</v>
+      </c>
+      <c r="E147" t="s">
+        <v>18</v>
+      </c>
+      <c r="F147" t="s">
+        <v>12</v>
+      </c>
+      <c r="G147" t="s">
+        <v>12</v>
+      </c>
+      <c r="H147" t="s">
+        <v>460</v>
+      </c>
+      <c r="I147" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="148" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A148">
+        <v>147</v>
+      </c>
+      <c r="B148" t="s">
+        <v>461</v>
+      </c>
+      <c r="C148" t="s">
+        <v>462</v>
+      </c>
+      <c r="D148" t="s">
+        <v>12</v>
+      </c>
+      <c r="E148" t="s">
+        <v>18</v>
+      </c>
+      <c r="F148" t="s">
+        <v>12</v>
+      </c>
+      <c r="G148" t="s">
+        <v>12</v>
+      </c>
+      <c r="H148" t="s">
+        <v>463</v>
+      </c>
+      <c r="I148" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="149" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A149">
+        <v>148</v>
+      </c>
+      <c r="B149" t="s">
+        <v>464</v>
+      </c>
+      <c r="C149" t="s">
+        <v>465</v>
+      </c>
+      <c r="D149" t="s">
+        <v>12</v>
+      </c>
+      <c r="E149" t="s">
+        <v>18</v>
+      </c>
+      <c r="F149" t="s">
+        <v>12</v>
+      </c>
+      <c r="G149" t="s">
+        <v>12</v>
+      </c>
+      <c r="H149" t="s">
+        <v>466</v>
+      </c>
+      <c r="I149" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="150" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A150">
+        <v>149</v>
+      </c>
+      <c r="B150" t="s">
+        <v>467</v>
+      </c>
+      <c r="C150" t="s">
+        <v>468</v>
+      </c>
+      <c r="D150" t="s">
+        <v>12</v>
+      </c>
+      <c r="E150" t="s">
+        <v>18</v>
+      </c>
+      <c r="F150" t="s">
+        <v>12</v>
+      </c>
+      <c r="G150" t="s">
+        <v>12</v>
+      </c>
+      <c r="H150" t="s">
+        <v>469</v>
+      </c>
+      <c r="I150" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="151" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A151">
+        <v>150</v>
+      </c>
+      <c r="B151" t="s">
+        <v>470</v>
+      </c>
+      <c r="C151" t="s">
+        <v>471</v>
+      </c>
+      <c r="D151" t="s">
+        <v>12</v>
+      </c>
+      <c r="E151" t="s">
+        <v>12</v>
+      </c>
+      <c r="F151" t="s">
+        <v>12</v>
+      </c>
+      <c r="G151" t="s">
+        <v>12</v>
+      </c>
+      <c r="H151" t="s">
+        <v>472</v>
+      </c>
+      <c r="I151" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="152" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A152">
+        <v>151</v>
+      </c>
+      <c r="B152" t="s">
+        <v>474</v>
+      </c>
+      <c r="C152" t="s">
+        <v>475</v>
+      </c>
+      <c r="D152" t="s">
+        <v>12</v>
+      </c>
+      <c r="E152" t="s">
+        <v>18</v>
+      </c>
+      <c r="F152" t="s">
+        <v>12</v>
+      </c>
+      <c r="G152" t="s">
+        <v>12</v>
+      </c>
+      <c r="H152" t="s">
+        <v>476</v>
+      </c>
+      <c r="I152" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="153" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A153">
+        <v>152</v>
+      </c>
+      <c r="B153" t="s">
+        <v>477</v>
+      </c>
+      <c r="C153" t="s">
+        <v>478</v>
+      </c>
+      <c r="D153" t="s">
+        <v>12</v>
+      </c>
+      <c r="E153" t="s">
+        <v>18</v>
+      </c>
+      <c r="F153" t="s">
+        <v>12</v>
+      </c>
+      <c r="G153" t="s">
+        <v>12</v>
+      </c>
+      <c r="H153" t="s">
+        <v>479</v>
+      </c>
+      <c r="I153" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="154" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A154">
+        <v>153</v>
+      </c>
+      <c r="B154" t="s">
+        <v>480</v>
+      </c>
+      <c r="C154" t="s">
+        <v>481</v>
+      </c>
+      <c r="D154" t="s">
+        <v>12</v>
+      </c>
+      <c r="E154" t="s">
+        <v>12</v>
+      </c>
+      <c r="F154" t="s">
+        <v>12</v>
+      </c>
+      <c r="G154" t="s">
+        <v>12</v>
+      </c>
+      <c r="H154" t="s">
+        <v>482</v>
+      </c>
+      <c r="I154" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="155" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A155">
+        <v>154</v>
+      </c>
+      <c r="B155" t="s">
+        <v>483</v>
+      </c>
+      <c r="C155" t="s">
+        <v>484</v>
+      </c>
+      <c r="D155" t="s">
+        <v>12</v>
+      </c>
+      <c r="E155" t="s">
+        <v>18</v>
+      </c>
+      <c r="F155" t="s">
+        <v>12</v>
+      </c>
+      <c r="G155" t="s">
+        <v>12</v>
+      </c>
+      <c r="H155" t="s">
+        <v>485</v>
+      </c>
+      <c r="I155" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="156" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A156">
+        <v>155</v>
+      </c>
+      <c r="B156" t="s">
+        <v>486</v>
+      </c>
+      <c r="C156" t="s">
+        <v>487</v>
+      </c>
+      <c r="D156" t="s">
+        <v>12</v>
+      </c>
+      <c r="E156" t="s">
+        <v>18</v>
+      </c>
+      <c r="F156" t="s">
+        <v>12</v>
+      </c>
+      <c r="G156" t="s">
+        <v>12</v>
+      </c>
+      <c r="H156" t="s">
+        <v>488</v>
+      </c>
+      <c r="I156" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="157" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A157">
+        <v>156</v>
+      </c>
+      <c r="B157" t="s">
+        <v>489</v>
+      </c>
+      <c r="C157" t="s">
+        <v>490</v>
+      </c>
+      <c r="D157" t="s">
+        <v>12</v>
+      </c>
+      <c r="E157" t="s">
+        <v>12</v>
+      </c>
+      <c r="F157" t="s">
+        <v>12</v>
+      </c>
+      <c r="G157" t="s">
+        <v>12</v>
+      </c>
+      <c r="H157" t="s">
+        <v>491</v>
+      </c>
+      <c r="I157" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="158" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A158">
+        <v>157</v>
+      </c>
+      <c r="B158" t="s">
+        <v>492</v>
+      </c>
+      <c r="C158" t="s">
+        <v>493</v>
+      </c>
+      <c r="D158" t="s">
+        <v>12</v>
+      </c>
+      <c r="E158" t="s">
+        <v>12</v>
+      </c>
+      <c r="F158" t="s">
+        <v>12</v>
+      </c>
+      <c r="G158" t="s">
+        <v>12</v>
+      </c>
+      <c r="H158" t="s">
+        <v>494</v>
+      </c>
+      <c r="I158" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="159" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A159">
+        <v>158</v>
+      </c>
+      <c r="B159" t="s">
+        <v>495</v>
+      </c>
+      <c r="C159" t="s">
+        <v>496</v>
+      </c>
+      <c r="D159" t="s">
+        <v>12</v>
+      </c>
+      <c r="E159" t="s">
+        <v>12</v>
+      </c>
+      <c r="F159" t="s">
+        <v>12</v>
+      </c>
+      <c r="G159" t="s">
+        <v>12</v>
+      </c>
+      <c r="H159" t="s">
+        <v>497</v>
+      </c>
+      <c r="I159" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="160" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A160">
+        <v>159</v>
+      </c>
+      <c r="B160" t="s">
+        <v>498</v>
+      </c>
+      <c r="C160" t="s">
+        <v>499</v>
+      </c>
+      <c r="D160" t="s">
+        <v>12</v>
+      </c>
+      <c r="E160" t="s">
+        <v>18</v>
+      </c>
+      <c r="F160" t="s">
+        <v>12</v>
+      </c>
+      <c r="G160" t="s">
+        <v>12</v>
+      </c>
+      <c r="H160" t="s">
+        <v>500</v>
+      </c>
+      <c r="I160" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="161" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A161">
+        <v>160</v>
+      </c>
+      <c r="B161" t="s">
+        <v>501</v>
+      </c>
+      <c r="C161" t="s">
+        <v>502</v>
+      </c>
+      <c r="D161" t="s">
+        <v>12</v>
+      </c>
+      <c r="E161" t="s">
+        <v>18</v>
+      </c>
+      <c r="F161" t="s">
+        <v>12</v>
+      </c>
+      <c r="G161" t="s">
+        <v>12</v>
+      </c>
+      <c r="H161" t="s">
+        <v>503</v>
+      </c>
+      <c r="I161" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="162" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A162">
+        <v>161</v>
+      </c>
+      <c r="B162" t="s">
+        <v>504</v>
+      </c>
+      <c r="C162" t="s">
+        <v>505</v>
+      </c>
+      <c r="D162" t="s">
+        <v>12</v>
+      </c>
+      <c r="E162" t="s">
+        <v>18</v>
+      </c>
+      <c r="F162" t="s">
+        <v>12</v>
+      </c>
+      <c r="G162" t="s">
+        <v>12</v>
+      </c>
+      <c r="H162" t="s">
+        <v>506</v>
+      </c>
+      <c r="I162" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="163" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A163">
+        <v>162</v>
+      </c>
+      <c r="B163" t="s">
+        <v>507</v>
+      </c>
+      <c r="C163" t="s">
+        <v>508</v>
+      </c>
+      <c r="D163" t="s">
+        <v>12</v>
+      </c>
+      <c r="E163" t="s">
+        <v>18</v>
+      </c>
+      <c r="F163" t="s">
+        <v>12</v>
+      </c>
+      <c r="G163" t="s">
+        <v>12</v>
+      </c>
+      <c r="H163" t="s">
+        <v>509</v>
+      </c>
+      <c r="I163" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="164" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A164">
+        <v>163</v>
+      </c>
+      <c r="B164" t="s">
+        <v>510</v>
+      </c>
+      <c r="C164" t="s">
+        <v>511</v>
+      </c>
+      <c r="D164" t="s">
+        <v>12</v>
+      </c>
+      <c r="E164" t="s">
+        <v>18</v>
+      </c>
+      <c r="F164" t="s">
+        <v>12</v>
+      </c>
+      <c r="G164" t="s">
+        <v>12</v>
+      </c>
+      <c r="H164" t="s">
+        <v>512</v>
+      </c>
+      <c r="I164" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="165" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A165">
+        <v>164</v>
+      </c>
+      <c r="B165" t="s">
+        <v>513</v>
+      </c>
+      <c r="C165" t="s">
+        <v>514</v>
+      </c>
+      <c r="D165" t="s">
+        <v>12</v>
+      </c>
+      <c r="E165" t="s">
+        <v>18</v>
+      </c>
+      <c r="F165" t="s">
+        <v>12</v>
+      </c>
+      <c r="G165" t="s">
+        <v>12</v>
+      </c>
+      <c r="H165" t="s">
+        <v>515</v>
+      </c>
+      <c r="I165" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="166" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A166">
+        <v>165</v>
+      </c>
+      <c r="B166" t="s">
+        <v>516</v>
+      </c>
+      <c r="C166" t="s">
+        <v>517</v>
+      </c>
+      <c r="D166" t="s">
+        <v>12</v>
+      </c>
+      <c r="E166" t="s">
+        <v>18</v>
+      </c>
+      <c r="F166" t="s">
+        <v>12</v>
+      </c>
+      <c r="G166" t="s">
+        <v>12</v>
+      </c>
+      <c r="H166" t="s">
+        <v>518</v>
+      </c>
+      <c r="I166" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="167" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A167">
+        <v>166</v>
+      </c>
+      <c r="B167" t="s">
+        <v>519</v>
+      </c>
+      <c r="C167" t="s">
+        <v>520</v>
+      </c>
+      <c r="D167" t="s">
+        <v>12</v>
+      </c>
+      <c r="E167" t="s">
+        <v>12</v>
+      </c>
+      <c r="F167" t="s">
+        <v>12</v>
+      </c>
+      <c r="G167" t="s">
+        <v>12</v>
+      </c>
+      <c r="H167" t="s">
+        <v>521</v>
+      </c>
+      <c r="I167" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="168" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A168">
+        <v>167</v>
+      </c>
+      <c r="B168" t="s">
+        <v>523</v>
+      </c>
+      <c r="C168" t="s">
+        <v>524</v>
+      </c>
+      <c r="D168" t="s">
+        <v>12</v>
+      </c>
+      <c r="E168" t="s">
+        <v>12</v>
+      </c>
+      <c r="F168" t="s">
+        <v>12</v>
+      </c>
+      <c r="G168" t="s">
+        <v>12</v>
+      </c>
+      <c r="H168" t="s">
+        <v>525</v>
+      </c>
+      <c r="I168" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="169" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A169">
+        <v>168</v>
+      </c>
+      <c r="B169" t="s">
+        <v>350</v>
+      </c>
+      <c r="C169" t="s">
+        <v>526</v>
+      </c>
+      <c r="D169" t="s">
+        <v>12</v>
+      </c>
+      <c r="E169" t="s">
+        <v>12</v>
+      </c>
+      <c r="F169" t="s">
+        <v>12</v>
+      </c>
+      <c r="G169" t="s">
+        <v>12</v>
+      </c>
+      <c r="H169" t="s">
+        <v>527</v>
+      </c>
+      <c r="I169" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="170" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A170">
+        <v>169</v>
+      </c>
+      <c r="B170" t="s">
+        <v>528</v>
+      </c>
+      <c r="C170" t="s">
+        <v>529</v>
+      </c>
+      <c r="D170" t="s">
+        <v>12</v>
+      </c>
+      <c r="E170" t="s">
+        <v>12</v>
+      </c>
+      <c r="F170" t="s">
+        <v>12</v>
+      </c>
+      <c r="G170" t="s">
+        <v>12</v>
+      </c>
+      <c r="H170" t="s">
+        <v>530</v>
+      </c>
+      <c r="I170" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="171" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A171">
+        <v>170</v>
+      </c>
+      <c r="B171" t="s">
+        <v>531</v>
+      </c>
+      <c r="C171" t="s">
+        <v>532</v>
+      </c>
+      <c r="D171" t="s">
+        <v>12</v>
+      </c>
+      <c r="E171" t="s">
+        <v>12</v>
+      </c>
+      <c r="F171" t="s">
+        <v>12</v>
+      </c>
+      <c r="G171" t="s">
+        <v>12</v>
+      </c>
+      <c r="H171" t="s">
+        <v>533</v>
+      </c>
+      <c r="I171" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="172" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A172">
+        <v>171</v>
+      </c>
+      <c r="B172" t="s">
+        <v>534</v>
+      </c>
+      <c r="C172" t="s">
+        <v>535</v>
+      </c>
+      <c r="D172" t="s">
+        <v>12</v>
+      </c>
+      <c r="E172" t="s">
+        <v>12</v>
+      </c>
+      <c r="F172" t="s">
+        <v>12</v>
+      </c>
+      <c r="G172" t="s">
+        <v>12</v>
+      </c>
+      <c r="H172" t="s">
+        <v>536</v>
+      </c>
+      <c r="I172" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="173" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A173">
+        <v>172</v>
+      </c>
+      <c r="B173" t="s">
+        <v>537</v>
+      </c>
+      <c r="C173" t="s">
+        <v>538</v>
+      </c>
+      <c r="D173" t="s">
+        <v>12</v>
+      </c>
+      <c r="E173" t="s">
+        <v>12</v>
+      </c>
+      <c r="F173" t="s">
+        <v>12</v>
+      </c>
+      <c r="G173" t="s">
+        <v>12</v>
+      </c>
+      <c r="H173" t="s">
+        <v>539</v>
+      </c>
+      <c r="I173" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="174" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A174">
+        <v>173</v>
+      </c>
+      <c r="B174" t="s">
+        <v>540</v>
+      </c>
+      <c r="C174" t="s">
+        <v>541</v>
+      </c>
+      <c r="D174" t="s">
+        <v>12</v>
+      </c>
+      <c r="E174" t="s">
+        <v>12</v>
+      </c>
+      <c r="F174" t="s">
+        <v>12</v>
+      </c>
+      <c r="G174" t="s">
+        <v>12</v>
+      </c>
+      <c r="H174" t="s">
+        <v>542</v>
+      </c>
+      <c r="I174" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="175" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A175">
+        <v>174</v>
+      </c>
+      <c r="B175" t="s">
+        <v>543</v>
+      </c>
+      <c r="C175" t="s">
+        <v>544</v>
+      </c>
+      <c r="D175" t="s">
+        <v>12</v>
+      </c>
+      <c r="E175" t="s">
+        <v>12</v>
+      </c>
+      <c r="F175" t="s">
+        <v>12</v>
+      </c>
+      <c r="G175" t="s">
+        <v>12</v>
+      </c>
+      <c r="H175" t="s">
+        <v>545</v>
+      </c>
+      <c r="I175" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="176" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A176">
+        <v>175</v>
+      </c>
+      <c r="B176" t="s">
+        <v>546</v>
+      </c>
+      <c r="C176" t="s">
+        <v>547</v>
+      </c>
+      <c r="D176" t="s">
+        <v>12</v>
+      </c>
+      <c r="E176" t="s">
+        <v>12</v>
+      </c>
+      <c r="F176" t="s">
+        <v>12</v>
+      </c>
+      <c r="G176" t="s">
+        <v>12</v>
+      </c>
+      <c r="H176" t="s">
+        <v>548</v>
+      </c>
+      <c r="I176" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="177" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A177">
+        <v>176</v>
+      </c>
+      <c r="B177" t="s">
+        <v>549</v>
+      </c>
+      <c r="C177" t="s">
+        <v>550</v>
+      </c>
+      <c r="D177" t="s">
+        <v>12</v>
+      </c>
+      <c r="E177" t="s">
+        <v>12</v>
+      </c>
+      <c r="F177" t="s">
+        <v>12</v>
+      </c>
+      <c r="G177" t="s">
+        <v>12</v>
+      </c>
+      <c r="H177" t="s">
+        <v>551</v>
+      </c>
+      <c r="I177" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="178" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A178">
+        <v>177</v>
+      </c>
+      <c r="B178" t="s">
+        <v>552</v>
+      </c>
+      <c r="C178" t="s">
+        <v>553</v>
+      </c>
+      <c r="D178" t="s">
+        <v>12</v>
+      </c>
+      <c r="E178" t="s">
+        <v>12</v>
+      </c>
+      <c r="F178" t="s">
+        <v>12</v>
+      </c>
+      <c r="G178" t="s">
+        <v>12</v>
+      </c>
+      <c r="H178" t="s">
+        <v>554</v>
+      </c>
+      <c r="I178" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="179" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A179">
+        <v>178</v>
+      </c>
+      <c r="B179" t="s">
+        <v>555</v>
+      </c>
+      <c r="C179" t="s">
+        <v>556</v>
+      </c>
+      <c r="D179" t="s">
+        <v>12</v>
+      </c>
+      <c r="E179" t="s">
+        <v>12</v>
+      </c>
+      <c r="F179" t="s">
+        <v>12</v>
+      </c>
+      <c r="G179" t="s">
+        <v>12</v>
+      </c>
+      <c r="H179" t="s">
+        <v>557</v>
+      </c>
+      <c r="I179" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="180" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A180">
+        <v>179</v>
+      </c>
+      <c r="B180" t="s">
+        <v>558</v>
+      </c>
+      <c r="C180" t="s">
+        <v>559</v>
+      </c>
+      <c r="D180" t="s">
+        <v>12</v>
+      </c>
+      <c r="E180" t="s">
+        <v>18</v>
+      </c>
+      <c r="F180" t="s">
+        <v>12</v>
+      </c>
+      <c r="G180" t="s">
+        <v>12</v>
+      </c>
+      <c r="H180" t="s">
+        <v>560</v>
+      </c>
+      <c r="I180" t="s">
+        <v>522</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H129" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>